<commit_message>
Add pinyin for Chinese names, addresses (153 suppliers)
</commit_message>
<xml_diff>
--- a/ipdf_suppliers.xlsx
+++ b/ipdf_suppliers.xlsx
@@ -505,7 +505,6 @@
           <t>amanda.pan@myc-production.com</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
           <t>No.99 Avenue of Wangjiang, Wangjiang County, Anqing City, Anhui Province, China.</t>
@@ -531,7 +530,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>刘金铃</t>
+          <t>刘金铃 (liú jīn líng)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -551,7 +550,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>江苏省吴江市 汾湖经济开发区临沪大道1999号, 215211No. 1999, Linhu Avenue, Fenhu Economic Development Zone, Wujiang City, Jiangsu Province, 215211</t>
+          <t>江苏省吴江市 (jiāng sū shěng wú jiāng shì) 汾湖经济开发区临沪大道 (fén hú jīng jì kāi fā qū lín hù dà dào)1999号 (hào), 215211No. 1999, Linhu Avenue, Fenhu Economic Development Zone, Wujiang City, Jiangsu Province, 215211</t>
         </is>
       </c>
       <c r="I3" t="n">
@@ -587,7 +586,6 @@
           <t>104872972@qq.com</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
           <t>No.4, 5 street, Nanling Gangpu Road, Baiyun district, Guangzhou city, Guangdong province, China</t>
@@ -613,7 +611,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>林显忠</t>
+          <t>林显忠 (lín xiǎn zhōng)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -633,7 +631,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>广州市白云区龙兴东南一横路3号No. 3, Longxing Southeast First Horizontal Road, Baiyun District, Guangzhou City</t>
+          <t>广州市白云区龙兴东南一横路 (guǎng zhōu shì bái yún qū lóng xīng dōng nán yī héng lù)3号 (hào)No. 3, Longxing Southeast First Horizontal Road, Baiyun District, Guangzhou City</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -646,7 +644,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>BOWEI博威</t>
+          <t>BOWEI博威 (bó wēi)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -656,7 +654,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>宋茜</t>
+          <t>宋茜 (sòng qiàn)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -664,7 +662,6 @@
           <t>19925699805</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
           <t>www.gzbowei.com</t>
@@ -672,7 +669,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>广州市花都区花东镇定邦空港产业园D栋Building D, Dingbang Airport Industrial Park, Huadong Town, Huadu District, Guangzhou</t>
+          <t>广州市花都区花东镇定邦空港产业园 (guǎng zhōu shì huā dōu qū huā dōng zhèn dìng bāng kōng gǎng chǎn yè yuán)D栋 (dòng)Building D, Dingbang Airport Industrial Park, Huadong Town, Huadu District, Guangzhou</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -715,7 +712,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>广东省开平市三埠街道新台路72号No. 72, Xintai Road, Sanbu Street, Kaiping City, Guangdong Province</t>
+          <t>广东省开平市三埠街道新台路 (guǎng dōng shěng kāi píng shì sān bù jiē dào xīn tái lù)72号 (hào)No. 72, Xintai Road, Sanbu Street, Kaiping City, Guangdong Province</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -738,7 +735,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>王耀峰</t>
+          <t>王耀峰 (wáng yào fēng)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -746,9 +743,6 @@
           <t>1380 7874 784</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
       <c r="I8" t="n">
         <v>2</v>
       </c>
@@ -769,7 +763,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>王媛媛</t>
+          <t>王媛媛 (wáng yuàn yuàn)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -789,7 +783,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>工厂广东省江门市新山市和情共建路305号座 公司地址:广州市白云区龙街尖路363号联边国际620单元Factory: Building 305, Heqing Gongjian Road, Xinshan City, Jiangmen City, Guangdong Province. Company Address: Unit 620, Lianbian International, No. 363, Longjie Jian Road, Baiyun District, Guangzhou</t>
+          <t>工厂广东省江门市新山市和情共建路 (gōng chǎng guǎng dōng shěng jiāng mén shì xīn shān shì hé qíng gòng jiàn lù)305号座 (hào zuò) 公司地址 (gōng sī dì zhǐ):广州市白云区龙街尖路 (guǎng zhōu shì bái yún qū lóng jiē jiān lù)363号联边国际 (hào lián biān guó jì)620单元 (dān yuán)Factory: Building 305, Heqing Gongjian Road, Xinshan City, Jiangmen City, Guangdong Province. Company Address: Unit 620, Lianbian International, No. 363, Longjie Jian Road, Baiyun District, Guangzhou</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -992,7 +986,6 @@
           <t>18126825966</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
           <t>https://feiming.1688.com</t>
@@ -1066,7 +1059,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Bella 陈丽霞</t>
+          <t>Bella 陈丽霞 (chén lì xiá)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1074,9 +1067,6 @@
           <t>+8618933938604</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
       <c r="I16" t="n">
         <v>3</v>
       </c>
@@ -1097,7 +1087,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>陈孔清</t>
+          <t>陈孔清 (chén kǒng qīng)</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1105,9 +1095,6 @@
           <t>400-008-9919, 13501547854</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
       <c r="I17" t="n">
         <v>2</v>
       </c>
@@ -1136,11 +1123,9 @@
           <t>13710501630</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr">
         <is>
-          <t>广东省广州市花都区秀全街道大布路29号峰华工业园Fenghua Industrial Park, No. 29 Dabu Road, Xiuquan Street, Huadu District, Guangzhou City, Guangdong Province</t>
+          <t>广东省广州市花都区秀全街道大布路 (guǎng dōng shěng guǎng zhōu shì huā dōu qū xiù quán jiē dào dà bù lù)29号峰华工业园 (hào fēng huá gōng yè yuán)Fenghua Industrial Park, No. 29 Dabu Road, Xiuquan Street, Huadu District, Guangzhou City, Guangdong Province</t>
         </is>
       </c>
       <c r="I18" t="n">
@@ -1163,7 +1148,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>胡明</t>
+          <t>胡明 (hú míng)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1171,11 +1156,9 @@
           <t>13570062455</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr">
         <is>
-          <t>广东省清远英德市英红镇万洋众创城D区37栋Building 37, Zone D, Wanyang Maker Town, Yinghong Town, Yingde City, Qingyuan City, Guangdong Province</t>
+          <t>广东省清远英德市英红镇万洋众创城 (guǎng dōng shěng qīng yuǎn yīng dé shì yīng hóng zhèn wàn yáng zhòng chuàng chéng)D区 (qū)37栋 (dòng)Building 37, Zone D, Wanyang Maker Town, Yinghong Town, Yingde City, Qingyuan City, Guangdong Province</t>
         </is>
       </c>
       <c r="I19" t="n">
@@ -1254,7 +1237,6 @@
           <t>lh1462836142@gmail.com</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr">
         <is>
           <t>42 floor, R &amp; F Dongshan New World Building, No.307 Guangzhou dadao zhong, Tianhe District, Guangzhou</t>
@@ -1280,7 +1262,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>谭玉雄</t>
+          <t>谭玉雄 (tán yù xióng)</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1300,7 +1282,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>广东省东莞市谢岗镇曹乐向阳路55号, 广东省东莞市樟木头镇塑料市场一期V栋1-2号, 广东省东莞市常平镇大京九塑料市场塑发东路53-54号No. 55, Caole Xiangyang Road, Xiegang Town, Dongguan City, Guangdong Province, Building V, Units 1-2, Phase 1, Plastic Market, Zhangmutou Town, Dongguan City, Guangdong Province, No. 53-54, Sufa East Road, Dajingjiu Plastic Market, Changping Town, Dongguan City, Guangdong Province</t>
+          <t>广东省东莞市谢岗镇曹乐向阳路 (guǎng dōng shěng dōng guǎn shì xiè gǎng zhèn cáo lè xiàng yáng lù)55号 (hào), 广东省东莞市樟木头镇塑料市场一期 (guǎng dōng shěng dōng guǎn shì zhāng mù tou zhèn sù liào shì chǎng yī qī)V栋 (dòng)1-2号 (hào), 广东省东莞市常平镇大京九塑料市场塑发东路 (guǎng dōng shěng dōng guǎn shì cháng píng zhèn dà jīng jiǔ sù liào shì chǎng sù fā dōng lù)53-54号 (hào)No. 55, Caole Xiangyang Road, Xiegang Town, Dongguan City, Guangdong Province, Building V, Units 1-2, Phase 1, Plastic Market, Zhangmutou Town, Dongguan City, Guangdong Province, No. 53-54, Sufa East Road, Dajingjiu Plastic Market, Changping Town, Dongguan City, Guangdong Province</t>
         </is>
       </c>
       <c r="I22" t="n">
@@ -1364,14 +1346,11 @@
           <t>Косметика и уход</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
           <t>020-83273747, 020-31523293</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr">
         <is>
           <t>Guangzhou City, Yuexiu District, Guangyuan West Road No. 121, Commercial Center C, 3rd Floor, Room 022, Guangzhou City, Baiyun District, Zhongluotan Town, Liantian North Road No. 9, Building 6, Chenmei Industrial Park</t>
@@ -1405,8 +1384,6 @@
           <t>15347449477</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr">
         <is>
           <t>Office | 4th Floor, 4024 Booth, Meiwan Square, Baiyun District, Guangzhou City, Guangdong Province</t>
@@ -1432,7 +1409,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>陈总</t>
+          <t>陈总 (chén zǒng)</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1440,11 +1417,9 @@
           <t>136-1010-8089, 135-3316-5675</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr">
         <is>
-          <t>广州市花都区先科一路金禾云创产业园Jinhe Yun Chuang Industrial Park, Xianke 1st Road, Huadu District, Guangzhou City</t>
+          <t>广州市花都区先科一路金禾云创产业园 (guǎng zhōu shì huā dōu qū xiān kē yī lù jīn hé yún chuàng chǎn yè yuán)Jinhe Yun Chuang Industrial Park, Xianke 1st Road, Huadu District, Guangzhou City</t>
         </is>
       </c>
       <c r="I26" t="n">
@@ -1480,10 +1455,9 @@
           <t>3031739800@qq.com</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr">
         <is>
-          <t>广州市越秀区先烈中路85号浙江大厦9楼9th Floor, Zhejiang Building, No. 85, Xianlie Middle Road, Yuexiu District, Guangzhou City</t>
+          <t>广州市越秀区先烈中路 (guǎng zhōu shì yuè xiù qū xiān liè zhōng lù)85号浙江大厦 (hào zhè jiāng dà shà)9楼 (lóu)9th Floor, Zhejiang Building, No. 85, Xianlie Middle Road, Yuexiu District, Guangzhou City</t>
         </is>
       </c>
       <c r="I27" t="n">
@@ -1506,7 +1480,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>吴月芳</t>
+          <t>吴月芳 (wú yuè fāng)</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1519,7 +1493,6 @@
           <t>2724754493@qq.com</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr">
         <is>
           <t>No. 339, Hengjiang Road, Conghua District, Guangzhou</t>
@@ -1631,7 +1604,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>陈泳</t>
+          <t>陈泳 (chén yǒng)</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1639,11 +1612,9 @@
           <t>+86 184 7567 6856, 020-36738536, 020-36739102</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr">
         <is>
-          <t>广州市白云区均禾街清湖村大山路6号No. 6, Dashan Road, Qinghu Village, Junhe Street, Baiyun District, Guangzhou City</t>
+          <t>广州市白云区均禾街清湖村大山路 (guǎng zhōu shì bái yún qū jūn hé jiē qīng hú cūn dà shān lù)6号 (hào)No. 6, Dashan Road, Qinghu Village, Junhe Street, Baiyun District, Guangzhou City</t>
         </is>
       </c>
       <c r="I31" t="n">
@@ -1709,7 +1680,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>赖梓浩</t>
+          <t>赖梓浩 (lài zǐ hào)</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1752,7 +1723,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>刘金连</t>
+          <t>刘金连 (liú jīn lián)</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -1760,13 +1731,11 @@
           <t>137 1082 1278</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr">
         <is>
           <t>https://202206.1688.com/</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr"/>
       <c r="I34" t="n">
         <v>2</v>
       </c>
@@ -1787,7 +1756,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>赵新亮</t>
+          <t>赵新亮 (zhào xīn liàng)</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1795,11 +1764,9 @@
           <t>176 7577 8864</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr"/>
-      <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr">
         <is>
-          <t>广州市白云区北村北大路22号四栋二楼Second Floor, Building 4, No. 22, Beicun Beida Road, Baiyun District, Guangzhou City</t>
+          <t>广州市白云区北村北大路 (guǎng zhōu shì bái yún qū běi cūn běi dà lù)22号四栋二楼 (hào sì dòng èr lóu)Second Floor, Building 4, No. 22, Beicun Beida Road, Baiyun District, Guangzhou City</t>
         </is>
       </c>
       <c r="I35" t="n">
@@ -1840,7 +1807,6 @@
           <t>www.qfpackage.com</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr"/>
       <c r="I36" t="n">
         <v>7</v>
       </c>
@@ -1950,7 +1916,6 @@
           <t>Dora Wong</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr"/>
       <c r="F39" t="inlineStr">
         <is>
           <t>dora.wong@simplerpackaging.com</t>
@@ -1961,7 +1926,6 @@
           <t>www.simplerpackaging.com</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr"/>
       <c r="I39" t="n">
         <v>1</v>
       </c>
@@ -1995,7 +1959,6 @@
           <t>603274975@qq.com</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr">
         <is>
           <t>Room 905/906/907, Building 2, Yuntuhui, No. 239, Yuncheng South Fourth Road, Baiyun District, Guangzhou</t>
@@ -2029,8 +1992,6 @@
           <t>15918480262, 3005008294</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr"/>
-      <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr">
         <is>
           <t>No. 2 Yinlan West Road, Xiejiazhuang, Taihe Town, Baiyun District, Guangzhou City</t>
@@ -2102,14 +2063,11 @@
           <t>Steven Lu</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr"/>
       <c r="F43" t="inlineStr">
         <is>
           <t>steven@yusupackaging.com</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr"/>
-      <c r="H43" t="inlineStr"/>
       <c r="I43" t="n">
         <v>1</v>
       </c>
@@ -2133,14 +2091,11 @@
           <t>David Ma</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr"/>
       <c r="F44" t="inlineStr">
         <is>
           <t>david@yutopackaging.com</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr"/>
-      <c r="H44" t="inlineStr"/>
       <c r="I44" t="n">
         <v>1</v>
       </c>
@@ -2174,7 +2129,6 @@
           <t>service003@gzzxplastic.com</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr"/>
       <c r="H45" t="inlineStr">
         <is>
           <t>No.78-1 Kaiyuan Road, Datang Town, Sanshui District, Foshan City, Guangdong Province, China</t>
@@ -2213,7 +2167,6 @@
           <t>jackey@zycosmeticmfg.com</t>
         </is>
       </c>
-      <c r="G46" t="inlineStr"/>
       <c r="H46" t="inlineStr">
         <is>
           <t>No. 15 Liangyuan Erheng Road, Zhonglustan Town, Baiyun District, Guangzhou, Guangdong Province, P.R. China</t>
@@ -2239,7 +2192,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>曹春</t>
+          <t>曹春 (cáo chūn)</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -2247,11 +2200,9 @@
           <t>13719223622</t>
         </is>
       </c>
-      <c r="F47" t="inlineStr"/>
-      <c r="G47" t="inlineStr"/>
       <c r="H47" t="inlineStr">
         <is>
-          <t>广州市白云区石井街石井大道634号No. 634, Shijing Avenue, Shijing Street, Baiyun District, Guangzhou City</t>
+          <t>广州市白云区石井街石井大道 (guǎng zhōu shì bái yún qū shí jǐng jiē shí jǐng dà dào)634号 (hào)No. 634, Shijing Avenue, Shijing Street, Baiyun District, Guangzhou City</t>
         </is>
       </c>
       <c r="I47" t="n">
@@ -2294,7 +2245,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>上海市浦东新区世纪大道100号No. 100, Century Avenue, Pudong New Area, Shanghai</t>
+          <t>上海市浦东新区世纪大道 (shàng hǎi shì pǔ dōng xīn qū shì jì dà dào)100号 (hào)No. 100, Century Avenue, Pudong New Area, Shanghai</t>
         </is>
       </c>
       <c r="I48" t="n">
@@ -2317,7 +2268,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>章海翰</t>
+          <t>章海翰 (zhāng hǎi hàn)</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2330,7 +2281,6 @@
           <t>88553355@qq.com</t>
         </is>
       </c>
-      <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr">
         <is>
           <t>Industrial Area No.3, Xiaqi Road and Hudi Road, Jinping District, Shantou city, Guangdong Province, China.</t>
@@ -2412,7 +2362,6 @@
           <t>henryxie@hontaipack.com</t>
         </is>
       </c>
-      <c r="G51" t="inlineStr"/>
       <c r="H51" t="inlineStr">
         <is>
           <t>No.191, Hudi Road, Shantou, Guangdong, China</t>
@@ -2458,7 +2407,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>上海市奉贤区大叶公路 6818号5A栋502Room 502, Building 5A, No. 6818, Daye Highway, Fengxian District, Shanghai City</t>
+          <t>上海市奉贤区大叶公路 (shàng hǎi shì fèng xián qū dà yè gōng lù) 6818号 (hào)5A栋 (dòng)502Room 502, Building 5A, No. 6818, Daye Highway, Fengxian District, Shanghai City</t>
         </is>
       </c>
       <c r="I52" t="n">
@@ -2481,7 +2430,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>陈雪萍</t>
+          <t>陈雪萍 (chén xuě píng)</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -2501,7 +2450,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>广东省惠州市博罗县石湾镇马石围路3号No. 3, Mashiwei Road, Shiwan Town, Boluo County, Huizhou City, Guangdong Province</t>
+          <t>广东省惠州市博罗县石湾镇马石围路 (guǎng dōng shěng huì zhōu shì bó luó xiàn shí wān zhèn mǎ shí wéi lù)3号 (hào)No. 3, Mashiwei Road, Shiwan Town, Boluo County, Huizhou City, Guangdong Province</t>
         </is>
       </c>
       <c r="I53" t="n">
@@ -2514,7 +2463,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>iGAO 丽高包装</t>
+          <t>iGAO 丽高包装 (lì gāo bāo zhuāng)</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2524,7 +2473,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>何丽银</t>
+          <t>何丽银 (hé lì yín)</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -2544,7 +2493,7 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>广东省清远市清城区石角镇广清产业园广创街6号No. 6, Guangchuang Street, Guangqing Industrial Park, Shijiao Town, Qingcheng District, Qingyuan City, Guangdong Province</t>
+          <t>广东省清远市清城区石角镇广清产业园广创街 (guǎng dōng shěng qīng yuǎn shì qīng chéng qū shí jiǎo zhèn guǎng qīng chǎn yè yuán guǎng chuàng jiē)6号 (hào)No. 6, Guangchuang Street, Guangqing Industrial Park, Shijiao Town, Qingcheng District, Qingyuan City, Guangdong Province</t>
         </is>
       </c>
       <c r="I54" t="n">
@@ -2567,7 +2516,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>冉露茜</t>
+          <t>冉露茜 (rǎn lù qiàn)</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -2587,7 +2536,7 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>黄浦区德必上海书城WE2101室Room WE2101, Debao Shanghai Book City, Huangpu District</t>
+          <t>黄浦区德必上海书城 (huáng pǔ qū dé bì shàng hǎi shū chéng)WE2101室 (shì)Room WE2101, Debao Shanghai Book City, Huangpu District</t>
         </is>
       </c>
       <c r="I55" t="n">
@@ -2623,10 +2572,9 @@
           <t>qiao.li@tensoar.com.cn</t>
         </is>
       </c>
-      <c r="G56" t="inlineStr"/>
       <c r="H56" t="inlineStr">
         <is>
-          <t>浙江省嘉兴市南湖区新丰镇新禾路158号No. 158, Xinhe Road, Xinfeng Town, Nanhu District, Jiaxing City, Zhejiang Province</t>
+          <t>浙江省嘉兴市南湖区新丰镇新禾路 (zhè jiāng shěng jiā xīng shì nán hú qū xīn fēng zhèn xīn hé lù)158号 (hào)No. 158, Xinhe Road, Xinfeng Town, Nanhu District, Jiaxing City, Zhejiang Province</t>
         </is>
       </c>
       <c r="I56" t="n">
@@ -2662,7 +2610,6 @@
           <t>19128957848@139.com</t>
         </is>
       </c>
-      <c r="G57" t="inlineStr"/>
       <c r="H57" t="inlineStr">
         <is>
           <t>No. 102, Qilongjie, Wulonggang, Zhongluotan Town, Baiyun District, Guangzhou, Guangdong Province China</t>
@@ -2731,7 +2678,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>陈铁文</t>
+          <t>陈铁文 (chén tiě wén)</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -2744,10 +2691,9 @@
           <t>chentiewen@kaidapack.com</t>
         </is>
       </c>
-      <c r="G59" t="inlineStr"/>
       <c r="H59" t="inlineStr">
         <is>
-          <t>福建省晋江市经济开发区 广东省深圳市龙华新区建设路与东环二路交汇处聚豪国际A栋2504室Room 2504, Building A, Juhuao International, Intersection of Jianshe Road and Donghuan 2nd Road, Longhua New District, Shenzhen City, Guangdong Province; Jinjiang Economic Development Zone, Jinjiang City, Fujian Province</t>
+          <t>福建省晋江市经济开发区 (fú jiàn shěng jìn jiāng shì jīng jì kāi fā qū) 广东省深圳市龙华新区建设路与东环二路交汇处聚豪国际 (guǎng dōng shěng shēn zhèn shì lóng huá xīn qū jiàn shè lù yǔ dōng huán èr lù jiāo huì chù jù háo guó jì)A栋 (dòng)2504室 (shì)Room 2504, Building A, Juhuao International, Intersection of Jianshe Road and Donghuan 2nd Road, Longhua New District, Shenzhen City, Guangdong Province; Jinjiang Economic Development Zone, Jinjiang City, Fujian Province</t>
         </is>
       </c>
       <c r="I59" t="n">
@@ -2813,7 +2759,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>周 亮</t>
+          <t>周 (zhōu) 亮 (liàng)</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -2831,7 +2777,6 @@
           <t>www.kingswin.com</t>
         </is>
       </c>
-      <c r="H61" t="inlineStr"/>
       <c r="I61" t="n">
         <v>1</v>
       </c>
@@ -2893,13 +2838,11 @@
           <t>Продукты на заказ / OEM</t>
         </is>
       </c>
-      <c r="D63" t="inlineStr"/>
       <c r="E63" t="inlineStr">
         <is>
           <t>17765635626</t>
         </is>
       </c>
-      <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr">
         <is>
           <t>www.mayacompany.com</t>
@@ -2943,8 +2886,6 @@
           <t>hyde@merrynewon.com</t>
         </is>
       </c>
-      <c r="G64" t="inlineStr"/>
-      <c r="H64" t="inlineStr"/>
       <c r="I64" t="n">
         <v>2</v>
       </c>
@@ -3064,10 +3005,9 @@
           <t>icy.ye@guangzhouhanjiang.com</t>
         </is>
       </c>
-      <c r="G67" t="inlineStr"/>
       <c r="H67" t="inlineStr">
         <is>
-          <t>广州市天河区林和东路285号中汇人寿901Room 901, Zhonghui Life Insurance, No. 285 Linhe East Road, Tianhe District, Guangzhou City</t>
+          <t>广州市天河区林和东路 (guǎng zhōu shì tiān hé qū lín hé dōng lù)285号中汇人寿 (hào zhōng huì rén shòu)901Room 901, Zhonghui Life Insurance, No. 285 Linhe East Road, Tianhe District, Guangzhou City</t>
         </is>
       </c>
       <c r="I67" t="n">
@@ -3090,7 +3030,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>李金花</t>
+          <t>李金花 (lǐ jīn huā)</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -3153,7 +3093,7 @@
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>广州市白云区鶴拳路一横路科我园3栋Building 3, Kewoyuan, Yiheng Road, Hequan Road, Baiyun District, Guangzhou City</t>
+          <t>广州市白云区鶴拳路一横路科我园 (guǎng zhōu shì bái yún qū hè quán lù yī héng lù kē wǒ yuán)3栋 (dòng)Building 3, Kewoyuan, Yiheng Road, Hequan Road, Baiyun District, Guangzhou City</t>
         </is>
       </c>
       <c r="I69" t="n">
@@ -3189,7 +3129,6 @@
           <t>jeff@gzqiyu.com</t>
         </is>
       </c>
-      <c r="G70" t="inlineStr"/>
       <c r="H70" t="inlineStr">
         <is>
           <t>No.107, Guanglong Road, Zhongluotan, Baiyun District, Guangzhou,China</t>
@@ -3309,8 +3248,6 @@
           <t>86-15017235618, 0754-83616788</t>
         </is>
       </c>
-      <c r="F73" t="inlineStr"/>
-      <c r="G73" t="inlineStr"/>
       <c r="H73" t="inlineStr">
         <is>
           <t>No. 1 Zizhong Road, Heping Town, Chaoyang District, Shantou515141, Guangdong, China</t>
@@ -3336,7 +3273,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Cécilia 叶思颖</t>
+          <t>Cécilia 叶思颖 (yè sī yǐng)</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -3392,7 +3329,6 @@
           <t>906845206@qq.com</t>
         </is>
       </c>
-      <c r="G75" t="inlineStr"/>
       <c r="H75" t="inlineStr">
         <is>
           <t>Floor 4, Building C, Shengmeng Industrial Park, No.70 Xiangxia Avenue, Longgui, Taihe Town, Baiyun District, Guangzhou, China</t>
@@ -3431,7 +3367,6 @@
           <t>hong46647426@gmail.com, 1154315619@qq.com</t>
         </is>
       </c>
-      <c r="G76" t="inlineStr"/>
       <c r="H76" t="inlineStr">
         <is>
           <t>Building F, North of Nan 'ao Road, Jinping District, Shantou City, Guangdong Province</t>
@@ -3457,7 +3392,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>洪碧虹</t>
+          <t>洪碧虹 (hóng bì hóng)</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -3470,10 +3405,9 @@
           <t>sale@lichaipk.com</t>
         </is>
       </c>
-      <c r="G77" t="inlineStr"/>
       <c r="H77" t="inlineStr">
         <is>
-          <t>汕头市金平区岐山街道中宫社区建明工业城11-12栋楼Buildings 11-12, Jianming Industrial City, Zhonggong Community, Qishan Street, Jinping District, Shantou City</t>
+          <t>汕头市金平区岐山街道中宫社区建明工业城 (shàn tóu shì jīn píng qū qí shān jiē dào zhōng gōng shè qū jiàn míng gōng yè chéng)11-12栋楼 (dòng lóu)Buildings 11-12, Jianming Industrial City, Zhonggong Community, Qishan Street, Jinping District, Shantou City</t>
         </is>
       </c>
       <c r="I77" t="n">
@@ -3552,7 +3486,6 @@
           <t>sales2@strongguang.com</t>
         </is>
       </c>
-      <c r="G79" t="inlineStr"/>
       <c r="H79" t="inlineStr">
         <is>
           <t>No.1 Zizhong Road, Heping Town, Chaoyang District, Shantou 515141, Guangdong, China</t>
@@ -3707,7 +3640,7 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>何燕芳 Orla</t>
+          <t>何燕芳 (hé yàn fāng) Orla</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -3725,7 +3658,6 @@
           <t>https://www.yastarplastic.com</t>
         </is>
       </c>
-      <c r="H83" t="inlineStr"/>
       <c r="I83" t="n">
         <v>1</v>
       </c>
@@ -3746,7 +3678,7 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>陈乐</t>
+          <t>陈乐 (chén lè)</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -3766,7 +3698,7 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>广州市赛康尼机械设备有限公司 广州市黄埔区南岗街道中南街10号联系中心办公室楼南面主楼南面Guangzhou Saikenni Machinery Equipment Co., Ltd. South side of the main building, south side of the Contact Center Office Building, No. 10, Zhongnan Street, Nangang Subdistrict, Huangpu District, Guangzhou</t>
+          <t>广州市赛康尼机械设备有限公司 (guǎng zhōu shì sài kāng ní jī xiè shè bèi yǒu xiàn gōng sī) 广州市黄埔区南岗街道中南街 (guǎng zhōu shì huáng pǔ qū nán gǎng jiē dào zhōng nán jiē)10号联系中心办公室楼南面主楼南面 (hào lián xì zhōng xīn bàn gōng shì lóu nán miàn zhǔ lóu nán miàn)Guangzhou Saikenni Machinery Equipment Co., Ltd. South side of the main building, south side of the Contact Center Office Building, No. 10, Zhongnan Street, Nangang Subdistrict, Huangpu District, Guangzhou</t>
         </is>
       </c>
       <c r="I84" t="n">
@@ -3789,7 +3721,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>鲍焕威 Bao huan wei</t>
+          <t>鲍焕威 (bào huàn wēi) Bao huan wei</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -3802,7 +3734,6 @@
           <t>289080492@qq.com</t>
         </is>
       </c>
-      <c r="G85" t="inlineStr"/>
       <c r="H85" t="inlineStr">
         <is>
           <t>Room 301, Building 6, 5th Indurstrial Park, Tianliao Community, Gongming Street, Guangming District, Shenzhen City, Guangdong Province, China</t>
@@ -3828,7 +3759,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>黄顺好</t>
+          <t>黄顺好 (huáng shùn hǎo)</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
@@ -3848,7 +3779,7 @@
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>广东佛山市顺德区伦教来涌工业区Laiyong Industrial Zone, Lunqiao, Shunde District, Foshan City, Guangdong</t>
+          <t>广东佛山市顺德区伦教来涌工业区 (guǎng dōng fó shān shì shùn dé qū lún jiào lái yǒng gōng yè qū)Laiyong Industrial Zone, Lunqiao, Shunde District, Foshan City, Guangdong</t>
         </is>
       </c>
       <c r="I86" t="n">
@@ -3871,7 +3802,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>邵仕华</t>
+          <t>邵仕华 (shào shì huá)</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
@@ -3889,7 +3820,6 @@
           <t>http://www.suicel.com</t>
         </is>
       </c>
-      <c r="H87" t="inlineStr"/>
       <c r="I87" t="n">
         <v>1</v>
       </c>
@@ -3910,7 +3840,7 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>陈晓雯</t>
+          <t>陈晓雯 (chén xiǎo wén)</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
@@ -3923,10 +3853,9 @@
           <t>mandy.c@gzsummitek.com</t>
         </is>
       </c>
-      <c r="G88" t="inlineStr"/>
       <c r="H88" t="inlineStr">
         <is>
-          <t>广东省清远市清城区石角镇(广清产业园)兴园路3号; 广州市花都区新雅街绿地空港五号地4栋1107室No. 3, Xingyuan Road, Shijiao Town (Guangqing Industrial Park), Qingcheng District, Qingyuan City, Guangdong Province; Room 1107, Building 4, Plot 5, Greenland Airport, Xinya Street, Huadu District, Guangzhou City</t>
+          <t>广东省清远市清城区石角镇 (guǎng dōng shěng qīng yuǎn shì qīng chéng qū shí jiǎo zhèn)(广清产业园 (guǎng qīng chǎn yè yuán))兴园路 (xīng yuán lù)3号 (hào); 广州市花都区新雅街绿地空港五号地 (guǎng zhōu shì huā dōu qū xīn yǎ jiē lǜ dì kōng gǎng wǔ hào dì)4栋 (dòng)1107室 (shì)No. 3, Xingyuan Road, Shijiao Town (Guangqing Industrial Park), Qingcheng District, Qingyuan City, Guangdong Province; Room 1107, Building 4, Plot 5, Greenland Airport, Xinya Street, Huadu District, Guangzhou City</t>
         </is>
       </c>
       <c r="I88" t="n">
@@ -3962,8 +3891,6 @@
           <t>GraceCheng@taolinpack.com</t>
         </is>
       </c>
-      <c r="G89" t="inlineStr"/>
-      <c r="H89" t="inlineStr"/>
       <c r="I89" t="n">
         <v>1</v>
       </c>
@@ -3984,7 +3911,7 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>徐春苗 Kavi</t>
+          <t>徐春苗 (xú chūn miáo) Kavi</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
@@ -3997,10 +3924,9 @@
           <t>chunmiao.xu@tensoar.com.cn</t>
         </is>
       </c>
-      <c r="G90" t="inlineStr"/>
       <c r="H90" t="inlineStr">
         <is>
-          <t>浙江省嘉兴市南湖区新丰镇新禾路158号No. 158, Xinhe Road, Xinfeng Town, Nanhu District, Jiaxing City, Zhejiang Province</t>
+          <t>浙江省嘉兴市南湖区新丰镇新禾路 (zhè jiāng shěng jiā xīng shì nán hú qū xīn fēng zhèn xīn hé lù)158号 (hào)No. 158, Xinhe Road, Xinfeng Town, Nanhu District, Jiaxing City, Zhejiang Province</t>
         </is>
       </c>
       <c r="I90" t="n">
@@ -4043,7 +3969,7 @@
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>江苏省泰兴市江平北路55号, 上海市徐汇区石龙路6号001室No. 55 Jiangping North Road, Taixing City, Jiangsu Province, Room 001, No. 6 Shilong Road, Xuhui District, Shanghai City</t>
+          <t>江苏省泰兴市江平北路 (jiāng sū shěng tài xīng shì jiāng píng běi lù)55号 (hào), 上海市徐汇区石龙路 (shàng hǎi shì xú huì qū shí lóng lù)6号 (hào)001室 (shì)No. 55 Jiangping North Road, Taixing City, Jiangsu Province, Room 001, No. 6 Shilong Road, Xuhui District, Shanghai City</t>
         </is>
       </c>
       <c r="I91" t="n">
@@ -4127,7 +4053,6 @@
           <t>www.tubest-packing.com</t>
         </is>
       </c>
-      <c r="H93" t="inlineStr"/>
       <c r="I93" t="n">
         <v>5</v>
       </c>
@@ -4148,7 +4073,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>翁铄桓</t>
+          <t>翁铄桓 (wēng shuò huán)</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
@@ -4161,10 +4086,9 @@
           <t>wengsh@unionwins.com.cn</t>
         </is>
       </c>
-      <c r="G94" t="inlineStr"/>
       <c r="H94" t="inlineStr">
         <is>
-          <t>佛山市三水区乐平镇博裕路34号1栋Building 1, No. 34, Boyu Road, Leping Town, Sanshui District, Foshan City</t>
+          <t>佛山市三水区乐平镇博裕路 (fó shān shì sān shuǐ qū lè píng zhèn bó yù lù)34号 (hào)1栋 (dòng)Building 1, No. 34, Boyu Road, Leping Town, Sanshui District, Foshan City</t>
         </is>
       </c>
       <c r="I94" t="n">
@@ -4187,7 +4111,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>顾友阳</t>
+          <t>顾友阳 (gù yǒu yáng)</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -4200,10 +4124,9 @@
           <t>aaron.gu@ronao.cn</t>
         </is>
       </c>
-      <c r="G95" t="inlineStr"/>
       <c r="H95" t="inlineStr">
         <is>
-          <t>上海市金山区漕泾开发区展业路288号一栋Building 1, No. 288, Zhanye Road, Caojing Development Zone, Jinshan District, Shanghai</t>
+          <t>上海市金山区漕泾开发区展业路 (shàng hǎi shì jīn shān qū cáo jīng kāi fā qū zhǎn yè lù)288号一栋 (hào yī dòng)Building 1, No. 288, Zhanye Road, Caojing Development Zone, Jinshan District, Shanghai</t>
         </is>
       </c>
       <c r="I95" t="n">
@@ -4224,19 +4147,16 @@
           <t>Упаковочные материалы и аксессуары, Дизайн и брендинг</t>
         </is>
       </c>
-      <c r="D96" t="inlineStr"/>
       <c r="E96" t="inlineStr">
         <is>
           <t>18830805081</t>
         </is>
       </c>
-      <c r="F96" t="inlineStr"/>
       <c r="G96" t="inlineStr">
         <is>
           <t>hongsheng1688.com</t>
         </is>
       </c>
-      <c r="H96" t="inlineStr"/>
       <c r="I96" t="n">
         <v>1</v>
       </c>
@@ -4343,7 +4263,7 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>林晓荣</t>
+          <t>林晓荣 (lín xiǎo róng)</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
@@ -4363,7 +4283,7 @@
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>广东省汕头市月浦龙洲路12号 Longzhou Road, Yuepu, Shantou City, Guangdong Province, China</t>
+          <t>广东省汕头市月浦龙洲路 (guǎng dōng shěng shàn tóu shì yuè pǔ lóng zhōu lù)12号 (hào) Longzhou Road, Yuepu, Shantou City, Guangdong Province, China</t>
         </is>
       </c>
       <c r="I99" t="n">
@@ -4386,7 +4306,7 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>谢榕宝</t>
+          <t>谢榕宝 (xiè róng bǎo)</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
@@ -4406,7 +4326,7 @@
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>广州市七星二号No. 2, Qixing, Guangzhou City</t>
+          <t>广州市七星二号 (guǎng zhōu shì qī xīng èr hào)No. 2, Qixing, Guangzhou City</t>
         </is>
       </c>
       <c r="I100" t="n">
@@ -4427,7 +4347,6 @@
           <t>Упаковочные материалы и аксессуары, Текстиль и нетканые материалы, Продукты на заказ / OEM</t>
         </is>
       </c>
-      <c r="D101" t="inlineStr"/>
       <c r="E101" t="inlineStr">
         <is>
           <t>021-62363736, 63287808, 189 1831 9995</t>
@@ -4445,7 +4364,7 @@
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>上海市嘉定区树屏路588弄财智金岸35号楼Building 35, Caizhi Jin'an, Lane 588, Shuping Road, Jiading District, Shanghai</t>
+          <t>上海市嘉定区树屏路 (shàng hǎi shì jiā dìng qū shù píng lù)588弄财智金岸 (nòng cái zhì jīn àn)35号楼 (hào lóu)Building 35, Caizhi Jin'an, Lane 588, Shuping Road, Jiading District, Shanghai</t>
         </is>
       </c>
       <c r="I101" t="n">
@@ -4524,7 +4443,6 @@
           <t>zettoruan@gmail.com</t>
         </is>
       </c>
-      <c r="G103" t="inlineStr"/>
       <c r="H103" t="inlineStr">
         <is>
           <t>Building 31, No.86, Maohai Road, Huangjiabu Town, Yuyao City, Zhejiang Province.</t>
@@ -4593,7 +4511,7 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>苏元元</t>
+          <t>苏元元 (sū yuán yuán)</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
@@ -4613,7 +4531,7 @@
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>浙江省绍兴市上虞区崧厦街道振兴路138号No. 138, Zhenxing Road, Songsha Street, Shangyu District, Shaoxing City, Zhejiang Province</t>
+          <t>浙江省绍兴市上虞区崧厦街道振兴路 (zhè jiāng shěng shào xīng shì shàng yú qū sōng shà jiē dào zhèn xīng lù)138号 (hào)No. 138, Zhenxing Road, Songsha Street, Shangyu District, Shaoxing City, Zhejiang Province</t>
         </is>
       </c>
       <c r="I105" t="n">
@@ -4636,7 +4554,7 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>刘艳霞</t>
+          <t>刘艳霞 (liú yàn xiá)</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
@@ -4644,9 +4562,6 @@
           <t>13515733610</t>
         </is>
       </c>
-      <c r="F106" t="inlineStr"/>
-      <c r="G106" t="inlineStr"/>
-      <c r="H106" t="inlineStr"/>
       <c r="I106" t="n">
         <v>1</v>
       </c>
@@ -4723,7 +4638,6 @@
           <t>nessani@foxmail.com</t>
         </is>
       </c>
-      <c r="G108" t="inlineStr"/>
       <c r="H108" t="inlineStr">
         <is>
           <t>Building NO.1, Wanyang creation city, NO.68 Maohai Road, Huangjiabu Town, Yuyao city, Ningbo, Zhejiang Province, China</t>
@@ -4749,7 +4663,7 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>张亮亮</t>
+          <t>张亮亮 (zhāng liàng liàng)</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
@@ -4762,7 +4676,6 @@
           <t>zhangliangliang@jusu-china.com</t>
         </is>
       </c>
-      <c r="G109" t="inlineStr"/>
       <c r="H109" t="inlineStr">
         <is>
           <t>No. 10, Xingye West Road, Xinxu Village, Sanxiang Town, Zhongshan City, Guangdong China</t>
@@ -4778,7 +4691,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>上海美涂化工科技有限公司 Shanghai Meitu Chemical Technology Co., Ltd.</t>
+          <t>上海美涂化工科技有限公司 (shàng hǎi měi tú huà gōng kē jì yǒu xiàn gōng sī) Shanghai Meitu Chemical Technology Co., Ltd.</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -4788,7 +4701,7 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>肖志坚</t>
+          <t>肖志坚 (xiào zhì jiān)</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
@@ -4801,10 +4714,9 @@
           <t>gf@mtchem.com</t>
         </is>
       </c>
-      <c r="G110" t="inlineStr"/>
       <c r="H110" t="inlineStr">
         <is>
-          <t>上海市松江区叶路133弄1-3号No. 1-3, Lane 133, Ye Road, Songjiang District, Shanghai</t>
+          <t>上海市松江区叶路 (shàng hǎi shì sōng jiāng qū yè lù)133弄 (nòng)1-3号 (hào)No. 1-3, Lane 133, Ye Road, Songjiang District, Shanghai</t>
         </is>
       </c>
       <c r="I110" t="n">
@@ -4817,7 +4729,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>东京品新材料科技有限公司 Tokyo Pin New Material Technology Co., Ltd.</t>
+          <t>东京品新材料科技有限公司 (dōng jīng pǐn xīn cái liào kē jì yǒu xiàn gōng sī) Tokyo Pin New Material Technology Co., Ltd.</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -4827,7 +4739,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>王馨苑</t>
+          <t>王馨苑 (wáng xīn yuàn)</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
@@ -4847,7 +4759,7 @@
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>广州市花都区花东镇微观产业园C栋Building C, Weiguan Industrial Park, Huadong Town, Huadu District, Guangzhou</t>
+          <t>广州市花都区花东镇微观产业园 (guǎng zhōu shì huā dōu qū huā dōng zhèn wēi guān chǎn yè yuán)C栋 (dòng)Building C, Weiguan Industrial Park, Huadong Town, Huadu District, Guangzhou</t>
         </is>
       </c>
       <c r="I111" t="n">
@@ -4860,7 +4772,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>余姚市叠天包装有限公司 YUYAO DIETIAN PACKAGING CO., LTD</t>
+          <t>余姚市叠天包装有限公司 (yú yáo shì dié tiān bāo zhuāng yǒu xiàn gōng sī) YUYAO DIETIAN PACKAGING CO., LTD</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -4870,7 +4782,7 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>王丽波</t>
+          <t>王丽波 (wáng lì bō)</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
@@ -4890,7 +4802,7 @@
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>浙江省余姚市牟山镇高车头 B67号肖西路西West of Xiaoxi Road, Gaochetou, Mushan Town, Yuyao City, Zhejiang Province, No. B67</t>
+          <t>浙江省余姚市牟山镇高车头 (zhè jiāng shěng yú yáo shì móu shān zhèn gāo chē tóu) B67号肖西路西 (hào xiào xī lù xī)West of Xiaoxi Road, Gaochetou, Mushan Town, Yuyao City, Zhejiang Province, No. B67</t>
         </is>
       </c>
       <c r="I112" t="n">
@@ -4903,7 +4815,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>余姚市银河日用品有限公司 YUYAO YINHE ARTICLES CO.,LTD.</t>
+          <t>余姚市银河日用品有限公司 (yú yáo shì yín hé rì yòng pǐn yǒu xiàn gōng sī) YUYAO YINHE ARTICLES CO.,LTD.</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -4913,7 +4825,7 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>刘锡蓉</t>
+          <t>刘锡蓉 (liú xī róng)</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
@@ -4933,7 +4845,7 @@
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>浙江省余姚市马渚镇北兴路183号No. 183, Beixing Road, Mazhu Town, Yuyao City, Zhejiang Province</t>
+          <t>浙江省余姚市马渚镇北兴路 (zhè jiāng shěng yú yáo shì mǎ zhǔ zhèn běi xīng lù)183号 (hào)No. 183, Beixing Road, Mazhu Town, Yuyao City, Zhejiang Province</t>
         </is>
       </c>
       <c r="I113" t="n">
@@ -4946,7 +4858,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>光正纸业有限公司 Guangzheng Paper Co., Ltd.</t>
+          <t>光正纸业有限公司 (guāng zhèng zhǐ yè yǒu xiàn gōng sī) Guangzheng Paper Co., Ltd.</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -4956,7 +4868,7 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>潘兴杰</t>
+          <t>潘兴杰 (pān xīng jié)</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
@@ -4976,7 +4888,7 @@
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>廣東省東莞市厚街鎮東業路2號No. 2, Dongye Road, Houjie Town, Dongguan City, Guangdong Province</t>
+          <t>廣東省東莞市厚街鎮東業路 (guǎng dōng shěng dōng guǎn shì hòu jiē zhèn dōng yè lù)2號 (hào)No. 2, Dongye Road, Houjie Town, Dongguan City, Guangdong Province</t>
         </is>
       </c>
       <c r="I114" t="n">
@@ -4989,7 +4901,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>吾道包装 Wudao Packaging</t>
+          <t>吾道包装 (wú dào bāo zhuāng) Wudao Packaging</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -4999,7 +4911,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>胡珍华</t>
+          <t>胡珍华 (hú zhēn huá)</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
@@ -5012,10 +4924,9 @@
           <t>wdpack888@163.com</t>
         </is>
       </c>
-      <c r="G115" t="inlineStr"/>
       <c r="H115" t="inlineStr">
         <is>
-          <t>广州市花都区绿港四街6号No. 6, Lvgong 4th Street, Huadu District, Guangzhou</t>
+          <t>广州市花都区绿港四街 (guǎng zhōu shì huā dōu qū lǜ gǎng sì jiē)6号 (hào)No. 6, Lvgong 4th Street, Huadu District, Guangzhou</t>
         </is>
       </c>
       <c r="I115" t="n">
@@ -5028,7 +4939,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>威美體造 Weimei Body Manufacturing</t>
+          <t>威美體造 (wēi měi tǐ zào) Weimei Body Manufacturing</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -5056,7 +4967,6 @@
           <t>https://chenmascosmetic.on.made-in-china.com</t>
         </is>
       </c>
-      <c r="H116" t="inlineStr"/>
       <c r="I116" t="n">
         <v>1</v>
       </c>
@@ -5067,7 +4977,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>宇然膜丽-YURANMOLI</t>
+          <t>宇然膜丽 (yǔ rán mó lì)-YURANMOLI</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
@@ -5077,7 +4987,7 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>刘扬娥</t>
+          <t>刘扬娥 (liú yáng é)</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
@@ -5085,7 +4995,6 @@
           <t>020-36090547, 181 2675 3479</t>
         </is>
       </c>
-      <c r="F117" t="inlineStr"/>
       <c r="G117" t="inlineStr">
         <is>
           <t>www.yuranmoli.com</t>
@@ -5093,7 +5002,7 @@
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>广州市白云区江高镇神山神石路41号No. 41, Shenshan Shishen Road, Jianggao Town, Baiyun District, Guangzhou</t>
+          <t>广州市白云区江高镇神山神石路 (guǎng zhōu shì bái yún qū jiāng gāo zhèn shén shān shén shí lù)41号 (hào)No. 41, Shenshan Shishen Road, Jianggao Town, Baiyun District, Guangzhou</t>
         </is>
       </c>
       <c r="I117" t="n">
@@ -5106,7 +5015,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>广东中源数字化技术有限公司 Guangdong Zhongyuan Digital Technology Co., Ltd.</t>
+          <t>广东中源数字化技术有限公司 (guǎng dōng zhōng yuán shù zì huà jì shù yǒu xiàn gōng sī) Guangdong Zhongyuan Digital Technology Co., Ltd.</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
@@ -5116,7 +5025,7 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>林帆</t>
+          <t>林帆 (lín fān)</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
@@ -5136,7 +5045,7 @@
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>广东省广州市天河区科韵路288号天盈创意园 C区3024-3027Rooms 3024-3027, Area C, Tianying Creative Park, No. 288 Keyun Road, Tianhe District, Guangzhou City, Guangdong Province</t>
+          <t>广东省广州市天河区科韵路 (guǎng dōng shěng guǎng zhōu shì tiān hé qū kē yùn lù)288号天盈创意园 (hào tiān yíng chuàng yì yuán) C区 (qū)3024-3027Rooms 3024-3027, Area C, Tianying Creative Park, No. 288 Keyun Road, Tianhe District, Guangzhou City, Guangdong Province</t>
         </is>
       </c>
       <c r="I118" t="n">
@@ -5149,7 +5058,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>广东全信医药科技有限公司 Guangdong Quanxin Pharmaceutical Technology Co., Ltd.</t>
+          <t>广东全信医药科技有限公司 (guǎng dōng quán xìn yī yào kē jì yǒu xiàn gōng sī) Guangdong Quanxin Pharmaceutical Technology Co., Ltd.</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -5159,7 +5068,7 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>刘丽红 Valerie</t>
+          <t>刘丽红 (liú lì hóng) Valerie</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
@@ -5167,11 +5076,9 @@
           <t>181-2245-2461</t>
         </is>
       </c>
-      <c r="F119" t="inlineStr"/>
-      <c r="G119" t="inlineStr"/>
       <c r="H119" t="inlineStr">
         <is>
-          <t>广东省广州市花都区金田路3号No. 3, Jintian Road, Huadu District, Guangzhou City, Guangdong Province</t>
+          <t>广东省广州市花都区金田路 (guǎng dōng shěng guǎng zhōu shì huā dōu qū jīn tián lù)3号 (hào)No. 3, Jintian Road, Huadu District, Guangzhou City, Guangdong Province</t>
         </is>
       </c>
       <c r="I119" t="n">
@@ -5184,7 +5091,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>广东华轻质量检测服务中心有限公司 Guangdong Huaqing Quality Inspection Service Center Co., Ltd.</t>
+          <t>广东华轻质量检测服务中心有限公司 (guǎng dōng huá qīng zhì liàng jiǎn cè fú wù zhōng xīn yǒu xiàn gōng sī) Guangdong Huaqing Quality Inspection Service Center Co., Ltd.</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
@@ -5194,7 +5101,7 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>梁冠文</t>
+          <t>梁冠文 (liáng guān wén)</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
@@ -5207,10 +5114,9 @@
           <t>liangguanwen@qtccn.com</t>
         </is>
       </c>
-      <c r="G120" t="inlineStr"/>
       <c r="H120" t="inlineStr">
         <is>
-          <t>广州市白云区北太路1633号广州民营科技园科园路2号凯铂中心D区1-4楼 1-4 F, Area D. Kaibo Center Building, No.2 Keyuan Road, Guangzhou Private Science and Technology Park, No. 1633 Beitai Road, Baiyun District, Guangzhou</t>
+          <t>广州市白云区北太路 (guǎng zhōu shì bái yún qū běi tài lù)1633号广州民营科技园科园路 (hào guǎng zhōu mín yíng kē jì yuán kē yuán lù)2号凯铂中心 (hào kǎi bó zhōng xīn)D区 (qū)1-4楼 (lóu) 1-4 F, Area D. Kaibo Center Building, No.2 Keyuan Road, Guangzhou Private Science and Technology Park, No. 1633 Beitai Road, Baiyun District, Guangzhou</t>
         </is>
       </c>
       <c r="I120" t="n">
@@ -5223,7 +5129,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>广东吾道创展塑业有限公司 Guangdong Wudao Chuangzhan Plastic Industry Co., Ltd.</t>
+          <t>广东吾道创展塑业有限公司 (guǎng dōng wú dào chuàng zhǎn sù yè yǒu xiàn gōng sī) Guangdong Wudao Chuangzhan Plastic Industry Co., Ltd.</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
@@ -5233,7 +5139,7 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>熊强 Xiong Qiang</t>
+          <t>熊强 (xióng qiáng) Xiong Qiang</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
@@ -5241,11 +5147,9 @@
           <t>159 0204 7142</t>
         </is>
       </c>
-      <c r="F121" t="inlineStr"/>
-      <c r="G121" t="inlineStr"/>
       <c r="H121" t="inlineStr">
         <is>
-          <t>广东省清远市佛冈县汤塘镇广佛产业园创业路7号 C区6栋101-501房Room 101-501, Building 6, Zone C, No. 7, Chuangye Road, Guangfo Industrial Park, Tangtang Town, Fogang County, Qingyuan City, Guangdong Province</t>
+          <t>广东省清远市佛冈县汤塘镇广佛产业园创业路 (guǎng dōng shěng qīng yuǎn shì fú gāng xiàn tāng táng zhèn guǎng fú chǎn yè yuán chuàng yè lù)7号 (hào) C区 (qū)6栋 (dòng)101-501房 (fáng)Room 101-501, Building 6, Zone C, No. 7, Chuangye Road, Guangfo Industrial Park, Tangtang Town, Fogang County, Qingyuan City, Guangdong Province</t>
         </is>
       </c>
       <c r="I121" t="n">
@@ -5258,7 +5162,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>广东坚固包装制品有限公司 Guangdong Jiangu Packaging Co., Ltd</t>
+          <t>广东坚固包装制品有限公司 (guǎng dōng jiān gù bāo zhuāng zhì pǐn yǒu xiàn gōng sī) Guangdong Jiangu Packaging Co., Ltd</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
@@ -5268,7 +5172,7 @@
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>李娟 LiJuan</t>
+          <t>李娟 (lǐ juān) LiJuan</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
@@ -5288,7 +5192,7 @@
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>广州市白云区江高镇408号工业园 A区 11/F Building 7 Awang Industrial Zone, Baiyun District, Guangzhou City</t>
+          <t>广州市白云区江高镇 (guǎng zhōu shì bái yún qū jiāng gāo zhèn)408号工业园 (hào gōng yè yuán) A区 (qū) 11/F Building 7 Awang Industrial Zone, Baiyun District, Guangzhou City</t>
         </is>
       </c>
       <c r="I122" t="n">
@@ -5301,7 +5205,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>广东尼特包装制品有限公司 Guangdong Nite Packaging Products Co., Ltd.</t>
+          <t>广东尼特包装制品有限公司 (guǎng dōng ní tè bāo zhuāng zhì pǐn yǒu xiàn gōng sī) Guangdong Nite Packaging Products Co., Ltd.</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
@@ -5311,7 +5215,7 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>肖海青</t>
+          <t>肖海青 (xiào hǎi qīng)</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
@@ -5331,7 +5235,7 @@
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>中山工厂:广东省中山市火炬开发区茂南路25号 惠州工厂:广东省惠州市龙门县金山工业园建设路2号Zhongshan Factory: No. 25, Maonan Road, Torch Development Zone, Zhongshan City, Guangdong Province; Huizhou Factory: No. 2, Jianshe Road, Jinshan Industrial Park, Longmen County, Huizhou City, Guangdong Province</t>
+          <t>中山工厂 (zhōng shān gōng chǎng):广东省中山市火炬开发区茂南路 (guǎng dōng shěng zhōng shān shì huǒ jù kāi fā qū mào nán lù)25号 (hào) 惠州工厂 (huì zhōu gōng chǎng):广东省惠州市龙门县金山工业园建设路 (guǎng dōng shěng huì zhōu shì lóng mén xiàn jīn shān gōng yè yuán jiàn shè lù)2号 (hào)Zhongshan Factory: No. 25, Maonan Road, Torch Development Zone, Zhongshan City, Guangdong Province; Huizhou Factory: No. 2, Jianshe Road, Jinshan Industrial Park, Longmen County, Huizhou City, Guangdong Province</t>
         </is>
       </c>
       <c r="I123" t="n">
@@ -5344,7 +5248,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>广东琴叶健康日用品科技有限公司 Guangdong Qinyue Health Daily Necessities Technology Co., Ltd.</t>
+          <t>广东琴叶健康日用品科技有限公司 (guǎng dōng qín yè jiàn kāng rì yòng pǐn kē jì yǒu xiàn gōng sī) Guangdong Qinyue Health Daily Necessities Technology Co., Ltd.</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
@@ -5354,7 +5258,7 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>郭武杰</t>
+          <t>郭武杰 (guō wǔ jié)</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
@@ -5367,10 +5271,9 @@
           <t>1023128601@qq.com</t>
         </is>
       </c>
-      <c r="G124" t="inlineStr"/>
       <c r="H124" t="inlineStr">
         <is>
-          <t>广州天河区广州大道中307号富力东山新天地中心42楼(总部营销中心)42nd Floor (Headquarters Marketing Center), Fuli Dongshan Xintiandi Center, No. 307 Guangzhou Avenue Middle, Tianhe District, Guangzhou</t>
+          <t>广州天河区广州大道中 (guǎng zhōu tiān hé qū guǎng zhōu dà dào zhōng)307号富力东山新天地中心 (hào fù lì dōng shān xīn tiān dì zhōng xīn)42楼 (lóu)(总部营销中心 (zǒng bù yíng xiāo zhōng xīn))42nd Floor (Headquarters Marketing Center), Fuli Dongshan Xintiandi Center, No. 307 Guangzhou Avenue Middle, Tianhe District, Guangzhou</t>
         </is>
       </c>
       <c r="I124" t="n">
@@ -5383,7 +5286,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>广东腾宇集团有限责任公司 Guangdong Tengyu Group Co., Ltd.</t>
+          <t>广东腾宇集团有限责任公司 (guǎng dōng téng yǔ jí tuán yǒu xiàn zé rèn gōng sī) Guangdong Tengyu Group Co., Ltd.</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
@@ -5393,7 +5296,7 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>陈花蕾 Chen Hualel</t>
+          <t>陈花蕾 (chén huā lěi) Chen Hualel</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
@@ -5413,7 +5316,7 @@
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>广州市白云区云城东路云理汇2栋3楼3rd Floor, Building 2, Yunlihui, Yuncheng East Road, Baiyun District, Guangzhou</t>
+          <t>广州市白云区云城东路云理汇 (guǎng zhōu shì bái yún qū yún chéng dōng lù yún lǐ huì)2栋 (dòng)3楼 (lóu)3rd Floor, Building 2, Yunlihui, Yuncheng East Road, Baiyun District, Guangzhou</t>
         </is>
       </c>
       <c r="I125" t="n">
@@ -5426,7 +5329,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>广州九圆塑业有限公司 Guangzhou Jiuyuan Plastic Industry Co., Ltd.</t>
+          <t>广州九圆塑业有限公司 (guǎng zhōu jiǔ yuán sù yè yǒu xiàn gōng sī) Guangzhou Jiuyuan Plastic Industry Co., Ltd.</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
@@ -5436,7 +5339,7 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>李小娜</t>
+          <t>李小娜 (lǐ xiǎo nà)</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
@@ -5444,7 +5347,6 @@
           <t>1992 7712 976</t>
         </is>
       </c>
-      <c r="F126" t="inlineStr"/>
       <c r="G126" t="inlineStr">
         <is>
           <t>https://jiuyuansuye04.1688.com/</t>
@@ -5452,7 +5354,7 @@
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>广州市从化区明珠工业园宝聚路二号No. 2, Baoju Road, Mingzhu Industrial Park, Conghua District, Guangzhou City</t>
+          <t>广州市从化区明珠工业园宝聚路二号 (guǎng zhōu shì cóng huà qū míng zhū gōng yè yuán bǎo jù lù èr hào)No. 2, Baoju Road, Mingzhu Industrial Park, Conghua District, Guangzhou City</t>
         </is>
       </c>
       <c r="I126" t="n">
@@ -5465,7 +5367,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>广州宇然膜丽无纺制品有限公司 Guangzhou Yuran Moli Non-woven Products Co., Ltd.</t>
+          <t>广州宇然膜丽无纺制品有限公司 (guǎng zhōu yǔ rán mó lì wú fǎng zhì pǐn yǒu xiàn gōng sī) Guangzhou Yuran Moli Non-woven Products Co., Ltd.</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -5475,7 +5377,7 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>彭练芝</t>
+          <t>彭练芝 (péng liàn zhī)</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
@@ -5483,7 +5385,6 @@
           <t>133 1885 5960, 020-36090547</t>
         </is>
       </c>
-      <c r="F127" t="inlineStr"/>
       <c r="G127" t="inlineStr">
         <is>
           <t>www.yuranmoli.com</t>
@@ -5491,7 +5392,7 @@
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>广州市白云区江高镇神山神石路41号No. 41, Shenshan Shishen Road, Jianggao Town, Baiyun District, Guangzhou</t>
+          <t>广州市白云区江高镇神山神石路 (guǎng zhōu shì bái yún qū jiāng gāo zhèn shén shān shén shí lù)41号 (hào)No. 41, Shenshan Shishen Road, Jianggao Town, Baiyun District, Guangzhou</t>
         </is>
       </c>
       <c r="I127" t="n">
@@ -5504,7 +5405,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>广州市捷盛隆纸品贸易有限公司 Guangzhou Jieshenglong Paper Products Trading Co., Ltd.</t>
+          <t>广州市捷盛隆纸品贸易有限公司 (guǎng zhōu shì jié shèng lóng zhǐ pǐn mào yì yǒu xiàn gōng sī) Guangzhou Jieshenglong Paper Products Trading Co., Ltd.</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
@@ -5514,7 +5415,7 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>李文慧</t>
+          <t>李文慧 (lǐ wén huì)</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
@@ -5522,11 +5423,9 @@
           <t>13202070184</t>
         </is>
       </c>
-      <c r="F128" t="inlineStr"/>
-      <c r="G128" t="inlineStr"/>
       <c r="H128" t="inlineStr">
         <is>
-          <t>广东省广州市花都区花东镇北兴北钟路54号No. 54, Beixing Beizhong Road, Huadong Town, Huadu District, Guangzhou City, Guangdong Province</t>
+          <t>广东省广州市花都区花东镇北兴北钟路 (guǎng dōng shěng guǎng zhōu shì huā dōu qū huā dōng zhèn běi xīng běi zhōng lù)54号 (hào)No. 54, Beixing Beizhong Road, Huadong Town, Huadu District, Guangzhou City, Guangdong Province</t>
         </is>
       </c>
       <c r="I128" t="n">
@@ -5539,7 +5438,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>广州市联惠科技有限公司 Guangzhou Lianhui Technology Co., Ltd.</t>
+          <t>广州市联惠科技有限公司 (guǎng zhōu shì lián huì kē jì yǒu xiàn gōng sī) Guangzhou Lianhui Technology Co., Ltd.</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
@@ -5549,7 +5448,7 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>刘绍伟</t>
+          <t>刘绍伟 (liú shào wěi)</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
@@ -5569,7 +5468,7 @@
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>佛山市三水区乐平镇博裕路34号1栋Building 1, No. 34, Boyu Road, Leping Town, Sanshui District, Foshan City</t>
+          <t>佛山市三水区乐平镇博裕路 (fó shān shì sān shuǐ qū lè píng zhèn bó yù lù)34号 (hào)1栋 (dòng)Building 1, No. 34, Boyu Road, Leping Town, Sanshui District, Foshan City</t>
         </is>
       </c>
       <c r="I129" t="n">
@@ -5582,7 +5481,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>广州市莱诺鸟智能科技有限公司 Guangzhou Lainuoniao Intelligent Technology Co., Ltd.</t>
+          <t>广州市莱诺鸟智能科技有限公司 (guǎng zhōu shì lái nuò niǎo zhì néng kē jì yǒu xiàn gōng sī) Guangzhou Lainuoniao Intelligent Technology Co., Ltd.</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
@@ -5592,7 +5491,7 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>陈坤</t>
+          <t>陈坤 (chén kūn)</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
@@ -5605,10 +5504,9 @@
           <t>kun.chen@lainuoniao.com</t>
         </is>
       </c>
-      <c r="G130" t="inlineStr"/>
       <c r="H130" t="inlineStr">
         <is>
-          <t>广州市白云区云城西路娇兰佳人大厦10楼10th Floor, Jiaolan Jiada Building, Yuncheng West Road, Baiyun District, Guangzhou City</t>
+          <t>广州市白云区云城西路娇兰佳人大厦 (guǎng zhōu shì bái yún qū yún chéng xī lù jiāo lán jiā rén dà shà)10楼 (lóu)10th Floor, Jiaolan Jiada Building, Yuncheng West Road, Baiyun District, Guangzhou City</t>
         </is>
       </c>
       <c r="I130" t="n">
@@ -5621,7 +5519,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>广州市贤俊龙彩印有限公司 Guangzhou Xianjunlong Color Printing Co., Ltd.</t>
+          <t>广州市贤俊龙彩印有限公司 (guǎng zhōu shì xián jùn lóng cǎi yìn yǒu xiàn gōng sī) Guangzhou Xianjunlong Color Printing Co., Ltd.</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
@@ -5631,7 +5529,7 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>卿慧</t>
+          <t>卿慧 (qīng huì)</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
@@ -5651,7 +5549,7 @@
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>广州市白云区三元里大道11号中港皮具城10楼1009室Room 1009, 10th Floor, Zhonggang Leather City, No. 11, Sanyuanli Avenue, Baiyun District, Guangzhou City</t>
+          <t>广州市白云区三元里大道 (guǎng zhōu shì bái yún qū sān yuán lǐ dà dào)11号中港皮具城 (hào zhōng gǎng pí jù chéng)10楼 (lóu)1009室 (shì)Room 1009, 10th Floor, Zhonggang Leather City, No. 11, Sanyuanli Avenue, Baiyun District, Guangzhou City</t>
         </is>
       </c>
       <c r="I131" t="n">
@@ -5664,7 +5562,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>广州市鸿亿防伪产品有限公司 Guangzhou Hongyi Anti-counterfeiting Products Co., Ltd.</t>
+          <t>广州市鸿亿防伪产品有限公司 (guǎng zhōu shì hóng yì fáng wěi chǎn pǐn yǒu xiàn gōng sī) Guangzhou Hongyi Anti-counterfeiting Products Co., Ltd.</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
@@ -5674,7 +5572,7 @@
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>邹永流</t>
+          <t>邹永流 (zōu yǒng liú)</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
@@ -5687,10 +5585,9 @@
           <t>go518@189.cn</t>
         </is>
       </c>
-      <c r="G132" t="inlineStr"/>
       <c r="H132" t="inlineStr">
         <is>
-          <t>广州市越秀区先烈中路85号浙江大厦9楼9th Floor, Zhejiang Building, No. 85, Xianlie Middle Road, Yuexiu District, Guangzhou City</t>
+          <t>广州市越秀区先烈中路 (guǎng zhōu shì yuè xiù qū xiān liè zhōng lù)85号浙江大厦 (hào zhè jiāng dà shà)9楼 (lóu)9th Floor, Zhejiang Building, No. 85, Xianlie Middle Road, Yuexiu District, Guangzhou City</t>
         </is>
       </c>
       <c r="I132" t="n">
@@ -5703,7 +5600,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>广州市鸿志包装材料有限公司 HERO TUBE</t>
+          <t>广州市鸿志包装材料有限公司 (guǎng zhōu shì hóng zhì bāo zhuāng cái liào yǒu xiàn gōng sī) HERO TUBE</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
@@ -5713,7 +5610,7 @@
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>罗文豪 Louis</t>
+          <t>罗文豪 (luó wén háo) Louis</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
@@ -5726,10 +5623,9 @@
           <t>luowenhao868@gmail.com</t>
         </is>
       </c>
-      <c r="G133" t="inlineStr"/>
       <c r="H133" t="inlineStr">
         <is>
-          <t>广州市从化区横江路339号 -36号鸿志软管Hongzhi Hose, No. 339-36, Hengjiang Road, Conghua District, Guangzhou City</t>
+          <t>广州市从化区横江路 (guǎng zhōu shì cóng huà qū héng jiāng lù)339号 (hào) -36号鸿志软管 (hào hóng zhì ruǎn guǎn)Hongzhi Hose, No. 339-36, Hengjiang Road, Conghua District, Guangzhou City</t>
         </is>
       </c>
       <c r="I133" t="n">
@@ -5742,7 +5638,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>广州心合包装科技制造有限公司 Guangzhou Xinhe Packaging Technology Manufacturing Co., Ltd.</t>
+          <t>广州心合包装科技制造有限公司 (guǎng zhōu xīn hé bāo zhuāng kē jì zhì zào yǒu xiàn gōng sī) Guangzhou Xinhe Packaging Technology Manufacturing Co., Ltd.</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
@@ -5765,10 +5661,9 @@
           <t>sales05@hspaperpackaging.com</t>
         </is>
       </c>
-      <c r="G134" t="inlineStr"/>
       <c r="H134" t="inlineStr">
         <is>
-          <t>广州市白云区太和镇谢家注兰西路2号 No. 2 Yinian West Road, Xielazhuang, Taihe Town layun District, Duangzhou City</t>
+          <t>广州市白云区太和镇谢家注兰西路 (guǎng zhōu shì bái yún qū tài hé zhèn xiè jiā zhù lán xī lù)2号 (hào) No. 2 Yinian West Road, Xielazhuang, Taihe Town layun District, Duangzhou City</t>
         </is>
       </c>
       <c r="I134" t="n">
@@ -5781,7 +5676,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>广州心合包装科技有限公司 Guangzhou Xinhe Packaging Technology Co., Ltd.</t>
+          <t>广州心合包装科技有限公司 (guǎng zhōu xīn hé bāo zhuāng kē jì yǒu xiàn gōng sī) Guangzhou Xinhe Packaging Technology Co., Ltd.</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
@@ -5791,7 +5686,7 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>于舒情</t>
+          <t>于舒情 (yú shū qíng)</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
@@ -5799,11 +5694,9 @@
           <t>+86-13660078608</t>
         </is>
       </c>
-      <c r="F135" t="inlineStr"/>
-      <c r="G135" t="inlineStr"/>
       <c r="H135" t="inlineStr">
         <is>
-          <t>广州市白云区太和镇谢家庄荫兰西路2号No. 2, Yinlan West Road, Xiejiazhuang, Taihe Town, Baiyun District, Guangzhou City</t>
+          <t>广州市白云区太和镇谢家庄荫兰西路 (guǎng zhōu shì bái yún qū tài hé zhèn xiè jiā zhuāng yīn lán xī lù)2号 (hào)No. 2, Yinlan West Road, Xiejiazhuang, Taihe Town, Baiyun District, Guangzhou City</t>
         </is>
       </c>
       <c r="I135" t="n">
@@ -5816,7 +5709,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>广州方和印刷有限公司 Guangzhou Fanghe Printing Co., Ltd.</t>
+          <t>广州方和印刷有限公司 (guǎng zhōu fāng hé yìn shuā yǒu xiàn gōng sī) Guangzhou Fanghe Printing Co., Ltd.</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
@@ -5826,7 +5719,7 @@
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>石小姐 SHI XIAOJIE</t>
+          <t>石小姐 (shí xiǎo jiě) SHI XIAOJIE</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
@@ -5846,7 +5739,7 @@
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>广州市白云区龙归街南岭村岗埔大道1号No. 1 Gangpu Avenue, Nanling Village, Longgui Street, Baiyun District, Guangzhou City</t>
+          <t>广州市白云区龙归街南岭村岗埔大道 (guǎng zhōu shì bái yún qū lóng guī jiē nán lǐng cūn gǎng pǔ dà dào)1号 (hào)No. 1 Gangpu Avenue, Nanling Village, Longgui Street, Baiyun District, Guangzhou City</t>
         </is>
       </c>
       <c r="I136" t="n">
@@ -5859,7 +5752,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>广州柯源塑料制品有限公司 Guangzhou Keyuan Plasticware Co., Ltd.</t>
+          <t>广州柯源塑料制品有限公司 (guǎng zhōu kē yuán sù liào zhì pǐn yǒu xiàn gōng sī) Guangzhou Keyuan Plasticware Co., Ltd.</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
@@ -5869,7 +5762,7 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>梁凯豪</t>
+          <t>梁凯豪 (liáng kǎi háo)</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
@@ -5877,7 +5770,6 @@
           <t>+86-13318898899</t>
         </is>
       </c>
-      <c r="F137" t="inlineStr"/>
       <c r="G137" t="inlineStr">
         <is>
           <t>www.keyuanbottle.com</t>
@@ -5898,7 +5790,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>广州语辰化妆品包装有限公司 Guangzhou Yucheng Cosmetics Packaging Co., Ltd.</t>
+          <t>广州语辰化妆品包装有限公司 (guǎng zhōu yǔ chén huà zhuāng pǐn bāo zhuāng yǒu xiàn gōng sī) Guangzhou Yucheng Cosmetics Packaging Co., Ltd.</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
@@ -5916,11 +5808,9 @@
           <t>18922244442</t>
         </is>
       </c>
-      <c r="F138" t="inlineStr"/>
-      <c r="G138" t="inlineStr"/>
       <c r="H138" t="inlineStr">
         <is>
-          <t>广州市花都区凤凰南路61号卓美大楼北楼307室Room 307, North Building, Zhuomei Building, No. 61, Fenghuang South Road, Huadu District, Guangzhou</t>
+          <t>广州市花都区凤凰南路 (guǎng zhōu shì huā dōu qū fèng huáng nán lù)61号卓美大楼北楼 (hào zhuó měi dà lóu běi lóu)307室 (shì)Room 307, North Building, Zhuomei Building, No. 61, Fenghuang South Road, Huadu District, Guangzhou</t>
         </is>
       </c>
       <c r="I138" t="n">
@@ -5933,7 +5823,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>廣州昌宏印務有限公司 Guangzhou Changhong Printing Co., Ltd.</t>
+          <t>廣州昌宏印務有限公司 (guǎng zhōu chāng hóng yìn wù yǒu xiàn gōng sī) Guangzhou Changhong Printing Co., Ltd.</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
@@ -5943,7 +5833,7 @@
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>黎金昌</t>
+          <t>黎金昌 (lí jīn chāng)</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
@@ -5963,7 +5853,7 @@
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>廣州市白雲區龍歸街夏良東路81號102房Room 102, No. 81, Xialiang East Road, Longgui Street, Baiyun District, Guangzhou</t>
+          <t>廣州市白雲區龍歸街夏良東路 (guǎng zhōu shì bái yún qū lóng guī jiē xià liáng dōng lù)81號 (hào)102房 (fáng)Room 102, No. 81, Xialiang East Road, Longgui Street, Baiyun District, Guangzhou</t>
         </is>
       </c>
       <c r="I139" t="n">
@@ -5976,7 +5866,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>廣州紅格智造包装有限公司 Guangzhou Hongge Intelligent Manufacturing Packaging Co., Ltd.</t>
+          <t>廣州紅格智造包装有限公司 (guǎng zhōu hóng gé zhì zào bāo zhuāng yǒu xiàn gōng sī) Guangzhou Hongge Intelligent Manufacturing Packaging Co., Ltd.</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
@@ -5999,10 +5889,9 @@
           <t>windy@gdcan.com.cn</t>
         </is>
       </c>
-      <c r="G140" t="inlineStr"/>
       <c r="H140" t="inlineStr">
         <is>
-          <t>廣州市花都區花山鎮城西村自編3號No. 3 (self-numbered), Chengxi Village, Huashan Town, Huadu District, Guangzhou City</t>
+          <t>廣州市花都區花山鎮城西村自編 (guǎng zhōu shì huā dōu qū huā shān zhèn chéng xī cūn zì biān)3號 (hào)No. 3 (self-numbered), Chengxi Village, Huashan Town, Huadu District, Guangzhou City</t>
         </is>
       </c>
       <c r="I140" t="n">
@@ -6015,13 +5904,12 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>护肤品OEM/ODM</t>
-        </is>
-      </c>
-      <c r="C141" t="inlineStr"/>
+          <t>护肤品 (hù fū pǐn)OEM/ODM</t>
+        </is>
+      </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>祝依婷 Carrie</t>
+          <t>祝依婷 (zhù yī tíng) Carrie</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
@@ -6029,11 +5917,9 @@
           <t>13926350387/+8613926350387</t>
         </is>
       </c>
-      <c r="F141" t="inlineStr"/>
-      <c r="G141" t="inlineStr"/>
       <c r="H141" t="inlineStr">
         <is>
-          <t>广东省广州市花都区金田路3号No. 3, Jintian Road, Huadu District, Guangzhou City, Guangdong Province</t>
+          <t>广东省广州市花都区金田路 (guǎng dōng shěng guǎng zhōu shì huā dōu qū jīn tián lù)3号 (hào)No. 3, Jintian Road, Huadu District, Guangzhou City, Guangdong Province</t>
         </is>
       </c>
       <c r="I141" t="n">
@@ -6046,7 +5932,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>正晟包装科技(广东)有限公司 Zhengsheng Packaging Technology (Guangdong) Co., Ltd.</t>
+          <t>正晟包装科技 (zhèng chéng bāo zhuāng kē jì)(广东 (guǎng dōng))有限公司 (yǒu xiàn gōng sī) Zhengsheng Packaging Technology (Guangdong) Co., Ltd.</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
@@ -6056,7 +5942,7 @@
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>邓思艺</t>
+          <t>邓思艺 (dèng sī yì)</t>
         </is>
       </c>
       <c r="E142" t="inlineStr">
@@ -6069,10 +5955,9 @@
           <t>Jenny08@gzsummitek.com</t>
         </is>
       </c>
-      <c r="G142" t="inlineStr"/>
       <c r="H142" t="inlineStr">
         <is>
-          <t>广东省清远市清城区石角镇(广清产业园)兴园路3号; 广州市花都区新雅街绿地空港五号地4栋1107室No. 3, Xingyuan Road, Shijiao Town (Guangqing Industrial Park), Qingcheng District, Qingyuan City, Guangdong Province; Room 1107, Building 4, Plot 5, Greenland Airport, Xinya Street, Huadu District, Guangzhou City</t>
+          <t>广东省清远市清城区石角镇 (guǎng dōng shěng qīng yuǎn shì qīng chéng qū shí jiǎo zhèn)(广清产业园 (guǎng qīng chǎn yè yuán))兴园路 (xīng yuán lù)3号 (hào); 广州市花都区新雅街绿地空港五号地 (guǎng zhōu shì huā dōu qū xīn yǎ jiē lǜ dì kōng gǎng wǔ hào dì)4栋 (dòng)1107室 (shì)No. 3, Xingyuan Road, Shijiao Town (Guangqing Industrial Park), Qingcheng District, Qingyuan City, Guangdong Province; Room 1107, Building 4, Plot 5, Greenland Airport, Xinya Street, Huadu District, Guangzhou City</t>
         </is>
       </c>
       <c r="I142" t="n">
@@ -6085,7 +5970,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>汕头市艺被塑胶模具有限公司 Shantou Yibei Plastic Mold Co., Ltd.</t>
+          <t>汕头市艺被塑胶模具有限公司 (shàn tóu shì yì bèi sù jiāo mú jù yǒu xiàn gōng sī) Shantou Yibei Plastic Mold Co., Ltd.</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
@@ -6095,7 +5980,7 @@
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>江思蓉</t>
+          <t>江思蓉 (jiāng sī róng)</t>
         </is>
       </c>
       <c r="E143" t="inlineStr">
@@ -6103,9 +5988,6 @@
           <t>18763000898</t>
         </is>
       </c>
-      <c r="F143" t="inlineStr"/>
-      <c r="G143" t="inlineStr"/>
-      <c r="H143" t="inlineStr"/>
       <c r="I143" t="n">
         <v>1</v>
       </c>
@@ -6116,7 +5998,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>汕头市艺骏塑胶模具有限公司 Shantou Yijun Plastic Mold Co., Ltd.</t>
+          <t>汕头市艺骏塑胶模具有限公司 (shàn tóu shì yì jùn sù jiāo mú jù yǒu xiàn gōng sī) Shantou Yijun Plastic Mold Co., Ltd.</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
@@ -6126,7 +6008,7 @@
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>刘键均</t>
+          <t>刘键均 (liú jiàn jūn)</t>
         </is>
       </c>
       <c r="E144" t="inlineStr">
@@ -6134,11 +6016,9 @@
           <t>16789429179</t>
         </is>
       </c>
-      <c r="F144" t="inlineStr"/>
-      <c r="G144" t="inlineStr"/>
       <c r="H144" t="inlineStr">
         <is>
-          <t>广州市白云区云城西路888号绿地中心2403Room 2403, Greenland Center, No. 888 Yuncheng West Road, Baiyun District, Guangzhou City</t>
+          <t>广州市白云区云城西路 (guǎng zhōu shì bái yún qū yún chéng xī lù)888号绿地中心 (hào lǜ dì zhōng xīn)2403Room 2403, Greenland Center, No. 888 Yuncheng West Road, Baiyun District, Guangzhou City</t>
         </is>
       </c>
       <c r="I144" t="n">
@@ -6151,7 +6031,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>汕头市金平区彩鸿塑业有限公司 Shantou Jinping District Caihong Plastic Industry Co., Ltd.</t>
+          <t>汕头市金平区彩鸿塑业有限公司 (shàn tóu shì jīn píng qū cǎi hóng sù yè yǒu xiàn gōng sī) Shantou Jinping District Caihong Plastic Industry Co., Ltd.</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
@@ -6161,7 +6041,7 @@
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>马壮茂</t>
+          <t>马壮茂 (mǎ zhuàng mào)</t>
         </is>
       </c>
       <c r="E145" t="inlineStr">
@@ -6174,8 +6054,6 @@
           <t>stcaihong2025@163.com</t>
         </is>
       </c>
-      <c r="G145" t="inlineStr"/>
-      <c r="H145" t="inlineStr"/>
       <c r="I145" t="n">
         <v>2</v>
       </c>
@@ -6186,7 +6064,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>浙江永锦科技有限公司 Zhejiang Yongjin Technology Co., Ltd.</t>
+          <t>浙江永锦科技有限公司 (zhè jiāng yǒng jǐn kē jì yǒu xiàn gōng sī) Zhejiang Yongjin Technology Co., Ltd.</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
@@ -6196,7 +6074,7 @@
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>谢雅琪</t>
+          <t>谢雅琪 (xiè yǎ qí)</t>
         </is>
       </c>
       <c r="E146" t="inlineStr">
@@ -6216,7 +6094,7 @@
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>浙江省绍兴市上虞区曹娥街道五星西路1999号联东U谷21栋C永, Add C tongin Bulding 21. Landong U Valley No. 1999, Wing West Road Cace Sheet, Shangyu District. Shocking City Zhellong ProvinceBuilding 21 C, Landong U Valley, No. 1999, Wuxing West Road, Cao'e Street, Shangyu District, Shaoxing City, Zhejiang Province</t>
+          <t>浙江省绍兴市上虞区曹娥街道五星西路 (zhè jiāng shěng shào xīng shì shàng yú qū cáo é jiē dào wǔ xīng xī lù)1999号联东 (hào lián dōng)U谷 (gǔ)21栋 (dòng)C永 (yǒng), Add C tongin Bulding 21. Landong U Valley No. 1999, Wing West Road Cace Sheet, Shangyu District. Shocking City Zhellong ProvinceBuilding 21 C, Landong U Valley, No. 1999, Wuxing West Road, Cao'e Street, Shangyu District, Shaoxing City, Zhejiang Province</t>
         </is>
       </c>
       <c r="I146" t="n">
@@ -6229,7 +6107,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>浙江赫宇包装科技有限公司 Zhejiang Heyu Packaging Technology Co., Ltd.</t>
+          <t>浙江赫宇包装科技有限公司 (zhè jiāng hè yǔ bāo zhuāng kē jì yǒu xiàn gōng sī) Zhejiang Heyu Packaging Technology Co., Ltd.</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
@@ -6239,7 +6117,7 @@
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>朱斌</t>
+          <t>朱斌 (zhū bīn)</t>
         </is>
       </c>
       <c r="E147" t="inlineStr">
@@ -6252,10 +6130,9 @@
           <t>bin.zhu@comsyns.com</t>
         </is>
       </c>
-      <c r="G147" t="inlineStr"/>
       <c r="H147" t="inlineStr">
         <is>
-          <t>浙江省平湖市新仓镇嘉创智谷远景产业园A7栋Building A7, Jia Chuang Zhi Gu Yuan Jing Industrial Park, Xincang Town, Pinghu City, Zhejiang Province</t>
+          <t>浙江省平湖市新仓镇嘉创智谷远景产业园 (zhè jiāng shěng píng hú shì xīn cāng zhèn jiā chuàng zhì gǔ yuǎn jǐng chǎn yè yuán)A7栋 (dòng)Building A7, Jia Chuang Zhi Gu Yuan Jing Industrial Park, Xincang Town, Pinghu City, Zhejiang Province</t>
         </is>
       </c>
       <c r="I147" t="n">
@@ -6268,7 +6145,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>淮安市永希金属制品有限公司 Huai'an Yongxi Metal Products Co., Ltd.</t>
+          <t>淮安市永希金属制品有限公司 (huái ān shì yǒng xī jīn shǔ zhì pǐn yǒu xiàn gōng sī) Huai'an Yongxi Metal Products Co., Ltd.</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
@@ -6278,7 +6155,7 @@
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>周晓娟</t>
+          <t>周晓娟 (zhōu xiǎo juān)</t>
         </is>
       </c>
       <c r="E148" t="inlineStr">
@@ -6291,10 +6168,9 @@
           <t>jane@yongxi-tech.com</t>
         </is>
       </c>
-      <c r="G148" t="inlineStr"/>
       <c r="H148" t="inlineStr">
         <is>
-          <t>江苏省淮安市洪泽区九牛路8号 邮政编号223100No. 8, Jiuniu Road, Hongze District, Huai'an City, Jiangsu Province, Postal Code 223100</t>
+          <t>江苏省淮安市洪泽区九牛路 (jiāng sū shěng huái ān shì hóng zé qū jiǔ niú lù)8号 (hào) 邮政编号 (yóu zhèng biān hào)223100No. 8, Jiuniu Road, Hongze District, Huai'an City, Jiangsu Province, Postal Code 223100</t>
         </is>
       </c>
       <c r="I148" t="n">
@@ -6307,7 +6183,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>粤成印刷 YUE CHENG</t>
+          <t>粤成印刷 (yuè chéng yìn shuā) YUE CHENG</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
@@ -6317,7 +6193,7 @@
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>章程</t>
+          <t>章程 (zhāng chéng)</t>
         </is>
       </c>
       <c r="E149" t="inlineStr">
@@ -6325,11 +6201,9 @@
           <t>134 3395 6098</t>
         </is>
       </c>
-      <c r="F149" t="inlineStr"/>
-      <c r="G149" t="inlineStr"/>
       <c r="H149" t="inlineStr">
         <is>
-          <t>广东省广州市花都区花山镇华辉路18号 微观化妆品创意产业园D栋整栋、H栋整栋Entire Building D and Entire Building H, Weiguan Cosmetics Creative Industrial Park, No. 18, Huahui Road, Huashan Town, Huadu District, Guangzhou City, Guangdong Province</t>
+          <t>广东省广州市花都区花山镇华辉路 (guǎng dōng shěng guǎng zhōu shì huā dōu qū huā shān zhèn huá huī lù)18号 (hào) 微观化妆品创意产业园 (wēi guān huà zhuāng pǐn chuàng yì chǎn yè yuán)D栋整栋 (dòng zhěng dòng)、H栋整栋 (dòng zhěng dòng)Entire Building D and Entire Building H, Weiguan Cosmetics Creative Industrial Park, No. 18, Huahui Road, Huashan Town, Huadu District, Guangzhou City, Guangdong Province</t>
         </is>
       </c>
       <c r="I149" t="n">
@@ -6342,7 +6216,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>精业 Jingye</t>
+          <t>精业 (jīng yè) Jingye</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
@@ -6365,8 +6239,6 @@
           <t>slana@wywbo.com</t>
         </is>
       </c>
-      <c r="G150" t="inlineStr"/>
-      <c r="H150" t="inlineStr"/>
       <c r="I150" t="n">
         <v>1</v>
       </c>
@@ -6377,7 +6249,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>精展软管 Jingzhan Hose</t>
+          <t>精展软管 (jīng zhǎn ruǎn guǎn) Jingzhan Hose</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
@@ -6387,7 +6259,7 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>游文聪</t>
+          <t>游文聪 (yóu wén cōng)</t>
         </is>
       </c>
       <c r="E151" t="inlineStr">
@@ -6395,11 +6267,9 @@
           <t>13808877295, 020-87817151</t>
         </is>
       </c>
-      <c r="F151" t="inlineStr"/>
-      <c r="G151" t="inlineStr"/>
       <c r="H151" t="inlineStr">
         <is>
-          <t>广州市从化区太平镇新兴路439号7栋Building 7, No. 439, Xinxing Road, Taiping Town, Conghua District, Guangzhou</t>
+          <t>广州市从化区太平镇新兴路 (guǎng zhōu shì cóng huà qū tài píng zhèn xīn xīng lù)439号 (hào)7栋 (dòng)Building 7, No. 439, Xinxing Road, Taiping Town, Conghua District, Guangzhou</t>
         </is>
       </c>
       <c r="I151" t="n">
@@ -6412,7 +6282,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>苏州海明包装科技有限公司 Suzhou Haiming Packaging Technology Co., Ltd.</t>
+          <t>苏州海明包装科技有限公司 (sū zhōu hǎi míng bāo zhuāng kē jì yǒu xiàn gōng sī) Suzhou Haiming Packaging Technology Co., Ltd.</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
@@ -6422,7 +6292,7 @@
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>贾均钊</t>
+          <t>贾均钊 (jiǎ jūn zhāo)</t>
         </is>
       </c>
       <c r="E152" t="inlineStr">
@@ -6442,7 +6312,7 @@
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>苏州市吴江区江陵街道益堂路10号No. 10 Yitang Road, Jiangling Street, Wujiang District, Suzhou City</t>
+          <t>苏州市吴江区江陵街道益堂路 (sū zhōu shì wú jiāng qū jiāng líng jiē dào yì táng lù)10号 (hào)No. 10 Yitang Road, Jiangling Street, Wujiang District, Suzhou City</t>
         </is>
       </c>
       <c r="I152" t="n">
@@ -6455,7 +6325,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>诚德科技股份有限公司 Chengde Technology Co., Ltd.</t>
+          <t>诚德科技股份有限公司 (chéng dé kē jì gǔ fèn yǒu xiàn gōng sī) Chengde Technology Co., Ltd.</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
@@ -6465,7 +6335,7 @@
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>郑国哲</t>
+          <t>郑国哲 (zhèng guó zhé)</t>
         </is>
       </c>
       <c r="E153" t="inlineStr">
@@ -6478,10 +6348,9 @@
           <t>haq@cdbz.cn</t>
         </is>
       </c>
-      <c r="G153" t="inlineStr"/>
       <c r="H153" t="inlineStr">
         <is>
-          <t>浙江省龙港市世纪大道888号No. 888, Century Avenue, Longgang City, Zhejiang Province</t>
+          <t>浙江省龙港市世纪大道 (zhè jiāng shěng lóng gǎng shì shì jì dà dào)888号 (hào)No. 888, Century Avenue, Longgang City, Zhejiang Province</t>
         </is>
       </c>
       <c r="I153" t="n">
@@ -6494,7 +6363,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>银脉玻璃 YINMAIBOLI</t>
+          <t>银脉玻璃 (yín mài bō lí) YINMAIBOLI</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
@@ -6504,7 +6373,7 @@
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>唐飞玲</t>
+          <t>唐飞玲 (táng fēi líng)</t>
         </is>
       </c>
       <c r="E154" t="inlineStr">
@@ -6524,7 +6393,7 @@
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>广州市白云区均禾街石马村桃红西街58号No. 58 Taohong West Street, Shima Village, Junhe Street, Baiyun District, Guangzhou City</t>
+          <t>广州市白云区均禾街石马村桃红西街 (guǎng zhōu shì bái yún qū jūn hé jiē shí mǎ cūn táo hóng xī jiē)58号 (hào)No. 58 Taohong West Street, Shima Village, Junhe Street, Baiyun District, Guangzhou City</t>
         </is>
       </c>
       <c r="I154" t="n">

</xml_diff>

<commit_message>
Add 5 new suppliers from exhibition photos + update to 158
</commit_message>
<xml_diff>
--- a/ipdf_suppliers.xlsx
+++ b/ipdf_suppliers.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I154"/>
+  <dimension ref="A1:I159"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -6400,6 +6400,180 @@
         <v>2</v>
       </c>
     </row>
+    <row r="155">
+      <c r="A155" t="n">
+        <v>154</v>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Shanghai Yingshuo / Ying Yu Packaging</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>Косметическая упаковка</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>+86 21 5988 5200</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr"/>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>www.yingshuo.com</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>188 Beiying Road, QingPu, Shanghai 201700</t>
+        </is>
+      </c>
+      <c r="I155" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="n">
+        <v>155</v>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>Hepuur New Material (Guangdong)</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>Новые материалы, Пластик</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>+86 769 8779 9839</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>info@hepuur.com</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>hepuur.com</t>
+        </is>
+      </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>No. 17 Langzhou Zhou Liao Road, Changping Town, Dongguan, Guangdong</t>
+        </is>
+      </c>
+      <c r="I156" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="n">
+        <v>156</v>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Zhejiang Z&amp;Z (Zhengzhuang)</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Пластиковая упаковка</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>+86-574-58122625</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>sales@z-z.cn</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>www.zzpkg.com</t>
+        </is>
+      </c>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>No.818 Shuanghe Road, Yuyao, Zhejiang</t>
+        </is>
+      </c>
+      <c r="I157" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="n">
+        <v>157</v>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>Ningbo Laoshi / LPI Packaging</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Пластиковая упаковка</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>+86-574-62465217</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>xu@jy-spayer.com</t>
+        </is>
+      </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>www.lpi-packaging.com</t>
+        </is>
+      </c>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>No. 888 Beixing Road, Mazhu Town, Yuyao, Zhejiang</t>
+        </is>
+      </c>
+      <c r="I158" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="n">
+        <v>158</v>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>Anhui Jusu Gaoke Packaging</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Пластиковая упаковка</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr"/>
+      <c r="F159" t="inlineStr"/>
+      <c r="G159" t="inlineStr"/>
+      <c r="H159" t="inlineStr">
+        <is>
+          <t>No. 1 Industrial Avenue, Yaoli Town, Lu'an City, Anhui</t>
+        </is>
+      </c>
+      <c r="I159" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I154"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Translate Chinese job titles, add product names to Excel
</commit_message>
<xml_diff>
--- a/ipdf_suppliers.xlsx
+++ b/ipdf_suppliers.xlsx
@@ -510,8 +510,10 @@
           <t>No.99 Avenue of Wangjiang, Wangjiang County, Anqing City, Anhui Province, China.</t>
         </is>
       </c>
-      <c r="I2" t="n">
-        <v>1</v>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>MOQ 3000. 20 rmb per piece. I was pleased with the meeting with this company. My</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -553,8 +555,10 @@
           <t>江苏省吴江市 (jiāng sū shěng wú jiāng shì) 汾湖经济开发区临沪大道 (fén hú jīng jì kāi fā qū lín hù dà dào)1999号 (hào), 215211No. 1999, Linhu Avenue, Fenhu Economic Development Zone, Wujiang City, Jiangsu Province, 215211</t>
         </is>
       </c>
-      <c r="I3" t="n">
-        <v>1</v>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>1 rmb, 5000 pcs, nice manager — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -591,8 +595,10 @@
           <t>No.4, 5 street, Nanling Gangpu Road, Baiyun district, Guangzhou city, Guangdong province, China</t>
         </is>
       </c>
-      <c r="I4" t="n">
-        <v>3</v>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>MOQ: 50 — покупатель / байер; MOQ 3000 RMB3 — покупатель / байер; 300 MOQ, 5 RMB per unit price. The prices are reasonable and packaging is really</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -634,8 +640,10 @@
           <t>广州市白云区龙兴东南一横路 (guǎng zhōu shì bái yún qū lóng xīng dōng nán yī héng lù)3号 (hào)No. 3, Longxing Southeast First Horizontal Road, Baiyun District, Guangzhou City</t>
         </is>
       </c>
-      <c r="I5" t="n">
-        <v>1</v>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>25rmb, 5000 pcs. Very friendly staff. — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -672,8 +680,10 @@
           <t>广州市花都区花东镇定邦空港产业园 (guǎng zhōu shì huā dōu qū huā dōng zhèn dìng bāng kōng gǎng chǎn yè yuán)D栋 (dòng)Building D, Dingbang Airport Industrial Park, Huadong Town, Huadu District, Guangzhou</t>
         </is>
       </c>
-      <c r="I6" t="n">
-        <v>1</v>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Interesting — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -715,8 +725,10 @@
           <t>广东省开平市三埠街道新台路 (guǎng dōng shěng kāi píng shì sān bù jiē dào xīn tái lù)72号 (hào)No. 72, Xintai Road, Sanbu Street, Kaiping City, Guangdong Province</t>
         </is>
       </c>
-      <c r="I7" t="n">
-        <v>1</v>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>10000 peices — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -743,8 +755,10 @@
           <t>1380 7874 784</t>
         </is>
       </c>
-      <c r="I8" t="n">
-        <v>2</v>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>20yuan/pcs, 500yuan moq — покупатель / байер; Good — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="9">
@@ -786,8 +800,10 @@
           <t>工厂广东省江门市新山市和情共建路 (gōng chǎng guǎng dōng shěng jiāng mén shì xīn shān shì hé qíng gòng jiàn lù)305号座 (hào zuò) 公司地址 (gōng sī dì zhǐ):广州市白云区龙街尖路 (guǎng zhōu shì bái yún qū lóng jiē jiān lù)363号联边国际 (hào lián biān guó jì)620单元 (dān yuán)Factory: Building 305, Heqing Gongjian Road, Xinshan City, Jiangmen City, Guangdong Province. Company Address: Unit 620, Lianbian International, No. 363, Longjie Jian Road, Baiyun District, Guangzhou</t>
         </is>
       </c>
-      <c r="I9" t="n">
-        <v>5</v>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Price=0.35..MOQ-500/COLOR..GOOD. — покупатель / байер; Under discussion price and moq — покупатель / байер; 1-09$ good — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -829,8 +845,10 @@
           <t>2nd Road, Chikan, ShipaiTown, Dongguan, Guangdong, 523346.China</t>
         </is>
       </c>
-      <c r="I10" t="n">
-        <v>1</v>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>30000USD — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="11">
@@ -872,8 +890,10 @@
           <t>No.6 East Lisha Road, Sha Tian Town, DongGuan, GuangDong 4713, Huijin International Financial Building. No. 660 Huangpu Avenue Middle, Tianhe District, Guangzhou</t>
         </is>
       </c>
-      <c r="I11" t="n">
-        <v>1</v>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>6000 MOQ. Very interesting. Something new — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="12">
@@ -915,8 +935,10 @@
           <t>SHANGHAI GUANGZHOU, SHANTOU</t>
         </is>
       </c>
-      <c r="I12" t="n">
-        <v>3</v>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>5,7¥ — покупатель / байер; 10-20 — покупатель / байер; 0.2$- Minimum MOQ 10000 pcs, offering customization — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="13">
@@ -958,8 +980,10 @@
           <t>No.9, Yongshun Avenue.M., Yonghe Zone. GETDZ.GuangZhou P.R.China 511356</t>
         </is>
       </c>
-      <c r="I13" t="n">
-        <v>1</v>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Aluminum foil/tin/10000msquare — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="14">
@@ -996,8 +1020,10 @@
           <t>Office add: Guangzhou Baiyun Beauty Bay Plaza, Room3028 Factory add: Tongzhou Bay Jianghai Linkage Development Demonstration Zone, Nanning City, Jiangsu Province</t>
         </is>
       </c>
-      <c r="I14" t="n">
-        <v>3</v>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>MOQ=12,000 products good — покупатель / байер; 12000 PCS MOQ — покупатель / байер; 6000 peices — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="15">
@@ -1039,8 +1065,10 @@
           <t>Factory Building One, Kewang Rd, Shishan Industrial Park Area A, Nanhal District, Foshan, Guangdong, China</t>
         </is>
       </c>
-      <c r="I15" t="n">
-        <v>1</v>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>0,8-1,2RMB, MOQ10000 — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="16">
@@ -1067,8 +1095,10 @@
           <t>+8618933938604</t>
         </is>
       </c>
-      <c r="I16" t="n">
-        <v>3</v>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>MOQ: 500 — покупатель / байер; MOQ: 500, Price: 220 RMB per price — покупатель / байер; MOQ: 4,1 — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="17">
@@ -1095,8 +1125,10 @@
           <t>400-008-9919, 13501547854</t>
         </is>
       </c>
-      <c r="I17" t="n">
-        <v>2</v>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>45-55 — покупатель / байер; 100-20-30юань от 1000 шт цена меньше — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="18">
@@ -1128,8 +1160,10 @@
           <t>广东省广州市花都区秀全街道大布路 (guǎng dōng shěng guǎng zhōu shì huā dōu qū xiù quán jiē dào dà bù lù)29号峰华工业园 (hào fēng huá gōng yè yuán)Fenghua Industrial Park, No. 29 Dabu Road, Xiuquan Street, Huadu District, Guangzhou City, Guangdong Province</t>
         </is>
       </c>
-      <c r="I18" t="n">
-        <v>1</v>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>MOQ 400, 16.3rmb/шт. — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="19">
@@ -1161,8 +1195,10 @@
           <t>广东省清远英德市英红镇万洋众创城 (guǎng dōng shěng qīng yuǎn yīng dé shì yīng hóng zhèn wàn yáng zhòng chuàng chéng)D区 (qū)37栋 (dòng)Building 37, Zone D, Wanyang Maker Town, Yinghong Town, Yingde City, Qingyuan City, Guangdong Province</t>
         </is>
       </c>
-      <c r="I19" t="n">
-        <v>1</v>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>6-12 RMB, MOQ 12000 — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="20">
@@ -1204,8 +1240,10 @@
           <t>Building C, Micro-Industrial Park, Huadong Town, Huadu District, Guangzhou City</t>
         </is>
       </c>
-      <c r="I20" t="n">
-        <v>2</v>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Good — покупатель / байер; Satisfied with the companies discussion is on the way — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="21">
@@ -1242,8 +1280,10 @@
           <t>42 floor, R &amp; F Dongshan New World Building, No.307 Guangzhou dadao zhong, Tianhe District, Guangzhou</t>
         </is>
       </c>
-      <c r="I21" t="n">
-        <v>2</v>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>20k — покупатель / байер; 20/item — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="22">
@@ -1285,8 +1325,10 @@
           <t>广东省东莞市谢岗镇曹乐向阳路 (guǎng dōng shěng dōng guǎn shì xiè gǎng zhèn cáo lè xiàng yáng lù)55号 (hào), 广东省东莞市樟木头镇塑料市场一期 (guǎng dōng shěng dōng guǎn shì zhāng mù tou zhèn sù liào shì chǎng yī qī)V栋 (dòng)1-2号 (hào), 广东省东莞市常平镇大京九塑料市场塑发东路 (guǎng dōng shěng dōng guǎn shì cháng píng zhèn dà jīng jiǔ sù liào shì chǎng sù fā dōng lù)53-54号 (hào)No. 55, Caole Xiangyang Road, Xiegang Town, Dongguan City, Guangdong Province, Building V, Units 1-2, Phase 1, Plastic Market, Zhangmutou Town, Dongguan City, Guangdong Province, No. 53-54, Sufa East Road, Dajingjiu Plastic Market, Changping Town, Dongguan City, Guangdong Province</t>
         </is>
       </c>
-      <c r="I22" t="n">
-        <v>2</v>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>1,9¥ — покупатель / байер; The streamline material is 130 to 150 rmb per kg. — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="23">
@@ -1328,8 +1370,10 @@
           <t>A46 3rd Floor, Building 3, Yunyinghui, Baiyun District, Guangzhou City, Guangdong Province</t>
         </is>
       </c>
-      <c r="I23" t="n">
-        <v>1</v>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>10000 MOQ. Like this factory too — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="24">
@@ -1356,8 +1400,10 @@
           <t>Guangzhou City, Yuexiu District, Guangyuan West Road No. 121, Commercial Center C, 3rd Floor, Room 022, Guangzhou City, Baiyun District, Zhongluotan Town, Liantian North Road No. 9, Building 6, Chenmei Industrial Park</t>
         </is>
       </c>
-      <c r="I24" t="n">
-        <v>1</v>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>They will send the price list after the exhibition — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="25">
@@ -1389,8 +1435,10 @@
           <t>Office | 4th Floor, 4024 Booth, Meiwan Square, Baiyun District, Guangzhou City, Guangdong Province</t>
         </is>
       </c>
-      <c r="I25" t="n">
-        <v>1</v>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>200Rmb set, 50 set — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="26">
@@ -1422,8 +1470,10 @@
           <t>广州市花都区先科一路金禾云创产业园 (guǎng zhōu shì huā dōu qū xiān kē yī lù jīn hé yún chuàng chǎn yè yuán)Jinhe Yun Chuang Industrial Park, Xianke 1st Road, Huadu District, Guangzhou City</t>
         </is>
       </c>
-      <c r="I26" t="n">
-        <v>1</v>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>35 RMB, MOQ 5000, Good company — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="27">
@@ -1460,8 +1510,10 @@
           <t>广州市越秀区先烈中路 (guǎng zhōu shì yuè xiù qū xiān liè zhōng lù)85号浙江大厦 (hào zhè jiāng dà shà)9楼 (lóu)9th Floor, Zhejiang Building, No. 85, Xianlie Middle Road, Yuexiu District, Guangzhou City</t>
         </is>
       </c>
-      <c r="I27" t="n">
-        <v>1</v>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>10k — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="28">
@@ -1498,8 +1550,10 @@
           <t>No. 339, Hengjiang Road, Conghua District, Guangzhou</t>
         </is>
       </c>
-      <c r="I28" t="n">
-        <v>1</v>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>400, 15rmb — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="29">
@@ -1541,8 +1595,10 @@
           <t>Room 4002, 4th Floor, Meiwan Square, Sanyuanli Street, Baiyun District, Guangzhou, Guangdong Province Ouyu Square, Huangjinling, Tangge Village, Baiyun Lake Street, Baiyun District, Guangzhou, Guangdong Province No. 18, Zone A, Hegui Industrial Park, Nanhai District, Foshan City, Guangdong Province</t>
         </is>
       </c>
-      <c r="I29" t="n">
-        <v>1</v>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>MOQ 5000. Price 7 yuanes — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="30">
@@ -1584,8 +1640,10 @@
           <t>No. 26 Longgui Nanling Central, Taihe Town, Baiyun District, Guangzhou, China</t>
         </is>
       </c>
-      <c r="I30" t="n">
-        <v>2</v>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Превосходные — покупатель / байер; MOQ: 1500 pcs — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="31">
@@ -1617,8 +1675,10 @@
           <t>广州市白云区均禾街清湖村大山路 (guǎng zhōu shì bái yún qū jūn hé jiē qīng hú cūn dà shān lù)6号 (hào)No. 6, Dashan Road, Qinghu Village, Junhe Street, Baiyun District, Guangzhou City</t>
         </is>
       </c>
-      <c r="I31" t="n">
-        <v>2</v>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>0.3 yuan/piece, хорошие впечатления — покупатель / байер; We need to talk on further details about the order — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="32">
@@ -1660,8 +1720,10 @@
           <t>Shajiao Industrial Park, Xiancun Town, Zengcheng District, Guangzhou City</t>
         </is>
       </c>
-      <c r="I32" t="n">
-        <v>2</v>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Anti-aging kit 35 rmb per piece MOQ 5000 pieces — покупатель / байер; 30 rmb one box, good — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="33">
@@ -1703,8 +1765,10 @@
           <t>Add. No. 88, Yongli Road, Xinhua Street, District, Guangzhou, China</t>
         </is>
       </c>
-      <c r="I33" t="n">
-        <v>1</v>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>200000 rmb, MOQ 1 — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="34">
@@ -1736,8 +1800,10 @@
           <t>https://202206.1688.com/</t>
         </is>
       </c>
-      <c r="I34" t="n">
-        <v>2</v>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>1.2RMB — покупатель / байер; 4 yuan, good feedback — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="35">
@@ -1769,8 +1835,10 @@
           <t>广州市白云区北村北大路 (guǎng zhōu shì bái yún qū běi cūn běi dà lù)22号四栋二楼 (hào sì dòng èr lóu)Second Floor, Building 4, No. 22, Beicun Beida Road, Baiyun District, Guangzhou City</t>
         </is>
       </c>
-      <c r="I35" t="n">
-        <v>2</v>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>20 thousand MOQ. 0.15 RMB per piece , the quality of paper mask is high. — покуп; 30 rmb. I take a few samples at home to try. I hope the products are good. The f</t>
+        </is>
       </c>
     </row>
     <row r="36">
@@ -1807,8 +1875,10 @@
           <t>www.qfpackage.com</t>
         </is>
       </c>
-      <c r="I36" t="n">
-        <v>7</v>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>14rmb, 500, visiting the factory — покупатель / байер; They promised to send me a catalogue of the — покупатель / байер; MOQ: 29 — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="37">
@@ -1850,8 +1920,10 @@
           <t>Add NO. 48 Dabu Road, Qinghu, Junhe street, Balyun District, Guangdong Province, China</t>
         </is>
       </c>
-      <c r="I37" t="n">
-        <v>1</v>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>1.2RMB/pc, 10000 pcs, contacts exchange — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="38">
@@ -1893,8 +1965,10 @@
           <t>No: 122, Wulonggang 4th Street, Zhongluotan Town, Baiyun District, Guangzhou, Guangdong, China 510545</t>
         </is>
       </c>
-      <c r="I38" t="n">
-        <v>1</v>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Цены разные, всё сложно, Хорошо — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="39">
@@ -1926,8 +2000,10 @@
           <t>www.simplerpackaging.com</t>
         </is>
       </c>
-      <c r="I39" t="n">
-        <v>1</v>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>They promised to send me a catalogue of the prices. — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="40">
@@ -1964,8 +2040,10 @@
           <t>Room 905/906/907, Building 2, Yuntuhui, No. 239, Yuncheng South Fourth Road, Baiyun District, Guangzhou</t>
         </is>
       </c>
-      <c r="I40" t="n">
-        <v>6</v>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>1,5 $ good — покупатель / байер; 0,08-0.15$/3000 — покупатель / байер; 0.85-1.20$/3000 — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="41">
@@ -1997,8 +2075,10 @@
           <t>No. 2 Yinlan West Road, Xiejiazhuang, Taihe Town, Baiyun District, Guangzhou City</t>
         </is>
       </c>
-      <c r="I41" t="n">
-        <v>2</v>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>2.8¥.MOQ-2000.ok. — покупатель / байер; We are fully satisfied with this supplier. The product range is extensive and we</t>
+        </is>
       </c>
     </row>
     <row r="42">
@@ -2040,8 +2120,10 @@
           <t>Building A5, Nanguo Industrial Park, 433 Helong 5th Road, Renhe Town, Baiyun District, Guangzhou</t>
         </is>
       </c>
-      <c r="I42" t="n">
-        <v>1</v>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>One machine we will talk about the price of the product later — покупатель / бай</t>
+        </is>
       </c>
     </row>
     <row r="43">
@@ -2068,8 +2150,10 @@
           <t>steven@yusupackaging.com</t>
         </is>
       </c>
-      <c r="I43" t="n">
-        <v>1</v>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Price is 3.5 RMB, MOQ is 15000 pieces, quality was outstanding — покупатель / ба</t>
+        </is>
       </c>
     </row>
     <row r="44">
@@ -2096,8 +2180,10 @@
           <t>david@yutopackaging.com</t>
         </is>
       </c>
-      <c r="I44" t="n">
-        <v>1</v>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>5-15 — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="45">
@@ -2134,8 +2220,10 @@
           <t>No.78-1 Kaiyuan Road, Datang Town, Sanshui District, Foshan City, Guangdong Province, China</t>
         </is>
       </c>
-      <c r="I45" t="n">
-        <v>1</v>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>2,9 MOQ 20,000 — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="46">
@@ -2172,8 +2260,10 @@
           <t>No. 15 Liangyuan Erheng Road, Zhonglustan Town, Baiyun District, Guangzhou, Guangdong Province, P.R. China</t>
         </is>
       </c>
-      <c r="I46" t="n">
-        <v>4</v>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>MOQ: 100 — покупатель / байер; MOQ: 1000 — покупатель / байер; 2.8 usd — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="47">
@@ -2205,8 +2295,10 @@
           <t>广州市白云区石井街石井大道 (guǎng zhōu shì bái yún qū shí jǐng jiē shí jǐng dà dào)634号 (hào)No. 634, Shijing Avenue, Shijing Street, Baiyun District, Guangzhou City</t>
         </is>
       </c>
-      <c r="I47" t="n">
-        <v>1</v>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Отлично — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="48">
@@ -2248,8 +2340,10 @@
           <t>上海市浦东新区世纪大道 (shàng hǎi shì pǔ dōng xīn qū shì jì dà dào)100号 (hào)No. 100, Century Avenue, Pudong New Area, Shanghai</t>
         </is>
       </c>
-      <c r="I48" t="n">
-        <v>1</v>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>7RMB 10,000piezas — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="49">
@@ -2286,8 +2380,10 @@
           <t>Industrial Area No.3, Xiaqi Road and Hudi Road, Jinping District, Shantou city, Guangdong Province, China.</t>
         </is>
       </c>
-      <c r="I49" t="n">
-        <v>1</v>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>12 Rmb, 500 pcs — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="50">
@@ -2329,8 +2425,10 @@
           <t>Guang Zhou</t>
         </is>
       </c>
-      <c r="I50" t="n">
-        <v>1</v>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Will send the price with catalog — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="51">
@@ -2367,8 +2465,10 @@
           <t>No.191, Hudi Road, Shantou, Guangdong, China</t>
         </is>
       </c>
-      <c r="I51" t="n">
-        <v>1</v>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>1,36 rmb, 100 pcs. Good price. — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="52">
@@ -2410,8 +2510,10 @@
           <t>上海市奉贤区大叶公路 (shàng hǎi shì fèng xián qū dà yè gōng lù) 6818号 (hào)5A栋 (dòng)502Room 502, Building 5A, No. 6818, Daye Highway, Fengxian District, Shanghai City</t>
         </is>
       </c>
-      <c r="I52" t="n">
-        <v>1</v>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>The price is 6-8 rmb, MOQ- 500-1000, I think the products are of good quality an</t>
+        </is>
       </c>
     </row>
     <row r="53">
@@ -2453,8 +2555,10 @@
           <t>广东省惠州市博罗县石湾镇马石围路 (guǎng dōng shěng huì zhōu shì bó luó xiàn shí wān zhèn mǎ shí wéi lù)3号 (hào)No. 3, Mashiwei Road, Shiwan Town, Boluo County, Huizhou City, Guangdong Province</t>
         </is>
       </c>
-      <c r="I53" t="n">
-        <v>2</v>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>They promised to send me a catalogue of the — покупатель / байер; .5$ depending upon MOQ, Minimum Moq 10000, good production facilities — покупате</t>
+        </is>
       </c>
     </row>
     <row r="54">
@@ -2496,8 +2600,10 @@
           <t>广东省清远市清城区石角镇广清产业园广创街 (guǎng dōng shěng qīng yuǎn shì qīng chéng qū shí jiǎo zhèn guǎng qīng chǎn yè yuán guǎng chuàng jiē)6号 (hào)No. 6, Guangchuang Street, Guangqing Industrial Park, Shijiao Town, Qingcheng District, Qingyuan City, Guangdong Province</t>
         </is>
       </c>
-      <c r="I54" t="n">
-        <v>1</v>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>The price is 3 rmb, MOQ- 10,000, reasonable prices and well experienced supplier</t>
+        </is>
       </c>
     </row>
     <row r="55">
@@ -2539,8 +2645,10 @@
           <t>黄浦区德必上海书城 (huáng pǔ qū dé bì shàng hǎi shū chéng)WE2101室 (shì)Room WE2101, Debao Shanghai Book City, Huangpu District</t>
         </is>
       </c>
-      <c r="I55" t="n">
-        <v>1</v>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>MOQ: 10000 pcs — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="56">
@@ -2577,8 +2685,10 @@
           <t>浙江省嘉兴市南湖区新丰镇新禾路 (zhè jiāng shěng jiā xīng shì nán hú qū xīn fēng zhèn xīn hé lù)158号 (hào)No. 158, Xinhe Road, Xinfeng Town, Nanhu District, Jiaxing City, Zhejiang Province</t>
         </is>
       </c>
-      <c r="I56" t="n">
-        <v>1</v>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>5000*7 RMB — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="57">
@@ -2615,8 +2725,10 @@
           <t>No. 102, Qilongjie, Wulonggang, Zhongluotan Town, Baiyun District, Guangzhou, Guangdong Province China</t>
         </is>
       </c>
-      <c r="I57" t="n">
-        <v>1</v>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Depends on the quantity — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="58">
@@ -2658,8 +2770,10 @@
           <t>No.69 Zhubei Rd. (E) Mazhu Town, Yuvac Zhejiang Province (P.C. 315450) No.888 Beixing Rd. Mazhu Town. Yuyao Zhejiang Province(P.C. 315450)</t>
         </is>
       </c>
-      <c r="I58" t="n">
-        <v>1</v>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>MOQ: 10000 — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="59">
@@ -2696,8 +2810,10 @@
           <t>福建省晋江市经济开发区 (fú jiàn shěng jìn jiāng shì jīng jì kāi fā qū) 广东省深圳市龙华新区建设路与东环二路交汇处聚豪国际 (guǎng dōng shěng shēn zhèn shì lóng huá xīn qū jiàn shè lù yǔ dōng huán èr lù jiāo huì chù jù háo guó jì)A栋 (dòng)2504室 (shì)Room 2504, Building A, Juhuao International, Intersection of Jianshe Road and Donghuan 2nd Road, Longhua New District, Shenzhen City, Guangdong Province; Jinjiang Economic Development Zone, Jinjiang City, Fujian Province</t>
         </is>
       </c>
-      <c r="I59" t="n">
-        <v>1</v>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Under discussion with suplier for customization — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="60">
@@ -2739,8 +2855,10 @@
           <t>3rd Floor, Building 6, No. 25, Fuyuan 1st Road, Xinya Subdistrict, Huadu District, Guangzhou City, Guangdong Province</t>
         </is>
       </c>
-      <c r="I60" t="n">
-        <v>1</v>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>MOQ: 0,3 — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="61">
@@ -2777,8 +2895,10 @@
           <t>www.kingswin.com</t>
         </is>
       </c>
-      <c r="I61" t="n">
-        <v>1</v>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>1.8-2RmbMoQ — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="62">
@@ -2820,8 +2940,10 @@
           <t>N2.Dongye Rd., Houjie Town, Dongguan City Guangdong Province China</t>
         </is>
       </c>
-      <c r="I62" t="n">
-        <v>1</v>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>0.8RMB — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="63">
@@ -2853,8 +2975,10 @@
           <t>Guangzhou, China</t>
         </is>
       </c>
-      <c r="I63" t="n">
-        <v>1</v>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>good — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="64">
@@ -2886,8 +3010,10 @@
           <t>hyde@merrynewon.com</t>
         </is>
       </c>
-      <c r="I64" t="n">
-        <v>2</v>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>MOQ 5000. Price 3 yuanes — покупатель / байер; Pump bottles for liquid lotion or foundation. Moq 5000 pieces — покупатель / бай</t>
+        </is>
       </c>
     </row>
     <row r="65">
@@ -2929,8 +3055,10 @@
           <t>The 2nd Industrial Zone, Tuanjie Road, Tuanjie Village, Xinya Street, Huadu District, Guangzhou Building Cle, Wanyang Zhongchuang City, 41 Dawang Avenue, High-tech Zone, Zhaoqing, Guangdong Province</t>
         </is>
       </c>
-      <c r="I65" t="n">
-        <v>1</v>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>2,12 rnb — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="66">
@@ -2972,8 +3100,10 @@
           <t>The 2nd Industrial Zone, Tuanjie Road, Tuanjie Village, Xinya Street, Huadu District, Guangzhou. Building C11#, Wanyang Zhongchuang City, 41 Dawang Avenue, High-tech Zone, Zhaoqing, Guangdong Province</t>
         </is>
       </c>
-      <c r="I66" t="n">
-        <v>2</v>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>6,5 per piece , MOQ 15,000 — покупатель / байер; Price is 3 RMB, MOQ is 15000 pieces, quality was outstanding — покупатель / байе</t>
+        </is>
       </c>
     </row>
     <row r="67">
@@ -3010,8 +3140,10 @@
           <t>广州市天河区林和东路 (guǎng zhōu shì tiān hé qū lín hé dōng lù)285号中汇人寿 (hào zhōng huì rén shòu)901Room 901, Zhonghui Life Insurance, No. 285 Linhe East Road, Tianhe District, Guangzhou City</t>
         </is>
       </c>
-      <c r="I67" t="n">
-        <v>1</v>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>Good — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="68">
@@ -3053,8 +3185,10 @@
           <t>Guangzhou Qian Zi non-woven products Co., LTD</t>
         </is>
       </c>
-      <c r="I68" t="n">
-        <v>1</v>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>0,8 yuan/piece, хорошие впечатления — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="69">
@@ -3096,8 +3230,10 @@
           <t>广州市白云区鶴拳路一横路科我园 (guǎng zhōu shì bái yún qū hè quán lù yī héng lù kē wǒ yuán)3栋 (dòng)Building 3, Kewoyuan, Yiheng Road, Hequan Road, Baiyun District, Guangzhou City</t>
         </is>
       </c>
-      <c r="I69" t="n">
-        <v>2</v>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>MOQ: 5000 pcs — покупатель / байер; 10, good — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="70">
@@ -3134,8 +3270,10 @@
           <t>No.107, Guanglong Road, Zhongluotan, Baiyun District, Guangzhou,China</t>
         </is>
       </c>
-      <c r="I70" t="n">
-        <v>1</v>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>3/item — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="71">
@@ -3177,8 +3315,10 @@
           <t>No. 120 Wai huan Road, Rong gui Shun de, Foshan City, Guangdong China</t>
         </is>
       </c>
-      <c r="I71" t="n">
-        <v>2</v>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>USD 1- 7 MOQ 10.000 — покупатель / байер; 1000 MOQ , 25rmb per piece — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="72">
@@ -3220,8 +3360,10 @@
           <t>No. 18, Nidong Road, Niliang Village, Xiaoyue Street, Shangyu District, Shaoxing City, Zhejiang Province 312367, China</t>
         </is>
       </c>
-      <c r="I72" t="n">
-        <v>1</v>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>MOQ 1000, price 10 yuanes — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="73">
@@ -3253,8 +3395,10 @@
           <t>No. 1 Zizhong Road, Heping Town, Chaoyang District, Shantou515141, Guangdong, China</t>
         </is>
       </c>
-      <c r="I73" t="n">
-        <v>2</v>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>0.9$ — покупатель / байер; Price 6.5; MOQ 5000 — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="74">
@@ -3296,8 +3440,10 @@
           <t>Building E1, Huangpu Technology Headquarters Port, Liandong U Valley, No. 10, Xicheng Middle Street, Nanwan, Huangpu District, Guangzhou, Guangdong, China</t>
         </is>
       </c>
-      <c r="I74" t="n">
-        <v>1</v>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>2/item — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="75">
@@ -3334,8 +3480,10 @@
           <t>Floor 4, Building C, Shengmeng Industrial Park, No.70 Xiangxia Avenue, Longgui, Taihe Town, Baiyun District, Guangzhou, China</t>
         </is>
       </c>
-      <c r="I75" t="n">
-        <v>4</v>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>Price 10-15 rmb — покупатель / байер; MOQ 3000 12 rmb good quality boxes many different design, quality good — покупат; 1.8 RMB, MOQ10000 for customized design — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="76">
@@ -3372,8 +3520,10 @@
           <t>Building F, North of Nan 'ao Road, Jinping District, Shantou City, Guangdong Province</t>
         </is>
       </c>
-      <c r="I76" t="n">
-        <v>2</v>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>10000*0.3USD — покупатель / байер; 2,8 rmb, MOQ 12000 — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="77">
@@ -3410,8 +3560,10 @@
           <t>汕头市金平区岐山街道中宫社区建明工业城 (shàn tóu shì jīn píng qū qí shān jiē dào zhōng gōng shè qū jiàn míng gōng yè chéng)11-12栋楼 (dòng lóu)Buildings 11-12, Jianming Industrial City, Zhonggong Community, Qishan Street, Jinping District, Shantou City</t>
         </is>
       </c>
-      <c r="I77" t="n">
-        <v>1</v>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>Fully satisfied — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="78">
@@ -3453,8 +3605,10 @@
           <t>Add:Dongfeng Link Town, South Jinjiang Rd, Shantou, Guangdong Province, China, Post Code: 521244</t>
         </is>
       </c>
-      <c r="I78" t="n">
-        <v>2</v>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>1.25RMB/pc, 30000 pcs, contacts exchange — покупатель / байер; 3.5 good — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="79">
@@ -3491,8 +3645,10 @@
           <t>No.1 Zizhong Road, Heping Town, Chaoyang District, Shantou 515141, Guangdong, China</t>
         </is>
       </c>
-      <c r="I79" t="n">
-        <v>3</v>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>MOQ: 12000 pcs — покупатель / байер; 5000USD — покупатель / байер; good — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="80">
@@ -3534,8 +3690,10 @@
           <t>B4, Baoyuan Industrial Zone, Jinping District, Shantou City, Guangdong Province</t>
         </is>
       </c>
-      <c r="I80" t="n">
-        <v>1</v>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>Price is 10 RMB, MOQ is 20000 pieces, quality was outstanding — покупатель / бай</t>
+        </is>
       </c>
     </row>
     <row r="81">
@@ -3577,8 +3735,10 @@
           <t>Umbrella Industrial Park, Songxia Town, Shangyu Dist., Shaoxing, Zhejiang, China (Mainland)</t>
         </is>
       </c>
-      <c r="I81" t="n">
-        <v>1</v>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>MOQ: 10000 — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="82">
@@ -3620,8 +3780,10 @@
           <t>Lihai Industry, Binhai New Town, Shaoxing City, Zhejiang Province, China</t>
         </is>
       </c>
-      <c r="I82" t="n">
-        <v>1</v>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>.5$, Minimum MOQ 3000pcs, only customization for bulk orders — покупатель / байе</t>
+        </is>
       </c>
     </row>
     <row r="83">
@@ -3658,8 +3820,10 @@
           <t>https://www.yastarplastic.com</t>
         </is>
       </c>
-      <c r="I83" t="n">
-        <v>1</v>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>MOQ: 8000 — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="84">
@@ -3701,8 +3865,10 @@
           <t>广州市赛康尼机械设备有限公司 (guǎng zhōu shì sài kāng ní jī xiè shè bèi yǒu xiàn gōng sī) 广州市黄埔区南岗街道中南街 (guǎng zhōu shì huáng pǔ qū nán gǎng jiē dào zhōng nán jiē)10号联系中心办公室楼南面主楼南面 (hào lián xì zhōng xīn bàn gōng shì lóu nán miàn zhǔ lóu nán miàn)Guangzhou Saikenni Machinery Equipment Co., Ltd. South side of the main building, south side of the Contact Center Office Building, No. 10, Zhongnan Street, Nangang Subdistrict, Huangpu District, Guangzhou</t>
         </is>
       </c>
-      <c r="I84" t="n">
-        <v>1</v>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>2 rmb 1000pcs — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="85">
@@ -3739,8 +3905,10 @@
           <t>Room 301, Building 6, 5th Indurstrial Park, Tianliao Community, Gongming Street, Guangming District, Shenzhen City, Guangdong Province, China</t>
         </is>
       </c>
-      <c r="I85" t="n">
-        <v>1</v>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>0.75 dollar per pieces, 1500 per pieces. — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="86">
@@ -3782,8 +3950,10 @@
           <t>广东佛山市顺德区伦教来涌工业区 (guǎng dōng fó shān shì shùn dé qū lún jiào lái yǒng gōng yè qū)Laiyong Industrial Zone, Lunqiao, Shunde District, Foshan City, Guangdong</t>
         </is>
       </c>
-      <c r="I86" t="n">
-        <v>2</v>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>Восхитительные — покупатель / байер; I liked the assortment and the prices — they offer good value for money — покупа</t>
+        </is>
       </c>
     </row>
     <row r="87">
@@ -3820,8 +3990,10 @@
           <t>http://www.suicel.com</t>
         </is>
       </c>
-      <c r="I87" t="n">
-        <v>1</v>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>5 yuan, good feedback — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="88">
@@ -3858,8 +4030,10 @@
           <t>广东省清远市清城区石角镇 (guǎng dōng shěng qīng yuǎn shì qīng chéng qū shí jiǎo zhèn)(广清产业园 (guǎng qīng chǎn yè yuán))兴园路 (xīng yuán lù)3号 (hào); 广州市花都区新雅街绿地空港五号地 (guǎng zhōu shì huā dōu qū xīn yǎ jiē lǜ dì kōng gǎng wǔ hào dì)4栋 (dòng)1107室 (shì)No. 3, Xingyuan Road, Shijiao Town (Guangqing Industrial Park), Qingcheng District, Qingyuan City, Guangdong Province; Room 1107, Building 4, Plot 5, Greenland Airport, Xinya Street, Huadu District, Guangzhou City</t>
         </is>
       </c>
-      <c r="I88" t="n">
-        <v>1</v>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>10 rmb — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="89">
@@ -3891,8 +4065,10 @@
           <t>GraceCheng@taolinpack.com</t>
         </is>
       </c>
-      <c r="I89" t="n">
-        <v>1</v>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MOQ 10000 шт но можно и меньше. Вполне можно сотрудничать, но думаю можно найти </t>
+        </is>
       </c>
     </row>
     <row r="90">
@@ -3929,8 +4105,10 @@
           <t>浙江省嘉兴市南湖区新丰镇新禾路 (zhè jiāng shěng jiā xīng shì nán hú qū xīn fēng zhèn xīn hé lù)158号 (hào)No. 158, Xinhe Road, Xinfeng Town, Nanhu District, Jiaxing City, Zhejiang Province</t>
         </is>
       </c>
-      <c r="I90" t="n">
-        <v>1</v>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>1500 - 25 — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="91">
@@ -3972,8 +4150,10 @@
           <t>江苏省泰兴市江平北路 (jiāng sū shěng tài xīng shì jiāng píng běi lù)55号 (hào), 上海市徐汇区石龙路 (shàng hǎi shì xú huì qū shí lóng lù)6号 (hào)001室 (shì)No. 55 Jiangping North Road, Taixing City, Jiangsu Province, Room 001, No. 6 Shilong Road, Xuhui District, Shanghai City</t>
         </is>
       </c>
-      <c r="I91" t="n">
-        <v>1</v>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>30 rmb per person with a MOQ 500 — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="92">
@@ -4015,8 +4195,10 @@
           <t>No. Room 2308, North Tower, Jinbin Dragonfly Building, 49 Huaxia Road, Tianhe District, Guangzhou China.510623</t>
         </is>
       </c>
-      <c r="I92" t="n">
-        <v>1</v>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>MOQ:6000 Pcs — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="93">
@@ -4053,8 +4235,10 @@
           <t>www.tubest-packing.com</t>
         </is>
       </c>
-      <c r="I93" t="n">
-        <v>5</v>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>Based on design and Customisation — покупатель / байер; MOQ=10,000 meeting was very budget friendly.. product i like most — покупатель /; 7 rmb, Quality packaging, interesting options that I have not seen before — поку</t>
+        </is>
       </c>
     </row>
     <row r="94">
@@ -4091,8 +4275,10 @@
           <t>佛山市三水区乐平镇博裕路 (fó shān shì sān shuǐ qū lè píng zhèn bó yù lù)34号 (hào)1栋 (dòng)Building 1, No. 34, Boyu Road, Leping Town, Sanshui District, Foshan City</t>
         </is>
       </c>
-      <c r="I94" t="n">
-        <v>1</v>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>Price 6.5; MOQ 5000 — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="95">
@@ -4129,8 +4315,10 @@
           <t>上海市金山区漕泾开发区展业路 (shàng hǎi shì jīn shān qū cáo jīng kāi fā qū zhǎn yè lù)288号一栋 (hào yī dòng)Building 1, No. 288, Zhanye Road, Caojing Development Zone, Jinshan District, Shanghai</t>
         </is>
       </c>
-      <c r="I95" t="n">
-        <v>17</v>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>The price is good — покупатель / байер; The price ranges from 1 to 2 Chinese yuan if the order is large — покупатель / б; MOQ: 5000 — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="96">
@@ -4157,8 +4345,10 @@
           <t>hongsheng1688.com</t>
         </is>
       </c>
-      <c r="I96" t="n">
-        <v>1</v>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>Наклейки с логотипом для тары, могут производить от любого количества. Цена - 15</t>
+        </is>
       </c>
     </row>
     <row r="97">
@@ -4200,8 +4390,10 @@
           <t>5F,No.268, Huandong Road, Xuxiake Town, Jiangyin, Jiangsu, China, 214407</t>
         </is>
       </c>
-      <c r="I97" t="n">
-        <v>2</v>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>1.25rmb/unit. For 5000 droppers it will be 6250 rmb. — покупатель / байер; 1-5 — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="98">
@@ -4243,8 +4435,10 @@
           <t>608, Building 2, Greenland Airport Center Huadu District, Guangzhou City</t>
         </is>
       </c>
-      <c r="I98" t="n">
-        <v>4</v>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>От 2000, от 2.2 — покупатель / байер; MOQ: 1800 pcs — покупатель / байер; MOQ: 11200 pcs — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="99">
@@ -4286,8 +4480,10 @@
           <t>广东省汕头市月浦龙洲路 (guǎng dōng shěng shàn tóu shì yuè pǔ lóng zhōu lù)12号 (hào) Longzhou Road, Yuepu, Shantou City, Guangdong Province, China</t>
         </is>
       </c>
-      <c r="I99" t="n">
-        <v>1</v>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>1-10 — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="100">
@@ -4329,8 +4525,10 @@
           <t>广州市七星二号 (guǎng zhōu shì qī xīng èr hào)No. 2, Qixing, Guangzhou City</t>
         </is>
       </c>
-      <c r="I100" t="n">
-        <v>1</v>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>MOQ 2000, 15 rmb high quality boxes many   different design cooperation with big</t>
+        </is>
       </c>
     </row>
     <row r="101">
@@ -4367,8 +4565,10 @@
           <t>上海市嘉定区树屏路 (shàng hǎi shì jiā dìng qū shù píng lù)588弄财智金岸 (nòng cái zhì jīn àn)35号楼 (hào lóu)Building 35, Caizhi Jin'an, Lane 588, Shuping Road, Jiading District, Shanghai</t>
         </is>
       </c>
-      <c r="I101" t="n">
-        <v>4</v>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>RMB 1.20  per 100,000 units — покупатель / байер; MOQ 1000 pieces, each oye 2.5 dola — покупатель / байер; MOQ 1000 , 2.5 dollar — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="102">
@@ -4410,8 +4610,10 @@
           <t>No 68, Dongling Road, Houxi Town, Jimei District, Xiamen City, China</t>
         </is>
       </c>
-      <c r="I102" t="n">
-        <v>4</v>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>0, 2 usd for 1 yard (25cm), MOQ 1000, huge right off sample options — покупатель; 2,6$ 100 yard roll ribbon very good quality and very big choice, can make a prin; 0.5 — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="103">
@@ -4448,8 +4650,10 @@
           <t>Building 31, No.86, Maohai Road, Huangjiabu Town, Yuyao City, Zhejiang Province.</t>
         </is>
       </c>
-      <c r="I103" t="n">
-        <v>1</v>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>Interesting — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="104">
@@ -4491,8 +4695,10 @@
           <t>No. 183 Beixing Road, Mazhu Town, Yuyao City, Zhejiang, China</t>
         </is>
       </c>
-      <c r="I104" t="n">
-        <v>2</v>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>8 rmb per sample — покупатель / байер; MOQ 10000шт, меньше производить не могут. Цена за интересующий продукт 2,1 юань.</t>
+        </is>
       </c>
     </row>
     <row r="105">
@@ -4534,8 +4740,10 @@
           <t>浙江省绍兴市上虞区崧厦街道振兴路 (zhè jiāng shěng shào xīng shì shàng yú qū sōng shà jiē dào zhèn xīng lù)138号 (hào)No. 138, Zhenxing Road, Songsha Street, Shangyu District, Shaoxing City, Zhejiang Province</t>
         </is>
       </c>
-      <c r="I105" t="n">
-        <v>1</v>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>5000*13,5RMB. Very nice sales managers — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="106">
@@ -4562,8 +4770,10 @@
           <t>13515733610</t>
         </is>
       </c>
-      <c r="I106" t="n">
-        <v>1</v>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>Moq  20HD, nice company — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="107">
@@ -4605,8 +4815,10 @@
           <t>15 Huachang Road, Mingwei Industrial Zone, Lizhou Street, Yuyao, Zhejiang, China. 168 Yuma Road, Mazhu Town, Yuyao, Zhejiang, China.</t>
         </is>
       </c>
-      <c r="I107" t="n">
-        <v>1</v>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>50000rmb ,the meeting was informative and helpfull. — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="108">
@@ -4643,8 +4855,10 @@
           <t>Building NO.1, Wanyang creation city, NO.68 Maohai Road, Huangjiabu Town, Yuyao city, Ningbo, Zhejiang Province, China</t>
         </is>
       </c>
-      <c r="I108" t="n">
-        <v>1</v>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>1-15 — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="109">
@@ -4681,8 +4895,10 @@
           <t>No. 10, Xingye West Road, Xinxu Village, Sanxiang Town, Zhongshan City, Guangdong China</t>
         </is>
       </c>
-      <c r="I109" t="n">
-        <v>1</v>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>4 RMB, 10000 pieces for MOQ, they have good quality products — покупатель / байе</t>
+        </is>
       </c>
     </row>
     <row r="110">
@@ -4719,8 +4935,10 @@
           <t>上海市松江区叶路 (shàng hǎi shì sōng jiāng qū yè lù)133弄 (nòng)1-3号 (hào)No. 1-3, Lane 133, Ye Road, Songjiang District, Shanghai</t>
         </is>
       </c>
-      <c r="I110" t="n">
-        <v>1</v>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>7rmb, 1000, very much interested in meeting — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="111">
@@ -4762,8 +4980,10 @@
           <t>广州市花都区花东镇微观产业园 (guǎng zhōu shì huā dōu qū huā dōng zhèn wēi guān chǎn yè yuán)C栋 (dòng)Building C, Weiguan Industrial Park, Huadong Town, Huadu District, Guangzhou</t>
         </is>
       </c>
-      <c r="I111" t="n">
-        <v>1</v>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>2.21$/pp — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="112">
@@ -4805,8 +5025,10 @@
           <t>浙江省余姚市牟山镇高车头 (zhè jiāng shěng yú yáo shì móu shān zhèn gāo chē tóu) B67号肖西路西 (hào xiào xī lù xī)West of Xiaoxi Road, Gaochetou, Mushan Town, Yuyao City, Zhejiang Province, No. B67</t>
         </is>
       </c>
-      <c r="I112" t="n">
-        <v>1</v>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>The price is 2.6 rmb, MOQ- 5000, good quality products and reasonable price. — п</t>
+        </is>
       </c>
     </row>
     <row r="113">
@@ -4848,8 +5070,10 @@
           <t>浙江省余姚市马渚镇北兴路 (zhè jiāng shěng yú yáo shì mǎ zhǔ zhèn běi xīng lù)183号 (hào)No. 183, Beixing Road, Mazhu Town, Yuyao City, Zhejiang Province</t>
         </is>
       </c>
-      <c r="I113" t="n">
-        <v>1</v>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>MOQ=10,000 meeting was friendly product good quality — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="114">
@@ -4891,8 +5115,10 @@
           <t>廣東省東莞市厚街鎮東業路 (guǎng dōng shěng dōng guǎn shì hòu jiē zhèn dōng yè lù)2號 (hào)No. 2, Dongye Road, Houjie Town, Dongguan City, Guangdong Province</t>
         </is>
       </c>
-      <c r="I114" t="n">
-        <v>1</v>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>9rmb , good quality — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="115">
@@ -4929,8 +5155,10 @@
           <t>广州市花都区绿港四街 (guǎng zhōu shì huā dōu qū lǜ gǎng sì jiē)6号 (hào)No. 6, Lvgong 4th Street, Huadu District, Guangzhou</t>
         </is>
       </c>
-      <c r="I115" t="n">
-        <v>6</v>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>2:5rmb 10000pcs — покупатель / байер; 5000p,  4.2y — покупатель / байер; 10000p, 2.5y — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="116">
@@ -4967,8 +5195,10 @@
           <t>https://chenmascosmetic.on.made-in-china.com</t>
         </is>
       </c>
-      <c r="I116" t="n">
-        <v>1</v>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>3RMB/pc, 1000 pcs, contacts exchange — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="117">
@@ -5005,8 +5235,10 @@
           <t>广州市白云区江高镇神山神石路 (guǎng zhōu shì bái yún qū jiāng gāo zhèn shén shān shén shí lù)41号 (hào)No. 41, Shenshan Shishen Road, Jianggao Town, Baiyun District, Guangzhou</t>
         </is>
       </c>
-      <c r="I117" t="n">
-        <v>1</v>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>2,4 yuan/piece. Отличные впечатления — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="118">
@@ -5048,8 +5280,10 @@
           <t>广东省广州市天河区科韵路 (guǎng dōng shěng guǎng zhōu shì tiān hé qū kē yùn lù)288号天盈创意园 (hào tiān yíng chuàng yì yuán) C区 (qū)3024-3027Rooms 3024-3027, Area C, Tianying Creative Park, No. 288 Keyun Road, Tianhe District, Guangzhou City, Guangdong Province</t>
         </is>
       </c>
-      <c r="I118" t="n">
-        <v>2</v>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>39rmb, 600 pcs — покупатель / байер; 20 Rmb , 15 pice — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="119">
@@ -5081,8 +5315,10 @@
           <t>广东省广州市花都区金田路 (guǎng dōng shěng guǎng zhōu shì huā dōu qū jīn tián lù)3号 (hào)No. 3, Jintian Road, Huadu District, Guangzhou City, Guangdong Province</t>
         </is>
       </c>
-      <c r="I119" t="n">
-        <v>4</v>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>13rmb , good quality — покупатель / байер; MOQ: 2000 — покупатель / байер; Sticker MOQ: 10k PCS — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="120">
@@ -5119,8 +5355,10 @@
           <t>广州市白云区北太路 (guǎng zhōu shì bái yún qū běi tài lù)1633号广州民营科技园科园路 (hào guǎng zhōu mín yíng kē jì yuán kē yuán lù)2号凯铂中心 (hào kǎi bó zhōng xīn)D区 (qū)1-4楼 (lóu) 1-4 F, Area D. Kaibo Center Building, No.2 Keyuan Road, Guangzhou Private Science and Technology Park, No. 1633 Beitai Road, Baiyun District, Guangzhou</t>
         </is>
       </c>
-      <c r="I120" t="n">
-        <v>1</v>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>depend on the product, good feedback — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="121">
@@ -5152,8 +5390,10 @@
           <t>广东省清远市佛冈县汤塘镇广佛产业园创业路 (guǎng dōng shěng qīng yuǎn shì fú gāng xiàn tāng táng zhèn guǎng fú chǎn yè yuán chuàng yè lù)7号 (hào) C区 (qū)6栋 (dòng)101-501房 (fáng)Room 101-501, Building 6, Zone C, No. 7, Chuangye Road, Guangfo Industrial Park, Tangtang Town, Fogang County, Qingyuan City, Guangdong Province</t>
         </is>
       </c>
-      <c r="I121" t="n">
-        <v>2</v>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>2,5 rmb, 10000 pcs, good quality — покупатель / байер; 45rmb, 400pcs — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="122">
@@ -5195,8 +5435,10 @@
           <t>广州市白云区江高镇 (guǎng zhōu shì bái yún qū jiāng gāo zhèn)408号工业园 (hào gōng yè yuán) A区 (qū) 11/F Building 7 Awang Industrial Zone, Baiyun District, Guangzhou City</t>
         </is>
       </c>
-      <c r="I122" t="n">
-        <v>1</v>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>5-10 — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="123">
@@ -5238,8 +5480,10 @@
           <t>中山工厂 (zhōng shān gōng chǎng):广东省中山市火炬开发区茂南路 (guǎng dōng shěng zhōng shān shì huǒ jù kāi fā qū mào nán lù)25号 (hào) 惠州工厂 (huì zhōu gōng chǎng):广东省惠州市龙门县金山工业园建设路 (guǎng dōng shěng huì zhōu shì lóng mén xiàn jīn shān gōng yè yuán jiàn shè lù)2号 (hào)Zhongshan Factory: No. 25, Maonan Road, Torch Development Zone, Zhongshan City, Guangdong Province; Huizhou Factory: No. 2, Jianshe Road, Jinshan Industrial Park, Longmen County, Huizhou City, Guangdong Province</t>
         </is>
       </c>
-      <c r="I123" t="n">
-        <v>2</v>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>MOQ: 12000 pcs — покупатель / байер; 7000USD — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="124">
@@ -5276,8 +5520,10 @@
           <t>广州天河区广州大道中 (guǎng zhōu tiān hé qū guǎng zhōu dà dào zhōng)307号富力东山新天地中心 (hào fù lì dōng shān xīn tiān dì zhōng xīn)42楼 (lóu)(总部营销中心 (zǒng bù yíng xiāo zhōng xīn))42nd Floor (Headquarters Marketing Center), Fuli Dongshan Xintiandi Center, No. 307 Guangzhou Avenue Middle, Tianhe District, Guangzhou</t>
         </is>
       </c>
-      <c r="I124" t="n">
-        <v>1</v>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>Mouth freshener 1RMB , MOQ 5000 — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="125">
@@ -5319,8 +5565,10 @@
           <t>广州市白云区云城东路云理汇 (guǎng zhōu shì bái yún qū yún chéng dōng lù yún lǐ huì)2栋 (dòng)3楼 (lóu)3rd Floor, Building 2, Yunlihui, Yuncheng East Road, Baiyun District, Guangzhou</t>
         </is>
       </c>
-      <c r="I125" t="n">
-        <v>1</v>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>20rmb, 1000, very much interested in making order — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="126">
@@ -5357,8 +5605,10 @@
           <t>广州市从化区明珠工业园宝聚路二号 (guǎng zhōu shì cóng huà qū míng zhū gōng yè yuán bǎo jù lù èr hào)No. 2, Baoju Road, Mingzhu Industrial Park, Conghua District, Guangzhou City</t>
         </is>
       </c>
-      <c r="I126" t="n">
-        <v>4</v>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>1000 MOQ, 0.25USD single piece — покупатель / байер; 1.5$ — покупатель / байер; Price 6 RMB; MOQ 5000 — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="127">
@@ -5395,8 +5645,10 @@
           <t>广州市白云区江高镇神山神石路 (guǎng zhōu shì bái yún qū jiāng gāo zhèn shén shān shén shí lù)41号 (hào)No. 41, Shenshan Shishen Road, Jianggao Town, Baiyun District, Guangzhou</t>
         </is>
       </c>
-      <c r="I127" t="n">
-        <v>2</v>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>0.045rmb , good quality — покупатель / байер; MOQ: 0,2 — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="128">
@@ -5428,8 +5680,10 @@
           <t>广东省广州市花都区花东镇北兴北钟路 (guǎng dōng shěng guǎng zhōu shì huā dōu qū huā dōng zhèn běi xīng běi zhōng lù)54号 (hào)No. 54, Beixing Beizhong Road, Huadong Town, Huadu District, Guangzhou City, Guangdong Province</t>
         </is>
       </c>
-      <c r="I128" t="n">
-        <v>1</v>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>Цены разные, всё сложно, Хорошо — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="129">
@@ -5471,8 +5725,10 @@
           <t>佛山市三水区乐平镇博裕路 (fó shān shì sān shuǐ qū lè píng zhèn bó yù lù)34号 (hào)1栋 (dòng)Building 1, No. 34, Boyu Road, Leping Town, Sanshui District, Foshan City</t>
         </is>
       </c>
-      <c r="I129" t="n">
-        <v>1</v>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>Price 4,8 MOQ 20,000 they were nice and welcoming — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="130">
@@ -5509,8 +5765,10 @@
           <t>广州市白云区云城西路娇兰佳人大厦 (guǎng zhōu shì bái yún qū yún chéng xī lù jiāo lán jiā rén dà shà)10楼 (lóu)10th Floor, Jiaolan Jiada Building, Yuncheng West Road, Baiyun District, Guangzhou City</t>
         </is>
       </c>
-      <c r="I130" t="n">
-        <v>1</v>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>Good — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="131">
@@ -5552,8 +5810,10 @@
           <t>广州市白云区三元里大道 (guǎng zhōu shì bái yún qū sān yuán lǐ dà dào)11号中港皮具城 (hào zhōng gǎng pí jù chéng)10楼 (lóu)1009室 (shì)Room 1009, 10th Floor, Zhonggang Leather City, No. 11, Sanyuanli Avenue, Baiyun District, Guangzhou City</t>
         </is>
       </c>
-      <c r="I131" t="n">
-        <v>1</v>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>USD 3-5 MOQ 3.000- 10.000 — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="132">
@@ -5590,8 +5850,10 @@
           <t>广州市越秀区先烈中路 (guǎng zhōu shì yuè xiù qū xiān liè zhōng lù)85号浙江大厦 (hào zhè jiāng dà shà)9楼 (lóu)9th Floor, Zhejiang Building, No. 85, Xianlie Middle Road, Yuexiu District, Guangzhou City</t>
         </is>
       </c>
-      <c r="I132" t="n">
-        <v>2</v>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>RMB 0.20  per 100,000 units — покупатель / байер; Brand Product QR code 0.001/ piece MOQ 100000 — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="133">
@@ -5628,8 +5890,10 @@
           <t>广州市从化区横江路 (guǎng zhōu shì cóng huà qū héng jiāng lù)339号 (hào) -36号鸿志软管 (hào hóng zhì ruǎn guǎn)Hongzhi Hose, No. 339-36, Hengjiang Road, Conghua District, Guangzhou City</t>
         </is>
       </c>
-      <c r="I133" t="n">
-        <v>1</v>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>30 RMB, MOQ 10000, good company — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="134">
@@ -5666,8 +5930,10 @@
           <t>广州市白云区太和镇谢家注兰西路 (guǎng zhōu shì bái yún qū tài hé zhèn xiè jiā zhù lán xī lù)2号 (hào) No. 2 Yinian West Road, Xielazhuang, Taihe Town layun District, Duangzhou City</t>
         </is>
       </c>
-      <c r="I134" t="n">
-        <v>1</v>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>5.5, good — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="135">
@@ -5699,8 +5965,10 @@
           <t>广州市白云区太和镇谢家庄荫兰西路 (guǎng zhōu shì bái yún qū tài hé zhèn xiè jiā zhuāng yīn lán xī lù)2号 (hào)No. 2, Yinlan West Road, Xiejiazhuang, Taihe Town, Baiyun District, Guangzhou City</t>
         </is>
       </c>
-      <c r="I135" t="n">
-        <v>1</v>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>3,5 rmb, MOQ 1000, good company — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="136">
@@ -5742,8 +6010,10 @@
           <t>广州市白云区龙归街南岭村岗埔大道 (guǎng zhōu shì bái yún qū lóng guī jiē nán lǐng cūn gǎng pǔ dà dào)1号 (hào)No. 1 Gangpu Avenue, Nanling Village, Longgui Street, Baiyun District, Guangzhou City</t>
         </is>
       </c>
-      <c r="I136" t="n">
-        <v>1</v>
+      <c r="I136" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10 - заказ от 100 единиц. очень качественно с нанесением фактуры — покупатель / </t>
+        </is>
       </c>
     </row>
     <row r="137">
@@ -5780,8 +6050,10 @@
           <t>No.1 Yongda Road, Huadong Town, Huadu District, Guangzhou City, Guangdong, China. Post Code510890</t>
         </is>
       </c>
-      <c r="I137" t="n">
-        <v>1</v>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>70000, feedback was fruitfull — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="138">
@@ -5813,8 +6085,10 @@
           <t>广州市花都区凤凰南路 (guǎng zhōu shì huā dōu qū fèng huáng nán lù)61号卓美大楼北楼 (hào zhuó měi dà lóu běi lóu)307室 (shì)Room 307, North Building, Zhuomei Building, No. 61, Fenghuang South Road, Huadu District, Guangzhou</t>
         </is>
       </c>
-      <c r="I138" t="n">
-        <v>2</v>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>5rmb 5000pcs — покупатель / байер; MIA 300, 18rmb — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="139">
@@ -5856,8 +6130,10 @@
           <t>廣州市白雲區龍歸街夏良東路 (guǎng zhōu shì bái yún qū lóng guī jiē xià liáng dōng lù)81號 (hào)102房 (fáng)Room 102, No. 81, Xialiang East Road, Longgui Street, Baiyun District, Guangzhou</t>
         </is>
       </c>
-      <c r="I139" t="n">
-        <v>1</v>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t>1000p, 1.5y — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="140">
@@ -5894,8 +6170,10 @@
           <t>廣州市花都區花山鎮城西村自編 (guǎng zhōu shì huā dōu qū huā shān zhèn chéng xī cūn zì biān)3號 (hào)No. 3 (self-numbered), Chengxi Village, Huashan Town, Huadu District, Guangzhou City</t>
         </is>
       </c>
-      <c r="I140" t="n">
-        <v>2</v>
+      <c r="I140" t="inlineStr">
+        <is>
+          <t>We need to talk on further details about the order — покупатель / байер; 0, 5 usd for MOQ 500, supplier with a nice quality — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="141">
@@ -5922,8 +6200,10 @@
           <t>广东省广州市花都区金田路 (guǎng dōng shěng guǎng zhōu shì huā dōu qū jīn tián lù)3号 (hào)No. 3, Jintian Road, Huadu District, Guangzhou City, Guangdong Province</t>
         </is>
       </c>
-      <c r="I141" t="n">
-        <v>1</v>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t>8 yuan for sunblock — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="142">
@@ -5960,8 +6240,10 @@
           <t>广东省清远市清城区石角镇 (guǎng dōng shěng qīng yuǎn shì qīng chéng qū shí jiǎo zhèn)(广清产业园 (guǎng qīng chǎn yè yuán))兴园路 (xīng yuán lù)3号 (hào); 广州市花都区新雅街绿地空港五号地 (guǎng zhōu shì huā dōu qū xīn yǎ jiē lǜ dì kōng gǎng wǔ hào dì)4栋 (dòng)1107室 (shì)No. 3, Xingyuan Road, Shijiao Town (Guangqing Industrial Park), Qingcheng District, Qingyuan City, Guangdong Province; Room 1107, Building 4, Plot 5, Greenland Airport, Xinya Street, Huadu District, Guangzhou City</t>
         </is>
       </c>
-      <c r="I142" t="n">
-        <v>1</v>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>0.65 dollar per pieces, 1000 pieces, the factory is really close the supplier ur</t>
+        </is>
       </c>
     </row>
     <row r="143">
@@ -5988,8 +6270,10 @@
           <t>18763000898</t>
         </is>
       </c>
-      <c r="I143" t="n">
-        <v>1</v>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>MOQ: 10000 pcs — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="144">
@@ -6021,8 +6305,10 @@
           <t>广州市白云区云城西路 (guǎng zhōu shì bái yún qū yún chéng xī lù)888号绿地中心 (hào lǜ dì zhōng xīn)2403Room 2403, Greenland Center, No. 888 Yuncheng West Road, Baiyun District, Guangzhou City</t>
         </is>
       </c>
-      <c r="I144" t="n">
-        <v>1</v>
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>12 RMB, 20000 pieces for MOQ, they have good quality products — покупатель / бай</t>
+        </is>
       </c>
     </row>
     <row r="145">
@@ -6054,8 +6340,10 @@
           <t>stcaihong2025@163.com</t>
         </is>
       </c>
-      <c r="I145" t="n">
-        <v>2</v>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>Невероятные — покупатель / байер; 10 rmb. Looks interesting, big choice — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="146">
@@ -6097,8 +6385,10 @@
           <t>浙江省绍兴市上虞区曹娥街道五星西路 (zhè jiāng shěng shào xīng shì shàng yú qū cáo é jiē dào wǔ xīng xī lù)1999号联东 (hào lián dōng)U谷 (gǔ)21栋 (dòng)C永 (yǒng), Add C tongin Bulding 21. Landong U Valley No. 1999, Wing West Road Cace Sheet, Shangyu District. Shocking City Zhellong ProvinceBuilding 21 C, Landong U Valley, No. 1999, Wuxing West Road, Cao'e Street, Shangyu District, Shaoxing City, Zhejiang Province</t>
         </is>
       </c>
-      <c r="I146" t="n">
-        <v>4</v>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1000 - 45 — покупатель / байер; Face roller 6.8 rmb per unit — покупатель / байер; 25rmb. . I was impressed by their professionalism and clear vision — покупатель </t>
+        </is>
       </c>
     </row>
     <row r="147">
@@ -6135,8 +6425,10 @@
           <t>浙江省平湖市新仓镇嘉创智谷远景产业园 (zhè jiāng shěng píng hú shì xīn cāng zhèn jiā chuàng zhì gǔ yuǎn jǐng chǎn yè yuán)A7栋 (dòng)Building A7, Jia Chuang Zhi Gu Yuan Jing Industrial Park, Xincang Town, Pinghu City, Zhejiang Province</t>
         </is>
       </c>
-      <c r="I147" t="n">
-        <v>2</v>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>0.1rmb, 5000pcs — покупатель / байер; 0,1 заказ от 1000 единиц — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="148">
@@ -6173,8 +6465,10 @@
           <t>江苏省淮安市洪泽区九牛路 (jiāng sū shěng huái ān shì hóng zé qū jiǔ niú lù)8号 (hào) 邮政编号 (yóu zhèng biān hào)223100No. 8, Jiuniu Road, Hongze District, Huai'an City, Jiangsu Province, Postal Code 223100</t>
         </is>
       </c>
-      <c r="I148" t="n">
-        <v>1</v>
+      <c r="I148" t="inlineStr">
+        <is>
+          <t>MOQ2000 USD0.20 — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="149">
@@ -6206,8 +6500,10 @@
           <t>广东省广州市花都区花山镇华辉路 (guǎng dōng shěng guǎng zhōu shì huā dōu qū huā shān zhèn huá huī lù)18号 (hào) 微观化妆品创意产业园 (wēi guān huà zhuāng pǐn chuàng yì chǎn yè yuán)D栋整栋 (dòng zhěng dòng)、H栋整栋 (dòng zhěng dòng)Entire Building D and Entire Building H, Weiguan Cosmetics Creative Industrial Park, No. 18, Huahui Road, Huashan Town, Huadu District, Guangzhou City, Guangdong Province</t>
         </is>
       </c>
-      <c r="I149" t="n">
-        <v>1</v>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>MOQ: 15 — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="150">
@@ -6239,8 +6535,10 @@
           <t>slana@wywbo.com</t>
         </is>
       </c>
-      <c r="I150" t="n">
-        <v>1</v>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>4 rmb — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="151">
@@ -6272,8 +6570,10 @@
           <t>广州市从化区太平镇新兴路 (guǎng zhōu shì cóng huà qū tài píng zhèn xīn xīng lù)439号 (hào)7栋 (dòng)Building 7, No. 439, Xinxing Road, Taiping Town, Conghua District, Guangzhou</t>
         </is>
       </c>
-      <c r="I151" t="n">
-        <v>2</v>
+      <c r="I151" t="inlineStr">
+        <is>
+          <t>MOQ: 10000 — покупатель / байер; Price: 5RMB, MOQ: 10000 — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="152">
@@ -6315,8 +6615,10 @@
           <t>苏州市吴江区江陵街道益堂路 (sū zhōu shì wú jiāng qū jiāng líng jiē dào yì táng lù)10号 (hào)No. 10 Yitang Road, Jiangling Street, Wujiang District, Suzhou City</t>
         </is>
       </c>
-      <c r="I152" t="n">
-        <v>1</v>
+      <c r="I152" t="inlineStr">
+        <is>
+          <t>8rmb, 200pcs — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="153">
@@ -6353,8 +6655,10 @@
           <t>浙江省龙港市世纪大道 (zhè jiāng shěng lóng gǎng shì shì jì dà dào)888号 (hào)No. 888, Century Avenue, Longgang City, Zhejiang Province</t>
         </is>
       </c>
-      <c r="I153" t="n">
-        <v>1</v>
+      <c r="I153" t="inlineStr">
+        <is>
+          <t>Under discussing — покупатель / байер</t>
+        </is>
       </c>
     </row>
     <row r="154">
@@ -6396,8 +6700,10 @@
           <t>广州市白云区均禾街石马村桃红西街 (guǎng zhōu shì bái yún qū jūn hé jiē shí mǎ cūn táo hóng xī jiē)58号 (hào)No. 58 Taohong West Street, Shima Village, Junhe Street, Baiyun District, Guangzhou City</t>
         </is>
       </c>
-      <c r="I154" t="n">
-        <v>2</v>
+      <c r="I154" t="inlineStr">
+        <is>
+          <t>10 RMB, 12000 pieces for MOQ, they have good quality products — покупатель / бай; 3000 MOQ, around 2rmb. Nice quality and company have VTB bank — покупатель / бай</t>
+        </is>
       </c>
     </row>
     <row r="155">
@@ -6419,7 +6725,6 @@
           <t>+86 21 5988 5200</t>
         </is>
       </c>
-      <c r="F155" t="inlineStr"/>
       <c r="G155" t="inlineStr">
         <is>
           <t>www.yingshuo.com</t>
@@ -6430,8 +6735,10 @@
           <t>188 Beiying Road, QingPu, Shanghai 201700</t>
         </is>
       </c>
-      <c r="I155" t="n">
-        <v>1</v>
+      <c r="I155" t="inlineStr">
+        <is>
+          <t>0 products</t>
+        </is>
       </c>
     </row>
     <row r="156">
@@ -6468,8 +6775,10 @@
           <t>No. 17 Langzhou Zhou Liao Road, Changping Town, Dongguan, Guangdong</t>
         </is>
       </c>
-      <c r="I156" t="n">
-        <v>1</v>
+      <c r="I156" t="inlineStr">
+        <is>
+          <t>0 products</t>
+        </is>
       </c>
     </row>
     <row r="157">
@@ -6506,8 +6815,10 @@
           <t>No.818 Shuanghe Road, Yuyao, Zhejiang</t>
         </is>
       </c>
-      <c r="I157" t="n">
-        <v>1</v>
+      <c r="I157" t="inlineStr">
+        <is>
+          <t>0 products</t>
+        </is>
       </c>
     </row>
     <row r="158">
@@ -6544,8 +6855,10 @@
           <t>No. 888 Beixing Road, Mazhu Town, Yuyao, Zhejiang</t>
         </is>
       </c>
-      <c r="I158" t="n">
-        <v>1</v>
+      <c r="I158" t="inlineStr">
+        <is>
+          <t>0 products</t>
+        </is>
       </c>
     </row>
     <row r="159">
@@ -6562,16 +6875,15 @@
           <t>Пластиковая упаковка</t>
         </is>
       </c>
-      <c r="E159" t="inlineStr"/>
-      <c r="F159" t="inlineStr"/>
-      <c r="G159" t="inlineStr"/>
       <c r="H159" t="inlineStr">
         <is>
           <t>No. 1 Industrial Avenue, Yaoli Town, Lu'an City, Anhui</t>
         </is>
       </c>
-      <c r="I159" t="n">
-        <v>1</v>
+      <c r="I159" t="inlineStr">
+        <is>
+          <t>0 products</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Remove duplicate Shanghai Yingshuo (#155)
</commit_message>
<xml_diff>
--- a/ipdf_suppliers.xlsx
+++ b/ipdf_suppliers.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I159"/>
+  <dimension ref="A1:I158"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -6743,36 +6743,36 @@
     </row>
     <row r="156">
       <c r="A156" t="n">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>Hepuur New Material (Guangdong)</t>
+          <t>Zhejiang Z&amp;Z (Zhengzhuang)</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>Новые материалы, Пластик</t>
+          <t>Пластиковая упаковка</t>
         </is>
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>+86 769 8779 9839</t>
+          <t>+86-574-58122625</t>
         </is>
       </c>
       <c r="F156" t="inlineStr">
         <is>
-          <t>info@hepuur.com</t>
+          <t>sales@z-z.cn</t>
         </is>
       </c>
       <c r="G156" t="inlineStr">
         <is>
-          <t>hepuur.com</t>
+          <t>www.zzpkg.com</t>
         </is>
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>No. 17 Langzhou Zhou Liao Road, Changping Town, Dongguan, Guangdong</t>
+          <t>No.818 Shuanghe Road, Yuyao, Zhejiang</t>
         </is>
       </c>
       <c r="I156" t="inlineStr">
@@ -6783,11 +6783,11 @@
     </row>
     <row r="157">
       <c r="A157" t="n">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>Zhejiang Z&amp;Z (Zhengzhuang)</t>
+          <t>Ningbo Laoshi / LPI Packaging</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
@@ -6797,22 +6797,22 @@
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>+86-574-58122625</t>
+          <t>+86-574-62465217</t>
         </is>
       </c>
       <c r="F157" t="inlineStr">
         <is>
-          <t>sales@z-z.cn</t>
+          <t>xu@jy-spayer.com</t>
         </is>
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>www.zzpkg.com</t>
+          <t>www.lpi-packaging.com</t>
         </is>
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>No.818 Shuanghe Road, Yuyao, Zhejiang</t>
+          <t>No. 888 Beixing Road, Mazhu Town, Yuyao, Zhejiang</t>
         </is>
       </c>
       <c r="I157" t="inlineStr">
@@ -6823,11 +6823,11 @@
     </row>
     <row r="158">
       <c r="A158" t="n">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>Ningbo Laoshi / LPI Packaging</t>
+          <t>Anhui Jusu Gaoke Packaging</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
@@ -6835,52 +6835,12 @@
           <t>Пластиковая упаковка</t>
         </is>
       </c>
-      <c r="E158" t="inlineStr">
-        <is>
-          <t>+86-574-62465217</t>
-        </is>
-      </c>
-      <c r="F158" t="inlineStr">
-        <is>
-          <t>xu@jy-spayer.com</t>
-        </is>
-      </c>
-      <c r="G158" t="inlineStr">
-        <is>
-          <t>www.lpi-packaging.com</t>
-        </is>
-      </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>No. 888 Beixing Road, Mazhu Town, Yuyao, Zhejiang</t>
+          <t>No. 1 Industrial Avenue, Yaoli Town, Lu'an City, Anhui</t>
         </is>
       </c>
       <c r="I158" t="inlineStr">
-        <is>
-          <t>0 products</t>
-        </is>
-      </c>
-    </row>
-    <row r="159">
-      <c r="A159" t="n">
-        <v>158</v>
-      </c>
-      <c r="B159" t="inlineStr">
-        <is>
-          <t>Anhui Jusu Gaoke Packaging</t>
-        </is>
-      </c>
-      <c r="C159" t="inlineStr">
-        <is>
-          <t>Пластиковая упаковка</t>
-        </is>
-      </c>
-      <c r="H159" t="inlineStr">
-        <is>
-          <t>No. 1 Industrial Avenue, Yaoli Town, Lu'an City, Anhui</t>
-        </is>
-      </c>
-      <c r="I159" t="inlineStr">
         <is>
           <t>0 products</t>
         </is>

</xml_diff>

<commit_message>
Translate all Excel: headers, categories, buyer comments for EN/ES/AR
</commit_message>
<xml_diff>
--- a/ipdf_suppliers.xlsx
+++ b/ipdf_suppliers.xlsx
@@ -487,7 +487,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Металлическая упаковка, Промышленное оборудование</t>
+          <t>Metal Packaging, Industrial Equipment</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -527,7 +527,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Металлическая упаковка, Пластиковая упаковка, Упаковочные материалы и аксессуары</t>
+          <t>Metal Packaging, Plastic Packaging, Packaging Materials &amp; Accessories</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -557,7 +557,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>1 rmb, 5000 pcs, nice manager — покупатель / байер</t>
+          <t>1 rmb, 5000 pcs, nice manager — buyer</t>
         </is>
       </c>
     </row>
@@ -572,7 +572,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Продукты на заказ / OEM, Упаковочные материалы и аксессуары, Промышленное оборудование</t>
+          <t>Custom Products / OEM, Packaging Materials &amp; Accessories, Industrial Equipment</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -597,7 +597,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>MOQ: 50 — покупатель / байер; MOQ 3000 RMB3 — покупатель / байер; 300 MOQ, 5 RMB per unit price. The prices are reasonable and packaging is really</t>
+          <t>MOQ: 50 — buyer; MOQ 3000 RMB3 — buyer; 300 MOQ, 5 RMB per unit price. The prices are reasonable and packaging is really</t>
         </is>
       </c>
     </row>
@@ -612,7 +612,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Упаковочные материалы и аксессуары, Промышленное оборудование</t>
+          <t>Packaging Materials &amp; Accessories, Industrial Equipment</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -642,7 +642,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>25rmb, 5000 pcs. Very friendly staff. — покупатель / байер</t>
+          <t>25rmb, 5000 pcs. Very friendly staff. — buyer</t>
         </is>
       </c>
     </row>
@@ -657,7 +657,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Продукты на заказ / OEM, Промышленное оборудование, Металлическая упаковка</t>
+          <t>Custom Products / OEM, Industrial Equipment, Metal Packaging</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -682,7 +682,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Interesting — покупатель / байер</t>
+          <t>Interesting — buyer</t>
         </is>
       </c>
     </row>
@@ -697,7 +697,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Продукты на заказ / OEM, Промышленное оборудование</t>
+          <t>Custom Products / OEM, Industrial Equipment</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -727,7 +727,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>10000 peices — покупатель / байер</t>
+          <t>10000 peices — buyer</t>
         </is>
       </c>
     </row>
@@ -742,7 +742,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Продукты на заказ / OEM</t>
+          <t>Custom Products / OEM</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -757,7 +757,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>20yuan/pcs, 500yuan moq — покупатель / байер; Good — покупатель / байер</t>
+          <t>20yuan/pcs, 500yuan moq — buyer; Good — buyer</t>
         </is>
       </c>
     </row>
@@ -772,7 +772,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Биотехнологии и фармацевтика, Косметика и уход, Продукты на заказ / OEM</t>
+          <t>Biotechnology &amp; Pharmaceuticals, Cosmetics &amp; Care, Custom Products / OEM</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -802,7 +802,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Price=0.35..MOQ-500/COLOR..GOOD. — покупатель / байер; Under discussion price and moq — покупатель / байер; 1-09$ good — покупатель / байер</t>
+          <t>Price=0.35..MOQ-500/COLOR..GOOD. — buyer; Under discussion price and moq — buyer; 1-09$ good — buyer</t>
         </is>
       </c>
     </row>
@@ -817,7 +817,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Косметика и уход, Упаковочные материалы и аксессуары, Промышленное оборудование</t>
+          <t>Cosmetics &amp; Care, Packaging Materials &amp; Accessories, Industrial Equipment</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -847,7 +847,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>30000USD — покупатель / байер</t>
+          <t>30000USD — buyer</t>
         </is>
       </c>
     </row>
@@ -862,7 +862,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Аэрозольная продукция, Упаковочные материалы и аксессуары, Продукты на заказ / OEM</t>
+          <t>Aerosol Products, Packaging Materials &amp; Accessories, Custom Products / OEM</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -892,7 +892,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>6000 MOQ. Very interesting. Something new — покупатель / байер</t>
+          <t>6000 MOQ. Very interesting. Something new — buyer</t>
         </is>
       </c>
     </row>
@@ -907,7 +907,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Упаковочные материалы и аксессуары, Продукты на заказ / OEM</t>
+          <t>Packaging Materials &amp; Accessories, Custom Products / OEM</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -937,7 +937,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>5,7¥ — покупатель / байер; 10-20 — покупатель / байер; 0.2$- Minimum MOQ 10000 pcs, offering customization — покупатель / байер</t>
+          <t>5,7¥ — buyer; 10-20 — buyer; 0.2$- Minimum MOQ 10000 pcs, offering customization — buyer</t>
         </is>
       </c>
     </row>
@@ -952,7 +952,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Металлическая упаковка, Гибкая упаковка и тубы</t>
+          <t>Metal Packaging, Flexible Packaging &amp; Tubes</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -982,7 +982,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Aluminum foil/tin/10000msquare — покупатель / байер</t>
+          <t>Aluminum foil/tin/10000msquare — buyer</t>
         </is>
       </c>
     </row>
@@ -997,7 +997,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Косметика и уход, Упаковочные материалы и аксессуары</t>
+          <t>Cosmetics &amp; Care, Packaging Materials &amp; Accessories</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1022,7 +1022,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>MOQ=12,000 products good — покупатель / байер; 12000 PCS MOQ — покупатель / байер; 6000 peices — покупатель / байер</t>
+          <t>MOQ=12,000 products good — buyer; 12000 PCS MOQ — buyer; 6000 peices — buyer</t>
         </is>
       </c>
     </row>
@@ -1037,7 +1037,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Пластиковая упаковка, Упаковочные материалы и аксессуары</t>
+          <t>Plastic Packaging, Packaging Materials &amp; Accessories</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1067,7 +1067,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>0,8-1,2RMB, MOQ10000 — покупатель / байер</t>
+          <t>0,8-1,2RMB, MOQ10000 — buyer</t>
         </is>
       </c>
     </row>
@@ -1082,7 +1082,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Электроника и цифровые решения</t>
+          <t>Electronics &amp; Digital Solutions</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1097,7 +1097,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>MOQ: 500 — покупатель / байер; MOQ: 500, Price: 220 RMB per price — покупатель / байер; MOQ: 4,1 — покупатель / байер</t>
+          <t>MOQ: 500 — buyer; MOQ: 500, Price: 220 RMB per price — buyer; MOQ: 4,1 — buyer</t>
         </is>
       </c>
     </row>
@@ -1112,7 +1112,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Бумажная упаковка и печать, Упаковочные материалы и аксессуары</t>
+          <t>Paper Packaging &amp; Printing, Packaging Materials &amp; Accessories</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1127,7 +1127,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>45-55 — покупатель / байер; 100-20-30юань от 1000 шт цена меньше — покупатель / байер</t>
+          <t>45-55 — buyer; 100-20-30юань от 1000 шт цена меньше — buyer</t>
         </is>
       </c>
     </row>
@@ -1142,7 +1142,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Биотехнологии и фармацевтика, Косметика и уход</t>
+          <t>Biotechnology &amp; Pharmaceuticals, Cosmetics &amp; Care</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1162,7 +1162,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>MOQ 400, 16.3rmb/шт. — покупатель / байер</t>
+          <t>MOQ 400, 16.3rmb/шт. — buyer</t>
         </is>
       </c>
     </row>
@@ -1177,7 +1177,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Упаковочные материалы и аксессуары, Пластиковая упаковка</t>
+          <t>Packaging Materials &amp; Accessories, Plastic Packaging</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1197,7 +1197,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>6-12 RMB, MOQ 12000 — покупатель / байер</t>
+          <t>6-12 RMB, MOQ 12000 — buyer</t>
         </is>
       </c>
     </row>
@@ -1212,7 +1212,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Упаковочные материалы и аксессуары, Электроника и цифровые решения</t>
+          <t>Packaging Materials &amp; Accessories, Electronics &amp; Digital Solutions</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1242,7 +1242,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Good — покупатель / байер; Satisfied with the companies discussion is on the way — покупатель / байер</t>
+          <t>Good — buyer; Satisfied with the companies discussion is on the way — buyer</t>
         </is>
       </c>
     </row>
@@ -1257,7 +1257,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Биотехнологии и фармацевтика, Косметика и уход</t>
+          <t>Biotechnology &amp; Pharmaceuticals, Cosmetics &amp; Care</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1282,7 +1282,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>20k — покупатель / байер; 20/item — покупатель / байер</t>
+          <t>20k — buyer; 20/item — buyer</t>
         </is>
       </c>
     </row>
@@ -1297,7 +1297,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Промышленное оборудование, Упаковочные материалы и аксессуары</t>
+          <t>Industrial Equipment, Packaging Materials &amp; Accessories</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1327,7 +1327,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>1,9¥ — покупатель / байер; The streamline material is 130 to 150 rmb per kg. — покупатель / байер</t>
+          <t>1,9¥ — buyer; The streamline material is 130 to 150 rmb per kg. — buyer</t>
         </is>
       </c>
     </row>
@@ -1342,7 +1342,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Косметика и уход</t>
+          <t>Cosmetics &amp; Care</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1372,7 +1372,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>10000 MOQ. Like this factory too — покупатель / байер</t>
+          <t>10000 MOQ. Like this factory too — buyer</t>
         </is>
       </c>
     </row>
@@ -1387,7 +1387,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Косметика и уход</t>
+          <t>Cosmetics &amp; Care</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1402,7 +1402,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>They will send the price list after the exhibition — покупатель / байер</t>
+          <t>They will send the price list after the exhibition — buyer</t>
         </is>
       </c>
     </row>
@@ -1417,7 +1417,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Упаковочные материалы и аксессуары</t>
+          <t>Packaging Materials &amp; Accessories</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1437,7 +1437,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>200Rmb set, 50 set — покупатель / байер</t>
+          <t>200Rmb set, 50 set — buyer</t>
         </is>
       </c>
     </row>
@@ -1452,7 +1452,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Биотехнологии и фармацевтика</t>
+          <t>Biotechnology &amp; Pharmaceuticals</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1472,7 +1472,7 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>35 RMB, MOQ 5000, Good company — покупатель / байер</t>
+          <t>35 RMB, MOQ 5000, Good company — buyer</t>
         </is>
       </c>
     </row>
@@ -1487,7 +1487,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Электроника и цифровые решения</t>
+          <t>Electronics &amp; Digital Solutions</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1512,7 +1512,7 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>10k — покупатель / байер</t>
+          <t>10k — buyer</t>
         </is>
       </c>
     </row>
@@ -1527,7 +1527,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Упаковочные материалы и аксессуары</t>
+          <t>Packaging Materials &amp; Accessories</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1552,7 +1552,7 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>400, 15rmb — покупатель / байер</t>
+          <t>400, 15rmb — buyer</t>
         </is>
       </c>
     </row>
@@ -1567,7 +1567,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Упаковочные материалы и аксессуары</t>
+          <t>Packaging Materials &amp; Accessories</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1597,7 +1597,7 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>MOQ 5000. Price 7 yuanes — покупатель / байер</t>
+          <t>MOQ 5000. Price 7 yuanes — buyer</t>
         </is>
       </c>
     </row>
@@ -1612,7 +1612,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Промышленное оборудование</t>
+          <t>Industrial Equipment</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1642,7 +1642,7 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Превосходные — покупатель / байер; MOQ: 1500 pcs — покупатель / байер</t>
+          <t>Превосходные — buyer; MOQ: 1500 pcs — buyer</t>
         </is>
       </c>
     </row>
@@ -1657,7 +1657,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Бумажная упаковка и печать</t>
+          <t>Paper Packaging &amp; Printing</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1677,7 +1677,7 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>0.3 yuan/piece, хорошие впечатления — покупатель / байер; We need to talk on further details about the order — покупатель / байер</t>
+          <t>0.3 yuan/piece, хорошие впечатления — buyer; We need to talk on further details about the order — buyer</t>
         </is>
       </c>
     </row>
@@ -1692,7 +1692,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Биотехнологии и фармацевтика, Косметика и уход</t>
+          <t>Biotechnology &amp; Pharmaceuticals, Cosmetics &amp; Care</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1722,7 +1722,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Anti-aging kit 35 rmb per piece MOQ 5000 pieces — покупатель / байер; 30 rmb one box, good — покупатель / байер</t>
+          <t>Anti-aging kit 35 rmb per piece MOQ 5000 pieces — buyer; 30 rmb one box, good — buyer</t>
         </is>
       </c>
     </row>
@@ -1737,7 +1737,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Косметика и уход</t>
+          <t>Cosmetics &amp; Care</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1767,7 +1767,7 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>200000 rmb, MOQ 1 — покупатель / байер</t>
+          <t>200000 rmb, MOQ 1 — buyer</t>
         </is>
       </c>
     </row>
@@ -1782,7 +1782,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Текстиль и нетканые материалы, Продукты на заказ / OEM, Косметика и уход</t>
+          <t>Textiles &amp; Nonwovens, Custom Products / OEM, Cosmetics &amp; Care</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1802,7 +1802,7 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>1.2RMB — покупатель / байер; 4 yuan, good feedback — покупатель / байер</t>
+          <t>1.2RMB — buyer; 4 yuan, good feedback — buyer</t>
         </is>
       </c>
     </row>
@@ -1817,7 +1817,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Текстиль и нетканые материалы, Косметика и уход, Бумажная упаковка и печать</t>
+          <t>Textiles &amp; Nonwovens, Cosmetics &amp; Care, Paper Packaging &amp; Printing</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1852,7 +1852,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Бумажная упаковка и печать, Упаковочные материалы и аксессуары</t>
+          <t>Paper Packaging &amp; Printing, Packaging Materials &amp; Accessories</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1877,7 +1877,7 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>14rmb, 500, visiting the factory — покупатель / байер; They promised to send me a catalogue of the — покупатель / байер; MOQ: 29 — покупатель / байер</t>
+          <t>14rmb, 500, visiting the factory — buyer; They promised to send me a catalogue of the — buyer; MOQ: 29 — buyer</t>
         </is>
       </c>
     </row>
@@ -1892,7 +1892,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Косметика и уход</t>
+          <t>Cosmetics &amp; Care</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1922,7 +1922,7 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>1.2RMB/pc, 10000 pcs, contacts exchange — покупатель / байер</t>
+          <t>1.2RMB/pc, 10000 pcs, contacts exchange — buyer</t>
         </is>
       </c>
     </row>
@@ -1937,7 +1937,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Косметика и уход</t>
+          <t>Cosmetics &amp; Care</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1967,7 +1967,7 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>Цены разные, всё сложно, Хорошо — покупатель / байер</t>
+          <t>Цены разные, всё сложно, Хорошо — buyer</t>
         </is>
       </c>
     </row>
@@ -1982,7 +1982,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Бумажная упаковка и печать, Упаковочные материалы и аксессуары</t>
+          <t>Paper Packaging &amp; Printing, Packaging Materials &amp; Accessories</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -2002,7 +2002,7 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>They promised to send me a catalogue of the prices. — покупатель / байер</t>
+          <t>They promised to send me a catalogue of the prices. — buyer</t>
         </is>
       </c>
     </row>
@@ -2017,7 +2017,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Электроника и цифровые решения, Промышленное оборудование</t>
+          <t>Electronics &amp; Digital Solutions, Industrial Equipment</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -2042,7 +2042,7 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>1,5 $ good — покупатель / байер; 0,08-0.15$/3000 — покупатель / байер; 0.85-1.20$/3000 — покупатель / байер</t>
+          <t>1,5 $ good — buyer; 0,08-0.15$/3000 — buyer; 0.85-1.20$/3000 — buyer</t>
         </is>
       </c>
     </row>
@@ -2057,7 +2057,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Упаковочные материалы и аксессуары, Промышленное оборудование, Продукты на заказ / OEM</t>
+          <t>Packaging Materials &amp; Accessories, Industrial Equipment, Custom Products / OEM</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -2077,7 +2077,7 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>2.8¥.MOQ-2000.ok. — покупатель / байер; We are fully satisfied with this supplier. The product range is extensive and we</t>
+          <t>2.8¥.MOQ-2000.ok. — buyer; We are fully satisfied with this supplier. The product range is extensive and we</t>
         </is>
       </c>
     </row>
@@ -2092,7 +2092,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Промышленное оборудование</t>
+          <t>Industrial Equipment</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -2137,7 +2137,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Пластиковая упаковка, Упаковочные материалы и аксессуары</t>
+          <t>Plastic Packaging, Packaging Materials &amp; Accessories</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -2167,7 +2167,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Пластиковая упаковка, Упаковочные материалы и аксессуары</t>
+          <t>Plastic Packaging, Packaging Materials &amp; Accessories</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -2182,7 +2182,7 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>5-15 — покупатель / байер</t>
+          <t>5-15 — buyer</t>
         </is>
       </c>
     </row>
@@ -2197,7 +2197,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Упаковочные материалы и аксессуары</t>
+          <t>Packaging Materials &amp; Accessories</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -2222,7 +2222,7 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>2,9 MOQ 20,000 — покупатель / байер</t>
+          <t>2,9 MOQ 20,000 — buyer</t>
         </is>
       </c>
     </row>
@@ -2237,7 +2237,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Косметика и уход</t>
+          <t>Cosmetics &amp; Care</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -2262,7 +2262,7 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>MOQ: 100 — покупатель / байер; MOQ: 1000 — покупатель / байер; 2.8 usd — покупатель / байер</t>
+          <t>MOQ: 100 — buyer; MOQ: 1000 — buyer; 2.8 usd — buyer</t>
         </is>
       </c>
     </row>
@@ -2277,7 +2277,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Упаковочные материалы и аксессуары</t>
+          <t>Packaging Materials &amp; Accessories</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -2297,7 +2297,7 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>Отлично — покупатель / байер</t>
+          <t>Отлично — buyer</t>
         </is>
       </c>
     </row>
@@ -2312,7 +2312,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Прочее</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -2342,7 +2342,7 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>7RMB 10,000piezas — покупатель / байер</t>
+          <t>7RMB 10,000piezas — buyer</t>
         </is>
       </c>
     </row>
@@ -2357,7 +2357,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Пластиковая упаковка, Продукты на заказ / OEM</t>
+          <t>Plastic Packaging, Custom Products / OEM</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -2382,7 +2382,7 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>12 Rmb, 500 pcs — покупатель / байер</t>
+          <t>12 Rmb, 500 pcs — buyer</t>
         </is>
       </c>
     </row>
@@ -2397,7 +2397,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Упаковочные материалы и аксессуары, Продукты на заказ / OEM</t>
+          <t>Packaging Materials &amp; Accessories, Custom Products / OEM</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>Will send the price with catalog — покупатель / байер</t>
+          <t>Will send the price with catalog — buyer</t>
         </is>
       </c>
     </row>
@@ -2442,7 +2442,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Упаковочные материалы и аксессуары</t>
+          <t>Packaging Materials &amp; Accessories</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -2467,7 +2467,7 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>1,36 rmb, 100 pcs. Good price. — покупатель / байер</t>
+          <t>1,36 rmb, 100 pcs. Good price. — buyer</t>
         </is>
       </c>
     </row>
@@ -2482,7 +2482,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Продукты на заказ / OEM, Электроника и цифровые решения</t>
+          <t>Custom Products / OEM, Electronics &amp; Digital Solutions</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -2527,7 +2527,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Упаковочные материалы и аксессуары, Продукты на заказ / OEM, Гибкая упаковка и тубы</t>
+          <t>Packaging Materials &amp; Accessories, Custom Products / OEM, Flexible Packaging &amp; Tubes</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -2557,7 +2557,7 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>They promised to send me a catalogue of the — покупатель / байер; .5$ depending upon MOQ, Minimum Moq 10000, good production facilities — покупате</t>
+          <t>They promised to send me a catalogue of the — buyer; .5$ depending upon MOQ, Minimum Moq 10000, good production facilities — покупате</t>
         </is>
       </c>
     </row>
@@ -2572,7 +2572,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Упаковочные материалы и аксессуары, Дизайн и брендинг</t>
+          <t>Packaging Materials &amp; Accessories, Design &amp; Branding</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -2617,7 +2617,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Косметика и уход</t>
+          <t>Cosmetics &amp; Care</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -2647,7 +2647,7 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>MOQ: 10000 pcs — покупатель / байер</t>
+          <t>MOQ: 10000 pcs — buyer</t>
         </is>
       </c>
     </row>
@@ -2662,7 +2662,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Электроника и цифровые решения, Промышленное оборудование</t>
+          <t>Electronics &amp; Digital Solutions, Industrial Equipment</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -2687,7 +2687,7 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>5000*7 RMB — покупатель / байер</t>
+          <t>5000*7 RMB — buyer</t>
         </is>
       </c>
     </row>
@@ -2702,7 +2702,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Упаковочные материалы и аксессуары, Продукты на заказ / OEM</t>
+          <t>Packaging Materials &amp; Accessories, Custom Products / OEM</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -2727,7 +2727,7 @@
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>Depends on the quantity — покупатель / байер</t>
+          <t>Depends on the quantity — buyer</t>
         </is>
       </c>
     </row>
@@ -2742,7 +2742,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Косметика и уход, Пластиковая упаковка</t>
+          <t>Cosmetics &amp; Care, Plastic Packaging</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -2772,7 +2772,7 @@
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>MOQ: 10000 — покупатель / байер</t>
+          <t>MOQ: 10000 — buyer</t>
         </is>
       </c>
     </row>
@@ -2787,7 +2787,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Продукты на заказ / OEM, Промышленное оборудование</t>
+          <t>Custom Products / OEM, Industrial Equipment</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -2812,7 +2812,7 @@
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>Under discussion with suplier for customization — покупатель / байер</t>
+          <t>Under discussion with suplier for customization — buyer</t>
         </is>
       </c>
     </row>
@@ -2827,7 +2827,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Косметика и уход, Биотехнологии и фармацевтика</t>
+          <t>Cosmetics &amp; Care, Biotechnology &amp; Pharmaceuticals</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -2857,7 +2857,7 @@
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>MOQ: 0,3 — покупатель / байер</t>
+          <t>MOQ: 0,3 — buyer</t>
         </is>
       </c>
     </row>
@@ -2872,7 +2872,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Промышленное оборудование, Продукты на заказ / OEM</t>
+          <t>Industrial Equipment, Custom Products / OEM</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -2897,7 +2897,7 @@
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>1.8-2RmbMoQ — покупатель / байер</t>
+          <t>1.8-2RmbMoQ — buyer</t>
         </is>
       </c>
     </row>
@@ -2912,7 +2912,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Бумажная упаковка и печать</t>
+          <t>Paper Packaging &amp; Printing</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -2942,7 +2942,7 @@
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>0.8RMB — покупатель / байер</t>
+          <t>0.8RMB — buyer</t>
         </is>
       </c>
     </row>
@@ -2957,7 +2957,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Продукты на заказ / OEM</t>
+          <t>Custom Products / OEM</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -2977,7 +2977,7 @@
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>good — покупатель / байер</t>
+          <t>good — buyer</t>
         </is>
       </c>
     </row>
@@ -2992,7 +2992,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Косметика и уход, Пластиковая упаковка</t>
+          <t>Cosmetics &amp; Care, Plastic Packaging</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -3012,7 +3012,7 @@
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>MOQ 5000. Price 3 yuanes — покупатель / байер; Pump bottles for liquid lotion or foundation. Moq 5000 pieces — покупатель / бай</t>
+          <t>MOQ 5000. Price 3 yuanes — buyer; Pump bottles for liquid lotion or foundation. Moq 5000 pieces — покупатель / бай</t>
         </is>
       </c>
     </row>
@@ -3027,7 +3027,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Пластиковая упаковка, Упаковочные материалы и аксессуары, Косметика и уход</t>
+          <t>Plastic Packaging, Packaging Materials &amp; Accessories, Cosmetics &amp; Care</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -3057,7 +3057,7 @@
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>2,12 rnb — покупатель / байер</t>
+          <t>2,12 rnb — buyer</t>
         </is>
       </c>
     </row>
@@ -3072,7 +3072,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Пластиковая упаковка, Упаковочные материалы и аксессуары, Продукты на заказ / OEM</t>
+          <t>Plastic Packaging, Packaging Materials &amp; Accessories, Custom Products / OEM</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -3102,7 +3102,7 @@
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>6,5 per piece , MOQ 15,000 — покупатель / байер; Price is 3 RMB, MOQ is 15000 pieces, quality was outstanding — покупатель / байе</t>
+          <t>6,5 per piece , MOQ 15,000 — buyer; Price is 3 RMB, MOQ is 15000 pieces, quality was outstanding — покупатель / байе</t>
         </is>
       </c>
     </row>
@@ -3117,7 +3117,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Косметика и уход, Электроника и цифровые решения, Продукты на заказ / OEM</t>
+          <t>Cosmetics &amp; Care, Electronics &amp; Digital Solutions, Custom Products / OEM</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -3142,7 +3142,7 @@
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>Good — покупатель / байер</t>
+          <t>Good — buyer</t>
         </is>
       </c>
     </row>
@@ -3157,7 +3157,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Текстиль и нетканые материалы</t>
+          <t>Textiles &amp; Nonwovens</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>0,8 yuan/piece, хорошие впечатления — покупатель / байер</t>
+          <t>0,8 yuan/piece, хорошие впечатления — buyer</t>
         </is>
       </c>
     </row>
@@ -3202,7 +3202,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Бумажная упаковка и печать, Продукты на заказ / OEM</t>
+          <t>Paper Packaging &amp; Printing, Custom Products / OEM</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -3232,7 +3232,7 @@
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>MOQ: 5000 pcs — покупатель / байер; 10, good — покупатель / байер</t>
+          <t>MOQ: 5000 pcs — buyer; 10, good — buyer</t>
         </is>
       </c>
     </row>
@@ -3247,7 +3247,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Упаковочные материалы и аксессуары, Гибкая упаковка и тубы, Продукты на заказ / OEM</t>
+          <t>Packaging Materials &amp; Accessories, Flexible Packaging &amp; Tubes, Custom Products / OEM</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -3272,7 +3272,7 @@
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>3/item — покупатель / байер</t>
+          <t>3/item — buyer</t>
         </is>
       </c>
     </row>
@@ -3287,7 +3287,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Пластиковая упаковка</t>
+          <t>Plastic Packaging</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -3317,7 +3317,7 @@
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>USD 1- 7 MOQ 10.000 — покупатель / байер; 1000 MOQ , 25rmb per piece — покупатель / байер</t>
+          <t>USD 1- 7 MOQ 10.000 — buyer; 1000 MOQ , 25rmb per piece — buyer</t>
         </is>
       </c>
     </row>
@@ -3332,7 +3332,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Упаковочные материалы и аксессуары</t>
+          <t>Packaging Materials &amp; Accessories</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -3362,7 +3362,7 @@
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>MOQ 1000, price 10 yuanes — покупатель / байер</t>
+          <t>MOQ 1000, price 10 yuanes — buyer</t>
         </is>
       </c>
     </row>
@@ -3377,7 +3377,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Пластиковая упаковка</t>
+          <t>Plastic Packaging</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -3397,7 +3397,7 @@
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>0.9$ — покупатель / байер; Price 6.5; MOQ 5000 — покупатель / байер</t>
+          <t>0.9$ — buyer; Price 6.5; MOQ 5000 — buyer</t>
         </is>
       </c>
     </row>
@@ -3412,7 +3412,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Упаковочные материалы и аксессуары, Гибкая упаковка и тубы</t>
+          <t>Packaging Materials &amp; Accessories, Flexible Packaging &amp; Tubes</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -3442,7 +3442,7 @@
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>2/item — покупатель / байер</t>
+          <t>2/item — buyer</t>
         </is>
       </c>
     </row>
@@ -3457,7 +3457,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Продукты на заказ / OEM, Бумажная упаковка и печать</t>
+          <t>Custom Products / OEM, Paper Packaging &amp; Printing</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -3482,7 +3482,7 @@
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>Price 10-15 rmb — покупатель / байер; MOQ 3000 12 rmb good quality boxes many different design, quality good — покупат; 1.8 RMB, MOQ10000 for customized design — покупатель / байер</t>
+          <t>Price 10-15 rmb — buyer; MOQ 3000 12 rmb good quality boxes many different design, quality good — покупат; 1.8 RMB, MOQ10000 for customized design — buyer</t>
         </is>
       </c>
     </row>
@@ -3497,7 +3497,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Промышленное оборудование, Электроника и цифровые решения</t>
+          <t>Industrial Equipment, Electronics &amp; Digital Solutions</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -3522,7 +3522,7 @@
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>10000*0.3USD — покупатель / байер; 2,8 rmb, MOQ 12000 — покупатель / байер</t>
+          <t>10000*0.3USD — buyer; 2,8 rmb, MOQ 12000 — buyer</t>
         </is>
       </c>
     </row>
@@ -3537,7 +3537,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Косметика и уход, Упаковочные материалы и аксессуары</t>
+          <t>Cosmetics &amp; Care, Packaging Materials &amp; Accessories</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -3562,7 +3562,7 @@
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>Fully satisfied — покупатель / байер</t>
+          <t>Fully satisfied — buyer</t>
         </is>
       </c>
     </row>
@@ -3577,7 +3577,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Электроника и цифровые решения, Промышленное оборудование</t>
+          <t>Electronics &amp; Digital Solutions, Industrial Equipment</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -3607,7 +3607,7 @@
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>1.25RMB/pc, 30000 pcs, contacts exchange — покупатель / байер; 3.5 good — покупатель / байер</t>
+          <t>1.25RMB/pc, 30000 pcs, contacts exchange — buyer; 3.5 good — buyer</t>
         </is>
       </c>
     </row>
@@ -3622,7 +3622,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Пластиковая упаковка</t>
+          <t>Plastic Packaging</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -3647,7 +3647,7 @@
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>MOQ: 12000 pcs — покупатель / байер; 5000USD — покупатель / байер; good — покупатель / байер</t>
+          <t>MOQ: 12000 pcs — buyer; 5000USD — buyer; good — buyer</t>
         </is>
       </c>
     </row>
@@ -3662,7 +3662,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Пластиковая упаковка</t>
+          <t>Plastic Packaging</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -3707,7 +3707,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Пластиковая упаковка</t>
+          <t>Plastic Packaging</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -3737,7 +3737,7 @@
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>MOQ: 10000 — покупатель / байер</t>
+          <t>MOQ: 10000 — buyer</t>
         </is>
       </c>
     </row>
@@ -3752,7 +3752,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Пластиковая упаковка</t>
+          <t>Plastic Packaging</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -3797,7 +3797,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Пластиковая упаковка</t>
+          <t>Plastic Packaging</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -3822,7 +3822,7 @@
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>MOQ: 8000 — покупатель / байер</t>
+          <t>MOQ: 8000 — buyer</t>
         </is>
       </c>
     </row>
@@ -3837,7 +3837,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Упаковочные материалы и аксессуары, Продукты на заказ / OEM</t>
+          <t>Packaging Materials &amp; Accessories, Custom Products / OEM</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -3867,7 +3867,7 @@
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>2 rmb 1000pcs — покупатель / байер</t>
+          <t>2 rmb 1000pcs — buyer</t>
         </is>
       </c>
     </row>
@@ -3882,7 +3882,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Электроника и цифровые решения, Продукты на заказ / OEM</t>
+          <t>Electronics &amp; Digital Solutions, Custom Products / OEM</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -3907,7 +3907,7 @@
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>0.75 dollar per pieces, 1500 per pieces. — покупатель / байер</t>
+          <t>0.75 dollar per pieces, 1500 per pieces. — buyer</t>
         </is>
       </c>
     </row>
@@ -3922,7 +3922,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Текстиль и нетканые материалы, Продукты на заказ / OEM</t>
+          <t>Textiles &amp; Nonwovens, Custom Products / OEM</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -3952,7 +3952,7 @@
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>Восхитительные — покупатель / байер; I liked the assortment and the prices — they offer good value for money — покупа</t>
+          <t>Восхитительные — buyer; I liked the assortment and the prices — they offer good value for money — покупа</t>
         </is>
       </c>
     </row>
@@ -3967,7 +3967,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Продукты на заказ / OEM</t>
+          <t>Custom Products / OEM</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -3992,7 +3992,7 @@
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>5 yuan, good feedback — покупатель / байер</t>
+          <t>5 yuan, good feedback — buyer</t>
         </is>
       </c>
     </row>
@@ -4007,7 +4007,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Упаковочные материалы и аксессуары</t>
+          <t>Packaging Materials &amp; Accessories</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -4032,7 +4032,7 @@
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>10 rmb — покупатель / байер</t>
+          <t>10 rmb — buyer</t>
         </is>
       </c>
     </row>
@@ -4047,7 +4047,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Пластиковая упаковка, Промышленное оборудование, Продукты на заказ / OEM</t>
+          <t>Plastic Packaging, Industrial Equipment, Custom Products / OEM</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -4082,7 +4082,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Электроника и цифровые решения, Промышленное оборудование</t>
+          <t>Electronics &amp; Digital Solutions, Industrial Equipment</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -4107,7 +4107,7 @@
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>1500 - 25 — покупатель / байер</t>
+          <t>1500 - 25 — buyer</t>
         </is>
       </c>
     </row>
@@ -4122,7 +4122,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Продукты на заказ / OEM</t>
+          <t>Custom Products / OEM</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -4152,7 +4152,7 @@
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>30 rmb per person with a MOQ 500 — покупатель / байер</t>
+          <t>30 rmb per person with a MOQ 500 — buyer</t>
         </is>
       </c>
     </row>
@@ -4167,7 +4167,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Продукты на заказ / OEM</t>
+          <t>Custom Products / OEM</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -4197,7 +4197,7 @@
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>MOQ:6000 Pcs — покупатель / байер</t>
+          <t>MOQ:6000 Pcs — buyer</t>
         </is>
       </c>
     </row>
@@ -4212,7 +4212,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Продукты на заказ / OEM, Упаковочные материалы и аксессуары, Дизайн и брендинг</t>
+          <t>Custom Products / OEM, Packaging Materials &amp; Accessories, Design &amp; Branding</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -4237,7 +4237,7 @@
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>Based on design and Customisation — покупатель / байер; MOQ=10,000 meeting was very budget friendly.. product i like most — покупатель /; 7 rmb, Quality packaging, interesting options that I have not seen before — поку</t>
+          <t>Based on design and Customisation — buyer; MOQ=10,000 meeting was very budget friendly.. product i like most — покупатель /; 7 rmb, Quality packaging, interesting options that I have not seen before — поку</t>
         </is>
       </c>
     </row>
@@ -4252,7 +4252,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Продукты на заказ / OEM</t>
+          <t>Custom Products / OEM</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -4277,7 +4277,7 @@
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>Price 6.5; MOQ 5000 — покупатель / байер</t>
+          <t>Price 6.5; MOQ 5000 — buyer</t>
         </is>
       </c>
     </row>
@@ -4292,7 +4292,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Продукты на заказ / OEM</t>
+          <t>Custom Products / OEM</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -4317,7 +4317,7 @@
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>The price is good — покупатель / байер; The price ranges from 1 to 2 Chinese yuan if the order is large — покупатель / б; MOQ: 5000 — покупатель / байер</t>
+          <t>The price is good — buyer; The price ranges from 1 to 2 Chinese yuan if the order is large — покупатель / б; MOQ: 5000 — buyer</t>
         </is>
       </c>
     </row>
@@ -4332,7 +4332,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Упаковочные материалы и аксессуары, Дизайн и брендинг</t>
+          <t>Packaging Materials &amp; Accessories, Design &amp; Branding</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
@@ -4362,7 +4362,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Биотехнологии и фармацевтика, Стеклянная упаковка</t>
+          <t>Biotechnology &amp; Pharmaceuticals, Glass Packaging</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -4392,7 +4392,7 @@
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>1.25rmb/unit. For 5000 droppers it will be 6250 rmb. — покупатель / байер; 1-5 — покупатель / байер</t>
+          <t>1.25rmb/unit. For 5000 droppers it will be 6250 rmb. — buyer; 1-5 — buyer</t>
         </is>
       </c>
     </row>
@@ -4407,7 +4407,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Косметика и уход</t>
+          <t>Cosmetics &amp; Care</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -4437,7 +4437,7 @@
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>От 2000, от 2.2 — покупатель / байер; MOQ: 1800 pcs — покупатель / байер; MOQ: 11200 pcs — покупатель / байер</t>
+          <t>От 2000, от 2.2 — buyer; MOQ: 1800 pcs — buyer; MOQ: 11200 pcs — buyer</t>
         </is>
       </c>
     </row>
@@ -4452,7 +4452,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Пластиковая упаковка</t>
+          <t>Plastic Packaging</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -4482,7 +4482,7 @@
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>1-10 — покупатель / байер</t>
+          <t>1-10 — buyer</t>
         </is>
       </c>
     </row>
@@ -4497,7 +4497,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Бумажная упаковка и печать</t>
+          <t>Paper Packaging &amp; Printing</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -4542,7 +4542,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Упаковочные материалы и аксессуары, Текстиль и нетканые материалы, Продукты на заказ / OEM</t>
+          <t>Packaging Materials &amp; Accessories, Textiles &amp; Nonwovens, Custom Products / OEM</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
@@ -4567,7 +4567,7 @@
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>RMB 1.20  per 100,000 units — покупатель / байер; MOQ 1000 pieces, each oye 2.5 dola — покупатель / байер; MOQ 1000 , 2.5 dollar — покупатель / байер</t>
+          <t>RMB 1.20  per 100,000 units — buyer; MOQ 1000 pieces, each oye 2.5 dola — buyer; MOQ 1000 , 2.5 dollar — buyer</t>
         </is>
       </c>
     </row>
@@ -4582,7 +4582,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Упаковочные материалы и аксессуары, Продукты на заказ / OEM, Текстиль и нетканые материалы</t>
+          <t>Packaging Materials &amp; Accessories, Custom Products / OEM, Textiles &amp; Nonwovens</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -4612,7 +4612,7 @@
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>0, 2 usd for 1 yard (25cm), MOQ 1000, huge right off sample options — покупатель; 2,6$ 100 yard roll ribbon very good quality and very big choice, can make a prin; 0.5 — покупатель / байер</t>
+          <t>0, 2 usd for 1 yard (25cm), MOQ 1000, huge right off sample options — покупатель; 2,6$ 100 yard roll ribbon very good quality and very big choice, can make a prin; 0.5 — buyer</t>
         </is>
       </c>
     </row>
@@ -4627,7 +4627,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Упаковочные материалы и аксессуары, Продукты на заказ / OEM</t>
+          <t>Packaging Materials &amp; Accessories, Custom Products / OEM</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -4652,7 +4652,7 @@
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>Interesting — покупатель / байер</t>
+          <t>Interesting — buyer</t>
         </is>
       </c>
     </row>
@@ -4667,7 +4667,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Пластиковая упаковка, Косметика и уход</t>
+          <t>Plastic Packaging, Cosmetics &amp; Care</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -4697,7 +4697,7 @@
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>8 rmb per sample — покупатель / байер; MOQ 10000шт, меньше производить не могут. Цена за интересующий продукт 2,1 юань.</t>
+          <t>8 rmb per sample — buyer; MOQ 10000шт, меньше производить не могут. Цена за интересующий продукт 2,1 юань.</t>
         </is>
       </c>
     </row>
@@ -4712,7 +4712,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Пластиковая упаковка</t>
+          <t>Plastic Packaging</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -4742,7 +4742,7 @@
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>5000*13,5RMB. Very nice sales managers — покупатель / байер</t>
+          <t>5000*13,5RMB. Very nice sales managers — buyer</t>
         </is>
       </c>
     </row>
@@ -4757,7 +4757,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Упаковочные материалы и аксессуары, Биотехнологии и фармацевтика</t>
+          <t>Packaging Materials &amp; Accessories, Biotechnology &amp; Pharmaceuticals</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -4772,7 +4772,7 @@
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>Moq  20HD, nice company — покупатель / байер</t>
+          <t>Moq  20HD, nice company — buyer</t>
         </is>
       </c>
     </row>
@@ -4787,7 +4787,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Промышленное оборудование, Продукты на заказ / OEM, Электроника и цифровые решения</t>
+          <t>Industrial Equipment, Custom Products / OEM, Electronics &amp; Digital Solutions</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -4817,7 +4817,7 @@
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>50000rmb ,the meeting was informative and helpfull. — покупатель / байер</t>
+          <t>50000rmb ,the meeting was informative and helpfull. — buyer</t>
         </is>
       </c>
     </row>
@@ -4832,7 +4832,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Упаковочные материалы и аксессуары, Продукты на заказ / OEM</t>
+          <t>Packaging Materials &amp; Accessories, Custom Products / OEM</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -4857,7 +4857,7 @@
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>1-15 — покупатель / байер</t>
+          <t>1-15 — buyer</t>
         </is>
       </c>
     </row>
@@ -4872,7 +4872,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Электроника и цифровые решения, Продукты на заказ / OEM</t>
+          <t>Electronics &amp; Digital Solutions, Custom Products / OEM</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -4912,7 +4912,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Биотехнологии и фармацевтика, Упаковочные материалы и аксессуары, Промышленное оборудование</t>
+          <t>Biotechnology &amp; Pharmaceuticals, Packaging Materials &amp; Accessories, Industrial Equipment</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -4937,7 +4937,7 @@
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>7rmb, 1000, very much interested in meeting — покупатель / байер</t>
+          <t>7rmb, 1000, very much interested in meeting — buyer</t>
         </is>
       </c>
     </row>
@@ -4952,7 +4952,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Упаковочные материалы и аксессуары, Электроника и цифровые решения, Промышленное оборудование</t>
+          <t>Packaging Materials &amp; Accessories, Electronics &amp; Digital Solutions, Industrial Equipment</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -4982,7 +4982,7 @@
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>2.21$/pp — покупатель / байер</t>
+          <t>2.21$/pp — buyer</t>
         </is>
       </c>
     </row>
@@ -4997,7 +4997,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Упаковочные материалы и аксессуары</t>
+          <t>Packaging Materials &amp; Accessories</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -5042,7 +5042,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Продукты на заказ / OEM, Косметика и уход, Пластиковая упаковка</t>
+          <t>Custom Products / OEM, Cosmetics &amp; Care, Plastic Packaging</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -5072,7 +5072,7 @@
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>MOQ=10,000 meeting was friendly product good quality — покупатель / байер</t>
+          <t>MOQ=10,000 meeting was friendly product good quality — buyer</t>
         </is>
       </c>
     </row>
@@ -5087,7 +5087,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Бумажная упаковка и печать</t>
+          <t>Paper Packaging &amp; Printing</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -5117,7 +5117,7 @@
       </c>
       <c r="I114" t="inlineStr">
         <is>
-          <t>9rmb , good quality — покупатель / байер</t>
+          <t>9rmb , good quality — buyer</t>
         </is>
       </c>
     </row>
@@ -5132,7 +5132,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Упаковочные материалы и аксессуары, Продукты на заказ / OEM</t>
+          <t>Packaging Materials &amp; Accessories, Custom Products / OEM</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -5157,7 +5157,7 @@
       </c>
       <c r="I115" t="inlineStr">
         <is>
-          <t>2:5rmb 10000pcs — покупатель / байер; 5000p,  4.2y — покупатель / байер; 10000p, 2.5y — покупатель / байер</t>
+          <t>2:5rmb 10000pcs — buyer; 5000p,  4.2y — buyer; 10000p, 2.5y — buyer</t>
         </is>
       </c>
     </row>
@@ -5172,7 +5172,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Косметика и уход</t>
+          <t>Cosmetics &amp; Care</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -5197,7 +5197,7 @@
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>3RMB/pc, 1000 pcs, contacts exchange — покупатель / байер</t>
+          <t>3RMB/pc, 1000 pcs, contacts exchange — buyer</t>
         </is>
       </c>
     </row>
@@ -5212,7 +5212,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Косметика и уход</t>
+          <t>Cosmetics &amp; Care</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -5237,7 +5237,7 @@
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>2,4 yuan/piece. Отличные впечатления — покупатель / байер</t>
+          <t>2,4 yuan/piece. Отличные впечатления — buyer</t>
         </is>
       </c>
     </row>
@@ -5252,7 +5252,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Электроника и цифровые решения</t>
+          <t>Electronics &amp; Digital Solutions</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -5282,7 +5282,7 @@
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>39rmb, 600 pcs — покупатель / байер; 20 Rmb , 15 pice — покупатель / байер</t>
+          <t>39rmb, 600 pcs — buyer; 20 Rmb , 15 pice — buyer</t>
         </is>
       </c>
     </row>
@@ -5297,7 +5297,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Биотехнологии и фармацевтика, Упаковочные материалы и аксессуары</t>
+          <t>Biotechnology &amp; Pharmaceuticals, Packaging Materials &amp; Accessories</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -5317,7 +5317,7 @@
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>13rmb , good quality — покупатель / байер; MOQ: 2000 — покупатель / байер; Sticker MOQ: 10k PCS — покупатель / байер</t>
+          <t>13rmb , good quality — buyer; MOQ: 2000 — buyer; Sticker MOQ: 10k PCS — buyer</t>
         </is>
       </c>
     </row>
@@ -5332,7 +5332,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Продукты на заказ / OEM</t>
+          <t>Custom Products / OEM</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -5357,7 +5357,7 @@
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>depend on the product, good feedback — покупатель / байер</t>
+          <t>depend on the product, good feedback — buyer</t>
         </is>
       </c>
     </row>
@@ -5372,7 +5372,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Пластиковая упаковка, Упаковочные материалы и аксессуары</t>
+          <t>Plastic Packaging, Packaging Materials &amp; Accessories</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -5392,7 +5392,7 @@
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>2,5 rmb, 10000 pcs, good quality — покупатель / байер; 45rmb, 400pcs — покупатель / байер</t>
+          <t>2,5 rmb, 10000 pcs, good quality — buyer; 45rmb, 400pcs — buyer</t>
         </is>
       </c>
     </row>
@@ -5407,7 +5407,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Упаковочные материалы и аксессуары, Пластиковая упаковка</t>
+          <t>Packaging Materials &amp; Accessories, Plastic Packaging</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
@@ -5437,7 +5437,7 @@
       </c>
       <c r="I122" t="inlineStr">
         <is>
-          <t>5-10 — покупатель / байер</t>
+          <t>5-10 — buyer</t>
         </is>
       </c>
     </row>
@@ -5452,7 +5452,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Упаковочные материалы и аксессуары</t>
+          <t>Packaging Materials &amp; Accessories</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
@@ -5482,7 +5482,7 @@
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>MOQ: 12000 pcs — покупатель / байер; 7000USD — покупатель / байер</t>
+          <t>MOQ: 12000 pcs — buyer; 7000USD — buyer</t>
         </is>
       </c>
     </row>
@@ -5497,7 +5497,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Косметика и уход</t>
+          <t>Cosmetics &amp; Care</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -5522,7 +5522,7 @@
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t>Mouth freshener 1RMB , MOQ 5000 — покупатель / байер</t>
+          <t>Mouth freshener 1RMB , MOQ 5000 — buyer</t>
         </is>
       </c>
     </row>
@@ -5537,7 +5537,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Продукты на заказ / OEM</t>
+          <t>Custom Products / OEM</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -5567,7 +5567,7 @@
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>20rmb, 1000, very much interested in making order — покупатель / байер</t>
+          <t>20rmb, 1000, very much interested in making order — buyer</t>
         </is>
       </c>
     </row>
@@ -5582,7 +5582,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Пластиковая упаковка, Промышленное оборудование</t>
+          <t>Plastic Packaging, Industrial Equipment</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
@@ -5607,7 +5607,7 @@
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>1000 MOQ, 0.25USD single piece — покупатель / байер; 1.5$ — покупатель / байер; Price 6 RMB; MOQ 5000 — покупатель / байер</t>
+          <t>1000 MOQ, 0.25USD single piece — buyer; 1.5$ — buyer; Price 6 RMB; MOQ 5000 — buyer</t>
         </is>
       </c>
     </row>
@@ -5622,7 +5622,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Текстиль и нетканые материалы, Гибкая упаковка и тубы</t>
+          <t>Textiles &amp; Nonwovens, Flexible Packaging &amp; Tubes</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
@@ -5647,7 +5647,7 @@
       </c>
       <c r="I127" t="inlineStr">
         <is>
-          <t>0.045rmb , good quality — покупатель / байер; MOQ: 0,2 — покупатель / байер</t>
+          <t>0.045rmb , good quality — buyer; MOQ: 0,2 — buyer</t>
         </is>
       </c>
     </row>
@@ -5662,7 +5662,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Бумажная упаковка и печать, Упаковочные материалы и аксессуары</t>
+          <t>Paper Packaging &amp; Printing, Packaging Materials &amp; Accessories</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
@@ -5682,7 +5682,7 @@
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>Цены разные, всё сложно, Хорошо — покупатель / байер</t>
+          <t>Цены разные, всё сложно, Хорошо — buyer</t>
         </is>
       </c>
     </row>
@@ -5697,7 +5697,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Электроника и цифровые решения, Продукты на заказ / OEM</t>
+          <t>Electronics &amp; Digital Solutions, Custom Products / OEM</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
@@ -5727,7 +5727,7 @@
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>Price 4,8 MOQ 20,000 they were nice and welcoming — покупатель / байер</t>
+          <t>Price 4,8 MOQ 20,000 they were nice and welcoming — buyer</t>
         </is>
       </c>
     </row>
@@ -5742,7 +5742,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Электроника и цифровые решения</t>
+          <t>Electronics &amp; Digital Solutions</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -5767,7 +5767,7 @@
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>Good — покупатель / байер</t>
+          <t>Good — buyer</t>
         </is>
       </c>
     </row>
@@ -5782,7 +5782,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>Бумажная упаковка и печать</t>
+          <t>Paper Packaging &amp; Printing</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
@@ -5812,7 +5812,7 @@
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>USD 3-5 MOQ 3.000- 10.000 — покупатель / байер</t>
+          <t>USD 3-5 MOQ 3.000- 10.000 — buyer</t>
         </is>
       </c>
     </row>
@@ -5827,7 +5827,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>Продукты на заказ / OEM, Электроника и цифровые решения, Дизайн и брендинг</t>
+          <t>Custom Products / OEM, Electronics &amp; Digital Solutions, Design &amp; Branding</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
@@ -5852,7 +5852,7 @@
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>RMB 0.20  per 100,000 units — покупатель / байер; Brand Product QR code 0.001/ piece MOQ 100000 — покупатель / байер</t>
+          <t>RMB 0.20  per 100,000 units — buyer; Brand Product QR code 0.001/ piece MOQ 100000 — buyer</t>
         </is>
       </c>
     </row>
@@ -5867,7 +5867,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>Упаковочные материалы и аксессуары, Гибкая упаковка и тубы</t>
+          <t>Packaging Materials &amp; Accessories, Flexible Packaging &amp; Tubes</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
@@ -5892,7 +5892,7 @@
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>30 RMB, MOQ 10000, good company — покупатель / байер</t>
+          <t>30 RMB, MOQ 10000, good company — buyer</t>
         </is>
       </c>
     </row>
@@ -5907,7 +5907,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>Упаковочные материалы и аксессуары, Промышленное оборудование, Продукты на заказ / OEM</t>
+          <t>Packaging Materials &amp; Accessories, Industrial Equipment, Custom Products / OEM</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
@@ -5932,7 +5932,7 @@
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>5.5, good — покупатель / байер</t>
+          <t>5.5, good — buyer</t>
         </is>
       </c>
     </row>
@@ -5947,7 +5947,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>Упаковочные материалы и аксессуары, Продукты на заказ / OEM, Промышленное оборудование</t>
+          <t>Packaging Materials &amp; Accessories, Custom Products / OEM, Industrial Equipment</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
@@ -5967,7 +5967,7 @@
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>3,5 rmb, MOQ 1000, good company — покупатель / байер</t>
+          <t>3,5 rmb, MOQ 1000, good company — buyer</t>
         </is>
       </c>
     </row>
@@ -5982,7 +5982,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>Бумажная упаковка и печать</t>
+          <t>Paper Packaging &amp; Printing</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
@@ -6027,7 +6027,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>Пластиковая упаковка</t>
+          <t>Plastic Packaging</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
@@ -6052,7 +6052,7 @@
       </c>
       <c r="I137" t="inlineStr">
         <is>
-          <t>70000, feedback was fruitfull — покупатель / байер</t>
+          <t>70000, feedback was fruitfull — buyer</t>
         </is>
       </c>
     </row>
@@ -6067,7 +6067,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>Косметика и уход, Упаковочные материалы и аксессуары</t>
+          <t>Cosmetics &amp; Care, Packaging Materials &amp; Accessories</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
@@ -6087,7 +6087,7 @@
       </c>
       <c r="I138" t="inlineStr">
         <is>
-          <t>5rmb 5000pcs — покупатель / байер; MIA 300, 18rmb — покупатель / байер</t>
+          <t>5rmb 5000pcs — buyer; MIA 300, 18rmb — buyer</t>
         </is>
       </c>
     </row>
@@ -6102,7 +6102,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>Бумажная упаковка и печать</t>
+          <t>Paper Packaging &amp; Printing</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
@@ -6132,7 +6132,7 @@
       </c>
       <c r="I139" t="inlineStr">
         <is>
-          <t>1000p, 1.5y — покупатель / байер</t>
+          <t>1000p, 1.5y — buyer</t>
         </is>
       </c>
     </row>
@@ -6147,7 +6147,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>Продукты на заказ / OEM, Упаковочные материалы и аксессуары</t>
+          <t>Custom Products / OEM, Packaging Materials &amp; Accessories</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
@@ -6172,7 +6172,7 @@
       </c>
       <c r="I140" t="inlineStr">
         <is>
-          <t>We need to talk on further details about the order — покупатель / байер; 0, 5 usd for MOQ 500, supplier with a nice quality — покупатель / байер</t>
+          <t>We need to talk on further details about the order — buyer; 0, 5 usd for MOQ 500, supplier with a nice quality — buyer</t>
         </is>
       </c>
     </row>
@@ -6202,7 +6202,7 @@
       </c>
       <c r="I141" t="inlineStr">
         <is>
-          <t>8 yuan for sunblock — покупатель / байер</t>
+          <t>8 yuan for sunblock — buyer</t>
         </is>
       </c>
     </row>
@@ -6217,7 +6217,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>Упаковочные материалы и аксессуары, Промышленное оборудование, Продукты на заказ / OEM</t>
+          <t>Packaging Materials &amp; Accessories, Industrial Equipment, Custom Products / OEM</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
@@ -6257,7 +6257,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>Промышленное оборудование</t>
+          <t>Industrial Equipment</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
@@ -6272,7 +6272,7 @@
       </c>
       <c r="I143" t="inlineStr">
         <is>
-          <t>MOQ: 10000 pcs — покупатель / байер</t>
+          <t>MOQ: 10000 pcs — buyer</t>
         </is>
       </c>
     </row>
@@ -6287,7 +6287,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>Промышленное оборудование, Пластиковая упаковка</t>
+          <t>Industrial Equipment, Plastic Packaging</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
@@ -6322,7 +6322,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>Пластиковая упаковка</t>
+          <t>Plastic Packaging</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
@@ -6342,7 +6342,7 @@
       </c>
       <c r="I145" t="inlineStr">
         <is>
-          <t>Невероятные — покупатель / байер; 10 rmb. Looks interesting, big choice — покупатель / байер</t>
+          <t>Невероятные — buyer; 10 rmb. Looks interesting, big choice — buyer</t>
         </is>
       </c>
     </row>
@@ -6357,7 +6357,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>Косметика и уход</t>
+          <t>Cosmetics &amp; Care</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
@@ -6387,7 +6387,7 @@
       </c>
       <c r="I146" t="inlineStr">
         <is>
-          <t xml:space="preserve">1000 - 45 — покупатель / байер; Face roller 6.8 rmb per unit — покупатель / байер; 25rmb. . I was impressed by their professionalism and clear vision — покупатель </t>
+          <t xml:space="preserve">1000 - 45 — buyer; Face roller 6.8 rmb per unit — buyer; 25rmb. . I was impressed by their professionalism and clear vision — покупатель </t>
         </is>
       </c>
     </row>
@@ -6402,7 +6402,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>Упаковочные материалы и аксессуары, Продукты на заказ / OEM</t>
+          <t>Packaging Materials &amp; Accessories, Custom Products / OEM</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
@@ -6427,7 +6427,7 @@
       </c>
       <c r="I147" t="inlineStr">
         <is>
-          <t>0.1rmb, 5000pcs — покупатель / байер; 0,1 заказ от 1000 единиц — покупатель / байер</t>
+          <t>0.1rmb, 5000pcs — buyer; 0,1 заказ от 1000 единиц — buyer</t>
         </is>
       </c>
     </row>
@@ -6442,7 +6442,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>Металлическая упаковка, Промышленное оборудование, Электроника и цифровые решения</t>
+          <t>Metal Packaging, Industrial Equipment, Electronics &amp; Digital Solutions</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
@@ -6467,7 +6467,7 @@
       </c>
       <c r="I148" t="inlineStr">
         <is>
-          <t>MOQ2000 USD0.20 — покупатель / байер</t>
+          <t>MOQ2000 USD0.20 — buyer</t>
         </is>
       </c>
     </row>
@@ -6482,7 +6482,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>Бумажная упаковка и печать</t>
+          <t>Paper Packaging &amp; Printing</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
@@ -6502,7 +6502,7 @@
       </c>
       <c r="I149" t="inlineStr">
         <is>
-          <t>MOQ: 15 — покупатель / байер</t>
+          <t>MOQ: 15 — buyer</t>
         </is>
       </c>
     </row>
@@ -6517,7 +6517,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>Продукты на заказ / OEM, Промышленное оборудование</t>
+          <t>Custom Products / OEM, Industrial Equipment</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
@@ -6537,7 +6537,7 @@
       </c>
       <c r="I150" t="inlineStr">
         <is>
-          <t>4 rmb — покупатель / байер</t>
+          <t>4 rmb — buyer</t>
         </is>
       </c>
     </row>
@@ -6552,7 +6552,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>Промышленное оборудование, Гибкая упаковка и тубы</t>
+          <t>Industrial Equipment, Flexible Packaging &amp; Tubes</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
@@ -6572,7 +6572,7 @@
       </c>
       <c r="I151" t="inlineStr">
         <is>
-          <t>MOQ: 10000 — покупатель / байер; Price: 5RMB, MOQ: 10000 — покупатель / байер</t>
+          <t>MOQ: 10000 — buyer; Price: 5RMB, MOQ: 10000 — buyer</t>
         </is>
       </c>
     </row>
@@ -6587,7 +6587,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>Упаковочные материалы и аксессуары, Продукты на заказ / OEM, Гибкая упаковка и тубы</t>
+          <t>Packaging Materials &amp; Accessories, Custom Products / OEM, Flexible Packaging &amp; Tubes</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
@@ -6617,7 +6617,7 @@
       </c>
       <c r="I152" t="inlineStr">
         <is>
-          <t>8rmb, 200pcs — покупатель / байер</t>
+          <t>8rmb, 200pcs — buyer</t>
         </is>
       </c>
     </row>
@@ -6632,7 +6632,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>Электроника и цифровые решения, Промышленное оборудование, Биотехнологии и фармацевтика</t>
+          <t>Electronics &amp; Digital Solutions, Industrial Equipment, Biotechnology &amp; Pharmaceuticals</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
@@ -6657,7 +6657,7 @@
       </c>
       <c r="I153" t="inlineStr">
         <is>
-          <t>Under discussing — покупатель / байер</t>
+          <t>Under discussing — buyer</t>
         </is>
       </c>
     </row>
@@ -6672,7 +6672,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>Стеклянная упаковка, Прочее, Продукты на заказ / OEM</t>
+          <t>Glass Packaging, Other, Custom Products / OEM</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
@@ -6717,7 +6717,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>Косметическая упаковка</t>
+          <t>Cosmetic Packaging</t>
         </is>
       </c>
       <c r="E155" t="inlineStr">
@@ -6752,7 +6752,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>Пластиковая упаковка</t>
+          <t>Plastic Packaging</t>
         </is>
       </c>
       <c r="E156" t="inlineStr">
@@ -6792,7 +6792,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>Пластиковая упаковка</t>
+          <t>Plastic Packaging</t>
         </is>
       </c>
       <c r="E157" t="inlineStr">
@@ -6832,7 +6832,7 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>Пластиковая упаковка</t>
+          <t>Plastic Packaging</t>
         </is>
       </c>
       <c r="H158" t="inlineStr">

</xml_diff>

<commit_message>
Remove Chinese chars from contacts + addresses in all Excel, keep Latin/pinyin + English address
</commit_message>
<xml_diff>
--- a/ipdf_suppliers.xlsx
+++ b/ipdf_suppliers.xlsx
@@ -532,7 +532,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>刘金铃 (liú jīn líng)</t>
+          <t>liú jīn líng</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -552,7 +552,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>江苏省吴江市 (jiāng sū shěng wú jiāng shì) 汾湖经济开发区临沪大道 (fén hú jīng jì kāi fā qū lín hù dà dào)1999号 (hào), 215211No. 1999, Linhu Avenue, Fenhu Economic Development Zone, Wujiang City, Jiangsu Province, 215211</t>
+          <t>No. 1999, Linhu Avenue, Fenhu Economic Development Zone, Wujiang City, Jiangsu Province, 215211</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -617,7 +617,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>林显忠 (lín xiǎn zhōng)</t>
+          <t>lín xiǎn zhōng</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -637,7 +637,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>广州市白云区龙兴东南一横路 (guǎng zhōu shì bái yún qū lóng xīng dōng nán yī héng lù)3号 (hào)No. 3, Longxing Southeast First Horizontal Road, Baiyun District, Guangzhou City</t>
+          <t>No. 3, Longxing Southeast First Horizontal Road, Baiyun District, Guangzhou City</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -662,7 +662,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>宋茜 (sòng qiàn)</t>
+          <t>sòng qiàn</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -677,7 +677,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>广州市花都区花东镇定邦空港产业园 (guǎng zhōu shì huā dōu qū huā dōng zhèn dìng bāng kōng gǎng chǎn yè yuán)D栋 (dòng)Building D, Dingbang Airport Industrial Park, Huadong Town, Huadu District, Guangzhou</t>
+          <t>D Building D, Dingbang Airport Industrial Park, Huadong Town, Huadu District, Guangzhou</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -722,7 +722,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>广东省开平市三埠街道新台路 (guǎng dōng shěng kāi píng shì sān bù jiē dào xīn tái lù)72号 (hào)No. 72, Xintai Road, Sanbu Street, Kaiping City, Guangdong Province</t>
+          <t>No. 72, Xintai Road, Sanbu Street, Kaiping City, Guangdong Province</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -747,7 +747,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>王耀峰 (wáng yào fēng)</t>
+          <t>wáng yào fēng</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -777,7 +777,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>王媛媛 (wáng yuàn yuàn)</t>
+          <t>wáng yuàn yuàn</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -797,7 +797,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>工厂广东省江门市新山市和情共建路 (gōng chǎng guǎng dōng shěng jiāng mén shì xīn shān shì hé qíng gòng jiàn lù)305号座 (hào zuò) 公司地址 (gōng sī dì zhǐ):广州市白云区龙街尖路 (guǎng zhōu shì bái yún qū lóng jiē jiān lù)363号联边国际 (hào lián biān guó jì)620单元 (dān yuán)Factory: Building 305, Heqing Gongjian Road, Xinshan City, Jiangmen City, Guangdong Province. Company Address: Unit 620, Lianbian International, No. 363, Longjie Jian Road, Baiyun District, Guangzhou</t>
+          <t>No. 363, Longjie Jian Road, Baiyun District, Guangzhou</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -842,7 +842,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2nd Road, Chikan, ShipaiTown, Dongguan, Guangdong, 523346.China</t>
+          <t>nd Road, Chikan, ShipaiTown, Dongguan, Guangdong, 523346.China</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1087,7 +1087,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Bella 陈丽霞 (chén lì xiá)</t>
+          <t>Bella chén lì xiá</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1117,7 +1117,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>陈孔清 (chén kǒng qīng)</t>
+          <t>chén kǒng qīng</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1157,7 +1157,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>广东省广州市花都区秀全街道大布路 (guǎng dōng shěng guǎng zhōu shì huā dōu qū xiù quán jiē dào dà bù lù)29号峰华工业园 (hào fēng huá gōng yè yuán)Fenghua Industrial Park, No. 29 Dabu Road, Xiuquan Street, Huadu District, Guangzhou City, Guangdong Province</t>
+          <t>No. 29 Dabu Road, Xiuquan Street, Huadu District, Guangzhou City, Guangdong Province</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1182,7 +1182,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>胡明 (hú míng)</t>
+          <t>hú míng</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1192,7 +1192,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>广东省清远英德市英红镇万洋众创城 (guǎng dōng shěng qīng yuǎn yīng dé shì yīng hóng zhèn wàn yáng zhòng chuàng chéng)D区 (qū)37栋 (dòng)Building 37, Zone D, Wanyang Maker Town, Yinghong Town, Yingde City, Qingyuan City, Guangdong Province</t>
+          <t>D 37 Building 37, Zone D, Wanyang Maker Town, Yinghong Town, Yingde City, Qingyuan City, Guangdong Province</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1277,7 +1277,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>42 floor, R &amp; F Dongshan New World Building, No.307 Guangzhou dadao zhong, Tianhe District, Guangzhou</t>
+          <t>No.307 Guangzhou dadao zhong, Tianhe District, Guangzhou</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1302,7 +1302,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>谭玉雄 (tán yù xióng)</t>
+          <t>tán yù xióng</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1322,7 +1322,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>广东省东莞市谢岗镇曹乐向阳路 (guǎng dōng shěng dōng guǎn shì xiè gǎng zhèn cáo lè xiàng yáng lù)55号 (hào), 广东省东莞市樟木头镇塑料市场一期 (guǎng dōng shěng dōng guǎn shì zhāng mù tou zhèn sù liào shì chǎng yī qī)V栋 (dòng)1-2号 (hào), 广东省东莞市常平镇大京九塑料市场塑发东路 (guǎng dōng shěng dōng guǎn shì cháng píng zhèn dà jīng jiǔ sù liào shì chǎng sù fā dōng lù)53-54号 (hào)No. 55, Caole Xiangyang Road, Xiegang Town, Dongguan City, Guangdong Province, Building V, Units 1-2, Phase 1, Plastic Market, Zhangmutou Town, Dongguan City, Guangdong Province, No. 53-54, Sufa East Road, Dajingjiu Plastic Market, Changping Town, Dongguan City, Guangdong Province</t>
+          <t>No. 55, Caole Xiangyang Road, Xiegang Town, Dongguan City, Guangdong Province, Building V, Units 1-2, Phase 1, Plastic Market, Zhangmutou Town, Dongguan City, Guangdong Province, No. 53-54, Sufa East Road, Dajingjiu Plastic Market, Changping Town, Dongguan City, Guangdong Province</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1397,7 +1397,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Guangzhou City, Yuexiu District, Guangyuan West Road No. 121, Commercial Center C, 3rd Floor, Room 022, Guangzhou City, Baiyun District, Zhongluotan Town, Liantian North Road No. 9, Building 6, Chenmei Industrial Park</t>
+          <t>No. 121, Commercial Center C, 3rd Floor, Room 022, Guangzhou City, Baiyun District, Zhongluotan Town, Liantian North Road No. 9, Building 6, Chenmei Industrial Park</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -1457,7 +1457,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>陈总 (chén zǒng)</t>
+          <t>chén zǒng</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1467,7 +1467,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>广州市花都区先科一路金禾云创产业园 (guǎng zhōu shì huā dōu qū xiān kē yī lù jīn hé yún chuàng chǎn yè yuán)Jinhe Yun Chuang Industrial Park, Xianke 1st Road, Huadu District, Guangzhou City</t>
+          <t>Jinhe Yun Chuang Industrial Park, Xianke 1st Road, Huadu District, Guangzhou City</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -1507,7 +1507,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>广州市越秀区先烈中路 (guǎng zhōu shì yuè xiù qū xiān liè zhōng lù)85号浙江大厦 (hào zhè jiāng dà shà)9楼 (lóu)9th Floor, Zhejiang Building, No. 85, Xianlie Middle Road, Yuexiu District, Guangzhou City</t>
+          <t>No. 85, Xianlie Middle Road, Yuexiu District, Guangzhou City</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -1532,7 +1532,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>吴月芳 (wú yuè fāng)</t>
+          <t>wú yuè fāng</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1592,7 +1592,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Room 4002, 4th Floor, Meiwan Square, Sanyuanli Street, Baiyun District, Guangzhou, Guangdong Province Ouyu Square, Huangjinling, Tangge Village, Baiyun Lake Street, Baiyun District, Guangzhou, Guangdong Province No. 18, Zone A, Hegui Industrial Park, Nanhai District, Foshan City, Guangdong Province</t>
+          <t>No. 18, Zone A, Hegui Industrial Park, Nanhai District, Foshan City, Guangdong Province</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -1662,7 +1662,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>陈泳 (chén yǒng)</t>
+          <t>chén yǒng</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1672,7 +1672,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>广州市白云区均禾街清湖村大山路 (guǎng zhōu shì bái yún qū jūn hé jiē qīng hú cūn dà shān lù)6号 (hào)No. 6, Dashan Road, Qinghu Village, Junhe Street, Baiyun District, Guangzhou City</t>
+          <t>No. 6, Dashan Road, Qinghu Village, Junhe Street, Baiyun District, Guangzhou City</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -1742,7 +1742,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>赖梓浩 (lài zǐ hào)</t>
+          <t>lài zǐ hào</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1762,7 +1762,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Add. No. 88, Yongli Road, Xinhua Street, District, Guangzhou, China</t>
+          <t>No. 88, Yongli Road, Xinhua Street, District, Guangzhou, China</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -1787,7 +1787,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>刘金连 (liú jīn lián)</t>
+          <t>liú jīn lián</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -1822,7 +1822,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>赵新亮 (zhào xīn liàng)</t>
+          <t>zhào xīn liàng</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1832,7 +1832,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>广州市白云区北村北大路 (guǎng zhōu shì bái yún qū běi cūn běi dà lù)22号四栋二楼 (hào sì dòng èr lóu)Second Floor, Building 4, No. 22, Beicun Beida Road, Baiyun District, Guangzhou City</t>
+          <t>No. 22, Beicun Beida Road, Baiyun District, Guangzhou City</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -2037,7 +2037,7 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Room 905/906/907, Building 2, Yuntuhui, No. 239, Yuncheng South Fourth Road, Baiyun District, Guangzhou</t>
+          <t>No. 239, Yuncheng South Fourth Road, Baiyun District, Guangzhou</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -2282,7 +2282,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>曹春 (cáo chūn)</t>
+          <t>cáo chūn</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -2292,7 +2292,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>广州市白云区石井街石井大道 (guǎng zhōu shì bái yún qū shí jǐng jiē shí jǐng dà dào)634号 (hào)No. 634, Shijing Avenue, Shijing Street, Baiyun District, Guangzhou City</t>
+          <t>No. 634, Shijing Avenue, Shijing Street, Baiyun District, Guangzhou City</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -2337,7 +2337,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>上海市浦东新区世纪大道 (shàng hǎi shì pǔ dōng xīn qū shì jì dà dào)100号 (hào)No. 100, Century Avenue, Pudong New Area, Shanghai</t>
+          <t>No. 100, Century Avenue, Pudong New Area, Shanghai</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -2362,7 +2362,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>章海翰 (zhāng hǎi hàn)</t>
+          <t>zhāng hǎi hàn</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2377,7 +2377,7 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>Industrial Area No.3, Xiaqi Road and Hudi Road, Jinping District, Shantou city, Guangdong Province, China.</t>
+          <t>No.3, Xiaqi Road and Hudi Road, Jinping District, Shantou city, Guangdong Province, China.</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -2507,7 +2507,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>上海市奉贤区大叶公路 (shàng hǎi shì fèng xián qū dà yè gōng lù) 6818号 (hào)5A栋 (dòng)502Room 502, Building 5A, No. 6818, Daye Highway, Fengxian District, Shanghai City</t>
+          <t>No. 6818, Daye Highway, Fengxian District, Shanghai City</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -2532,7 +2532,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>陈雪萍 (chén xuě píng)</t>
+          <t>chén xuě píng</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -2552,7 +2552,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>广东省惠州市博罗县石湾镇马石围路 (guǎng dōng shěng huì zhōu shì bó luó xiàn shí wān zhèn mǎ shí wéi lù)3号 (hào)No. 3, Mashiwei Road, Shiwan Town, Boluo County, Huizhou City, Guangdong Province</t>
+          <t>No. 3, Mashiwei Road, Shiwan Town, Boluo County, Huizhou City, Guangdong Province</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -2577,7 +2577,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>何丽银 (hé lì yín)</t>
+          <t>hé lì yín</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -2597,7 +2597,7 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>广东省清远市清城区石角镇广清产业园广创街 (guǎng dōng shěng qīng yuǎn shì qīng chéng qū shí jiǎo zhèn guǎng qīng chǎn yè yuán guǎng chuàng jiē)6号 (hào)No. 6, Guangchuang Street, Guangqing Industrial Park, Shijiao Town, Qingcheng District, Qingyuan City, Guangdong Province</t>
+          <t>No. 6, Guangchuang Street, Guangqing Industrial Park, Shijiao Town, Qingcheng District, Qingyuan City, Guangdong Province</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -2622,7 +2622,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>冉露茜 (rǎn lù qiàn)</t>
+          <t>rǎn lù qiàn</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -2642,7 +2642,7 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>黄浦区德必上海书城 (huáng pǔ qū dé bì shàng hǎi shū chéng)WE2101室 (shì)Room WE2101, Debao Shanghai Book City, Huangpu District</t>
+          <t>WE2101 Room WE2101, Debao Shanghai Book City, Huangpu District</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -2682,7 +2682,7 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>浙江省嘉兴市南湖区新丰镇新禾路 (zhè jiāng shěng jiā xīng shì nán hú qū xīn fēng zhèn xīn hé lù)158号 (hào)No. 158, Xinhe Road, Xinfeng Town, Nanhu District, Jiaxing City, Zhejiang Province</t>
+          <t>No. 158, Xinhe Road, Xinfeng Town, Nanhu District, Jiaxing City, Zhejiang Province</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -2767,7 +2767,7 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>No.69 Zhubei Rd. (E) Mazhu Town, Yuvac Zhejiang Province (P.C. 315450) No.888 Beixing Rd. Mazhu Town. Yuyao Zhejiang Province(P.C. 315450)</t>
+          <t>No.69 Zhubei Rd. Mazhu Town, Yuvac Zhejiang Province No.888 Beixing Rd. Mazhu Town. Yuyao Zhejiang Province</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -2792,7 +2792,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>陈铁文 (chén tiě wén)</t>
+          <t>chén tiě wén</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -2807,7 +2807,7 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>福建省晋江市经济开发区 (fú jiàn shěng jìn jiāng shì jīng jì kāi fā qū) 广东省深圳市龙华新区建设路与东环二路交汇处聚豪国际 (guǎng dōng shěng shēn zhèn shì lóng huá xīn qū jiàn shè lù yǔ dōng huán èr lù jiāo huì chù jù háo guó jì)A栋 (dòng)2504室 (shì)Room 2504, Building A, Juhuao International, Intersection of Jianshe Road and Donghuan 2nd Road, Longhua New District, Shenzhen City, Guangdong Province; Jinjiang Economic Development Zone, Jinjiang City, Fujian Province</t>
+          <t>A 2504 Room 2504, Building A, Juhuao International, Intersection of Jianshe Road and Donghuan 2nd Road, Longhua New District, Shenzhen City, Guangdong Province; Jinjiang Economic Development Zone, Jinjiang City, Fujian Province</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -2852,7 +2852,7 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>3rd Floor, Building 6, No. 25, Fuyuan 1st Road, Xinya Subdistrict, Huadu District, Guangzhou City, Guangdong Province</t>
+          <t>No. 25, Fuyuan 1st Road, Xinya Subdistrict, Huadu District, Guangzhou City, Guangdong Province</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -2877,7 +2877,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>周 (zhōu) 亮 (liàng)</t>
+          <t>zhōu liàng</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -3137,7 +3137,7 @@
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>广州市天河区林和东路 (guǎng zhōu shì tiān hé qū lín hé dōng lù)285号中汇人寿 (hào zhōng huì rén shòu)901Room 901, Zhonghui Life Insurance, No. 285 Linhe East Road, Tianhe District, Guangzhou City</t>
+          <t>No. 285 Linhe East Road, Tianhe District, Guangzhou City</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -3162,7 +3162,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>李金花 (lǐ jīn huā)</t>
+          <t>lǐ jīn huā</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -3227,7 +3227,7 @@
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>广州市白云区鶴拳路一横路科我园 (guǎng zhōu shì bái yún qū hè quán lù yī héng lù kē wǒ yuán)3栋 (dòng)Building 3, Kewoyuan, Yiheng Road, Hequan Road, Baiyun District, Guangzhou City</t>
+          <t>Building 3, Kewoyuan, Yiheng Road, Hequan Road, Baiyun District, Guangzhou City</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
@@ -3417,7 +3417,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Cécilia 叶思颖 (yè sī yǐng)</t>
+          <t>Cécilia yè sī yǐng</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -3437,7 +3437,7 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>Building E1, Huangpu Technology Headquarters Port, Liandong U Valley, No. 10, Xicheng Middle Street, Nanwan, Huangpu District, Guangzhou, Guangdong, China</t>
+          <t>No. 10, Xicheng Middle Street, Nanwan, Huangpu District, Guangzhou, Guangdong, China</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -3477,7 +3477,7 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>Floor 4, Building C, Shengmeng Industrial Park, No.70 Xiangxia Avenue, Longgui, Taihe Town, Baiyun District, Guangzhou, China</t>
+          <t>No.70 Xiangxia Avenue, Longgui, Taihe Town, Baiyun District, Guangzhou, China</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
@@ -3542,7 +3542,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>洪碧虹 (hóng bì hóng)</t>
+          <t>hóng bì hóng</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -3557,7 +3557,7 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>汕头市金平区岐山街道中宫社区建明工业城 (shàn tóu shì jīn píng qū qí shān jiē dào zhōng gōng shè qū jiàn míng gōng yè chéng)11-12栋楼 (dòng lóu)Buildings 11-12, Jianming Industrial City, Zhonggong Community, Qishan Street, Jinping District, Shantou City</t>
+          <t>-12 Buildings 11-12, Jianming Industrial City, Zhonggong Community, Qishan Street, Jinping District, Shantou City</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
@@ -3732,7 +3732,7 @@
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>Umbrella Industrial Park, Songxia Town, Shangyu Dist., Shaoxing, Zhejiang, China (Mainland)</t>
+          <t>Umbrella Industrial Park, Songxia Town, Shangyu Dist., Shaoxing, Zhejiang, China</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
@@ -3802,7 +3802,7 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>何燕芳 (hé yàn fāng) Orla</t>
+          <t>hé yàn fāng Orla</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -3842,7 +3842,7 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>陈乐 (chén lè)</t>
+          <t>chén lè</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -3862,7 +3862,7 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>广州市赛康尼机械设备有限公司 (guǎng zhōu shì sài kāng ní jī xiè shè bèi yǒu xiàn gōng sī) 广州市黄埔区南岗街道中南街 (guǎng zhōu shì huáng pǔ qū nán gǎng jiē dào zhōng nán jiē)10号联系中心办公室楼南面主楼南面 (hào lián xì zhōng xīn bàn gōng shì lóu nán miàn zhǔ lóu nán miàn)Guangzhou Saikenni Machinery Equipment Co., Ltd. South side of the main building, south side of the Contact Center Office Building, No. 10, Zhongnan Street, Nangang Subdistrict, Huangpu District, Guangzhou</t>
+          <t>No. 10, Zhongnan Street, Nangang Subdistrict, Huangpu District, Guangzhou</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
@@ -3887,7 +3887,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>鲍焕威 (bào huàn wēi) Bao huan wei</t>
+          <t>bào huàn wēi Bao huan wei</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -3927,7 +3927,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>黄顺好 (huáng shùn hǎo)</t>
+          <t>huáng shùn hǎo</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
@@ -3947,7 +3947,7 @@
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>广东佛山市顺德区伦教来涌工业区 (guǎng dōng fó shān shì shùn dé qū lún jiào lái yǒng gōng yè qū)Laiyong Industrial Zone, Lunqiao, Shunde District, Foshan City, Guangdong</t>
+          <t>Laiyong Industrial Zone, Lunqiao, Shunde District, Foshan City, Guangdong</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
@@ -3972,7 +3972,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>邵仕华 (shào shì huá)</t>
+          <t>shào shì huá</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
@@ -4012,7 +4012,7 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>陈晓雯 (chén xiǎo wén)</t>
+          <t>chén xiǎo wén</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
@@ -4027,7 +4027,7 @@
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>广东省清远市清城区石角镇 (guǎng dōng shěng qīng yuǎn shì qīng chéng qū shí jiǎo zhèn)(广清产业园 (guǎng qīng chǎn yè yuán))兴园路 (xīng yuán lù)3号 (hào); 广州市花都区新雅街绿地空港五号地 (guǎng zhōu shì huā dōu qū xīn yǎ jiē lǜ dì kōng gǎng wǔ hào dì)4栋 (dòng)1107室 (shì)No. 3, Xingyuan Road, Shijiao Town (Guangqing Industrial Park), Qingcheng District, Qingyuan City, Guangdong Province; Room 1107, Building 4, Plot 5, Greenland Airport, Xinya Street, Huadu District, Guangzhou City</t>
+          <t>No. 3, Xingyuan Road, Shijiao Town , Qingcheng District, Qingyuan City, Guangdong Province; Room 1107, Building 4, Plot 5, Greenland Airport, Xinya Street, Huadu District, Guangzhou City</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
@@ -4087,7 +4087,7 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>徐春苗 (xú chūn miáo) Kavi</t>
+          <t>xú chūn miáo Kavi</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
@@ -4102,7 +4102,7 @@
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>浙江省嘉兴市南湖区新丰镇新禾路 (zhè jiāng shěng jiā xīng shì nán hú qū xīn fēng zhèn xīn hé lù)158号 (hào)No. 158, Xinhe Road, Xinfeng Town, Nanhu District, Jiaxing City, Zhejiang Province</t>
+          <t>No. 158, Xinhe Road, Xinfeng Town, Nanhu District, Jiaxing City, Zhejiang Province</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
@@ -4147,7 +4147,7 @@
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>江苏省泰兴市江平北路 (jiāng sū shěng tài xīng shì jiāng píng běi lù)55号 (hào), 上海市徐汇区石龙路 (shàng hǎi shì xú huì qū shí lóng lù)6号 (hào)001室 (shì)No. 55 Jiangping North Road, Taixing City, Jiangsu Province, Room 001, No. 6 Shilong Road, Xuhui District, Shanghai City</t>
+          <t>No. 55 Jiangping North Road, Taixing City, Jiangsu Province, Room 001, No. 6 Shilong Road, Xuhui District, Shanghai City</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
@@ -4257,7 +4257,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>翁铄桓 (wēng shuò huán)</t>
+          <t>wēng shuò huán</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
@@ -4272,7 +4272,7 @@
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>佛山市三水区乐平镇博裕路 (fó shān shì sān shuǐ qū lè píng zhèn bó yù lù)34号 (hào)1栋 (dòng)Building 1, No. 34, Boyu Road, Leping Town, Sanshui District, Foshan City</t>
+          <t>No. 34, Boyu Road, Leping Town, Sanshui District, Foshan City</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
@@ -4297,7 +4297,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>顾友阳 (gù yǒu yáng)</t>
+          <t>gù yǒu yáng</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -4312,7 +4312,7 @@
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>上海市金山区漕泾开发区展业路 (shàng hǎi shì jīn shān qū cáo jīng kāi fā qū zhǎn yè lù)288号一栋 (hào yī dòng)Building 1, No. 288, Zhanye Road, Caojing Development Zone, Jinshan District, Shanghai</t>
+          <t>No. 288, Zhanye Road, Caojing Development Zone, Jinshan District, Shanghai</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
@@ -4387,7 +4387,7 @@
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>5F,No.268, Huandong Road, Xuxiake Town, Jiangyin, Jiangsu, China, 214407</t>
+          <t>No.268, Huandong Road, Xuxiake Town, Jiangyin, Jiangsu, China, 214407</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
@@ -4432,7 +4432,7 @@
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>608, Building 2, Greenland Airport Center Huadu District, Guangzhou City</t>
+          <t>Building 2, Greenland Airport Center Huadu District, Guangzhou City</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
@@ -4457,7 +4457,7 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>林晓荣 (lín xiǎo róng)</t>
+          <t>lín xiǎo róng</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
@@ -4477,7 +4477,7 @@
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>广东省汕头市月浦龙洲路 (guǎng dōng shěng shàn tóu shì yuè pǔ lóng zhōu lù)12号 (hào) Longzhou Road, Yuepu, Shantou City, Guangdong Province, China</t>
+          <t>Longzhou Road, Yuepu, Shantou City, Guangdong Province, China</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
@@ -4502,7 +4502,7 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>谢榕宝 (xiè róng bǎo)</t>
+          <t>xiè róng bǎo</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
@@ -4522,7 +4522,7 @@
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>广州市七星二号 (guǎng zhōu shì qī xīng èr hào)No. 2, Qixing, Guangzhou City</t>
+          <t>No. 2, Qixing, Guangzhou City</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
@@ -4562,7 +4562,7 @@
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>上海市嘉定区树屏路 (shàng hǎi shì jiā dìng qū shù píng lù)588弄财智金岸 (nòng cái zhì jīn àn)35号楼 (hào lóu)Building 35, Caizhi Jin'an, Lane 588, Shuping Road, Jiading District, Shanghai</t>
+          <t>Building 35, Caizhi Jin'an, Lane 588, Shuping Road, Jiading District, Shanghai</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -4647,7 +4647,7 @@
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>Building 31, No.86, Maohai Road, Huangjiabu Town, Yuyao City, Zhejiang Province.</t>
+          <t>No.86, Maohai Road, Huangjiabu Town, Yuyao City, Zhejiang Province.</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
@@ -4717,7 +4717,7 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>苏元元 (sū yuán yuán)</t>
+          <t>sū yuán yuán</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
@@ -4737,7 +4737,7 @@
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>浙江省绍兴市上虞区崧厦街道振兴路 (zhè jiāng shěng shào xīng shì shàng yú qū sōng shà jiē dào zhèn xīng lù)138号 (hào)No. 138, Zhenxing Road, Songsha Street, Shangyu District, Shaoxing City, Zhejiang Province</t>
+          <t>No. 138, Zhenxing Road, Songsha Street, Shangyu District, Shaoxing City, Zhejiang Province</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
@@ -4762,7 +4762,7 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>刘艳霞 (liú yàn xiá)</t>
+          <t>liú yàn xiá</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
@@ -4812,7 +4812,7 @@
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>15 Huachang Road, Mingwei Industrial Zone, Lizhou Street, Yuyao, Zhejiang, China. 168 Yuma Road, Mazhu Town, Yuyao, Zhejiang, China.</t>
+          <t>Huachang Road, Mingwei Industrial Zone, Lizhou Street, Yuyao, Zhejiang, China. 168 Yuma Road, Mazhu Town, Yuyao, Zhejiang, China.</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
@@ -4877,7 +4877,7 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>张亮亮 (zhāng liàng liàng)</t>
+          <t>zhāng liàng liàng</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
@@ -4917,7 +4917,7 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>肖志坚 (xiào zhì jiān)</t>
+          <t>xiào zhì jiān</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
@@ -4932,7 +4932,7 @@
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>上海市松江区叶路 (shàng hǎi shì sōng jiāng qū yè lù)133弄 (nòng)1-3号 (hào)No. 1-3, Lane 133, Ye Road, Songjiang District, Shanghai</t>
+          <t>No. 1-3, Lane 133, Ye Road, Songjiang District, Shanghai</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
@@ -4957,7 +4957,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>王馨苑 (wáng xīn yuàn)</t>
+          <t>wáng xīn yuàn</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
@@ -4977,7 +4977,7 @@
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>广州市花都区花东镇微观产业园 (guǎng zhōu shì huā dōu qū huā dōng zhèn wēi guān chǎn yè yuán)C栋 (dòng)Building C, Weiguan Industrial Park, Huadong Town, Huadu District, Guangzhou</t>
+          <t>C Building C, Weiguan Industrial Park, Huadong Town, Huadu District, Guangzhou</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
@@ -5002,7 +5002,7 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>王丽波 (wáng lì bō)</t>
+          <t>wáng lì bō</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
@@ -5022,7 +5022,7 @@
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>浙江省余姚市牟山镇高车头 (zhè jiāng shěng yú yáo shì móu shān zhèn gāo chē tóu) B67号肖西路西 (hào xiào xī lù xī)West of Xiaoxi Road, Gaochetou, Mushan Town, Yuyao City, Zhejiang Province, No. B67</t>
+          <t>B67 West of Xiaoxi Road, Gaochetou, Mushan Town, Yuyao City, Zhejiang Province, No. B67</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
@@ -5047,7 +5047,7 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>刘锡蓉 (liú xī róng)</t>
+          <t>liú xī róng</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
@@ -5067,7 +5067,7 @@
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>浙江省余姚市马渚镇北兴路 (zhè jiāng shěng yú yáo shì mǎ zhǔ zhèn běi xīng lù)183号 (hào)No. 183, Beixing Road, Mazhu Town, Yuyao City, Zhejiang Province</t>
+          <t>No. 183, Beixing Road, Mazhu Town, Yuyao City, Zhejiang Province</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
@@ -5092,7 +5092,7 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>潘兴杰 (pān xīng jié)</t>
+          <t>pān xīng jié</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
@@ -5112,7 +5112,7 @@
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>廣東省東莞市厚街鎮東業路 (guǎng dōng shěng dōng guǎn shì hòu jiē zhèn dōng yè lù)2號 (hào)No. 2, Dongye Road, Houjie Town, Dongguan City, Guangdong Province</t>
+          <t>No. 2, Dongye Road, Houjie Town, Dongguan City, Guangdong Province</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
@@ -5137,7 +5137,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>胡珍华 (hú zhēn huá)</t>
+          <t>hú zhēn huá</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
@@ -5152,7 +5152,7 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>广州市花都区绿港四街 (guǎng zhōu shì huā dōu qū lǜ gǎng sì jiē)6号 (hào)No. 6, Lvgong 4th Street, Huadu District, Guangzhou</t>
+          <t>No. 6, Lvgong 4th Street, Huadu District, Guangzhou</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -5217,7 +5217,7 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>刘扬娥 (liú yáng é)</t>
+          <t>liú yáng é</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
@@ -5232,7 +5232,7 @@
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>广州市白云区江高镇神山神石路 (guǎng zhōu shì bái yún qū jiāng gāo zhèn shén shān shén shí lù)41号 (hào)No. 41, Shenshan Shishen Road, Jianggao Town, Baiyun District, Guangzhou</t>
+          <t>No. 41, Shenshan Shishen Road, Jianggao Town, Baiyun District, Guangzhou</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
@@ -5257,7 +5257,7 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>林帆 (lín fān)</t>
+          <t>lín fān</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
@@ -5277,7 +5277,7 @@
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>广东省广州市天河区科韵路 (guǎng dōng shěng guǎng zhōu shì tiān hé qū kē yùn lù)288号天盈创意园 (hào tiān yíng chuàng yì yuán) C区 (qū)3024-3027Rooms 3024-3027, Area C, Tianying Creative Park, No. 288 Keyun Road, Tianhe District, Guangzhou City, Guangdong Province</t>
+          <t>No. 288 Keyun Road, Tianhe District, Guangzhou City, Guangdong Province</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
@@ -5302,7 +5302,7 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>刘丽红 (liú lì hóng) Valerie</t>
+          <t>liú lì hóng Valerie</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
@@ -5312,7 +5312,7 @@
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>广东省广州市花都区金田路 (guǎng dōng shěng guǎng zhōu shì huā dōu qū jīn tián lù)3号 (hào)No. 3, Jintian Road, Huadu District, Guangzhou City, Guangdong Province</t>
+          <t>No. 3, Jintian Road, Huadu District, Guangzhou City, Guangdong Province</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
@@ -5337,7 +5337,7 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>梁冠文 (liáng guān wén)</t>
+          <t>liáng guān wén</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
@@ -5352,7 +5352,7 @@
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>广州市白云区北太路 (guǎng zhōu shì bái yún qū běi tài lù)1633号广州民营科技园科园路 (hào guǎng zhōu mín yíng kē jì yuán kē yuán lù)2号凯铂中心 (hào kǎi bó zhōng xīn)D区 (qū)1-4楼 (lóu) 1-4 F, Area D. Kaibo Center Building, No.2 Keyuan Road, Guangzhou Private Science and Technology Park, No. 1633 Beitai Road, Baiyun District, Guangzhou</t>
+          <t>No.2 Keyuan Road, Guangzhou Private Science and Technology Park, No. 1633 Beitai Road, Baiyun District, Guangzhou</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
@@ -5377,7 +5377,7 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>熊强 (xióng qiáng) Xiong Qiang</t>
+          <t>xióng qiáng Xiong Qiang</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
@@ -5387,7 +5387,7 @@
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>广东省清远市佛冈县汤塘镇广佛产业园创业路 (guǎng dōng shěng qīng yuǎn shì fú gāng xiàn tāng táng zhèn guǎng fú chǎn yè yuán chuàng yè lù)7号 (hào) C区 (qū)6栋 (dòng)101-501房 (fáng)Room 101-501, Building 6, Zone C, No. 7, Chuangye Road, Guangfo Industrial Park, Tangtang Town, Fogang County, Qingyuan City, Guangdong Province</t>
+          <t>No. 7, Chuangye Road, Guangfo Industrial Park, Tangtang Town, Fogang County, Qingyuan City, Guangdong Province</t>
         </is>
       </c>
       <c r="I121" t="inlineStr">
@@ -5412,7 +5412,7 @@
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>李娟 (lǐ juān) LiJuan</t>
+          <t>lǐ juān LiJuan</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
@@ -5432,7 +5432,7 @@
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>广州市白云区江高镇 (guǎng zhōu shì bái yún qū jiāng gāo zhèn)408号工业园 (hào gōng yè yuán) A区 (qū) 11/F Building 7 Awang Industrial Zone, Baiyun District, Guangzhou City</t>
+          <t>A 11/F Building 7 Awang Industrial Zone, Baiyun District, Guangzhou City</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
@@ -5457,7 +5457,7 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>肖海青 (xiào hǎi qīng)</t>
+          <t>xiào hǎi qīng</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
@@ -5477,7 +5477,7 @@
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>中山工厂 (zhōng shān gōng chǎng):广东省中山市火炬开发区茂南路 (guǎng dōng shěng zhōng shān shì huǒ jù kāi fā qū mào nán lù)25号 (hào) 惠州工厂 (huì zhōu gōng chǎng):广东省惠州市龙门县金山工业园建设路 (guǎng dōng shěng huì zhōu shì lóng mén xiàn jīn shān gōng yè yuán jiàn shè lù)2号 (hào)Zhongshan Factory: No. 25, Maonan Road, Torch Development Zone, Zhongshan City, Guangdong Province; Huizhou Factory: No. 2, Jianshe Road, Jinshan Industrial Park, Longmen County, Huizhou City, Guangdong Province</t>
+          <t>No. 25, Maonan Road, Torch Development Zone, Zhongshan City, Guangdong Province; Huizhou Factory: No. 2, Jianshe Road, Jinshan Industrial Park, Longmen County, Huizhou City, Guangdong Province</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
@@ -5502,7 +5502,7 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>郭武杰 (guō wǔ jié)</t>
+          <t>guō wǔ jié</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
@@ -5517,7 +5517,7 @@
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>广州天河区广州大道中 (guǎng zhōu tiān hé qū guǎng zhōu dà dào zhōng)307号富力东山新天地中心 (hào fù lì dōng shān xīn tiān dì zhōng xīn)42楼 (lóu)(总部营销中心 (zǒng bù yíng xiāo zhōng xīn))42nd Floor (Headquarters Marketing Center), Fuli Dongshan Xintiandi Center, No. 307 Guangzhou Avenue Middle, Tianhe District, Guangzhou</t>
+          <t>No. 307 Guangzhou Avenue Middle, Tianhe District, Guangzhou</t>
         </is>
       </c>
       <c r="I124" t="inlineStr">
@@ -5542,7 +5542,7 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>陈花蕾 (chén huā lěi) Chen Hualel</t>
+          <t>chén huā lěi Chen Hualel</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
@@ -5562,7 +5562,7 @@
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>广州市白云区云城东路云理汇 (guǎng zhōu shì bái yún qū yún chéng dōng lù yún lǐ huì)2栋 (dòng)3楼 (lóu)3rd Floor, Building 2, Yunlihui, Yuncheng East Road, Baiyun District, Guangzhou</t>
+          <t>3rd Floor, Building 2, Yunlihui, Yuncheng East Road, Baiyun District, Guangzhou</t>
         </is>
       </c>
       <c r="I125" t="inlineStr">
@@ -5587,7 +5587,7 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>李小娜 (lǐ xiǎo nà)</t>
+          <t>lǐ xiǎo nà</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
@@ -5602,7 +5602,7 @@
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>广州市从化区明珠工业园宝聚路二号 (guǎng zhōu shì cóng huà qū míng zhū gōng yè yuán bǎo jù lù èr hào)No. 2, Baoju Road, Mingzhu Industrial Park, Conghua District, Guangzhou City</t>
+          <t>No. 2, Baoju Road, Mingzhu Industrial Park, Conghua District, Guangzhou City</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
@@ -5627,7 +5627,7 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>彭练芝 (péng liàn zhī)</t>
+          <t>péng liàn zhī</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
@@ -5642,7 +5642,7 @@
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>广州市白云区江高镇神山神石路 (guǎng zhōu shì bái yún qū jiāng gāo zhèn shén shān shén shí lù)41号 (hào)No. 41, Shenshan Shishen Road, Jianggao Town, Baiyun District, Guangzhou</t>
+          <t>No. 41, Shenshan Shishen Road, Jianggao Town, Baiyun District, Guangzhou</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
@@ -5667,7 +5667,7 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>李文慧 (lǐ wén huì)</t>
+          <t>lǐ wén huì</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
@@ -5677,7 +5677,7 @@
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>广东省广州市花都区花东镇北兴北钟路 (guǎng dōng shěng guǎng zhōu shì huā dōu qū huā dōng zhèn běi xīng běi zhōng lù)54号 (hào)No. 54, Beixing Beizhong Road, Huadong Town, Huadu District, Guangzhou City, Guangdong Province</t>
+          <t>No. 54, Beixing Beizhong Road, Huadong Town, Huadu District, Guangzhou City, Guangdong Province</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
@@ -5702,7 +5702,7 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>刘绍伟 (liú shào wěi)</t>
+          <t>liú shào wěi</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
@@ -5722,7 +5722,7 @@
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>佛山市三水区乐平镇博裕路 (fó shān shì sān shuǐ qū lè píng zhèn bó yù lù)34号 (hào)1栋 (dòng)Building 1, No. 34, Boyu Road, Leping Town, Sanshui District, Foshan City</t>
+          <t>No. 34, Boyu Road, Leping Town, Sanshui District, Foshan City</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
@@ -5747,7 +5747,7 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>陈坤 (chén kūn)</t>
+          <t>chén kūn</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
@@ -5762,7 +5762,7 @@
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>广州市白云区云城西路娇兰佳人大厦 (guǎng zhōu shì bái yún qū yún chéng xī lù jiāo lán jiā rén dà shà)10楼 (lóu)10th Floor, Jiaolan Jiada Building, Yuncheng West Road, Baiyun District, Guangzhou City</t>
+          <t>th Floor, Jiaolan Jiada Building, Yuncheng West Road, Baiyun District, Guangzhou City</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
@@ -5787,7 +5787,7 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>卿慧 (qīng huì)</t>
+          <t>qīng huì</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
@@ -5807,7 +5807,7 @@
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>广州市白云区三元里大道 (guǎng zhōu shì bái yún qū sān yuán lǐ dà dào)11号中港皮具城 (hào zhōng gǎng pí jù chéng)10楼 (lóu)1009室 (shì)Room 1009, 10th Floor, Zhonggang Leather City, No. 11, Sanyuanli Avenue, Baiyun District, Guangzhou City</t>
+          <t>No. 11, Sanyuanli Avenue, Baiyun District, Guangzhou City</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
@@ -5832,7 +5832,7 @@
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>邹永流 (zōu yǒng liú)</t>
+          <t>zōu yǒng liú</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
@@ -5847,7 +5847,7 @@
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>广州市越秀区先烈中路 (guǎng zhōu shì yuè xiù qū xiān liè zhōng lù)85号浙江大厦 (hào zhè jiāng dà shà)9楼 (lóu)9th Floor, Zhejiang Building, No. 85, Xianlie Middle Road, Yuexiu District, Guangzhou City</t>
+          <t>No. 85, Xianlie Middle Road, Yuexiu District, Guangzhou City</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
@@ -5872,7 +5872,7 @@
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>罗文豪 (luó wén háo) Louis</t>
+          <t>luó wén háo Louis</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
@@ -5887,7 +5887,7 @@
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>广州市从化区横江路 (guǎng zhōu shì cóng huà qū héng jiāng lù)339号 (hào) -36号鸿志软管 (hào hóng zhì ruǎn guǎn)Hongzhi Hose, No. 339-36, Hengjiang Road, Conghua District, Guangzhou City</t>
+          <t>No. 339-36, Hengjiang Road, Conghua District, Guangzhou City</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
@@ -5927,7 +5927,7 @@
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>广州市白云区太和镇谢家注兰西路 (guǎng zhōu shì bái yún qū tài hé zhèn xiè jiā zhù lán xī lù)2号 (hào) No. 2 Yinian West Road, Xielazhuang, Taihe Town layun District, Duangzhou City</t>
+          <t>No. 2 Yinian West Road, Xielazhuang, Taihe Town layun District, Duangzhou City</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
@@ -5952,7 +5952,7 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>于舒情 (yú shū qíng)</t>
+          <t>yú shū qíng</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
@@ -5962,7 +5962,7 @@
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>广州市白云区太和镇谢家庄荫兰西路 (guǎng zhōu shì bái yún qū tài hé zhèn xiè jiā zhuāng yīn lán xī lù)2号 (hào)No. 2, Yinlan West Road, Xiejiazhuang, Taihe Town, Baiyun District, Guangzhou City</t>
+          <t>No. 2, Yinlan West Road, Xiejiazhuang, Taihe Town, Baiyun District, Guangzhou City</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
@@ -5987,7 +5987,7 @@
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>石小姐 (shí xiǎo jiě) SHI XIAOJIE</t>
+          <t>shí xiǎo jiě SHI XIAOJIE</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
@@ -6007,7 +6007,7 @@
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>广州市白云区龙归街南岭村岗埔大道 (guǎng zhōu shì bái yún qū lóng guī jiē nán lǐng cūn gǎng pǔ dà dào)1号 (hào)No. 1 Gangpu Avenue, Nanling Village, Longgui Street, Baiyun District, Guangzhou City</t>
+          <t>No. 1 Gangpu Avenue, Nanling Village, Longgui Street, Baiyun District, Guangzhou City</t>
         </is>
       </c>
       <c r="I136" t="inlineStr">
@@ -6032,7 +6032,7 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>梁凯豪 (liáng kǎi háo)</t>
+          <t>liáng kǎi háo</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
@@ -6082,7 +6082,7 @@
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>广州市花都区凤凰南路 (guǎng zhōu shì huā dōu qū fèng huáng nán lù)61号卓美大楼北楼 (hào zhuó měi dà lóu běi lóu)307室 (shì)Room 307, North Building, Zhuomei Building, No. 61, Fenghuang South Road, Huadu District, Guangzhou</t>
+          <t>No. 61, Fenghuang South Road, Huadu District, Guangzhou</t>
         </is>
       </c>
       <c r="I138" t="inlineStr">
@@ -6107,7 +6107,7 @@
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>黎金昌 (lí jīn chāng)</t>
+          <t>lí jīn chāng</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
@@ -6127,7 +6127,7 @@
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>廣州市白雲區龍歸街夏良東路 (guǎng zhōu shì bái yún qū lóng guī jiē xià liáng dōng lù)81號 (hào)102房 (fáng)Room 102, No. 81, Xialiang East Road, Longgui Street, Baiyun District, Guangzhou</t>
+          <t>No. 81, Xialiang East Road, Longgui Street, Baiyun District, Guangzhou</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
@@ -6167,7 +6167,7 @@
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>廣州市花都區花山鎮城西村自編 (guǎng zhōu shì huā dōu qū huā shān zhèn chéng xī cūn zì biān)3號 (hào)No. 3 (self-numbered), Chengxi Village, Huashan Town, Huadu District, Guangzhou City</t>
+          <t>No. 3 , Chengxi Village, Huashan Town, Huadu District, Guangzhou City</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
@@ -6187,7 +6187,7 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>祝依婷 (zhù yī tíng) Carrie</t>
+          <t>zhù yī tíng Carrie</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
@@ -6197,7 +6197,7 @@
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>广东省广州市花都区金田路 (guǎng dōng shěng guǎng zhōu shì huā dōu qū jīn tián lù)3号 (hào)No. 3, Jintian Road, Huadu District, Guangzhou City, Guangdong Province</t>
+          <t>No. 3, Jintian Road, Huadu District, Guangzhou City, Guangdong Province</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
@@ -6222,7 +6222,7 @@
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>邓思艺 (dèng sī yì)</t>
+          <t>dèng sī yì</t>
         </is>
       </c>
       <c r="E142" t="inlineStr">
@@ -6237,7 +6237,7 @@
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>广东省清远市清城区石角镇 (guǎng dōng shěng qīng yuǎn shì qīng chéng qū shí jiǎo zhèn)(广清产业园 (guǎng qīng chǎn yè yuán))兴园路 (xīng yuán lù)3号 (hào); 广州市花都区新雅街绿地空港五号地 (guǎng zhōu shì huā dōu qū xīn yǎ jiē lǜ dì kōng gǎng wǔ hào dì)4栋 (dòng)1107室 (shì)No. 3, Xingyuan Road, Shijiao Town (Guangqing Industrial Park), Qingcheng District, Qingyuan City, Guangdong Province; Room 1107, Building 4, Plot 5, Greenland Airport, Xinya Street, Huadu District, Guangzhou City</t>
+          <t>No. 3, Xingyuan Road, Shijiao Town , Qingcheng District, Qingyuan City, Guangdong Province; Room 1107, Building 4, Plot 5, Greenland Airport, Xinya Street, Huadu District, Guangzhou City</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
@@ -6262,7 +6262,7 @@
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>江思蓉 (jiāng sī róng)</t>
+          <t>jiāng sī róng</t>
         </is>
       </c>
       <c r="E143" t="inlineStr">
@@ -6292,7 +6292,7 @@
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>刘键均 (liú jiàn jūn)</t>
+          <t>liú jiàn jūn</t>
         </is>
       </c>
       <c r="E144" t="inlineStr">
@@ -6302,7 +6302,7 @@
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>广州市白云区云城西路 (guǎng zhōu shì bái yún qū yún chéng xī lù)888号绿地中心 (hào lǜ dì zhōng xīn)2403Room 2403, Greenland Center, No. 888 Yuncheng West Road, Baiyun District, Guangzhou City</t>
+          <t>No. 888 Yuncheng West Road, Baiyun District, Guangzhou City</t>
         </is>
       </c>
       <c r="I144" t="inlineStr">
@@ -6327,7 +6327,7 @@
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>马壮茂 (mǎ zhuàng mào)</t>
+          <t>mǎ zhuàng mào</t>
         </is>
       </c>
       <c r="E145" t="inlineStr">
@@ -6362,7 +6362,7 @@
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>谢雅琪 (xiè yǎ qí)</t>
+          <t>xiè yǎ qí</t>
         </is>
       </c>
       <c r="E146" t="inlineStr">
@@ -6382,7 +6382,7 @@
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>浙江省绍兴市上虞区曹娥街道五星西路 (zhè jiāng shěng shào xīng shì shàng yú qū cáo é jiē dào wǔ xīng xī lù)1999号联东 (hào lián dōng)U谷 (gǔ)21栋 (dòng)C永 (yǒng), Add C tongin Bulding 21. Landong U Valley No. 1999, Wing West Road Cace Sheet, Shangyu District. Shocking City Zhellong ProvinceBuilding 21 C, Landong U Valley, No. 1999, Wuxing West Road, Cao'e Street, Shangyu District, Shaoxing City, Zhejiang Province</t>
+          <t>No. 1999, Wing West Road Cace Sheet, Shangyu District. Shocking City Zhellong ProvinceBuilding 21 C, Landong U Valley, No. 1999, Wuxing West Road, Cao'e Street, Shangyu District, Shaoxing City, Zhejiang Province</t>
         </is>
       </c>
       <c r="I146" t="inlineStr">
@@ -6407,7 +6407,7 @@
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>朱斌 (zhū bīn)</t>
+          <t>zhū bīn</t>
         </is>
       </c>
       <c r="E147" t="inlineStr">
@@ -6422,7 +6422,7 @@
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>浙江省平湖市新仓镇嘉创智谷远景产业园 (zhè jiāng shěng píng hú shì xīn cāng zhèn jiā chuàng zhì gǔ yuǎn jǐng chǎn yè yuán)A7栋 (dòng)Building A7, Jia Chuang Zhi Gu Yuan Jing Industrial Park, Xincang Town, Pinghu City, Zhejiang Province</t>
+          <t>A7 Building A7, Jia Chuang Zhi Gu Yuan Jing Industrial Park, Xincang Town, Pinghu City, Zhejiang Province</t>
         </is>
       </c>
       <c r="I147" t="inlineStr">
@@ -6447,7 +6447,7 @@
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>周晓娟 (zhōu xiǎo juān)</t>
+          <t>zhōu xiǎo juān</t>
         </is>
       </c>
       <c r="E148" t="inlineStr">
@@ -6462,7 +6462,7 @@
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>江苏省淮安市洪泽区九牛路 (jiāng sū shěng huái ān shì hóng zé qū jiǔ niú lù)8号 (hào) 邮政编号 (yóu zhèng biān hào)223100No. 8, Jiuniu Road, Hongze District, Huai'an City, Jiangsu Province, Postal Code 223100</t>
+          <t>No. 8, Jiuniu Road, Hongze District, Huai'an City, Jiangsu Province, Postal Code 223100</t>
         </is>
       </c>
       <c r="I148" t="inlineStr">
@@ -6487,7 +6487,7 @@
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>章程 (zhāng chéng)</t>
+          <t>zhāng chéng</t>
         </is>
       </c>
       <c r="E149" t="inlineStr">
@@ -6497,7 +6497,7 @@
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>广东省广州市花都区花山镇华辉路 (guǎng dōng shěng guǎng zhōu shì huā dōu qū huā shān zhèn huá huī lù)18号 (hào) 微观化妆品创意产业园 (wēi guān huà zhuāng pǐn chuàng yì chǎn yè yuán)D栋整栋 (dòng zhěng dòng)、H栋整栋 (dòng zhěng dòng)Entire Building D and Entire Building H, Weiguan Cosmetics Creative Industrial Park, No. 18, Huahui Road, Huashan Town, Huadu District, Guangzhou City, Guangdong Province</t>
+          <t>No. 18, Huahui Road, Huashan Town, Huadu District, Guangzhou City, Guangdong Province</t>
         </is>
       </c>
       <c r="I149" t="inlineStr">
@@ -6557,7 +6557,7 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>游文聪 (yóu wén cōng)</t>
+          <t>yóu wén cōng</t>
         </is>
       </c>
       <c r="E151" t="inlineStr">
@@ -6567,7 +6567,7 @@
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>广州市从化区太平镇新兴路 (guǎng zhōu shì cóng huà qū tài píng zhèn xīn xīng lù)439号 (hào)7栋 (dòng)Building 7, No. 439, Xinxing Road, Taiping Town, Conghua District, Guangzhou</t>
+          <t>No. 439, Xinxing Road, Taiping Town, Conghua District, Guangzhou</t>
         </is>
       </c>
       <c r="I151" t="inlineStr">
@@ -6592,7 +6592,7 @@
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>贾均钊 (jiǎ jūn zhāo)</t>
+          <t>jiǎ jūn zhāo</t>
         </is>
       </c>
       <c r="E152" t="inlineStr">
@@ -6612,7 +6612,7 @@
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>苏州市吴江区江陵街道益堂路 (sū zhōu shì wú jiāng qū jiāng líng jiē dào yì táng lù)10号 (hào)No. 10 Yitang Road, Jiangling Street, Wujiang District, Suzhou City</t>
+          <t>No. 10 Yitang Road, Jiangling Street, Wujiang District, Suzhou City</t>
         </is>
       </c>
       <c r="I152" t="inlineStr">
@@ -6637,7 +6637,7 @@
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>郑国哲 (zhèng guó zhé)</t>
+          <t>zhèng guó zhé</t>
         </is>
       </c>
       <c r="E153" t="inlineStr">
@@ -6652,7 +6652,7 @@
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>浙江省龙港市世纪大道 (zhè jiāng shěng lóng gǎng shì shì jì dà dào)888号 (hào)No. 888, Century Avenue, Longgang City, Zhejiang Province</t>
+          <t>No. 888, Century Avenue, Longgang City, Zhejiang Province</t>
         </is>
       </c>
       <c r="I153" t="inlineStr">
@@ -6677,7 +6677,7 @@
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>唐飞玲 (táng fēi líng)</t>
+          <t>táng fēi líng</t>
         </is>
       </c>
       <c r="E154" t="inlineStr">
@@ -6697,7 +6697,7 @@
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>广州市白云区均禾街石马村桃红西街 (guǎng zhōu shì bái yún qū jūn hé jiē shí mǎ cūn táo hóng xī jiē)58号 (hào)No. 58 Taohong West Street, Shima Village, Junhe Street, Baiyun District, Guangzhou City</t>
+          <t>No. 58 Taohong West Street, Shima Village, Junhe Street, Baiyun District, Guangzhou City</t>
         </is>
       </c>
       <c r="I154" t="inlineStr">
@@ -6732,7 +6732,7 @@
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>188 Beiying Road, QingPu, Shanghai 201700</t>
+          <t>Beiying Road, QingPu, Shanghai 201700</t>
         </is>
       </c>
       <c r="I155" t="inlineStr">

</xml_diff>

<commit_message>
Revert "Remove Chinese chars from contacts + addresses in all Excel, keep Latin/pinyin + English address"
This reverts commit edb4912692f6cb89d57f56ca31b1d9d63bc1b928.
</commit_message>
<xml_diff>
--- a/ipdf_suppliers.xlsx
+++ b/ipdf_suppliers.xlsx
@@ -532,7 +532,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>liú jīn líng</t>
+          <t>刘金铃 (liú jīn líng)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -552,7 +552,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>No. 1999, Linhu Avenue, Fenhu Economic Development Zone, Wujiang City, Jiangsu Province, 215211</t>
+          <t>江苏省吴江市 (jiāng sū shěng wú jiāng shì) 汾湖经济开发区临沪大道 (fén hú jīng jì kāi fā qū lín hù dà dào)1999号 (hào), 215211No. 1999, Linhu Avenue, Fenhu Economic Development Zone, Wujiang City, Jiangsu Province, 215211</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -617,7 +617,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>lín xiǎn zhōng</t>
+          <t>林显忠 (lín xiǎn zhōng)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -637,7 +637,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>No. 3, Longxing Southeast First Horizontal Road, Baiyun District, Guangzhou City</t>
+          <t>广州市白云区龙兴东南一横路 (guǎng zhōu shì bái yún qū lóng xīng dōng nán yī héng lù)3号 (hào)No. 3, Longxing Southeast First Horizontal Road, Baiyun District, Guangzhou City</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -662,7 +662,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>sòng qiàn</t>
+          <t>宋茜 (sòng qiàn)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -677,7 +677,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>D Building D, Dingbang Airport Industrial Park, Huadong Town, Huadu District, Guangzhou</t>
+          <t>广州市花都区花东镇定邦空港产业园 (guǎng zhōu shì huā dōu qū huā dōng zhèn dìng bāng kōng gǎng chǎn yè yuán)D栋 (dòng)Building D, Dingbang Airport Industrial Park, Huadong Town, Huadu District, Guangzhou</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -722,7 +722,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>No. 72, Xintai Road, Sanbu Street, Kaiping City, Guangdong Province</t>
+          <t>广东省开平市三埠街道新台路 (guǎng dōng shěng kāi píng shì sān bù jiē dào xīn tái lù)72号 (hào)No. 72, Xintai Road, Sanbu Street, Kaiping City, Guangdong Province</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -747,7 +747,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>wáng yào fēng</t>
+          <t>王耀峰 (wáng yào fēng)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -777,7 +777,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>wáng yuàn yuàn</t>
+          <t>王媛媛 (wáng yuàn yuàn)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -797,7 +797,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>No. 363, Longjie Jian Road, Baiyun District, Guangzhou</t>
+          <t>工厂广东省江门市新山市和情共建路 (gōng chǎng guǎng dōng shěng jiāng mén shì xīn shān shì hé qíng gòng jiàn lù)305号座 (hào zuò) 公司地址 (gōng sī dì zhǐ):广州市白云区龙街尖路 (guǎng zhōu shì bái yún qū lóng jiē jiān lù)363号联边国际 (hào lián biān guó jì)620单元 (dān yuán)Factory: Building 305, Heqing Gongjian Road, Xinshan City, Jiangmen City, Guangdong Province. Company Address: Unit 620, Lianbian International, No. 363, Longjie Jian Road, Baiyun District, Guangzhou</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -842,7 +842,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>nd Road, Chikan, ShipaiTown, Dongguan, Guangdong, 523346.China</t>
+          <t>2nd Road, Chikan, ShipaiTown, Dongguan, Guangdong, 523346.China</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1087,7 +1087,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Bella chén lì xiá</t>
+          <t>Bella 陈丽霞 (chén lì xiá)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1117,7 +1117,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>chén kǒng qīng</t>
+          <t>陈孔清 (chén kǒng qīng)</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1157,7 +1157,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>No. 29 Dabu Road, Xiuquan Street, Huadu District, Guangzhou City, Guangdong Province</t>
+          <t>广东省广州市花都区秀全街道大布路 (guǎng dōng shěng guǎng zhōu shì huā dōu qū xiù quán jiē dào dà bù lù)29号峰华工业园 (hào fēng huá gōng yè yuán)Fenghua Industrial Park, No. 29 Dabu Road, Xiuquan Street, Huadu District, Guangzhou City, Guangdong Province</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1182,7 +1182,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>hú míng</t>
+          <t>胡明 (hú míng)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1192,7 +1192,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>D 37 Building 37, Zone D, Wanyang Maker Town, Yinghong Town, Yingde City, Qingyuan City, Guangdong Province</t>
+          <t>广东省清远英德市英红镇万洋众创城 (guǎng dōng shěng qīng yuǎn yīng dé shì yīng hóng zhèn wàn yáng zhòng chuàng chéng)D区 (qū)37栋 (dòng)Building 37, Zone D, Wanyang Maker Town, Yinghong Town, Yingde City, Qingyuan City, Guangdong Province</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1277,7 +1277,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>No.307 Guangzhou dadao zhong, Tianhe District, Guangzhou</t>
+          <t>42 floor, R &amp; F Dongshan New World Building, No.307 Guangzhou dadao zhong, Tianhe District, Guangzhou</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1302,7 +1302,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>tán yù xióng</t>
+          <t>谭玉雄 (tán yù xióng)</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1322,7 +1322,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>No. 55, Caole Xiangyang Road, Xiegang Town, Dongguan City, Guangdong Province, Building V, Units 1-2, Phase 1, Plastic Market, Zhangmutou Town, Dongguan City, Guangdong Province, No. 53-54, Sufa East Road, Dajingjiu Plastic Market, Changping Town, Dongguan City, Guangdong Province</t>
+          <t>广东省东莞市谢岗镇曹乐向阳路 (guǎng dōng shěng dōng guǎn shì xiè gǎng zhèn cáo lè xiàng yáng lù)55号 (hào), 广东省东莞市樟木头镇塑料市场一期 (guǎng dōng shěng dōng guǎn shì zhāng mù tou zhèn sù liào shì chǎng yī qī)V栋 (dòng)1-2号 (hào), 广东省东莞市常平镇大京九塑料市场塑发东路 (guǎng dōng shěng dōng guǎn shì cháng píng zhèn dà jīng jiǔ sù liào shì chǎng sù fā dōng lù)53-54号 (hào)No. 55, Caole Xiangyang Road, Xiegang Town, Dongguan City, Guangdong Province, Building V, Units 1-2, Phase 1, Plastic Market, Zhangmutou Town, Dongguan City, Guangdong Province, No. 53-54, Sufa East Road, Dajingjiu Plastic Market, Changping Town, Dongguan City, Guangdong Province</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1397,7 +1397,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>No. 121, Commercial Center C, 3rd Floor, Room 022, Guangzhou City, Baiyun District, Zhongluotan Town, Liantian North Road No. 9, Building 6, Chenmei Industrial Park</t>
+          <t>Guangzhou City, Yuexiu District, Guangyuan West Road No. 121, Commercial Center C, 3rd Floor, Room 022, Guangzhou City, Baiyun District, Zhongluotan Town, Liantian North Road No. 9, Building 6, Chenmei Industrial Park</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -1457,7 +1457,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>chén zǒng</t>
+          <t>陈总 (chén zǒng)</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1467,7 +1467,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Jinhe Yun Chuang Industrial Park, Xianke 1st Road, Huadu District, Guangzhou City</t>
+          <t>广州市花都区先科一路金禾云创产业园 (guǎng zhōu shì huā dōu qū xiān kē yī lù jīn hé yún chuàng chǎn yè yuán)Jinhe Yun Chuang Industrial Park, Xianke 1st Road, Huadu District, Guangzhou City</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -1507,7 +1507,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>No. 85, Xianlie Middle Road, Yuexiu District, Guangzhou City</t>
+          <t>广州市越秀区先烈中路 (guǎng zhōu shì yuè xiù qū xiān liè zhōng lù)85号浙江大厦 (hào zhè jiāng dà shà)9楼 (lóu)9th Floor, Zhejiang Building, No. 85, Xianlie Middle Road, Yuexiu District, Guangzhou City</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -1532,7 +1532,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>wú yuè fāng</t>
+          <t>吴月芳 (wú yuè fāng)</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1592,7 +1592,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>No. 18, Zone A, Hegui Industrial Park, Nanhai District, Foshan City, Guangdong Province</t>
+          <t>Room 4002, 4th Floor, Meiwan Square, Sanyuanli Street, Baiyun District, Guangzhou, Guangdong Province Ouyu Square, Huangjinling, Tangge Village, Baiyun Lake Street, Baiyun District, Guangzhou, Guangdong Province No. 18, Zone A, Hegui Industrial Park, Nanhai District, Foshan City, Guangdong Province</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -1662,7 +1662,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>chén yǒng</t>
+          <t>陈泳 (chén yǒng)</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1672,7 +1672,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>No. 6, Dashan Road, Qinghu Village, Junhe Street, Baiyun District, Guangzhou City</t>
+          <t>广州市白云区均禾街清湖村大山路 (guǎng zhōu shì bái yún qū jūn hé jiē qīng hú cūn dà shān lù)6号 (hào)No. 6, Dashan Road, Qinghu Village, Junhe Street, Baiyun District, Guangzhou City</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -1742,7 +1742,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>lài zǐ hào</t>
+          <t>赖梓浩 (lài zǐ hào)</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1762,7 +1762,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>No. 88, Yongli Road, Xinhua Street, District, Guangzhou, China</t>
+          <t>Add. No. 88, Yongli Road, Xinhua Street, District, Guangzhou, China</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -1787,7 +1787,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>liú jīn lián</t>
+          <t>刘金连 (liú jīn lián)</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -1822,7 +1822,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>zhào xīn liàng</t>
+          <t>赵新亮 (zhào xīn liàng)</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1832,7 +1832,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>No. 22, Beicun Beida Road, Baiyun District, Guangzhou City</t>
+          <t>广州市白云区北村北大路 (guǎng zhōu shì bái yún qū běi cūn běi dà lù)22号四栋二楼 (hào sì dòng èr lóu)Second Floor, Building 4, No. 22, Beicun Beida Road, Baiyun District, Guangzhou City</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -2037,7 +2037,7 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>No. 239, Yuncheng South Fourth Road, Baiyun District, Guangzhou</t>
+          <t>Room 905/906/907, Building 2, Yuntuhui, No. 239, Yuncheng South Fourth Road, Baiyun District, Guangzhou</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -2282,7 +2282,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>cáo chūn</t>
+          <t>曹春 (cáo chūn)</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -2292,7 +2292,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>No. 634, Shijing Avenue, Shijing Street, Baiyun District, Guangzhou City</t>
+          <t>广州市白云区石井街石井大道 (guǎng zhōu shì bái yún qū shí jǐng jiē shí jǐng dà dào)634号 (hào)No. 634, Shijing Avenue, Shijing Street, Baiyun District, Guangzhou City</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -2337,7 +2337,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>No. 100, Century Avenue, Pudong New Area, Shanghai</t>
+          <t>上海市浦东新区世纪大道 (shàng hǎi shì pǔ dōng xīn qū shì jì dà dào)100号 (hào)No. 100, Century Avenue, Pudong New Area, Shanghai</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -2362,7 +2362,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>zhāng hǎi hàn</t>
+          <t>章海翰 (zhāng hǎi hàn)</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2377,7 +2377,7 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>No.3, Xiaqi Road and Hudi Road, Jinping District, Shantou city, Guangdong Province, China.</t>
+          <t>Industrial Area No.3, Xiaqi Road and Hudi Road, Jinping District, Shantou city, Guangdong Province, China.</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -2507,7 +2507,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>No. 6818, Daye Highway, Fengxian District, Shanghai City</t>
+          <t>上海市奉贤区大叶公路 (shàng hǎi shì fèng xián qū dà yè gōng lù) 6818号 (hào)5A栋 (dòng)502Room 502, Building 5A, No. 6818, Daye Highway, Fengxian District, Shanghai City</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -2532,7 +2532,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>chén xuě píng</t>
+          <t>陈雪萍 (chén xuě píng)</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -2552,7 +2552,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>No. 3, Mashiwei Road, Shiwan Town, Boluo County, Huizhou City, Guangdong Province</t>
+          <t>广东省惠州市博罗县石湾镇马石围路 (guǎng dōng shěng huì zhōu shì bó luó xiàn shí wān zhèn mǎ shí wéi lù)3号 (hào)No. 3, Mashiwei Road, Shiwan Town, Boluo County, Huizhou City, Guangdong Province</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -2577,7 +2577,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>hé lì yín</t>
+          <t>何丽银 (hé lì yín)</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -2597,7 +2597,7 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>No. 6, Guangchuang Street, Guangqing Industrial Park, Shijiao Town, Qingcheng District, Qingyuan City, Guangdong Province</t>
+          <t>广东省清远市清城区石角镇广清产业园广创街 (guǎng dōng shěng qīng yuǎn shì qīng chéng qū shí jiǎo zhèn guǎng qīng chǎn yè yuán guǎng chuàng jiē)6号 (hào)No. 6, Guangchuang Street, Guangqing Industrial Park, Shijiao Town, Qingcheng District, Qingyuan City, Guangdong Province</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -2622,7 +2622,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>rǎn lù qiàn</t>
+          <t>冉露茜 (rǎn lù qiàn)</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -2642,7 +2642,7 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>WE2101 Room WE2101, Debao Shanghai Book City, Huangpu District</t>
+          <t>黄浦区德必上海书城 (huáng pǔ qū dé bì shàng hǎi shū chéng)WE2101室 (shì)Room WE2101, Debao Shanghai Book City, Huangpu District</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -2682,7 +2682,7 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>No. 158, Xinhe Road, Xinfeng Town, Nanhu District, Jiaxing City, Zhejiang Province</t>
+          <t>浙江省嘉兴市南湖区新丰镇新禾路 (zhè jiāng shěng jiā xīng shì nán hú qū xīn fēng zhèn xīn hé lù)158号 (hào)No. 158, Xinhe Road, Xinfeng Town, Nanhu District, Jiaxing City, Zhejiang Province</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -2767,7 +2767,7 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>No.69 Zhubei Rd. Mazhu Town, Yuvac Zhejiang Province No.888 Beixing Rd. Mazhu Town. Yuyao Zhejiang Province</t>
+          <t>No.69 Zhubei Rd. (E) Mazhu Town, Yuvac Zhejiang Province (P.C. 315450) No.888 Beixing Rd. Mazhu Town. Yuyao Zhejiang Province(P.C. 315450)</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -2792,7 +2792,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>chén tiě wén</t>
+          <t>陈铁文 (chén tiě wén)</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -2807,7 +2807,7 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>A 2504 Room 2504, Building A, Juhuao International, Intersection of Jianshe Road and Donghuan 2nd Road, Longhua New District, Shenzhen City, Guangdong Province; Jinjiang Economic Development Zone, Jinjiang City, Fujian Province</t>
+          <t>福建省晋江市经济开发区 (fú jiàn shěng jìn jiāng shì jīng jì kāi fā qū) 广东省深圳市龙华新区建设路与东环二路交汇处聚豪国际 (guǎng dōng shěng shēn zhèn shì lóng huá xīn qū jiàn shè lù yǔ dōng huán èr lù jiāo huì chù jù háo guó jì)A栋 (dòng)2504室 (shì)Room 2504, Building A, Juhuao International, Intersection of Jianshe Road and Donghuan 2nd Road, Longhua New District, Shenzhen City, Guangdong Province; Jinjiang Economic Development Zone, Jinjiang City, Fujian Province</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -2852,7 +2852,7 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>No. 25, Fuyuan 1st Road, Xinya Subdistrict, Huadu District, Guangzhou City, Guangdong Province</t>
+          <t>3rd Floor, Building 6, No. 25, Fuyuan 1st Road, Xinya Subdistrict, Huadu District, Guangzhou City, Guangdong Province</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -2877,7 +2877,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>zhōu liàng</t>
+          <t>周 (zhōu) 亮 (liàng)</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -3137,7 +3137,7 @@
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>No. 285 Linhe East Road, Tianhe District, Guangzhou City</t>
+          <t>广州市天河区林和东路 (guǎng zhōu shì tiān hé qū lín hé dōng lù)285号中汇人寿 (hào zhōng huì rén shòu)901Room 901, Zhonghui Life Insurance, No. 285 Linhe East Road, Tianhe District, Guangzhou City</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -3162,7 +3162,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>lǐ jīn huā</t>
+          <t>李金花 (lǐ jīn huā)</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -3227,7 +3227,7 @@
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>Building 3, Kewoyuan, Yiheng Road, Hequan Road, Baiyun District, Guangzhou City</t>
+          <t>广州市白云区鶴拳路一横路科我园 (guǎng zhōu shì bái yún qū hè quán lù yī héng lù kē wǒ yuán)3栋 (dòng)Building 3, Kewoyuan, Yiheng Road, Hequan Road, Baiyun District, Guangzhou City</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
@@ -3417,7 +3417,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Cécilia yè sī yǐng</t>
+          <t>Cécilia 叶思颖 (yè sī yǐng)</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -3437,7 +3437,7 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>No. 10, Xicheng Middle Street, Nanwan, Huangpu District, Guangzhou, Guangdong, China</t>
+          <t>Building E1, Huangpu Technology Headquarters Port, Liandong U Valley, No. 10, Xicheng Middle Street, Nanwan, Huangpu District, Guangzhou, Guangdong, China</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -3477,7 +3477,7 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>No.70 Xiangxia Avenue, Longgui, Taihe Town, Baiyun District, Guangzhou, China</t>
+          <t>Floor 4, Building C, Shengmeng Industrial Park, No.70 Xiangxia Avenue, Longgui, Taihe Town, Baiyun District, Guangzhou, China</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
@@ -3542,7 +3542,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>hóng bì hóng</t>
+          <t>洪碧虹 (hóng bì hóng)</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -3557,7 +3557,7 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>-12 Buildings 11-12, Jianming Industrial City, Zhonggong Community, Qishan Street, Jinping District, Shantou City</t>
+          <t>汕头市金平区岐山街道中宫社区建明工业城 (shàn tóu shì jīn píng qū qí shān jiē dào zhōng gōng shè qū jiàn míng gōng yè chéng)11-12栋楼 (dòng lóu)Buildings 11-12, Jianming Industrial City, Zhonggong Community, Qishan Street, Jinping District, Shantou City</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
@@ -3732,7 +3732,7 @@
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>Umbrella Industrial Park, Songxia Town, Shangyu Dist., Shaoxing, Zhejiang, China</t>
+          <t>Umbrella Industrial Park, Songxia Town, Shangyu Dist., Shaoxing, Zhejiang, China (Mainland)</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
@@ -3802,7 +3802,7 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>hé yàn fāng Orla</t>
+          <t>何燕芳 (hé yàn fāng) Orla</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -3842,7 +3842,7 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>chén lè</t>
+          <t>陈乐 (chén lè)</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -3862,7 +3862,7 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>No. 10, Zhongnan Street, Nangang Subdistrict, Huangpu District, Guangzhou</t>
+          <t>广州市赛康尼机械设备有限公司 (guǎng zhōu shì sài kāng ní jī xiè shè bèi yǒu xiàn gōng sī) 广州市黄埔区南岗街道中南街 (guǎng zhōu shì huáng pǔ qū nán gǎng jiē dào zhōng nán jiē)10号联系中心办公室楼南面主楼南面 (hào lián xì zhōng xīn bàn gōng shì lóu nán miàn zhǔ lóu nán miàn)Guangzhou Saikenni Machinery Equipment Co., Ltd. South side of the main building, south side of the Contact Center Office Building, No. 10, Zhongnan Street, Nangang Subdistrict, Huangpu District, Guangzhou</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
@@ -3887,7 +3887,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>bào huàn wēi Bao huan wei</t>
+          <t>鲍焕威 (bào huàn wēi) Bao huan wei</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -3927,7 +3927,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>huáng shùn hǎo</t>
+          <t>黄顺好 (huáng shùn hǎo)</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
@@ -3947,7 +3947,7 @@
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>Laiyong Industrial Zone, Lunqiao, Shunde District, Foshan City, Guangdong</t>
+          <t>广东佛山市顺德区伦教来涌工业区 (guǎng dōng fó shān shì shùn dé qū lún jiào lái yǒng gōng yè qū)Laiyong Industrial Zone, Lunqiao, Shunde District, Foshan City, Guangdong</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
@@ -3972,7 +3972,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>shào shì huá</t>
+          <t>邵仕华 (shào shì huá)</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
@@ -4012,7 +4012,7 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>chén xiǎo wén</t>
+          <t>陈晓雯 (chén xiǎo wén)</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
@@ -4027,7 +4027,7 @@
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>No. 3, Xingyuan Road, Shijiao Town , Qingcheng District, Qingyuan City, Guangdong Province; Room 1107, Building 4, Plot 5, Greenland Airport, Xinya Street, Huadu District, Guangzhou City</t>
+          <t>广东省清远市清城区石角镇 (guǎng dōng shěng qīng yuǎn shì qīng chéng qū shí jiǎo zhèn)(广清产业园 (guǎng qīng chǎn yè yuán))兴园路 (xīng yuán lù)3号 (hào); 广州市花都区新雅街绿地空港五号地 (guǎng zhōu shì huā dōu qū xīn yǎ jiē lǜ dì kōng gǎng wǔ hào dì)4栋 (dòng)1107室 (shì)No. 3, Xingyuan Road, Shijiao Town (Guangqing Industrial Park), Qingcheng District, Qingyuan City, Guangdong Province; Room 1107, Building 4, Plot 5, Greenland Airport, Xinya Street, Huadu District, Guangzhou City</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
@@ -4087,7 +4087,7 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>xú chūn miáo Kavi</t>
+          <t>徐春苗 (xú chūn miáo) Kavi</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
@@ -4102,7 +4102,7 @@
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>No. 158, Xinhe Road, Xinfeng Town, Nanhu District, Jiaxing City, Zhejiang Province</t>
+          <t>浙江省嘉兴市南湖区新丰镇新禾路 (zhè jiāng shěng jiā xīng shì nán hú qū xīn fēng zhèn xīn hé lù)158号 (hào)No. 158, Xinhe Road, Xinfeng Town, Nanhu District, Jiaxing City, Zhejiang Province</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
@@ -4147,7 +4147,7 @@
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>No. 55 Jiangping North Road, Taixing City, Jiangsu Province, Room 001, No. 6 Shilong Road, Xuhui District, Shanghai City</t>
+          <t>江苏省泰兴市江平北路 (jiāng sū shěng tài xīng shì jiāng píng běi lù)55号 (hào), 上海市徐汇区石龙路 (shàng hǎi shì xú huì qū shí lóng lù)6号 (hào)001室 (shì)No. 55 Jiangping North Road, Taixing City, Jiangsu Province, Room 001, No. 6 Shilong Road, Xuhui District, Shanghai City</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
@@ -4257,7 +4257,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>wēng shuò huán</t>
+          <t>翁铄桓 (wēng shuò huán)</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
@@ -4272,7 +4272,7 @@
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>No. 34, Boyu Road, Leping Town, Sanshui District, Foshan City</t>
+          <t>佛山市三水区乐平镇博裕路 (fó shān shì sān shuǐ qū lè píng zhèn bó yù lù)34号 (hào)1栋 (dòng)Building 1, No. 34, Boyu Road, Leping Town, Sanshui District, Foshan City</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
@@ -4297,7 +4297,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>gù yǒu yáng</t>
+          <t>顾友阳 (gù yǒu yáng)</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -4312,7 +4312,7 @@
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>No. 288, Zhanye Road, Caojing Development Zone, Jinshan District, Shanghai</t>
+          <t>上海市金山区漕泾开发区展业路 (shàng hǎi shì jīn shān qū cáo jīng kāi fā qū zhǎn yè lù)288号一栋 (hào yī dòng)Building 1, No. 288, Zhanye Road, Caojing Development Zone, Jinshan District, Shanghai</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
@@ -4387,7 +4387,7 @@
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>No.268, Huandong Road, Xuxiake Town, Jiangyin, Jiangsu, China, 214407</t>
+          <t>5F,No.268, Huandong Road, Xuxiake Town, Jiangyin, Jiangsu, China, 214407</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
@@ -4432,7 +4432,7 @@
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>Building 2, Greenland Airport Center Huadu District, Guangzhou City</t>
+          <t>608, Building 2, Greenland Airport Center Huadu District, Guangzhou City</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
@@ -4457,7 +4457,7 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>lín xiǎo róng</t>
+          <t>林晓荣 (lín xiǎo róng)</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
@@ -4477,7 +4477,7 @@
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>Longzhou Road, Yuepu, Shantou City, Guangdong Province, China</t>
+          <t>广东省汕头市月浦龙洲路 (guǎng dōng shěng shàn tóu shì yuè pǔ lóng zhōu lù)12号 (hào) Longzhou Road, Yuepu, Shantou City, Guangdong Province, China</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
@@ -4502,7 +4502,7 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>xiè róng bǎo</t>
+          <t>谢榕宝 (xiè róng bǎo)</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
@@ -4522,7 +4522,7 @@
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>No. 2, Qixing, Guangzhou City</t>
+          <t>广州市七星二号 (guǎng zhōu shì qī xīng èr hào)No. 2, Qixing, Guangzhou City</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
@@ -4562,7 +4562,7 @@
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>Building 35, Caizhi Jin'an, Lane 588, Shuping Road, Jiading District, Shanghai</t>
+          <t>上海市嘉定区树屏路 (shàng hǎi shì jiā dìng qū shù píng lù)588弄财智金岸 (nòng cái zhì jīn àn)35号楼 (hào lóu)Building 35, Caizhi Jin'an, Lane 588, Shuping Road, Jiading District, Shanghai</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -4647,7 +4647,7 @@
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>No.86, Maohai Road, Huangjiabu Town, Yuyao City, Zhejiang Province.</t>
+          <t>Building 31, No.86, Maohai Road, Huangjiabu Town, Yuyao City, Zhejiang Province.</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
@@ -4717,7 +4717,7 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>sū yuán yuán</t>
+          <t>苏元元 (sū yuán yuán)</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
@@ -4737,7 +4737,7 @@
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>No. 138, Zhenxing Road, Songsha Street, Shangyu District, Shaoxing City, Zhejiang Province</t>
+          <t>浙江省绍兴市上虞区崧厦街道振兴路 (zhè jiāng shěng shào xīng shì shàng yú qū sōng shà jiē dào zhèn xīng lù)138号 (hào)No. 138, Zhenxing Road, Songsha Street, Shangyu District, Shaoxing City, Zhejiang Province</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
@@ -4762,7 +4762,7 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>liú yàn xiá</t>
+          <t>刘艳霞 (liú yàn xiá)</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
@@ -4812,7 +4812,7 @@
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>Huachang Road, Mingwei Industrial Zone, Lizhou Street, Yuyao, Zhejiang, China. 168 Yuma Road, Mazhu Town, Yuyao, Zhejiang, China.</t>
+          <t>15 Huachang Road, Mingwei Industrial Zone, Lizhou Street, Yuyao, Zhejiang, China. 168 Yuma Road, Mazhu Town, Yuyao, Zhejiang, China.</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
@@ -4877,7 +4877,7 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>zhāng liàng liàng</t>
+          <t>张亮亮 (zhāng liàng liàng)</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
@@ -4917,7 +4917,7 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>xiào zhì jiān</t>
+          <t>肖志坚 (xiào zhì jiān)</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
@@ -4932,7 +4932,7 @@
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>No. 1-3, Lane 133, Ye Road, Songjiang District, Shanghai</t>
+          <t>上海市松江区叶路 (shàng hǎi shì sōng jiāng qū yè lù)133弄 (nòng)1-3号 (hào)No. 1-3, Lane 133, Ye Road, Songjiang District, Shanghai</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
@@ -4957,7 +4957,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>wáng xīn yuàn</t>
+          <t>王馨苑 (wáng xīn yuàn)</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
@@ -4977,7 +4977,7 @@
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>C Building C, Weiguan Industrial Park, Huadong Town, Huadu District, Guangzhou</t>
+          <t>广州市花都区花东镇微观产业园 (guǎng zhōu shì huā dōu qū huā dōng zhèn wēi guān chǎn yè yuán)C栋 (dòng)Building C, Weiguan Industrial Park, Huadong Town, Huadu District, Guangzhou</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
@@ -5002,7 +5002,7 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>wáng lì bō</t>
+          <t>王丽波 (wáng lì bō)</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
@@ -5022,7 +5022,7 @@
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>B67 West of Xiaoxi Road, Gaochetou, Mushan Town, Yuyao City, Zhejiang Province, No. B67</t>
+          <t>浙江省余姚市牟山镇高车头 (zhè jiāng shěng yú yáo shì móu shān zhèn gāo chē tóu) B67号肖西路西 (hào xiào xī lù xī)West of Xiaoxi Road, Gaochetou, Mushan Town, Yuyao City, Zhejiang Province, No. B67</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
@@ -5047,7 +5047,7 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>liú xī róng</t>
+          <t>刘锡蓉 (liú xī róng)</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
@@ -5067,7 +5067,7 @@
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>No. 183, Beixing Road, Mazhu Town, Yuyao City, Zhejiang Province</t>
+          <t>浙江省余姚市马渚镇北兴路 (zhè jiāng shěng yú yáo shì mǎ zhǔ zhèn běi xīng lù)183号 (hào)No. 183, Beixing Road, Mazhu Town, Yuyao City, Zhejiang Province</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
@@ -5092,7 +5092,7 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>pān xīng jié</t>
+          <t>潘兴杰 (pān xīng jié)</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
@@ -5112,7 +5112,7 @@
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>No. 2, Dongye Road, Houjie Town, Dongguan City, Guangdong Province</t>
+          <t>廣東省東莞市厚街鎮東業路 (guǎng dōng shěng dōng guǎn shì hòu jiē zhèn dōng yè lù)2號 (hào)No. 2, Dongye Road, Houjie Town, Dongguan City, Guangdong Province</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
@@ -5137,7 +5137,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>hú zhēn huá</t>
+          <t>胡珍华 (hú zhēn huá)</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
@@ -5152,7 +5152,7 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>No. 6, Lvgong 4th Street, Huadu District, Guangzhou</t>
+          <t>广州市花都区绿港四街 (guǎng zhōu shì huā dōu qū lǜ gǎng sì jiē)6号 (hào)No. 6, Lvgong 4th Street, Huadu District, Guangzhou</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -5217,7 +5217,7 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>liú yáng é</t>
+          <t>刘扬娥 (liú yáng é)</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
@@ -5232,7 +5232,7 @@
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>No. 41, Shenshan Shishen Road, Jianggao Town, Baiyun District, Guangzhou</t>
+          <t>广州市白云区江高镇神山神石路 (guǎng zhōu shì bái yún qū jiāng gāo zhèn shén shān shén shí lù)41号 (hào)No. 41, Shenshan Shishen Road, Jianggao Town, Baiyun District, Guangzhou</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
@@ -5257,7 +5257,7 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>lín fān</t>
+          <t>林帆 (lín fān)</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
@@ -5277,7 +5277,7 @@
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>No. 288 Keyun Road, Tianhe District, Guangzhou City, Guangdong Province</t>
+          <t>广东省广州市天河区科韵路 (guǎng dōng shěng guǎng zhōu shì tiān hé qū kē yùn lù)288号天盈创意园 (hào tiān yíng chuàng yì yuán) C区 (qū)3024-3027Rooms 3024-3027, Area C, Tianying Creative Park, No. 288 Keyun Road, Tianhe District, Guangzhou City, Guangdong Province</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
@@ -5302,7 +5302,7 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>liú lì hóng Valerie</t>
+          <t>刘丽红 (liú lì hóng) Valerie</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
@@ -5312,7 +5312,7 @@
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>No. 3, Jintian Road, Huadu District, Guangzhou City, Guangdong Province</t>
+          <t>广东省广州市花都区金田路 (guǎng dōng shěng guǎng zhōu shì huā dōu qū jīn tián lù)3号 (hào)No. 3, Jintian Road, Huadu District, Guangzhou City, Guangdong Province</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
@@ -5337,7 +5337,7 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>liáng guān wén</t>
+          <t>梁冠文 (liáng guān wén)</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
@@ -5352,7 +5352,7 @@
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>No.2 Keyuan Road, Guangzhou Private Science and Technology Park, No. 1633 Beitai Road, Baiyun District, Guangzhou</t>
+          <t>广州市白云区北太路 (guǎng zhōu shì bái yún qū běi tài lù)1633号广州民营科技园科园路 (hào guǎng zhōu mín yíng kē jì yuán kē yuán lù)2号凯铂中心 (hào kǎi bó zhōng xīn)D区 (qū)1-4楼 (lóu) 1-4 F, Area D. Kaibo Center Building, No.2 Keyuan Road, Guangzhou Private Science and Technology Park, No. 1633 Beitai Road, Baiyun District, Guangzhou</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
@@ -5377,7 +5377,7 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>xióng qiáng Xiong Qiang</t>
+          <t>熊强 (xióng qiáng) Xiong Qiang</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
@@ -5387,7 +5387,7 @@
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>No. 7, Chuangye Road, Guangfo Industrial Park, Tangtang Town, Fogang County, Qingyuan City, Guangdong Province</t>
+          <t>广东省清远市佛冈县汤塘镇广佛产业园创业路 (guǎng dōng shěng qīng yuǎn shì fú gāng xiàn tāng táng zhèn guǎng fú chǎn yè yuán chuàng yè lù)7号 (hào) C区 (qū)6栋 (dòng)101-501房 (fáng)Room 101-501, Building 6, Zone C, No. 7, Chuangye Road, Guangfo Industrial Park, Tangtang Town, Fogang County, Qingyuan City, Guangdong Province</t>
         </is>
       </c>
       <c r="I121" t="inlineStr">
@@ -5412,7 +5412,7 @@
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>lǐ juān LiJuan</t>
+          <t>李娟 (lǐ juān) LiJuan</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
@@ -5432,7 +5432,7 @@
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>A 11/F Building 7 Awang Industrial Zone, Baiyun District, Guangzhou City</t>
+          <t>广州市白云区江高镇 (guǎng zhōu shì bái yún qū jiāng gāo zhèn)408号工业园 (hào gōng yè yuán) A区 (qū) 11/F Building 7 Awang Industrial Zone, Baiyun District, Guangzhou City</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
@@ -5457,7 +5457,7 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>xiào hǎi qīng</t>
+          <t>肖海青 (xiào hǎi qīng)</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
@@ -5477,7 +5477,7 @@
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>No. 25, Maonan Road, Torch Development Zone, Zhongshan City, Guangdong Province; Huizhou Factory: No. 2, Jianshe Road, Jinshan Industrial Park, Longmen County, Huizhou City, Guangdong Province</t>
+          <t>中山工厂 (zhōng shān gōng chǎng):广东省中山市火炬开发区茂南路 (guǎng dōng shěng zhōng shān shì huǒ jù kāi fā qū mào nán lù)25号 (hào) 惠州工厂 (huì zhōu gōng chǎng):广东省惠州市龙门县金山工业园建设路 (guǎng dōng shěng huì zhōu shì lóng mén xiàn jīn shān gōng yè yuán jiàn shè lù)2号 (hào)Zhongshan Factory: No. 25, Maonan Road, Torch Development Zone, Zhongshan City, Guangdong Province; Huizhou Factory: No. 2, Jianshe Road, Jinshan Industrial Park, Longmen County, Huizhou City, Guangdong Province</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
@@ -5502,7 +5502,7 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>guō wǔ jié</t>
+          <t>郭武杰 (guō wǔ jié)</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
@@ -5517,7 +5517,7 @@
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>No. 307 Guangzhou Avenue Middle, Tianhe District, Guangzhou</t>
+          <t>广州天河区广州大道中 (guǎng zhōu tiān hé qū guǎng zhōu dà dào zhōng)307号富力东山新天地中心 (hào fù lì dōng shān xīn tiān dì zhōng xīn)42楼 (lóu)(总部营销中心 (zǒng bù yíng xiāo zhōng xīn))42nd Floor (Headquarters Marketing Center), Fuli Dongshan Xintiandi Center, No. 307 Guangzhou Avenue Middle, Tianhe District, Guangzhou</t>
         </is>
       </c>
       <c r="I124" t="inlineStr">
@@ -5542,7 +5542,7 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>chén huā lěi Chen Hualel</t>
+          <t>陈花蕾 (chén huā lěi) Chen Hualel</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
@@ -5562,7 +5562,7 @@
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>3rd Floor, Building 2, Yunlihui, Yuncheng East Road, Baiyun District, Guangzhou</t>
+          <t>广州市白云区云城东路云理汇 (guǎng zhōu shì bái yún qū yún chéng dōng lù yún lǐ huì)2栋 (dòng)3楼 (lóu)3rd Floor, Building 2, Yunlihui, Yuncheng East Road, Baiyun District, Guangzhou</t>
         </is>
       </c>
       <c r="I125" t="inlineStr">
@@ -5587,7 +5587,7 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>lǐ xiǎo nà</t>
+          <t>李小娜 (lǐ xiǎo nà)</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
@@ -5602,7 +5602,7 @@
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>No. 2, Baoju Road, Mingzhu Industrial Park, Conghua District, Guangzhou City</t>
+          <t>广州市从化区明珠工业园宝聚路二号 (guǎng zhōu shì cóng huà qū míng zhū gōng yè yuán bǎo jù lù èr hào)No. 2, Baoju Road, Mingzhu Industrial Park, Conghua District, Guangzhou City</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
@@ -5627,7 +5627,7 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>péng liàn zhī</t>
+          <t>彭练芝 (péng liàn zhī)</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
@@ -5642,7 +5642,7 @@
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>No. 41, Shenshan Shishen Road, Jianggao Town, Baiyun District, Guangzhou</t>
+          <t>广州市白云区江高镇神山神石路 (guǎng zhōu shì bái yún qū jiāng gāo zhèn shén shān shén shí lù)41号 (hào)No. 41, Shenshan Shishen Road, Jianggao Town, Baiyun District, Guangzhou</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
@@ -5667,7 +5667,7 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>lǐ wén huì</t>
+          <t>李文慧 (lǐ wén huì)</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
@@ -5677,7 +5677,7 @@
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>No. 54, Beixing Beizhong Road, Huadong Town, Huadu District, Guangzhou City, Guangdong Province</t>
+          <t>广东省广州市花都区花东镇北兴北钟路 (guǎng dōng shěng guǎng zhōu shì huā dōu qū huā dōng zhèn běi xīng běi zhōng lù)54号 (hào)No. 54, Beixing Beizhong Road, Huadong Town, Huadu District, Guangzhou City, Guangdong Province</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
@@ -5702,7 +5702,7 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>liú shào wěi</t>
+          <t>刘绍伟 (liú shào wěi)</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
@@ -5722,7 +5722,7 @@
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>No. 34, Boyu Road, Leping Town, Sanshui District, Foshan City</t>
+          <t>佛山市三水区乐平镇博裕路 (fó shān shì sān shuǐ qū lè píng zhèn bó yù lù)34号 (hào)1栋 (dòng)Building 1, No. 34, Boyu Road, Leping Town, Sanshui District, Foshan City</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
@@ -5747,7 +5747,7 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>chén kūn</t>
+          <t>陈坤 (chén kūn)</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
@@ -5762,7 +5762,7 @@
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>th Floor, Jiaolan Jiada Building, Yuncheng West Road, Baiyun District, Guangzhou City</t>
+          <t>广州市白云区云城西路娇兰佳人大厦 (guǎng zhōu shì bái yún qū yún chéng xī lù jiāo lán jiā rén dà shà)10楼 (lóu)10th Floor, Jiaolan Jiada Building, Yuncheng West Road, Baiyun District, Guangzhou City</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
@@ -5787,7 +5787,7 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>qīng huì</t>
+          <t>卿慧 (qīng huì)</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
@@ -5807,7 +5807,7 @@
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>No. 11, Sanyuanli Avenue, Baiyun District, Guangzhou City</t>
+          <t>广州市白云区三元里大道 (guǎng zhōu shì bái yún qū sān yuán lǐ dà dào)11号中港皮具城 (hào zhōng gǎng pí jù chéng)10楼 (lóu)1009室 (shì)Room 1009, 10th Floor, Zhonggang Leather City, No. 11, Sanyuanli Avenue, Baiyun District, Guangzhou City</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
@@ -5832,7 +5832,7 @@
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>zōu yǒng liú</t>
+          <t>邹永流 (zōu yǒng liú)</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
@@ -5847,7 +5847,7 @@
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>No. 85, Xianlie Middle Road, Yuexiu District, Guangzhou City</t>
+          <t>广州市越秀区先烈中路 (guǎng zhōu shì yuè xiù qū xiān liè zhōng lù)85号浙江大厦 (hào zhè jiāng dà shà)9楼 (lóu)9th Floor, Zhejiang Building, No. 85, Xianlie Middle Road, Yuexiu District, Guangzhou City</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
@@ -5872,7 +5872,7 @@
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>luó wén háo Louis</t>
+          <t>罗文豪 (luó wén háo) Louis</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
@@ -5887,7 +5887,7 @@
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>No. 339-36, Hengjiang Road, Conghua District, Guangzhou City</t>
+          <t>广州市从化区横江路 (guǎng zhōu shì cóng huà qū héng jiāng lù)339号 (hào) -36号鸿志软管 (hào hóng zhì ruǎn guǎn)Hongzhi Hose, No. 339-36, Hengjiang Road, Conghua District, Guangzhou City</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
@@ -5927,7 +5927,7 @@
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>No. 2 Yinian West Road, Xielazhuang, Taihe Town layun District, Duangzhou City</t>
+          <t>广州市白云区太和镇谢家注兰西路 (guǎng zhōu shì bái yún qū tài hé zhèn xiè jiā zhù lán xī lù)2号 (hào) No. 2 Yinian West Road, Xielazhuang, Taihe Town layun District, Duangzhou City</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
@@ -5952,7 +5952,7 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>yú shū qíng</t>
+          <t>于舒情 (yú shū qíng)</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
@@ -5962,7 +5962,7 @@
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>No. 2, Yinlan West Road, Xiejiazhuang, Taihe Town, Baiyun District, Guangzhou City</t>
+          <t>广州市白云区太和镇谢家庄荫兰西路 (guǎng zhōu shì bái yún qū tài hé zhèn xiè jiā zhuāng yīn lán xī lù)2号 (hào)No. 2, Yinlan West Road, Xiejiazhuang, Taihe Town, Baiyun District, Guangzhou City</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
@@ -5987,7 +5987,7 @@
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>shí xiǎo jiě SHI XIAOJIE</t>
+          <t>石小姐 (shí xiǎo jiě) SHI XIAOJIE</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
@@ -6007,7 +6007,7 @@
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>No. 1 Gangpu Avenue, Nanling Village, Longgui Street, Baiyun District, Guangzhou City</t>
+          <t>广州市白云区龙归街南岭村岗埔大道 (guǎng zhōu shì bái yún qū lóng guī jiē nán lǐng cūn gǎng pǔ dà dào)1号 (hào)No. 1 Gangpu Avenue, Nanling Village, Longgui Street, Baiyun District, Guangzhou City</t>
         </is>
       </c>
       <c r="I136" t="inlineStr">
@@ -6032,7 +6032,7 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>liáng kǎi háo</t>
+          <t>梁凯豪 (liáng kǎi háo)</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
@@ -6082,7 +6082,7 @@
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>No. 61, Fenghuang South Road, Huadu District, Guangzhou</t>
+          <t>广州市花都区凤凰南路 (guǎng zhōu shì huā dōu qū fèng huáng nán lù)61号卓美大楼北楼 (hào zhuó měi dà lóu běi lóu)307室 (shì)Room 307, North Building, Zhuomei Building, No. 61, Fenghuang South Road, Huadu District, Guangzhou</t>
         </is>
       </c>
       <c r="I138" t="inlineStr">
@@ -6107,7 +6107,7 @@
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>lí jīn chāng</t>
+          <t>黎金昌 (lí jīn chāng)</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
@@ -6127,7 +6127,7 @@
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>No. 81, Xialiang East Road, Longgui Street, Baiyun District, Guangzhou</t>
+          <t>廣州市白雲區龍歸街夏良東路 (guǎng zhōu shì bái yún qū lóng guī jiē xià liáng dōng lù)81號 (hào)102房 (fáng)Room 102, No. 81, Xialiang East Road, Longgui Street, Baiyun District, Guangzhou</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
@@ -6167,7 +6167,7 @@
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>No. 3 , Chengxi Village, Huashan Town, Huadu District, Guangzhou City</t>
+          <t>廣州市花都區花山鎮城西村自編 (guǎng zhōu shì huā dōu qū huā shān zhèn chéng xī cūn zì biān)3號 (hào)No. 3 (self-numbered), Chengxi Village, Huashan Town, Huadu District, Guangzhou City</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
@@ -6187,7 +6187,7 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>zhù yī tíng Carrie</t>
+          <t>祝依婷 (zhù yī tíng) Carrie</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
@@ -6197,7 +6197,7 @@
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>No. 3, Jintian Road, Huadu District, Guangzhou City, Guangdong Province</t>
+          <t>广东省广州市花都区金田路 (guǎng dōng shěng guǎng zhōu shì huā dōu qū jīn tián lù)3号 (hào)No. 3, Jintian Road, Huadu District, Guangzhou City, Guangdong Province</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
@@ -6222,7 +6222,7 @@
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>dèng sī yì</t>
+          <t>邓思艺 (dèng sī yì)</t>
         </is>
       </c>
       <c r="E142" t="inlineStr">
@@ -6237,7 +6237,7 @@
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>No. 3, Xingyuan Road, Shijiao Town , Qingcheng District, Qingyuan City, Guangdong Province; Room 1107, Building 4, Plot 5, Greenland Airport, Xinya Street, Huadu District, Guangzhou City</t>
+          <t>广东省清远市清城区石角镇 (guǎng dōng shěng qīng yuǎn shì qīng chéng qū shí jiǎo zhèn)(广清产业园 (guǎng qīng chǎn yè yuán))兴园路 (xīng yuán lù)3号 (hào); 广州市花都区新雅街绿地空港五号地 (guǎng zhōu shì huā dōu qū xīn yǎ jiē lǜ dì kōng gǎng wǔ hào dì)4栋 (dòng)1107室 (shì)No. 3, Xingyuan Road, Shijiao Town (Guangqing Industrial Park), Qingcheng District, Qingyuan City, Guangdong Province; Room 1107, Building 4, Plot 5, Greenland Airport, Xinya Street, Huadu District, Guangzhou City</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
@@ -6262,7 +6262,7 @@
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>jiāng sī róng</t>
+          <t>江思蓉 (jiāng sī róng)</t>
         </is>
       </c>
       <c r="E143" t="inlineStr">
@@ -6292,7 +6292,7 @@
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>liú jiàn jūn</t>
+          <t>刘键均 (liú jiàn jūn)</t>
         </is>
       </c>
       <c r="E144" t="inlineStr">
@@ -6302,7 +6302,7 @@
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>No. 888 Yuncheng West Road, Baiyun District, Guangzhou City</t>
+          <t>广州市白云区云城西路 (guǎng zhōu shì bái yún qū yún chéng xī lù)888号绿地中心 (hào lǜ dì zhōng xīn)2403Room 2403, Greenland Center, No. 888 Yuncheng West Road, Baiyun District, Guangzhou City</t>
         </is>
       </c>
       <c r="I144" t="inlineStr">
@@ -6327,7 +6327,7 @@
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>mǎ zhuàng mào</t>
+          <t>马壮茂 (mǎ zhuàng mào)</t>
         </is>
       </c>
       <c r="E145" t="inlineStr">
@@ -6362,7 +6362,7 @@
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>xiè yǎ qí</t>
+          <t>谢雅琪 (xiè yǎ qí)</t>
         </is>
       </c>
       <c r="E146" t="inlineStr">
@@ -6382,7 +6382,7 @@
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>No. 1999, Wing West Road Cace Sheet, Shangyu District. Shocking City Zhellong ProvinceBuilding 21 C, Landong U Valley, No. 1999, Wuxing West Road, Cao'e Street, Shangyu District, Shaoxing City, Zhejiang Province</t>
+          <t>浙江省绍兴市上虞区曹娥街道五星西路 (zhè jiāng shěng shào xīng shì shàng yú qū cáo é jiē dào wǔ xīng xī lù)1999号联东 (hào lián dōng)U谷 (gǔ)21栋 (dòng)C永 (yǒng), Add C tongin Bulding 21. Landong U Valley No. 1999, Wing West Road Cace Sheet, Shangyu District. Shocking City Zhellong ProvinceBuilding 21 C, Landong U Valley, No. 1999, Wuxing West Road, Cao'e Street, Shangyu District, Shaoxing City, Zhejiang Province</t>
         </is>
       </c>
       <c r="I146" t="inlineStr">
@@ -6407,7 +6407,7 @@
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>zhū bīn</t>
+          <t>朱斌 (zhū bīn)</t>
         </is>
       </c>
       <c r="E147" t="inlineStr">
@@ -6422,7 +6422,7 @@
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>A7 Building A7, Jia Chuang Zhi Gu Yuan Jing Industrial Park, Xincang Town, Pinghu City, Zhejiang Province</t>
+          <t>浙江省平湖市新仓镇嘉创智谷远景产业园 (zhè jiāng shěng píng hú shì xīn cāng zhèn jiā chuàng zhì gǔ yuǎn jǐng chǎn yè yuán)A7栋 (dòng)Building A7, Jia Chuang Zhi Gu Yuan Jing Industrial Park, Xincang Town, Pinghu City, Zhejiang Province</t>
         </is>
       </c>
       <c r="I147" t="inlineStr">
@@ -6447,7 +6447,7 @@
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>zhōu xiǎo juān</t>
+          <t>周晓娟 (zhōu xiǎo juān)</t>
         </is>
       </c>
       <c r="E148" t="inlineStr">
@@ -6462,7 +6462,7 @@
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>No. 8, Jiuniu Road, Hongze District, Huai'an City, Jiangsu Province, Postal Code 223100</t>
+          <t>江苏省淮安市洪泽区九牛路 (jiāng sū shěng huái ān shì hóng zé qū jiǔ niú lù)8号 (hào) 邮政编号 (yóu zhèng biān hào)223100No. 8, Jiuniu Road, Hongze District, Huai'an City, Jiangsu Province, Postal Code 223100</t>
         </is>
       </c>
       <c r="I148" t="inlineStr">
@@ -6487,7 +6487,7 @@
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>zhāng chéng</t>
+          <t>章程 (zhāng chéng)</t>
         </is>
       </c>
       <c r="E149" t="inlineStr">
@@ -6497,7 +6497,7 @@
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>No. 18, Huahui Road, Huashan Town, Huadu District, Guangzhou City, Guangdong Province</t>
+          <t>广东省广州市花都区花山镇华辉路 (guǎng dōng shěng guǎng zhōu shì huā dōu qū huā shān zhèn huá huī lù)18号 (hào) 微观化妆品创意产业园 (wēi guān huà zhuāng pǐn chuàng yì chǎn yè yuán)D栋整栋 (dòng zhěng dòng)、H栋整栋 (dòng zhěng dòng)Entire Building D and Entire Building H, Weiguan Cosmetics Creative Industrial Park, No. 18, Huahui Road, Huashan Town, Huadu District, Guangzhou City, Guangdong Province</t>
         </is>
       </c>
       <c r="I149" t="inlineStr">
@@ -6557,7 +6557,7 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>yóu wén cōng</t>
+          <t>游文聪 (yóu wén cōng)</t>
         </is>
       </c>
       <c r="E151" t="inlineStr">
@@ -6567,7 +6567,7 @@
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>No. 439, Xinxing Road, Taiping Town, Conghua District, Guangzhou</t>
+          <t>广州市从化区太平镇新兴路 (guǎng zhōu shì cóng huà qū tài píng zhèn xīn xīng lù)439号 (hào)7栋 (dòng)Building 7, No. 439, Xinxing Road, Taiping Town, Conghua District, Guangzhou</t>
         </is>
       </c>
       <c r="I151" t="inlineStr">
@@ -6592,7 +6592,7 @@
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>jiǎ jūn zhāo</t>
+          <t>贾均钊 (jiǎ jūn zhāo)</t>
         </is>
       </c>
       <c r="E152" t="inlineStr">
@@ -6612,7 +6612,7 @@
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>No. 10 Yitang Road, Jiangling Street, Wujiang District, Suzhou City</t>
+          <t>苏州市吴江区江陵街道益堂路 (sū zhōu shì wú jiāng qū jiāng líng jiē dào yì táng lù)10号 (hào)No. 10 Yitang Road, Jiangling Street, Wujiang District, Suzhou City</t>
         </is>
       </c>
       <c r="I152" t="inlineStr">
@@ -6637,7 +6637,7 @@
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>zhèng guó zhé</t>
+          <t>郑国哲 (zhèng guó zhé)</t>
         </is>
       </c>
       <c r="E153" t="inlineStr">
@@ -6652,7 +6652,7 @@
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>No. 888, Century Avenue, Longgang City, Zhejiang Province</t>
+          <t>浙江省龙港市世纪大道 (zhè jiāng shěng lóng gǎng shì shì jì dà dào)888号 (hào)No. 888, Century Avenue, Longgang City, Zhejiang Province</t>
         </is>
       </c>
       <c r="I153" t="inlineStr">
@@ -6677,7 +6677,7 @@
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>táng fēi líng</t>
+          <t>唐飞玲 (táng fēi líng)</t>
         </is>
       </c>
       <c r="E154" t="inlineStr">
@@ -6697,7 +6697,7 @@
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>No. 58 Taohong West Street, Shima Village, Junhe Street, Baiyun District, Guangzhou City</t>
+          <t>广州市白云区均禾街石马村桃红西街 (guǎng zhōu shì bái yún qū jūn hé jiē shí mǎ cūn táo hóng xī jiē)58号 (hào)No. 58 Taohong West Street, Shima Village, Junhe Street, Baiyun District, Guangzhou City</t>
         </is>
       </c>
       <c r="I154" t="inlineStr">
@@ -6732,7 +6732,7 @@
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>Beiying Road, QingPu, Shanghai 201700</t>
+          <t>188 Beiying Road, QingPu, Shanghai 201700</t>
         </is>
       </c>
       <c r="I155" t="inlineStr">

</xml_diff>

<commit_message>
Strip pinyin tone marks, keep Chinese characters in all Excel
</commit_message>
<xml_diff>
--- a/ipdf_suppliers.xlsx
+++ b/ipdf_suppliers.xlsx
@@ -532,7 +532,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>刘金铃 (liú jīn líng)</t>
+          <t>刘金铃 (liu jin ling)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -552,7 +552,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>江苏省吴江市 (jiāng sū shěng wú jiāng shì) 汾湖经济开发区临沪大道 (fén hú jīng jì kāi fā qū lín hù dà dào)1999号 (hào), 215211No. 1999, Linhu Avenue, Fenhu Economic Development Zone, Wujiang City, Jiangsu Province, 215211</t>
+          <t>江苏省吴江市 (jiang su sheng wu jiang shi) 汾湖经济开发区临沪大道 (fen hu jing ji kai fa qu lin hu da dao)1999号 (hao), 215211No. 1999, Linhu Avenue, Fenhu Economic Development Zone, Wujiang City, Jiangsu Province, 215211</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -617,7 +617,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>林显忠 (lín xiǎn zhōng)</t>
+          <t>林显忠 (lin xian zhong)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -637,7 +637,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>广州市白云区龙兴东南一横路 (guǎng zhōu shì bái yún qū lóng xīng dōng nán yī héng lù)3号 (hào)No. 3, Longxing Southeast First Horizontal Road, Baiyun District, Guangzhou City</t>
+          <t>广州市白云区龙兴东南一横路 (guang zhou shi bai yun qu long xing dong nan yi heng lu)3号 (hao)No. 3, Longxing Southeast First Horizontal Road, Baiyun District, Guangzhou City</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -652,7 +652,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>BOWEI博威 (bó wēi)</t>
+          <t>BOWEI博威 (bo wei)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -662,7 +662,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>宋茜 (sòng qiàn)</t>
+          <t>宋茜 (song qian)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -677,7 +677,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>广州市花都区花东镇定邦空港产业园 (guǎng zhōu shì huā dōu qū huā dōng zhèn dìng bāng kōng gǎng chǎn yè yuán)D栋 (dòng)Building D, Dingbang Airport Industrial Park, Huadong Town, Huadu District, Guangzhou</t>
+          <t>广州市花都区花东镇定邦空港产业园 (guang zhou shi hua dou qu hua dong zhen ding bang kong gang chan ye yuan)D栋 (dong)Building D, Dingbang Airport Industrial Park, Huadong Town, Huadu District, Guangzhou</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -722,7 +722,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>广东省开平市三埠街道新台路 (guǎng dōng shěng kāi píng shì sān bù jiē dào xīn tái lù)72号 (hào)No. 72, Xintai Road, Sanbu Street, Kaiping City, Guangdong Province</t>
+          <t>广东省开平市三埠街道新台路 (guang dong sheng kai ping shi san bu jie dao xin tai lu)72号 (hao)No. 72, Xintai Road, Sanbu Street, Kaiping City, Guangdong Province</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -747,7 +747,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>王耀峰 (wáng yào fēng)</t>
+          <t>王耀峰 (wang yao feng)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -777,7 +777,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>王媛媛 (wáng yuàn yuàn)</t>
+          <t>王媛媛 (wang yuan yuan)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -797,7 +797,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>工厂广东省江门市新山市和情共建路 (gōng chǎng guǎng dōng shěng jiāng mén shì xīn shān shì hé qíng gòng jiàn lù)305号座 (hào zuò) 公司地址 (gōng sī dì zhǐ):广州市白云区龙街尖路 (guǎng zhōu shì bái yún qū lóng jiē jiān lù)363号联边国际 (hào lián biān guó jì)620单元 (dān yuán)Factory: Building 305, Heqing Gongjian Road, Xinshan City, Jiangmen City, Guangdong Province. Company Address: Unit 620, Lianbian International, No. 363, Longjie Jian Road, Baiyun District, Guangzhou</t>
+          <t>工厂广东省江门市新山市和情共建路 (gong chang guang dong sheng jiang men shi xin shan shi he qing gong jian lu)305号座 (hao zuo) 公司地址 (gong si di zhi):广州市白云区龙街尖路 (guang zhou shi bai yun qu long jie jian lu)363号联边国际 (hao lian bian guo ji)620单元 (dan yuan)Factory: Building 305, Heqing Gongjian Road, Xinshan City, Jiangmen City, Guangdong Province. Company Address: Unit 620, Lianbian International, No. 363, Longjie Jian Road, Baiyun District, Guangzhou</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1087,7 +1087,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Bella 陈丽霞 (chén lì xiá)</t>
+          <t>Bella 陈丽霞 (chen li xia)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1117,7 +1117,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>陈孔清 (chén kǒng qīng)</t>
+          <t>陈孔清 (chen kong qing)</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1157,7 +1157,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>广东省广州市花都区秀全街道大布路 (guǎng dōng shěng guǎng zhōu shì huā dōu qū xiù quán jiē dào dà bù lù)29号峰华工业园 (hào fēng huá gōng yè yuán)Fenghua Industrial Park, No. 29 Dabu Road, Xiuquan Street, Huadu District, Guangzhou City, Guangdong Province</t>
+          <t>广东省广州市花都区秀全街道大布路 (guang dong sheng guang zhou shi hua dou qu xiu quan jie dao da bu lu)29号峰华工业园 (hao feng hua gong ye yuan)Fenghua Industrial Park, No. 29 Dabu Road, Xiuquan Street, Huadu District, Guangzhou City, Guangdong Province</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1182,7 +1182,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>胡明 (hú míng)</t>
+          <t>胡明 (hu ming)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1192,7 +1192,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>广东省清远英德市英红镇万洋众创城 (guǎng dōng shěng qīng yuǎn yīng dé shì yīng hóng zhèn wàn yáng zhòng chuàng chéng)D区 (qū)37栋 (dòng)Building 37, Zone D, Wanyang Maker Town, Yinghong Town, Yingde City, Qingyuan City, Guangdong Province</t>
+          <t>广东省清远英德市英红镇万洋众创城 (guang dong sheng qing yuan ying de shi ying hong zhen wan yang zhong chuang cheng)D区 (qu)37栋 (dong)Building 37, Zone D, Wanyang Maker Town, Yinghong Town, Yingde City, Qingyuan City, Guangdong Province</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1302,7 +1302,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>谭玉雄 (tán yù xióng)</t>
+          <t>谭玉雄 (tan yu xiong)</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1322,7 +1322,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>广东省东莞市谢岗镇曹乐向阳路 (guǎng dōng shěng dōng guǎn shì xiè gǎng zhèn cáo lè xiàng yáng lù)55号 (hào), 广东省东莞市樟木头镇塑料市场一期 (guǎng dōng shěng dōng guǎn shì zhāng mù tou zhèn sù liào shì chǎng yī qī)V栋 (dòng)1-2号 (hào), 广东省东莞市常平镇大京九塑料市场塑发东路 (guǎng dōng shěng dōng guǎn shì cháng píng zhèn dà jīng jiǔ sù liào shì chǎng sù fā dōng lù)53-54号 (hào)No. 55, Caole Xiangyang Road, Xiegang Town, Dongguan City, Guangdong Province, Building V, Units 1-2, Phase 1, Plastic Market, Zhangmutou Town, Dongguan City, Guangdong Province, No. 53-54, Sufa East Road, Dajingjiu Plastic Market, Changping Town, Dongguan City, Guangdong Province</t>
+          <t>广东省东莞市谢岗镇曹乐向阳路 (guang dong sheng dong guan shi xie gang zhen cao le xiang yang lu)55号 (hao), 广东省东莞市樟木头镇塑料市场一期 (guang dong sheng dong guan shi zhang mu tou zhen su liao shi chang yi qi)V栋 (dong)1-2号 (hao), 广东省东莞市常平镇大京九塑料市场塑发东路 (guang dong sheng dong guan shi chang ping zhen da jing jiu su liao shi chang su fa dong lu)53-54号 (hao)No. 55, Caole Xiangyang Road, Xiegang Town, Dongguan City, Guangdong Province, Building V, Units 1-2, Phase 1, Plastic Market, Zhangmutou Town, Dongguan City, Guangdong Province, No. 53-54, Sufa East Road, Dajingjiu Plastic Market, Changping Town, Dongguan City, Guangdong Province</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1457,7 +1457,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>陈总 (chén zǒng)</t>
+          <t>陈总 (chen zong)</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1467,7 +1467,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>广州市花都区先科一路金禾云创产业园 (guǎng zhōu shì huā dōu qū xiān kē yī lù jīn hé yún chuàng chǎn yè yuán)Jinhe Yun Chuang Industrial Park, Xianke 1st Road, Huadu District, Guangzhou City</t>
+          <t>广州市花都区先科一路金禾云创产业园 (guang zhou shi hua dou qu xian ke yi lu jin he yun chuang chan ye yuan)Jinhe Yun Chuang Industrial Park, Xianke 1st Road, Huadu District, Guangzhou City</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -1507,7 +1507,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>广州市越秀区先烈中路 (guǎng zhōu shì yuè xiù qū xiān liè zhōng lù)85号浙江大厦 (hào zhè jiāng dà shà)9楼 (lóu)9th Floor, Zhejiang Building, No. 85, Xianlie Middle Road, Yuexiu District, Guangzhou City</t>
+          <t>广州市越秀区先烈中路 (guang zhou shi yue xiu qu xian lie zhong lu)85号浙江大厦 (hao zhe jiang da sha)9楼 (lou)9th Floor, Zhejiang Building, No. 85, Xianlie Middle Road, Yuexiu District, Guangzhou City</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -1532,7 +1532,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>吴月芳 (wú yuè fāng)</t>
+          <t>吴月芳 (wu yue fang)</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1662,7 +1662,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>陈泳 (chén yǒng)</t>
+          <t>陈泳 (chen yong)</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1672,7 +1672,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>广州市白云区均禾街清湖村大山路 (guǎng zhōu shì bái yún qū jūn hé jiē qīng hú cūn dà shān lù)6号 (hào)No. 6, Dashan Road, Qinghu Village, Junhe Street, Baiyun District, Guangzhou City</t>
+          <t>广州市白云区均禾街清湖村大山路 (guang zhou shi bai yun qu jun he jie qing hu cun da shan lu)6号 (hao)No. 6, Dashan Road, Qinghu Village, Junhe Street, Baiyun District, Guangzhou City</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -1742,7 +1742,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>赖梓浩 (lài zǐ hào)</t>
+          <t>赖梓浩 (lai zi hao)</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1787,7 +1787,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>刘金连 (liú jīn lián)</t>
+          <t>刘金连 (liu jin lian)</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -1822,7 +1822,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>赵新亮 (zhào xīn liàng)</t>
+          <t>赵新亮 (zhao xin liang)</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1832,7 +1832,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>广州市白云区北村北大路 (guǎng zhōu shì bái yún qū běi cūn běi dà lù)22号四栋二楼 (hào sì dòng èr lóu)Second Floor, Building 4, No. 22, Beicun Beida Road, Baiyun District, Guangzhou City</t>
+          <t>广州市白云区北村北大路 (guang zhou shi bai yun qu bei cun bei da lu)22号四栋二楼 (hao si dong er lou)Second Floor, Building 4, No. 22, Beicun Beida Road, Baiyun District, Guangzhou City</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -2282,7 +2282,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>曹春 (cáo chūn)</t>
+          <t>曹春 (cao chun)</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -2292,7 +2292,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>广州市白云区石井街石井大道 (guǎng zhōu shì bái yún qū shí jǐng jiē shí jǐng dà dào)634号 (hào)No. 634, Shijing Avenue, Shijing Street, Baiyun District, Guangzhou City</t>
+          <t>广州市白云区石井街石井大道 (guang zhou shi bai yun qu shi jing jie shi jing da dao)634号 (hao)No. 634, Shijing Avenue, Shijing Street, Baiyun District, Guangzhou City</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -2337,7 +2337,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>上海市浦东新区世纪大道 (shàng hǎi shì pǔ dōng xīn qū shì jì dà dào)100号 (hào)No. 100, Century Avenue, Pudong New Area, Shanghai</t>
+          <t>上海市浦东新区世纪大道 (shang hai shi pu dong xin qu shi ji da dao)100号 (hao)No. 100, Century Avenue, Pudong New Area, Shanghai</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -2362,7 +2362,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>章海翰 (zhāng hǎi hàn)</t>
+          <t>章海翰 (zhang hai han)</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2507,7 +2507,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>上海市奉贤区大叶公路 (shàng hǎi shì fèng xián qū dà yè gōng lù) 6818号 (hào)5A栋 (dòng)502Room 502, Building 5A, No. 6818, Daye Highway, Fengxian District, Shanghai City</t>
+          <t>上海市奉贤区大叶公路 (shang hai shi feng xian qu da ye gong lu) 6818号 (hao)5A栋 (dong)502Room 502, Building 5A, No. 6818, Daye Highway, Fengxian District, Shanghai City</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -2532,7 +2532,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>陈雪萍 (chén xuě píng)</t>
+          <t>陈雪萍 (chen xue ping)</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -2552,7 +2552,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>广东省惠州市博罗县石湾镇马石围路 (guǎng dōng shěng huì zhōu shì bó luó xiàn shí wān zhèn mǎ shí wéi lù)3号 (hào)No. 3, Mashiwei Road, Shiwan Town, Boluo County, Huizhou City, Guangdong Province</t>
+          <t>广东省惠州市博罗县石湾镇马石围路 (guang dong sheng hui zhou shi bo luo xian shi wan zhen ma shi wei lu)3号 (hao)No. 3, Mashiwei Road, Shiwan Town, Boluo County, Huizhou City, Guangdong Province</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -2567,7 +2567,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>iGAO 丽高包装 (lì gāo bāo zhuāng)</t>
+          <t>iGAO 丽高包装 (li gao bao zhuang)</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2577,7 +2577,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>何丽银 (hé lì yín)</t>
+          <t>何丽银 (he li yin)</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -2597,7 +2597,7 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>广东省清远市清城区石角镇广清产业园广创街 (guǎng dōng shěng qīng yuǎn shì qīng chéng qū shí jiǎo zhèn guǎng qīng chǎn yè yuán guǎng chuàng jiē)6号 (hào)No. 6, Guangchuang Street, Guangqing Industrial Park, Shijiao Town, Qingcheng District, Qingyuan City, Guangdong Province</t>
+          <t>广东省清远市清城区石角镇广清产业园广创街 (guang dong sheng qing yuan shi qing cheng qu shi jiao zhen guang qing chan ye yuan guang chuang jie)6号 (hao)No. 6, Guangchuang Street, Guangqing Industrial Park, Shijiao Town, Qingcheng District, Qingyuan City, Guangdong Province</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -2622,7 +2622,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>冉露茜 (rǎn lù qiàn)</t>
+          <t>冉露茜 (ran lu qian)</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -2642,7 +2642,7 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>黄浦区德必上海书城 (huáng pǔ qū dé bì shàng hǎi shū chéng)WE2101室 (shì)Room WE2101, Debao Shanghai Book City, Huangpu District</t>
+          <t>黄浦区德必上海书城 (huang pu qu de bi shang hai shu cheng)WE2101室 (shi)Room WE2101, Debao Shanghai Book City, Huangpu District</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -2682,7 +2682,7 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>浙江省嘉兴市南湖区新丰镇新禾路 (zhè jiāng shěng jiā xīng shì nán hú qū xīn fēng zhèn xīn hé lù)158号 (hào)No. 158, Xinhe Road, Xinfeng Town, Nanhu District, Jiaxing City, Zhejiang Province</t>
+          <t>浙江省嘉兴市南湖区新丰镇新禾路 (zhe jiang sheng jia xing shi nan hu qu xin feng zhen xin he lu)158号 (hao)No. 158, Xinhe Road, Xinfeng Town, Nanhu District, Jiaxing City, Zhejiang Province</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -2792,7 +2792,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>陈铁文 (chén tiě wén)</t>
+          <t>陈铁文 (chen tie wen)</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -2807,7 +2807,7 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>福建省晋江市经济开发区 (fú jiàn shěng jìn jiāng shì jīng jì kāi fā qū) 广东省深圳市龙华新区建设路与东环二路交汇处聚豪国际 (guǎng dōng shěng shēn zhèn shì lóng huá xīn qū jiàn shè lù yǔ dōng huán èr lù jiāo huì chù jù háo guó jì)A栋 (dòng)2504室 (shì)Room 2504, Building A, Juhuao International, Intersection of Jianshe Road and Donghuan 2nd Road, Longhua New District, Shenzhen City, Guangdong Province; Jinjiang Economic Development Zone, Jinjiang City, Fujian Province</t>
+          <t>福建省晋江市经济开发区 (fu jian sheng jin jiang shi jing ji kai fa qu) 广东省深圳市龙华新区建设路与东环二路交汇处聚豪国际 (guang dong sheng shen zhen shi long hua xin qu jian she lu yu dong huan er lu jiao hui chu ju hao guo ji)A栋 (dong)2504室 (shi)Room 2504, Building A, Juhuao International, Intersection of Jianshe Road and Donghuan 2nd Road, Longhua New District, Shenzhen City, Guangdong Province; Jinjiang Economic Development Zone, Jinjiang City, Fujian Province</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -2877,7 +2877,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>周 (zhōu) 亮 (liàng)</t>
+          <t>周 (zhou) 亮 (liang)</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -3112,7 +3112,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>NATUTÈCH</t>
+          <t>NATUTECH</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -3137,7 +3137,7 @@
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>广州市天河区林和东路 (guǎng zhōu shì tiān hé qū lín hé dōng lù)285号中汇人寿 (hào zhōng huì rén shòu)901Room 901, Zhonghui Life Insurance, No. 285 Linhe East Road, Tianhe District, Guangzhou City</t>
+          <t>广州市天河区林和东路 (guang zhou shi tian he qu lin he dong lu)285号中汇人寿 (hao zhong hui ren shou)901Room 901, Zhonghui Life Insurance, No. 285 Linhe East Road, Tianhe District, Guangzhou City</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -3162,7 +3162,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>李金花 (lǐ jīn huā)</t>
+          <t>李金花 (li jin hua)</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -3227,7 +3227,7 @@
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>广州市白云区鶴拳路一横路科我园 (guǎng zhōu shì bái yún qū hè quán lù yī héng lù kē wǒ yuán)3栋 (dòng)Building 3, Kewoyuan, Yiheng Road, Hequan Road, Baiyun District, Guangzhou City</t>
+          <t>广州市白云区鶴拳路一横路科我园 (guang zhou shi bai yun qu he quan lu yi heng lu ke wo yuan)3栋 (dong)Building 3, Kewoyuan, Yiheng Road, Hequan Road, Baiyun District, Guangzhou City</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
@@ -3417,7 +3417,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Cécilia 叶思颖 (yè sī yǐng)</t>
+          <t>Cecilia 叶思颖 (ye si ying)</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -3542,7 +3542,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>洪碧虹 (hóng bì hóng)</t>
+          <t>洪碧虹 (hong bi hong)</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -3557,7 +3557,7 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>汕头市金平区岐山街道中宫社区建明工业城 (shàn tóu shì jīn píng qū qí shān jiē dào zhōng gōng shè qū jiàn míng gōng yè chéng)11-12栋楼 (dòng lóu)Buildings 11-12, Jianming Industrial City, Zhonggong Community, Qishan Street, Jinping District, Shantou City</t>
+          <t>汕头市金平区岐山街道中宫社区建明工业城 (shan tou shi jin ping qu qi shan jie dao zhong gong she qu jian ming gong ye cheng)11-12栋楼 (dong lou)Buildings 11-12, Jianming Industrial City, Zhonggong Community, Qishan Street, Jinping District, Shantou City</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
@@ -3802,7 +3802,7 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>何燕芳 (hé yàn fāng) Orla</t>
+          <t>何燕芳 (he yan fang) Orla</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -3842,7 +3842,7 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>陈乐 (chén lè)</t>
+          <t>陈乐 (chen le)</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -3862,7 +3862,7 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>广州市赛康尼机械设备有限公司 (guǎng zhōu shì sài kāng ní jī xiè shè bèi yǒu xiàn gōng sī) 广州市黄埔区南岗街道中南街 (guǎng zhōu shì huáng pǔ qū nán gǎng jiē dào zhōng nán jiē)10号联系中心办公室楼南面主楼南面 (hào lián xì zhōng xīn bàn gōng shì lóu nán miàn zhǔ lóu nán miàn)Guangzhou Saikenni Machinery Equipment Co., Ltd. South side of the main building, south side of the Contact Center Office Building, No. 10, Zhongnan Street, Nangang Subdistrict, Huangpu District, Guangzhou</t>
+          <t>广州市赛康尼机械设备有限公司 (guang zhou shi sai kang ni ji xie she bei you xian gong si) 广州市黄埔区南岗街道中南街 (guang zhou shi huang pu qu nan gang jie dao zhong nan jie)10号联系中心办公室楼南面主楼南面 (hao lian xi zhong xin ban gong shi lou nan mian zhu lou nan mian)Guangzhou Saikenni Machinery Equipment Co., Ltd. South side of the main building, south side of the Contact Center Office Building, No. 10, Zhongnan Street, Nangang Subdistrict, Huangpu District, Guangzhou</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
@@ -3887,7 +3887,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>鲍焕威 (bào huàn wēi) Bao huan wei</t>
+          <t>鲍焕威 (bao huan wei) Bao huan wei</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -3927,7 +3927,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>黄顺好 (huáng shùn hǎo)</t>
+          <t>黄顺好 (huang shun hao)</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
@@ -3947,7 +3947,7 @@
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>广东佛山市顺德区伦教来涌工业区 (guǎng dōng fó shān shì shùn dé qū lún jiào lái yǒng gōng yè qū)Laiyong Industrial Zone, Lunqiao, Shunde District, Foshan City, Guangdong</t>
+          <t>广东佛山市顺德区伦教来涌工业区 (guang dong fo shan shi shun de qu lun jiao lai yong gong ye qu)Laiyong Industrial Zone, Lunqiao, Shunde District, Foshan City, Guangdong</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
@@ -3972,7 +3972,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>邵仕华 (shào shì huá)</t>
+          <t>邵仕华 (shao shi hua)</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
@@ -4012,7 +4012,7 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>陈晓雯 (chén xiǎo wén)</t>
+          <t>陈晓雯 (chen xiao wen)</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
@@ -4027,7 +4027,7 @@
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>广东省清远市清城区石角镇 (guǎng dōng shěng qīng yuǎn shì qīng chéng qū shí jiǎo zhèn)(广清产业园 (guǎng qīng chǎn yè yuán))兴园路 (xīng yuán lù)3号 (hào); 广州市花都区新雅街绿地空港五号地 (guǎng zhōu shì huā dōu qū xīn yǎ jiē lǜ dì kōng gǎng wǔ hào dì)4栋 (dòng)1107室 (shì)No. 3, Xingyuan Road, Shijiao Town (Guangqing Industrial Park), Qingcheng District, Qingyuan City, Guangdong Province; Room 1107, Building 4, Plot 5, Greenland Airport, Xinya Street, Huadu District, Guangzhou City</t>
+          <t>广东省清远市清城区石角镇 (guang dong sheng qing yuan shi qing cheng qu shi jiao zhen)(广清产业园 (guang qing chan ye yuan))兴园路 (xing yuan lu)3号 (hao); 广州市花都区新雅街绿地空港五号地 (guang zhou shi hua dou qu xin ya jie lv di kong gang wu hao di)4栋 (dong)1107室 (shi)No. 3, Xingyuan Road, Shijiao Town (Guangqing Industrial Park), Qingcheng District, Qingyuan City, Guangdong Province; Room 1107, Building 4, Plot 5, Greenland Airport, Xinya Street, Huadu District, Guangzhou City</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
@@ -4087,7 +4087,7 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>徐春苗 (xú chūn miáo) Kavi</t>
+          <t>徐春苗 (xu chun miao) Kavi</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
@@ -4102,7 +4102,7 @@
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>浙江省嘉兴市南湖区新丰镇新禾路 (zhè jiāng shěng jiā xīng shì nán hú qū xīn fēng zhèn xīn hé lù)158号 (hào)No. 158, Xinhe Road, Xinfeng Town, Nanhu District, Jiaxing City, Zhejiang Province</t>
+          <t>浙江省嘉兴市南湖区新丰镇新禾路 (zhe jiang sheng jia xing shi nan hu qu xin feng zhen xin he lu)158号 (hao)No. 158, Xinhe Road, Xinfeng Town, Nanhu District, Jiaxing City, Zhejiang Province</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
@@ -4147,7 +4147,7 @@
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>江苏省泰兴市江平北路 (jiāng sū shěng tài xīng shì jiāng píng běi lù)55号 (hào), 上海市徐汇区石龙路 (shàng hǎi shì xú huì qū shí lóng lù)6号 (hào)001室 (shì)No. 55 Jiangping North Road, Taixing City, Jiangsu Province, Room 001, No. 6 Shilong Road, Xuhui District, Shanghai City</t>
+          <t>江苏省泰兴市江平北路 (jiang su sheng tai xing shi jiang ping bei lu)55号 (hao), 上海市徐汇区石龙路 (shang hai shi xu hui qu shi long lu)6号 (hao)001室 (shi)No. 55 Jiangping North Road, Taixing City, Jiangsu Province, Room 001, No. 6 Shilong Road, Xuhui District, Shanghai City</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
@@ -4257,7 +4257,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>翁铄桓 (wēng shuò huán)</t>
+          <t>翁铄桓 (weng shuo huan)</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
@@ -4272,7 +4272,7 @@
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>佛山市三水区乐平镇博裕路 (fó shān shì sān shuǐ qū lè píng zhèn bó yù lù)34号 (hào)1栋 (dòng)Building 1, No. 34, Boyu Road, Leping Town, Sanshui District, Foshan City</t>
+          <t>佛山市三水区乐平镇博裕路 (fo shan shi san shui qu le ping zhen bo yu lu)34号 (hao)1栋 (dong)Building 1, No. 34, Boyu Road, Leping Town, Sanshui District, Foshan City</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
@@ -4297,7 +4297,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>顾友阳 (gù yǒu yáng)</t>
+          <t>顾友阳 (gu you yang)</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -4312,7 +4312,7 @@
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>上海市金山区漕泾开发区展业路 (shàng hǎi shì jīn shān qū cáo jīng kāi fā qū zhǎn yè lù)288号一栋 (hào yī dòng)Building 1, No. 288, Zhanye Road, Caojing Development Zone, Jinshan District, Shanghai</t>
+          <t>上海市金山区漕泾开发区展业路 (shang hai shi jin shan qu cao jing kai fa qu zhan ye lu)288号一栋 (hao yi dong)Building 1, No. 288, Zhanye Road, Caojing Development Zone, Jinshan District, Shanghai</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
@@ -4457,7 +4457,7 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>林晓荣 (lín xiǎo róng)</t>
+          <t>林晓荣 (lin xiao rong)</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
@@ -4477,7 +4477,7 @@
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>广东省汕头市月浦龙洲路 (guǎng dōng shěng shàn tóu shì yuè pǔ lóng zhōu lù)12号 (hào) Longzhou Road, Yuepu, Shantou City, Guangdong Province, China</t>
+          <t>广东省汕头市月浦龙洲路 (guang dong sheng shan tou shi yue pu long zhou lu)12号 (hao) Longzhou Road, Yuepu, Shantou City, Guangdong Province, China</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
@@ -4502,7 +4502,7 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>谢榕宝 (xiè róng bǎo)</t>
+          <t>谢榕宝 (xie rong bao)</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
@@ -4522,7 +4522,7 @@
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>广州市七星二号 (guǎng zhōu shì qī xīng èr hào)No. 2, Qixing, Guangzhou City</t>
+          <t>广州市七星二号 (guang zhou shi qi xing er hao)No. 2, Qixing, Guangzhou City</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
@@ -4562,7 +4562,7 @@
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>上海市嘉定区树屏路 (shàng hǎi shì jiā dìng qū shù píng lù)588弄财智金岸 (nòng cái zhì jīn àn)35号楼 (hào lóu)Building 35, Caizhi Jin'an, Lane 588, Shuping Road, Jiading District, Shanghai</t>
+          <t>上海市嘉定区树屏路 (shang hai shi jia ding qu shu ping lu)588弄财智金岸 (nong cai zhi jin an)35号楼 (hao lou)Building 35, Caizhi Jin'an, Lane 588, Shuping Road, Jiading District, Shanghai</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -4717,7 +4717,7 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>苏元元 (sū yuán yuán)</t>
+          <t>苏元元 (su yuan yuan)</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
@@ -4737,7 +4737,7 @@
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>浙江省绍兴市上虞区崧厦街道振兴路 (zhè jiāng shěng shào xīng shì shàng yú qū sōng shà jiē dào zhèn xīng lù)138号 (hào)No. 138, Zhenxing Road, Songsha Street, Shangyu District, Shaoxing City, Zhejiang Province</t>
+          <t>浙江省绍兴市上虞区崧厦街道振兴路 (zhe jiang sheng shao xing shi shang yu qu song sha jie dao zhen xing lu)138号 (hao)No. 138, Zhenxing Road, Songsha Street, Shangyu District, Shaoxing City, Zhejiang Province</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
@@ -4762,7 +4762,7 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>刘艳霞 (liú yàn xiá)</t>
+          <t>刘艳霞 (liu yan xia)</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
@@ -4877,7 +4877,7 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>张亮亮 (zhāng liàng liàng)</t>
+          <t>张亮亮 (zhang liang liang)</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
@@ -4907,7 +4907,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>上海美涂化工科技有限公司 (shàng hǎi měi tú huà gōng kē jì yǒu xiàn gōng sī) Shanghai Meitu Chemical Technology Co., Ltd.</t>
+          <t>上海美涂化工科技有限公司 (shang hai mei tu hua gong ke ji you xian gong si) Shanghai Meitu Chemical Technology Co., Ltd.</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -4917,7 +4917,7 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>肖志坚 (xiào zhì jiān)</t>
+          <t>肖志坚 (xiao zhi jian)</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
@@ -4932,7 +4932,7 @@
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>上海市松江区叶路 (shàng hǎi shì sōng jiāng qū yè lù)133弄 (nòng)1-3号 (hào)No. 1-3, Lane 133, Ye Road, Songjiang District, Shanghai</t>
+          <t>上海市松江区叶路 (shang hai shi song jiang qu ye lu)133弄 (nong)1-3号 (hao)No. 1-3, Lane 133, Ye Road, Songjiang District, Shanghai</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
@@ -4947,7 +4947,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>东京品新材料科技有限公司 (dōng jīng pǐn xīn cái liào kē jì yǒu xiàn gōng sī) Tokyo Pin New Material Technology Co., Ltd.</t>
+          <t>东京品新材料科技有限公司 (dong jing pin xin cai liao ke ji you xian gong si) Tokyo Pin New Material Technology Co., Ltd.</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -4957,7 +4957,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>王馨苑 (wáng xīn yuàn)</t>
+          <t>王馨苑 (wang xin yuan)</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
@@ -4977,7 +4977,7 @@
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>广州市花都区花东镇微观产业园 (guǎng zhōu shì huā dōu qū huā dōng zhèn wēi guān chǎn yè yuán)C栋 (dòng)Building C, Weiguan Industrial Park, Huadong Town, Huadu District, Guangzhou</t>
+          <t>广州市花都区花东镇微观产业园 (guang zhou shi hua dou qu hua dong zhen wei guan chan ye yuan)C栋 (dong)Building C, Weiguan Industrial Park, Huadong Town, Huadu District, Guangzhou</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
@@ -4992,7 +4992,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>余姚市叠天包装有限公司 (yú yáo shì dié tiān bāo zhuāng yǒu xiàn gōng sī) YUYAO DIETIAN PACKAGING CO., LTD</t>
+          <t>余姚市叠天包装有限公司 (yu yao shi die tian bao zhuang you xian gong si) YUYAO DIETIAN PACKAGING CO., LTD</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -5002,7 +5002,7 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>王丽波 (wáng lì bō)</t>
+          <t>王丽波 (wang li bo)</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
@@ -5022,7 +5022,7 @@
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>浙江省余姚市牟山镇高车头 (zhè jiāng shěng yú yáo shì móu shān zhèn gāo chē tóu) B67号肖西路西 (hào xiào xī lù xī)West of Xiaoxi Road, Gaochetou, Mushan Town, Yuyao City, Zhejiang Province, No. B67</t>
+          <t>浙江省余姚市牟山镇高车头 (zhe jiang sheng yu yao shi mou shan zhen gao che tou) B67号肖西路西 (hao xiao xi lu xi)West of Xiaoxi Road, Gaochetou, Mushan Town, Yuyao City, Zhejiang Province, No. B67</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
@@ -5037,7 +5037,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>余姚市银河日用品有限公司 (yú yáo shì yín hé rì yòng pǐn yǒu xiàn gōng sī) YUYAO YINHE ARTICLES CO.,LTD.</t>
+          <t>余姚市银河日用品有限公司 (yu yao shi yin he ri yong pin you xian gong si) YUYAO YINHE ARTICLES CO.,LTD.</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -5047,7 +5047,7 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>刘锡蓉 (liú xī róng)</t>
+          <t>刘锡蓉 (liu xi rong)</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
@@ -5067,7 +5067,7 @@
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>浙江省余姚市马渚镇北兴路 (zhè jiāng shěng yú yáo shì mǎ zhǔ zhèn běi xīng lù)183号 (hào)No. 183, Beixing Road, Mazhu Town, Yuyao City, Zhejiang Province</t>
+          <t>浙江省余姚市马渚镇北兴路 (zhe jiang sheng yu yao shi ma zhu zhen bei xing lu)183号 (hao)No. 183, Beixing Road, Mazhu Town, Yuyao City, Zhejiang Province</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
@@ -5082,7 +5082,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>光正纸业有限公司 (guāng zhèng zhǐ yè yǒu xiàn gōng sī) Guangzheng Paper Co., Ltd.</t>
+          <t>光正纸业有限公司 (guang zheng zhi ye you xian gong si) Guangzheng Paper Co., Ltd.</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -5092,7 +5092,7 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>潘兴杰 (pān xīng jié)</t>
+          <t>潘兴杰 (pan xing jie)</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
@@ -5112,7 +5112,7 @@
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>廣東省東莞市厚街鎮東業路 (guǎng dōng shěng dōng guǎn shì hòu jiē zhèn dōng yè lù)2號 (hào)No. 2, Dongye Road, Houjie Town, Dongguan City, Guangdong Province</t>
+          <t>廣東省東莞市厚街鎮東業路 (guang dong sheng dong guan shi hou jie zhen dong ye lu)2號 (hao)No. 2, Dongye Road, Houjie Town, Dongguan City, Guangdong Province</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
@@ -5127,7 +5127,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>吾道包装 (wú dào bāo zhuāng) Wudao Packaging</t>
+          <t>吾道包装 (wu dao bao zhuang) Wudao Packaging</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -5137,7 +5137,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>胡珍华 (hú zhēn huá)</t>
+          <t>胡珍华 (hu zhen hua)</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
@@ -5152,7 +5152,7 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>广州市花都区绿港四街 (guǎng zhōu shì huā dōu qū lǜ gǎng sì jiē)6号 (hào)No. 6, Lvgong 4th Street, Huadu District, Guangzhou</t>
+          <t>广州市花都区绿港四街 (guang zhou shi hua dou qu lv gang si jie)6号 (hao)No. 6, Lvgong 4th Street, Huadu District, Guangzhou</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -5167,7 +5167,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>威美體造 (wēi měi tǐ zào) Weimei Body Manufacturing</t>
+          <t>威美體造 (wei mei ti zao) Weimei Body Manufacturing</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -5207,7 +5207,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>宇然膜丽 (yǔ rán mó lì)-YURANMOLI</t>
+          <t>宇然膜丽 (yu ran mo li)-YURANMOLI</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
@@ -5217,7 +5217,7 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>刘扬娥 (liú yáng é)</t>
+          <t>刘扬娥 (liu yang e)</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
@@ -5232,7 +5232,7 @@
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>广州市白云区江高镇神山神石路 (guǎng zhōu shì bái yún qū jiāng gāo zhèn shén shān shén shí lù)41号 (hào)No. 41, Shenshan Shishen Road, Jianggao Town, Baiyun District, Guangzhou</t>
+          <t>广州市白云区江高镇神山神石路 (guang zhou shi bai yun qu jiang gao zhen shen shan shen shi lu)41号 (hao)No. 41, Shenshan Shishen Road, Jianggao Town, Baiyun District, Guangzhou</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
@@ -5247,7 +5247,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>广东中源数字化技术有限公司 (guǎng dōng zhōng yuán shù zì huà jì shù yǒu xiàn gōng sī) Guangdong Zhongyuan Digital Technology Co., Ltd.</t>
+          <t>广东中源数字化技术有限公司 (guang dong zhong yuan shu zi hua ji shu you xian gong si) Guangdong Zhongyuan Digital Technology Co., Ltd.</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
@@ -5257,7 +5257,7 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>林帆 (lín fān)</t>
+          <t>林帆 (lin fan)</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
@@ -5277,7 +5277,7 @@
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>广东省广州市天河区科韵路 (guǎng dōng shěng guǎng zhōu shì tiān hé qū kē yùn lù)288号天盈创意园 (hào tiān yíng chuàng yì yuán) C区 (qū)3024-3027Rooms 3024-3027, Area C, Tianying Creative Park, No. 288 Keyun Road, Tianhe District, Guangzhou City, Guangdong Province</t>
+          <t>广东省广州市天河区科韵路 (guang dong sheng guang zhou shi tian he qu ke yun lu)288号天盈创意园 (hao tian ying chuang yi yuan) C区 (qu)3024-3027Rooms 3024-3027, Area C, Tianying Creative Park, No. 288 Keyun Road, Tianhe District, Guangzhou City, Guangdong Province</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
@@ -5292,7 +5292,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>广东全信医药科技有限公司 (guǎng dōng quán xìn yī yào kē jì yǒu xiàn gōng sī) Guangdong Quanxin Pharmaceutical Technology Co., Ltd.</t>
+          <t>广东全信医药科技有限公司 (guang dong quan xin yi yao ke ji you xian gong si) Guangdong Quanxin Pharmaceutical Technology Co., Ltd.</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -5302,7 +5302,7 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>刘丽红 (liú lì hóng) Valerie</t>
+          <t>刘丽红 (liu li hong) Valerie</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
@@ -5312,7 +5312,7 @@
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>广东省广州市花都区金田路 (guǎng dōng shěng guǎng zhōu shì huā dōu qū jīn tián lù)3号 (hào)No. 3, Jintian Road, Huadu District, Guangzhou City, Guangdong Province</t>
+          <t>广东省广州市花都区金田路 (guang dong sheng guang zhou shi hua dou qu jin tian lu)3号 (hao)No. 3, Jintian Road, Huadu District, Guangzhou City, Guangdong Province</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
@@ -5327,7 +5327,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>广东华轻质量检测服务中心有限公司 (guǎng dōng huá qīng zhì liàng jiǎn cè fú wù zhōng xīn yǒu xiàn gōng sī) Guangdong Huaqing Quality Inspection Service Center Co., Ltd.</t>
+          <t>广东华轻质量检测服务中心有限公司 (guang dong hua qing zhi liang jian ce fu wu zhong xin you xian gong si) Guangdong Huaqing Quality Inspection Service Center Co., Ltd.</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
@@ -5337,7 +5337,7 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>梁冠文 (liáng guān wén)</t>
+          <t>梁冠文 (liang guan wen)</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
@@ -5352,7 +5352,7 @@
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>广州市白云区北太路 (guǎng zhōu shì bái yún qū běi tài lù)1633号广州民营科技园科园路 (hào guǎng zhōu mín yíng kē jì yuán kē yuán lù)2号凯铂中心 (hào kǎi bó zhōng xīn)D区 (qū)1-4楼 (lóu) 1-4 F, Area D. Kaibo Center Building, No.2 Keyuan Road, Guangzhou Private Science and Technology Park, No. 1633 Beitai Road, Baiyun District, Guangzhou</t>
+          <t>广州市白云区北太路 (guang zhou shi bai yun qu bei tai lu)1633号广州民营科技园科园路 (hao guang zhou min ying ke ji yuan ke yuan lu)2号凯铂中心 (hao kai bo zhong xin)D区 (qu)1-4楼 (lou) 1-4 F, Area D. Kaibo Center Building, No.2 Keyuan Road, Guangzhou Private Science and Technology Park, No. 1633 Beitai Road, Baiyun District, Guangzhou</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
@@ -5367,7 +5367,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>广东吾道创展塑业有限公司 (guǎng dōng wú dào chuàng zhǎn sù yè yǒu xiàn gōng sī) Guangdong Wudao Chuangzhan Plastic Industry Co., Ltd.</t>
+          <t>广东吾道创展塑业有限公司 (guang dong wu dao chuang zhan su ye you xian gong si) Guangdong Wudao Chuangzhan Plastic Industry Co., Ltd.</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
@@ -5377,7 +5377,7 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>熊强 (xióng qiáng) Xiong Qiang</t>
+          <t>熊强 (xiong qiang) Xiong Qiang</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
@@ -5387,7 +5387,7 @@
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>广东省清远市佛冈县汤塘镇广佛产业园创业路 (guǎng dōng shěng qīng yuǎn shì fú gāng xiàn tāng táng zhèn guǎng fú chǎn yè yuán chuàng yè lù)7号 (hào) C区 (qū)6栋 (dòng)101-501房 (fáng)Room 101-501, Building 6, Zone C, No. 7, Chuangye Road, Guangfo Industrial Park, Tangtang Town, Fogang County, Qingyuan City, Guangdong Province</t>
+          <t>广东省清远市佛冈县汤塘镇广佛产业园创业路 (guang dong sheng qing yuan shi fu gang xian tang tang zhen guang fu chan ye yuan chuang ye lu)7号 (hao) C区 (qu)6栋 (dong)101-501房 (fang)Room 101-501, Building 6, Zone C, No. 7, Chuangye Road, Guangfo Industrial Park, Tangtang Town, Fogang County, Qingyuan City, Guangdong Province</t>
         </is>
       </c>
       <c r="I121" t="inlineStr">
@@ -5402,7 +5402,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>广东坚固包装制品有限公司 (guǎng dōng jiān gù bāo zhuāng zhì pǐn yǒu xiàn gōng sī) Guangdong Jiangu Packaging Co., Ltd</t>
+          <t>广东坚固包装制品有限公司 (guang dong jian gu bao zhuang zhi pin you xian gong si) Guangdong Jiangu Packaging Co., Ltd</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
@@ -5412,7 +5412,7 @@
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>李娟 (lǐ juān) LiJuan</t>
+          <t>李娟 (li juan) LiJuan</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
@@ -5432,7 +5432,7 @@
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>广州市白云区江高镇 (guǎng zhōu shì bái yún qū jiāng gāo zhèn)408号工业园 (hào gōng yè yuán) A区 (qū) 11/F Building 7 Awang Industrial Zone, Baiyun District, Guangzhou City</t>
+          <t>广州市白云区江高镇 (guang zhou shi bai yun qu jiang gao zhen)408号工业园 (hao gong ye yuan) A区 (qu) 11/F Building 7 Awang Industrial Zone, Baiyun District, Guangzhou City</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
@@ -5447,7 +5447,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>广东尼特包装制品有限公司 (guǎng dōng ní tè bāo zhuāng zhì pǐn yǒu xiàn gōng sī) Guangdong Nite Packaging Products Co., Ltd.</t>
+          <t>广东尼特包装制品有限公司 (guang dong ni te bao zhuang zhi pin you xian gong si) Guangdong Nite Packaging Products Co., Ltd.</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
@@ -5457,7 +5457,7 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>肖海青 (xiào hǎi qīng)</t>
+          <t>肖海青 (xiao hai qing)</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
@@ -5477,7 +5477,7 @@
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>中山工厂 (zhōng shān gōng chǎng):广东省中山市火炬开发区茂南路 (guǎng dōng shěng zhōng shān shì huǒ jù kāi fā qū mào nán lù)25号 (hào) 惠州工厂 (huì zhōu gōng chǎng):广东省惠州市龙门县金山工业园建设路 (guǎng dōng shěng huì zhōu shì lóng mén xiàn jīn shān gōng yè yuán jiàn shè lù)2号 (hào)Zhongshan Factory: No. 25, Maonan Road, Torch Development Zone, Zhongshan City, Guangdong Province; Huizhou Factory: No. 2, Jianshe Road, Jinshan Industrial Park, Longmen County, Huizhou City, Guangdong Province</t>
+          <t>中山工厂 (zhong shan gong chang):广东省中山市火炬开发区茂南路 (guang dong sheng zhong shan shi huo ju kai fa qu mao nan lu)25号 (hao) 惠州工厂 (hui zhou gong chang):广东省惠州市龙门县金山工业园建设路 (guang dong sheng hui zhou shi long men xian jin shan gong ye yuan jian she lu)2号 (hao)Zhongshan Factory: No. 25, Maonan Road, Torch Development Zone, Zhongshan City, Guangdong Province; Huizhou Factory: No. 2, Jianshe Road, Jinshan Industrial Park, Longmen County, Huizhou City, Guangdong Province</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
@@ -5492,7 +5492,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>广东琴叶健康日用品科技有限公司 (guǎng dōng qín yè jiàn kāng rì yòng pǐn kē jì yǒu xiàn gōng sī) Guangdong Qinyue Health Daily Necessities Technology Co., Ltd.</t>
+          <t>广东琴叶健康日用品科技有限公司 (guang dong qin ye jian kang ri yong pin ke ji you xian gong si) Guangdong Qinyue Health Daily Necessities Technology Co., Ltd.</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
@@ -5502,7 +5502,7 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>郭武杰 (guō wǔ jié)</t>
+          <t>郭武杰 (guo wu jie)</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
@@ -5517,7 +5517,7 @@
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>广州天河区广州大道中 (guǎng zhōu tiān hé qū guǎng zhōu dà dào zhōng)307号富力东山新天地中心 (hào fù lì dōng shān xīn tiān dì zhōng xīn)42楼 (lóu)(总部营销中心 (zǒng bù yíng xiāo zhōng xīn))42nd Floor (Headquarters Marketing Center), Fuli Dongshan Xintiandi Center, No. 307 Guangzhou Avenue Middle, Tianhe District, Guangzhou</t>
+          <t>广州天河区广州大道中 (guang zhou tian he qu guang zhou da dao zhong)307号富力东山新天地中心 (hao fu li dong shan xin tian di zhong xin)42楼 (lou)(总部营销中心 (zong bu ying xiao zhong xin))42nd Floor (Headquarters Marketing Center), Fuli Dongshan Xintiandi Center, No. 307 Guangzhou Avenue Middle, Tianhe District, Guangzhou</t>
         </is>
       </c>
       <c r="I124" t="inlineStr">
@@ -5532,7 +5532,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>广东腾宇集团有限责任公司 (guǎng dōng téng yǔ jí tuán yǒu xiàn zé rèn gōng sī) Guangdong Tengyu Group Co., Ltd.</t>
+          <t>广东腾宇集团有限责任公司 (guang dong teng yu ji tuan you xian ze ren gong si) Guangdong Tengyu Group Co., Ltd.</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
@@ -5542,7 +5542,7 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>陈花蕾 (chén huā lěi) Chen Hualel</t>
+          <t>陈花蕾 (chen hua lei) Chen Hualel</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
@@ -5562,7 +5562,7 @@
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>广州市白云区云城东路云理汇 (guǎng zhōu shì bái yún qū yún chéng dōng lù yún lǐ huì)2栋 (dòng)3楼 (lóu)3rd Floor, Building 2, Yunlihui, Yuncheng East Road, Baiyun District, Guangzhou</t>
+          <t>广州市白云区云城东路云理汇 (guang zhou shi bai yun qu yun cheng dong lu yun li hui)2栋 (dong)3楼 (lou)3rd Floor, Building 2, Yunlihui, Yuncheng East Road, Baiyun District, Guangzhou</t>
         </is>
       </c>
       <c r="I125" t="inlineStr">
@@ -5577,7 +5577,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>广州九圆塑业有限公司 (guǎng zhōu jiǔ yuán sù yè yǒu xiàn gōng sī) Guangzhou Jiuyuan Plastic Industry Co., Ltd.</t>
+          <t>广州九圆塑业有限公司 (guang zhou jiu yuan su ye you xian gong si) Guangzhou Jiuyuan Plastic Industry Co., Ltd.</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
@@ -5587,7 +5587,7 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>李小娜 (lǐ xiǎo nà)</t>
+          <t>李小娜 (li xiao na)</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
@@ -5602,7 +5602,7 @@
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>广州市从化区明珠工业园宝聚路二号 (guǎng zhōu shì cóng huà qū míng zhū gōng yè yuán bǎo jù lù èr hào)No. 2, Baoju Road, Mingzhu Industrial Park, Conghua District, Guangzhou City</t>
+          <t>广州市从化区明珠工业园宝聚路二号 (guang zhou shi cong hua qu ming zhu gong ye yuan bao ju lu er hao)No. 2, Baoju Road, Mingzhu Industrial Park, Conghua District, Guangzhou City</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
@@ -5617,7 +5617,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>广州宇然膜丽无纺制品有限公司 (guǎng zhōu yǔ rán mó lì wú fǎng zhì pǐn yǒu xiàn gōng sī) Guangzhou Yuran Moli Non-woven Products Co., Ltd.</t>
+          <t>广州宇然膜丽无纺制品有限公司 (guang zhou yu ran mo li wu fang zhi pin you xian gong si) Guangzhou Yuran Moli Non-woven Products Co., Ltd.</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -5627,7 +5627,7 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>彭练芝 (péng liàn zhī)</t>
+          <t>彭练芝 (peng lian zhi)</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
@@ -5642,7 +5642,7 @@
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>广州市白云区江高镇神山神石路 (guǎng zhōu shì bái yún qū jiāng gāo zhèn shén shān shén shí lù)41号 (hào)No. 41, Shenshan Shishen Road, Jianggao Town, Baiyun District, Guangzhou</t>
+          <t>广州市白云区江高镇神山神石路 (guang zhou shi bai yun qu jiang gao zhen shen shan shen shi lu)41号 (hao)No. 41, Shenshan Shishen Road, Jianggao Town, Baiyun District, Guangzhou</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
@@ -5657,7 +5657,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>广州市捷盛隆纸品贸易有限公司 (guǎng zhōu shì jié shèng lóng zhǐ pǐn mào yì yǒu xiàn gōng sī) Guangzhou Jieshenglong Paper Products Trading Co., Ltd.</t>
+          <t>广州市捷盛隆纸品贸易有限公司 (guang zhou shi jie sheng long zhi pin mao yi you xian gong si) Guangzhou Jieshenglong Paper Products Trading Co., Ltd.</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
@@ -5667,7 +5667,7 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>李文慧 (lǐ wén huì)</t>
+          <t>李文慧 (li wen hui)</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
@@ -5677,7 +5677,7 @@
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>广东省广州市花都区花东镇北兴北钟路 (guǎng dōng shěng guǎng zhōu shì huā dōu qū huā dōng zhèn běi xīng běi zhōng lù)54号 (hào)No. 54, Beixing Beizhong Road, Huadong Town, Huadu District, Guangzhou City, Guangdong Province</t>
+          <t>广东省广州市花都区花东镇北兴北钟路 (guang dong sheng guang zhou shi hua dou qu hua dong zhen bei xing bei zhong lu)54号 (hao)No. 54, Beixing Beizhong Road, Huadong Town, Huadu District, Guangzhou City, Guangdong Province</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
@@ -5692,7 +5692,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>广州市联惠科技有限公司 (guǎng zhōu shì lián huì kē jì yǒu xiàn gōng sī) Guangzhou Lianhui Technology Co., Ltd.</t>
+          <t>广州市联惠科技有限公司 (guang zhou shi lian hui ke ji you xian gong si) Guangzhou Lianhui Technology Co., Ltd.</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
@@ -5702,7 +5702,7 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>刘绍伟 (liú shào wěi)</t>
+          <t>刘绍伟 (liu shao wei)</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
@@ -5722,7 +5722,7 @@
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>佛山市三水区乐平镇博裕路 (fó shān shì sān shuǐ qū lè píng zhèn bó yù lù)34号 (hào)1栋 (dòng)Building 1, No. 34, Boyu Road, Leping Town, Sanshui District, Foshan City</t>
+          <t>佛山市三水区乐平镇博裕路 (fo shan shi san shui qu le ping zhen bo yu lu)34号 (hao)1栋 (dong)Building 1, No. 34, Boyu Road, Leping Town, Sanshui District, Foshan City</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
@@ -5737,7 +5737,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>广州市莱诺鸟智能科技有限公司 (guǎng zhōu shì lái nuò niǎo zhì néng kē jì yǒu xiàn gōng sī) Guangzhou Lainuoniao Intelligent Technology Co., Ltd.</t>
+          <t>广州市莱诺鸟智能科技有限公司 (guang zhou shi lai nuo niao zhi neng ke ji you xian gong si) Guangzhou Lainuoniao Intelligent Technology Co., Ltd.</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
@@ -5747,7 +5747,7 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>陈坤 (chén kūn)</t>
+          <t>陈坤 (chen kun)</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
@@ -5762,7 +5762,7 @@
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>广州市白云区云城西路娇兰佳人大厦 (guǎng zhōu shì bái yún qū yún chéng xī lù jiāo lán jiā rén dà shà)10楼 (lóu)10th Floor, Jiaolan Jiada Building, Yuncheng West Road, Baiyun District, Guangzhou City</t>
+          <t>广州市白云区云城西路娇兰佳人大厦 (guang zhou shi bai yun qu yun cheng xi lu jiao lan jia ren da sha)10楼 (lou)10th Floor, Jiaolan Jiada Building, Yuncheng West Road, Baiyun District, Guangzhou City</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
@@ -5777,7 +5777,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>广州市贤俊龙彩印有限公司 (guǎng zhōu shì xián jùn lóng cǎi yìn yǒu xiàn gōng sī) Guangzhou Xianjunlong Color Printing Co., Ltd.</t>
+          <t>广州市贤俊龙彩印有限公司 (guang zhou shi xian jun long cai yin you xian gong si) Guangzhou Xianjunlong Color Printing Co., Ltd.</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
@@ -5787,7 +5787,7 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>卿慧 (qīng huì)</t>
+          <t>卿慧 (qing hui)</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
@@ -5807,7 +5807,7 @@
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>广州市白云区三元里大道 (guǎng zhōu shì bái yún qū sān yuán lǐ dà dào)11号中港皮具城 (hào zhōng gǎng pí jù chéng)10楼 (lóu)1009室 (shì)Room 1009, 10th Floor, Zhonggang Leather City, No. 11, Sanyuanli Avenue, Baiyun District, Guangzhou City</t>
+          <t>广州市白云区三元里大道 (guang zhou shi bai yun qu san yuan li da dao)11号中港皮具城 (hao zhong gang pi ju cheng)10楼 (lou)1009室 (shi)Room 1009, 10th Floor, Zhonggang Leather City, No. 11, Sanyuanli Avenue, Baiyun District, Guangzhou City</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
@@ -5822,7 +5822,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>广州市鸿亿防伪产品有限公司 (guǎng zhōu shì hóng yì fáng wěi chǎn pǐn yǒu xiàn gōng sī) Guangzhou Hongyi Anti-counterfeiting Products Co., Ltd.</t>
+          <t>广州市鸿亿防伪产品有限公司 (guang zhou shi hong yi fang wei chan pin you xian gong si) Guangzhou Hongyi Anti-counterfeiting Products Co., Ltd.</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
@@ -5832,7 +5832,7 @@
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>邹永流 (zōu yǒng liú)</t>
+          <t>邹永流 (zou yong liu)</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
@@ -5847,7 +5847,7 @@
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>广州市越秀区先烈中路 (guǎng zhōu shì yuè xiù qū xiān liè zhōng lù)85号浙江大厦 (hào zhè jiāng dà shà)9楼 (lóu)9th Floor, Zhejiang Building, No. 85, Xianlie Middle Road, Yuexiu District, Guangzhou City</t>
+          <t>广州市越秀区先烈中路 (guang zhou shi yue xiu qu xian lie zhong lu)85号浙江大厦 (hao zhe jiang da sha)9楼 (lou)9th Floor, Zhejiang Building, No. 85, Xianlie Middle Road, Yuexiu District, Guangzhou City</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
@@ -5862,7 +5862,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>广州市鸿志包装材料有限公司 (guǎng zhōu shì hóng zhì bāo zhuāng cái liào yǒu xiàn gōng sī) HERO TUBE</t>
+          <t>广州市鸿志包装材料有限公司 (guang zhou shi hong zhi bao zhuang cai liao you xian gong si) HERO TUBE</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
@@ -5872,7 +5872,7 @@
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>罗文豪 (luó wén háo) Louis</t>
+          <t>罗文豪 (luo wen hao) Louis</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
@@ -5887,7 +5887,7 @@
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>广州市从化区横江路 (guǎng zhōu shì cóng huà qū héng jiāng lù)339号 (hào) -36号鸿志软管 (hào hóng zhì ruǎn guǎn)Hongzhi Hose, No. 339-36, Hengjiang Road, Conghua District, Guangzhou City</t>
+          <t>广州市从化区横江路 (guang zhou shi cong hua qu heng jiang lu)339号 (hao) -36号鸿志软管 (hao hong zhi ruan guan)Hongzhi Hose, No. 339-36, Hengjiang Road, Conghua District, Guangzhou City</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
@@ -5902,7 +5902,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>广州心合包装科技制造有限公司 (guǎng zhōu xīn hé bāo zhuāng kē jì zhì zào yǒu xiàn gōng sī) Guangzhou Xinhe Packaging Technology Manufacturing Co., Ltd.</t>
+          <t>广州心合包装科技制造有限公司 (guang zhou xin he bao zhuang ke ji zhi zao you xian gong si) Guangzhou Xinhe Packaging Technology Manufacturing Co., Ltd.</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
@@ -5927,7 +5927,7 @@
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>广州市白云区太和镇谢家注兰西路 (guǎng zhōu shì bái yún qū tài hé zhèn xiè jiā zhù lán xī lù)2号 (hào) No. 2 Yinian West Road, Xielazhuang, Taihe Town layun District, Duangzhou City</t>
+          <t>广州市白云区太和镇谢家注兰西路 (guang zhou shi bai yun qu tai he zhen xie jia zhu lan xi lu)2号 (hao) No. 2 Yinian West Road, Xielazhuang, Taihe Town layun District, Duangzhou City</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
@@ -5942,7 +5942,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>广州心合包装科技有限公司 (guǎng zhōu xīn hé bāo zhuāng kē jì yǒu xiàn gōng sī) Guangzhou Xinhe Packaging Technology Co., Ltd.</t>
+          <t>广州心合包装科技有限公司 (guang zhou xin he bao zhuang ke ji you xian gong si) Guangzhou Xinhe Packaging Technology Co., Ltd.</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
@@ -5952,7 +5952,7 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>于舒情 (yú shū qíng)</t>
+          <t>于舒情 (yu shu qing)</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
@@ -5962,7 +5962,7 @@
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>广州市白云区太和镇谢家庄荫兰西路 (guǎng zhōu shì bái yún qū tài hé zhèn xiè jiā zhuāng yīn lán xī lù)2号 (hào)No. 2, Yinlan West Road, Xiejiazhuang, Taihe Town, Baiyun District, Guangzhou City</t>
+          <t>广州市白云区太和镇谢家庄荫兰西路 (guang zhou shi bai yun qu tai he zhen xie jia zhuang yin lan xi lu)2号 (hao)No. 2, Yinlan West Road, Xiejiazhuang, Taihe Town, Baiyun District, Guangzhou City</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
@@ -5977,7 +5977,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>广州方和印刷有限公司 (guǎng zhōu fāng hé yìn shuā yǒu xiàn gōng sī) Guangzhou Fanghe Printing Co., Ltd.</t>
+          <t>广州方和印刷有限公司 (guang zhou fang he yin shua you xian gong si) Guangzhou Fanghe Printing Co., Ltd.</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
@@ -5987,7 +5987,7 @@
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>石小姐 (shí xiǎo jiě) SHI XIAOJIE</t>
+          <t>石小姐 (shi xiao jie) SHI XIAOJIE</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
@@ -6007,7 +6007,7 @@
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>广州市白云区龙归街南岭村岗埔大道 (guǎng zhōu shì bái yún qū lóng guī jiē nán lǐng cūn gǎng pǔ dà dào)1号 (hào)No. 1 Gangpu Avenue, Nanling Village, Longgui Street, Baiyun District, Guangzhou City</t>
+          <t>广州市白云区龙归街南岭村岗埔大道 (guang zhou shi bai yun qu long gui jie nan ling cun gang pu da dao)1号 (hao)No. 1 Gangpu Avenue, Nanling Village, Longgui Street, Baiyun District, Guangzhou City</t>
         </is>
       </c>
       <c r="I136" t="inlineStr">
@@ -6022,7 +6022,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>广州柯源塑料制品有限公司 (guǎng zhōu kē yuán sù liào zhì pǐn yǒu xiàn gōng sī) Guangzhou Keyuan Plasticware Co., Ltd.</t>
+          <t>广州柯源塑料制品有限公司 (guang zhou ke yuan su liao zhi pin you xian gong si) Guangzhou Keyuan Plasticware Co., Ltd.</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
@@ -6032,7 +6032,7 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>梁凯豪 (liáng kǎi háo)</t>
+          <t>梁凯豪 (liang kai hao)</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
@@ -6062,7 +6062,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>广州语辰化妆品包装有限公司 (guǎng zhōu yǔ chén huà zhuāng pǐn bāo zhuāng yǒu xiàn gōng sī) Guangzhou Yucheng Cosmetics Packaging Co., Ltd.</t>
+          <t>广州语辰化妆品包装有限公司 (guang zhou yu chen hua zhuang pin bao zhuang you xian gong si) Guangzhou Yucheng Cosmetics Packaging Co., Ltd.</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
@@ -6082,7 +6082,7 @@
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>广州市花都区凤凰南路 (guǎng zhōu shì huā dōu qū fèng huáng nán lù)61号卓美大楼北楼 (hào zhuó měi dà lóu běi lóu)307室 (shì)Room 307, North Building, Zhuomei Building, No. 61, Fenghuang South Road, Huadu District, Guangzhou</t>
+          <t>广州市花都区凤凰南路 (guang zhou shi hua dou qu feng huang nan lu)61号卓美大楼北楼 (hao zhuo mei da lou bei lou)307室 (shi)Room 307, North Building, Zhuomei Building, No. 61, Fenghuang South Road, Huadu District, Guangzhou</t>
         </is>
       </c>
       <c r="I138" t="inlineStr">
@@ -6097,7 +6097,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>廣州昌宏印務有限公司 (guǎng zhōu chāng hóng yìn wù yǒu xiàn gōng sī) Guangzhou Changhong Printing Co., Ltd.</t>
+          <t>廣州昌宏印務有限公司 (guang zhou chang hong yin wu you xian gong si) Guangzhou Changhong Printing Co., Ltd.</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
@@ -6107,7 +6107,7 @@
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>黎金昌 (lí jīn chāng)</t>
+          <t>黎金昌 (li jin chang)</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
@@ -6127,7 +6127,7 @@
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>廣州市白雲區龍歸街夏良東路 (guǎng zhōu shì bái yún qū lóng guī jiē xià liáng dōng lù)81號 (hào)102房 (fáng)Room 102, No. 81, Xialiang East Road, Longgui Street, Baiyun District, Guangzhou</t>
+          <t>廣州市白雲區龍歸街夏良東路 (guang zhou shi bai yun qu long gui jie xia liang dong lu)81號 (hao)102房 (fang)Room 102, No. 81, Xialiang East Road, Longgui Street, Baiyun District, Guangzhou</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
@@ -6142,7 +6142,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>廣州紅格智造包装有限公司 (guǎng zhōu hóng gé zhì zào bāo zhuāng yǒu xiàn gōng sī) Guangzhou Hongge Intelligent Manufacturing Packaging Co., Ltd.</t>
+          <t>廣州紅格智造包装有限公司 (guang zhou hong ge zhi zao bao zhuang you xian gong si) Guangzhou Hongge Intelligent Manufacturing Packaging Co., Ltd.</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
@@ -6167,7 +6167,7 @@
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>廣州市花都區花山鎮城西村自編 (guǎng zhōu shì huā dōu qū huā shān zhèn chéng xī cūn zì biān)3號 (hào)No. 3 (self-numbered), Chengxi Village, Huashan Town, Huadu District, Guangzhou City</t>
+          <t>廣州市花都區花山鎮城西村自編 (guang zhou shi hua dou qu hua shan zhen cheng xi cun zi bian)3號 (hao)No. 3 (self-numbered), Chengxi Village, Huashan Town, Huadu District, Guangzhou City</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
@@ -6182,12 +6182,12 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>护肤品 (hù fū pǐn)OEM/ODM</t>
+          <t>护肤品 (hu fu pin)OEM/ODM</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>祝依婷 (zhù yī tíng) Carrie</t>
+          <t>祝依婷 (zhu yi ting) Carrie</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
@@ -6197,7 +6197,7 @@
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>广东省广州市花都区金田路 (guǎng dōng shěng guǎng zhōu shì huā dōu qū jīn tián lù)3号 (hào)No. 3, Jintian Road, Huadu District, Guangzhou City, Guangdong Province</t>
+          <t>广东省广州市花都区金田路 (guang dong sheng guang zhou shi hua dou qu jin tian lu)3号 (hao)No. 3, Jintian Road, Huadu District, Guangzhou City, Guangdong Province</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
@@ -6212,7 +6212,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>正晟包装科技 (zhèng chéng bāo zhuāng kē jì)(广东 (guǎng dōng))有限公司 (yǒu xiàn gōng sī) Zhengsheng Packaging Technology (Guangdong) Co., Ltd.</t>
+          <t>正晟包装科技 (zheng cheng bao zhuang ke ji)(广东 (guang dong))有限公司 (you xian gong si) Zhengsheng Packaging Technology (Guangdong) Co., Ltd.</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
@@ -6222,7 +6222,7 @@
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>邓思艺 (dèng sī yì)</t>
+          <t>邓思艺 (deng si yi)</t>
         </is>
       </c>
       <c r="E142" t="inlineStr">
@@ -6237,7 +6237,7 @@
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>广东省清远市清城区石角镇 (guǎng dōng shěng qīng yuǎn shì qīng chéng qū shí jiǎo zhèn)(广清产业园 (guǎng qīng chǎn yè yuán))兴园路 (xīng yuán lù)3号 (hào); 广州市花都区新雅街绿地空港五号地 (guǎng zhōu shì huā dōu qū xīn yǎ jiē lǜ dì kōng gǎng wǔ hào dì)4栋 (dòng)1107室 (shì)No. 3, Xingyuan Road, Shijiao Town (Guangqing Industrial Park), Qingcheng District, Qingyuan City, Guangdong Province; Room 1107, Building 4, Plot 5, Greenland Airport, Xinya Street, Huadu District, Guangzhou City</t>
+          <t>广东省清远市清城区石角镇 (guang dong sheng qing yuan shi qing cheng qu shi jiao zhen)(广清产业园 (guang qing chan ye yuan))兴园路 (xing yuan lu)3号 (hao); 广州市花都区新雅街绿地空港五号地 (guang zhou shi hua dou qu xin ya jie lv di kong gang wu hao di)4栋 (dong)1107室 (shi)No. 3, Xingyuan Road, Shijiao Town (Guangqing Industrial Park), Qingcheng District, Qingyuan City, Guangdong Province; Room 1107, Building 4, Plot 5, Greenland Airport, Xinya Street, Huadu District, Guangzhou City</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
@@ -6252,7 +6252,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>汕头市艺被塑胶模具有限公司 (shàn tóu shì yì bèi sù jiāo mú jù yǒu xiàn gōng sī) Shantou Yibei Plastic Mold Co., Ltd.</t>
+          <t>汕头市艺被塑胶模具有限公司 (shan tou shi yi bei su jiao mu ju you xian gong si) Shantou Yibei Plastic Mold Co., Ltd.</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
@@ -6262,7 +6262,7 @@
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>江思蓉 (jiāng sī róng)</t>
+          <t>江思蓉 (jiang si rong)</t>
         </is>
       </c>
       <c r="E143" t="inlineStr">
@@ -6282,7 +6282,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>汕头市艺骏塑胶模具有限公司 (shàn tóu shì yì jùn sù jiāo mú jù yǒu xiàn gōng sī) Shantou Yijun Plastic Mold Co., Ltd.</t>
+          <t>汕头市艺骏塑胶模具有限公司 (shan tou shi yi jun su jiao mu ju you xian gong si) Shantou Yijun Plastic Mold Co., Ltd.</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
@@ -6292,7 +6292,7 @@
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>刘键均 (liú jiàn jūn)</t>
+          <t>刘键均 (liu jian jun)</t>
         </is>
       </c>
       <c r="E144" t="inlineStr">
@@ -6302,7 +6302,7 @@
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>广州市白云区云城西路 (guǎng zhōu shì bái yún qū yún chéng xī lù)888号绿地中心 (hào lǜ dì zhōng xīn)2403Room 2403, Greenland Center, No. 888 Yuncheng West Road, Baiyun District, Guangzhou City</t>
+          <t>广州市白云区云城西路 (guang zhou shi bai yun qu yun cheng xi lu)888号绿地中心 (hao lv di zhong xin)2403Room 2403, Greenland Center, No. 888 Yuncheng West Road, Baiyun District, Guangzhou City</t>
         </is>
       </c>
       <c r="I144" t="inlineStr">
@@ -6317,7 +6317,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>汕头市金平区彩鸿塑业有限公司 (shàn tóu shì jīn píng qū cǎi hóng sù yè yǒu xiàn gōng sī) Shantou Jinping District Caihong Plastic Industry Co., Ltd.</t>
+          <t>汕头市金平区彩鸿塑业有限公司 (shan tou shi jin ping qu cai hong su ye you xian gong si) Shantou Jinping District Caihong Plastic Industry Co., Ltd.</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
@@ -6327,7 +6327,7 @@
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>马壮茂 (mǎ zhuàng mào)</t>
+          <t>马壮茂 (ma zhuang mao)</t>
         </is>
       </c>
       <c r="E145" t="inlineStr">
@@ -6352,7 +6352,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>浙江永锦科技有限公司 (zhè jiāng yǒng jǐn kē jì yǒu xiàn gōng sī) Zhejiang Yongjin Technology Co., Ltd.</t>
+          <t>浙江永锦科技有限公司 (zhe jiang yong jin ke ji you xian gong si) Zhejiang Yongjin Technology Co., Ltd.</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
@@ -6362,7 +6362,7 @@
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>谢雅琪 (xiè yǎ qí)</t>
+          <t>谢雅琪 (xie ya qi)</t>
         </is>
       </c>
       <c r="E146" t="inlineStr">
@@ -6382,7 +6382,7 @@
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>浙江省绍兴市上虞区曹娥街道五星西路 (zhè jiāng shěng shào xīng shì shàng yú qū cáo é jiē dào wǔ xīng xī lù)1999号联东 (hào lián dōng)U谷 (gǔ)21栋 (dòng)C永 (yǒng), Add C tongin Bulding 21. Landong U Valley No. 1999, Wing West Road Cace Sheet, Shangyu District. Shocking City Zhellong ProvinceBuilding 21 C, Landong U Valley, No. 1999, Wuxing West Road, Cao'e Street, Shangyu District, Shaoxing City, Zhejiang Province</t>
+          <t>浙江省绍兴市上虞区曹娥街道五星西路 (zhe jiang sheng shao xing shi shang yu qu cao e jie dao wu xing xi lu)1999号联东 (hao lian dong)U谷 (gu)21栋 (dong)C永 (yong), Add C tongin Bulding 21. Landong U Valley No. 1999, Wing West Road Cace Sheet, Shangyu District. Shocking City Zhellong ProvinceBuilding 21 C, Landong U Valley, No. 1999, Wuxing West Road, Cao'e Street, Shangyu District, Shaoxing City, Zhejiang Province</t>
         </is>
       </c>
       <c r="I146" t="inlineStr">
@@ -6397,7 +6397,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>浙江赫宇包装科技有限公司 (zhè jiāng hè yǔ bāo zhuāng kē jì yǒu xiàn gōng sī) Zhejiang Heyu Packaging Technology Co., Ltd.</t>
+          <t>浙江赫宇包装科技有限公司 (zhe jiang he yu bao zhuang ke ji you xian gong si) Zhejiang Heyu Packaging Technology Co., Ltd.</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
@@ -6407,7 +6407,7 @@
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>朱斌 (zhū bīn)</t>
+          <t>朱斌 (zhu bin)</t>
         </is>
       </c>
       <c r="E147" t="inlineStr">
@@ -6422,7 +6422,7 @@
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>浙江省平湖市新仓镇嘉创智谷远景产业园 (zhè jiāng shěng píng hú shì xīn cāng zhèn jiā chuàng zhì gǔ yuǎn jǐng chǎn yè yuán)A7栋 (dòng)Building A7, Jia Chuang Zhi Gu Yuan Jing Industrial Park, Xincang Town, Pinghu City, Zhejiang Province</t>
+          <t>浙江省平湖市新仓镇嘉创智谷远景产业园 (zhe jiang sheng ping hu shi xin cang zhen jia chuang zhi gu yuan jing chan ye yuan)A7栋 (dong)Building A7, Jia Chuang Zhi Gu Yuan Jing Industrial Park, Xincang Town, Pinghu City, Zhejiang Province</t>
         </is>
       </c>
       <c r="I147" t="inlineStr">
@@ -6437,7 +6437,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>淮安市永希金属制品有限公司 (huái ān shì yǒng xī jīn shǔ zhì pǐn yǒu xiàn gōng sī) Huai'an Yongxi Metal Products Co., Ltd.</t>
+          <t>淮安市永希金属制品有限公司 (huai an shi yong xi jin shu zhi pin you xian gong si) Huai'an Yongxi Metal Products Co., Ltd.</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
@@ -6447,7 +6447,7 @@
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>周晓娟 (zhōu xiǎo juān)</t>
+          <t>周晓娟 (zhou xiao juan)</t>
         </is>
       </c>
       <c r="E148" t="inlineStr">
@@ -6462,7 +6462,7 @@
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>江苏省淮安市洪泽区九牛路 (jiāng sū shěng huái ān shì hóng zé qū jiǔ niú lù)8号 (hào) 邮政编号 (yóu zhèng biān hào)223100No. 8, Jiuniu Road, Hongze District, Huai'an City, Jiangsu Province, Postal Code 223100</t>
+          <t>江苏省淮安市洪泽区九牛路 (jiang su sheng huai an shi hong ze qu jiu niu lu)8号 (hao) 邮政编号 (you zheng bian hao)223100No. 8, Jiuniu Road, Hongze District, Huai'an City, Jiangsu Province, Postal Code 223100</t>
         </is>
       </c>
       <c r="I148" t="inlineStr">
@@ -6477,7 +6477,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>粤成印刷 (yuè chéng yìn shuā) YUE CHENG</t>
+          <t>粤成印刷 (yue cheng yin shua) YUE CHENG</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
@@ -6487,7 +6487,7 @@
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>章程 (zhāng chéng)</t>
+          <t>章程 (zhang cheng)</t>
         </is>
       </c>
       <c r="E149" t="inlineStr">
@@ -6497,7 +6497,7 @@
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>广东省广州市花都区花山镇华辉路 (guǎng dōng shěng guǎng zhōu shì huā dōu qū huā shān zhèn huá huī lù)18号 (hào) 微观化妆品创意产业园 (wēi guān huà zhuāng pǐn chuàng yì chǎn yè yuán)D栋整栋 (dòng zhěng dòng)、H栋整栋 (dòng zhěng dòng)Entire Building D and Entire Building H, Weiguan Cosmetics Creative Industrial Park, No. 18, Huahui Road, Huashan Town, Huadu District, Guangzhou City, Guangdong Province</t>
+          <t>广东省广州市花都区花山镇华辉路 (guang dong sheng guang zhou shi hua dou qu hua shan zhen hua hui lu)18号 (hao) 微观化妆品创意产业园 (wei guan hua zhuang pin chuang yi chan ye yuan)D栋整栋 (dong zheng dong)、H栋整栋 (dong zheng dong)Entire Building D and Entire Building H, Weiguan Cosmetics Creative Industrial Park, No. 18, Huahui Road, Huashan Town, Huadu District, Guangzhou City, Guangdong Province</t>
         </is>
       </c>
       <c r="I149" t="inlineStr">
@@ -6512,7 +6512,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>精业 (jīng yè) Jingye</t>
+          <t>精业 (jing ye) Jingye</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
@@ -6547,7 +6547,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>精展软管 (jīng zhǎn ruǎn guǎn) Jingzhan Hose</t>
+          <t>精展软管 (jing zhan ruan guan) Jingzhan Hose</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
@@ -6557,7 +6557,7 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>游文聪 (yóu wén cōng)</t>
+          <t>游文聪 (you wen cong)</t>
         </is>
       </c>
       <c r="E151" t="inlineStr">
@@ -6567,7 +6567,7 @@
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>广州市从化区太平镇新兴路 (guǎng zhōu shì cóng huà qū tài píng zhèn xīn xīng lù)439号 (hào)7栋 (dòng)Building 7, No. 439, Xinxing Road, Taiping Town, Conghua District, Guangzhou</t>
+          <t>广州市从化区太平镇新兴路 (guang zhou shi cong hua qu tai ping zhen xin xing lu)439号 (hao)7栋 (dong)Building 7, No. 439, Xinxing Road, Taiping Town, Conghua District, Guangzhou</t>
         </is>
       </c>
       <c r="I151" t="inlineStr">
@@ -6582,7 +6582,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>苏州海明包装科技有限公司 (sū zhōu hǎi míng bāo zhuāng kē jì yǒu xiàn gōng sī) Suzhou Haiming Packaging Technology Co., Ltd.</t>
+          <t>苏州海明包装科技有限公司 (su zhou hai ming bao zhuang ke ji you xian gong si) Suzhou Haiming Packaging Technology Co., Ltd.</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
@@ -6592,7 +6592,7 @@
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>贾均钊 (jiǎ jūn zhāo)</t>
+          <t>贾均钊 (jia jun zhao)</t>
         </is>
       </c>
       <c r="E152" t="inlineStr">
@@ -6612,7 +6612,7 @@
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>苏州市吴江区江陵街道益堂路 (sū zhōu shì wú jiāng qū jiāng líng jiē dào yì táng lù)10号 (hào)No. 10 Yitang Road, Jiangling Street, Wujiang District, Suzhou City</t>
+          <t>苏州市吴江区江陵街道益堂路 (su zhou shi wu jiang qu jiang ling jie dao yi tang lu)10号 (hao)No. 10 Yitang Road, Jiangling Street, Wujiang District, Suzhou City</t>
         </is>
       </c>
       <c r="I152" t="inlineStr">
@@ -6627,7 +6627,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>诚德科技股份有限公司 (chéng dé kē jì gǔ fèn yǒu xiàn gōng sī) Chengde Technology Co., Ltd.</t>
+          <t>诚德科技股份有限公司 (cheng de ke ji gu fen you xian gong si) Chengde Technology Co., Ltd.</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
@@ -6637,7 +6637,7 @@
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>郑国哲 (zhèng guó zhé)</t>
+          <t>郑国哲 (zheng guo zhe)</t>
         </is>
       </c>
       <c r="E153" t="inlineStr">
@@ -6652,7 +6652,7 @@
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>浙江省龙港市世纪大道 (zhè jiāng shěng lóng gǎng shì shì jì dà dào)888号 (hào)No. 888, Century Avenue, Longgang City, Zhejiang Province</t>
+          <t>浙江省龙港市世纪大道 (zhe jiang sheng long gang shi shi ji da dao)888号 (hao)No. 888, Century Avenue, Longgang City, Zhejiang Province</t>
         </is>
       </c>
       <c r="I153" t="inlineStr">
@@ -6667,7 +6667,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>银脉玻璃 (yín mài bō lí) YINMAIBOLI</t>
+          <t>银脉玻璃 (yin mai bo li) YINMAIBOLI</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
@@ -6677,7 +6677,7 @@
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>唐飞玲 (táng fēi líng)</t>
+          <t>唐飞玲 (tang fei ling)</t>
         </is>
       </c>
       <c r="E154" t="inlineStr">
@@ -6697,7 +6697,7 @@
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>广州市白云区均禾街石马村桃红西街 (guǎng zhōu shì bái yún qū jūn hé jiē shí mǎ cūn táo hóng xī jiē)58号 (hào)No. 58 Taohong West Street, Shima Village, Junhe Street, Baiyun District, Guangzhou City</t>
+          <t>广州市白云区均禾街石马村桃红西街 (guang zhou shi bai yun qu jun he jie shi ma cun tao hong xi jie)58号 (hao)No. 58 Taohong West Street, Shima Village, Junhe Street, Baiyun District, Guangzhou City</t>
         </is>
       </c>
       <c r="I154" t="inlineStr">

</xml_diff>